<commit_message>
Scraper de Sentenciados: busqueda incondicional (Natural: cedula+RUC derivado+nombre; Juridica: razon social+RUC, ambas siempre). Fix espera de loaderDiv antes del clic en Buscar (evitaba cierre inesperado del navegador)
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{478E3C43-5028-4AA3-B796-3BB4517629F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11978BAD-3976-4872-9F6B-204F5F872079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Revision" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Revision!$A$3:$GE$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Revision!$A$3:$GQ$5</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -284,7 +284,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FK3" authorId="1" shapeId="0" xr:uid="{4B658DD9-EA7C-4527-82E1-C9110A8EA055}">
+    <comment ref="FW3" authorId="1" shapeId="0" xr:uid="{4B658DD9-EA7C-4527-82E1-C9110A8EA055}">
       <text>
         <r>
           <rPr>
@@ -343,7 +343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="243">
   <si>
     <t>IDENTIFICACIÓN BÁSICA</t>
   </si>
@@ -884,9 +884,6 @@
     <t>Supercias</t>
   </si>
   <si>
-    <t>No cumple sus obligaciones, Actualización de Información General. Del sector societario</t>
-  </si>
-  <si>
     <t>SRI DEUDAS</t>
   </si>
   <si>
@@ -959,9 +956,6 @@
     <t>VILLACIS OLIVO ROMMEL JOERICK</t>
   </si>
   <si>
-    <t>Razon Social de Empresa</t>
-  </si>
-  <si>
     <t>Nombre Persona Natural / Juridica</t>
   </si>
   <si>
@@ -1001,7 +995,85 @@
     <t>afiliado seguro general tiempo completo</t>
   </si>
   <si>
-    <t>No existen registros de sentencias dentro del sistema sobre el usuario consultado.!, por favor de click en el botón VISUALIZAR para imprimir el acta.!</t>
+    <t>17230-2024-00186</t>
+  </si>
+  <si>
+    <t>FACTURAS O DOCUMENTOS ART. 356 NUM.2</t>
+  </si>
+  <si>
+    <t>09286-2026-03113</t>
+  </si>
+  <si>
+    <t>DERECHOS FUNDAMENTALES DEL CONSUMIDOR</t>
+  </si>
+  <si>
+    <t>09286-2026-01247</t>
+  </si>
+  <si>
+    <t>200 USURPACIÓN, INC.1</t>
+  </si>
+  <si>
+    <t>(RESUMEN AI)</t>
+  </si>
+  <si>
+    <t>09359-2026-00154</t>
+  </si>
+  <si>
+    <t>IMPUGNACIÓN DE VISTO BUENO</t>
+  </si>
+  <si>
+    <t>17371-2022-02501</t>
+  </si>
+  <si>
+    <t>INDEMNIZACIÓN POR DESPIDO INTEMPESTIVO</t>
+  </si>
+  <si>
+    <t>Razon Social (Empresa)</t>
+  </si>
+  <si>
+    <t>ALVAREZ HENRIQUES AQUILES DAVID</t>
+  </si>
+  <si>
+    <t>0911788289</t>
+  </si>
+  <si>
+    <t>Infracción Sentenciados</t>
+  </si>
+  <si>
+    <t>Fecha de Resolucion de Sentencia</t>
+  </si>
+  <si>
+    <t>No. Sentencias</t>
+  </si>
+  <si>
+    <t>No. Proceso</t>
+  </si>
+  <si>
+    <t>17U05202600018</t>
+  </si>
+  <si>
+    <t>09333202600398</t>
+  </si>
+  <si>
+    <t>02/04/2026</t>
+  </si>
+  <si>
+    <t>369 DELICUENCIA ORGANIZADA INC 3</t>
+  </si>
+  <si>
+    <t>282 INCUMPLIMIENTO DE DECISIONES LEGÍTIMAS DE AUTORIDAD COMPETENTE, INC.1</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>23281202303069</t>
+  </si>
+  <si>
+    <t>235 ENGAÑO AL COMPRADOR RESPECTO A LA IDENTIDAD O CALIDAD DE LAS COSAS O SERVICIOS VENDIDOS</t>
+  </si>
+  <si>
+    <t>SENTENCIADOS</t>
   </si>
 </sst>
 </file>
@@ -1011,8 +1083,8 @@
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_ &quot;$&quot;* #,##0.00_ ;_ &quot;$&quot;* \-#,##0.00_ ;_ &quot;$&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -1204,7 +1276,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -1615,12 +1687,73 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="120">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1755,6 +1888,9 @@
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1773,15 +1909,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1974,7 +2101,31 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2579,7 +2730,7 @@
         <v>115</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2736,7 +2887,7 @@
         <v>136</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -2850,54 +3001,60 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3838F483-03F0-4F1D-B50C-3B9C5206BD2F}">
-  <dimension ref="A1:GE6"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:GQ7"/>
+  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="70.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.5546875" style="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.5546875" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="31.21875" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.44140625" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="18.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="16.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.88671875" style="5" customWidth="1"/>
-    <col min="19" max="20" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="44.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="16.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.88671875" style="45" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="16.88671875" style="45" customWidth="1"/>
-    <col min="27" max="27" width="20.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.5546875" style="47" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.88671875" style="47" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.88671875" style="47" customWidth="1"/>
+    <col min="19" max="19" width="24" style="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="24.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="46.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="16.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="24.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.5546875" style="47" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.88671875" style="47" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.44140625" style="47" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="140" style="5" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="25.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="25.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="30" max="32" width="25.44140625" style="5" customWidth="1"/>
-    <col min="33" max="33" width="25.44140625" style="46" customWidth="1"/>
-    <col min="34" max="37" width="25.44140625" style="5" customWidth="1"/>
+    <col min="29" max="29" width="29.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="27.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="24.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14" style="45" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="24.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="29.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="19.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="23.21875" style="5" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="29" style="5" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="28.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="11.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="23.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="22.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="44" max="44" width="25.88671875" style="9" bestFit="1" customWidth="1"/>
-    <col min="45" max="46" width="30.6640625" style="5" bestFit="1" customWidth="1"/>
+    <col min="45" max="46" width="34.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="47" max="47" width="27.21875" style="5" bestFit="1" customWidth="1"/>
     <col min="48" max="48" width="26.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="49" max="49" width="10.77734375" style="4" bestFit="1" customWidth="1"/>
     <col min="50" max="50" width="11.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="51" max="51" width="23.21875" style="9" bestFit="1" customWidth="1"/>
     <col min="52" max="52" width="21" style="5" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="26.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="27.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="54" max="54" width="20.21875" style="5" bestFit="1" customWidth="1"/>
     <col min="55" max="55" width="30" style="9" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="27.21875" style="5" bestFit="1" customWidth="1"/>
@@ -2910,7 +3067,7 @@
     <col min="63" max="63" width="20.21875" style="5" bestFit="1" customWidth="1"/>
     <col min="64" max="64" width="30" style="9" bestFit="1" customWidth="1"/>
     <col min="65" max="65" width="27.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="25.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="26.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="67" max="67" width="10.77734375" style="4" bestFit="1" customWidth="1"/>
     <col min="68" max="68" width="11.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="23.21875" style="9" bestFit="1" customWidth="1"/>
@@ -2984,482 +3141,515 @@
     <col min="137" max="137" width="21.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="138" max="138" width="20.77734375" style="9" bestFit="1" customWidth="1"/>
     <col min="139" max="139" width="12.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="140" max="140" width="20.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="141" max="141" width="21.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="142" max="142" width="19.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="140" max="140" width="25.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="141" max="141" width="22.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="142" max="142" width="24.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="143" max="143" width="16.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="144" max="144" width="19.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="145" max="145" width="18.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="146" max="146" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="147" max="147" width="21.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="148" max="148" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="149" max="149" width="22.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="150" max="150" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="151" max="151" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="152" max="152" width="20.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="153" max="153" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="154" max="154" width="22.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="155" max="155" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="156" max="156" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="157" max="157" width="20.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="158" max="158" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="159" max="159" width="22.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="160" max="160" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="161" max="161" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="162" max="162" width="20.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="163" max="163" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="164" max="164" width="24.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="165" max="165" width="10.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="166" max="166" width="22.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="167" max="167" width="15.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="168" max="168" width="22.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="169" max="169" width="16.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="170" max="170" width="21.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="171" max="171" width="28.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="172" max="172" width="28.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="173" max="173" width="12.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="174" max="174" width="11.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="175" max="175" width="15.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="176" max="176" width="13.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="177" max="177" width="23.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="178" max="178" width="25.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="179" max="179" width="28.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="180" max="182" width="11.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="183" max="183" width="21.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="184" max="184" width="15" style="5" bestFit="1" customWidth="1"/>
-    <col min="185" max="185" width="17.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="186" max="186" width="6.88671875" style="11" bestFit="1" customWidth="1"/>
-    <col min="187" max="187" width="9.88671875" style="11" bestFit="1" customWidth="1"/>
-    <col min="188" max="16384" width="11.44140625" style="5"/>
+    <col min="145" max="145" width="19.109375" style="5" customWidth="1"/>
+    <col min="146" max="147" width="19.109375" style="4" customWidth="1"/>
+    <col min="148" max="148" width="19.109375" style="47" customWidth="1"/>
+    <col min="149" max="151" width="19.109375" style="4" customWidth="1"/>
+    <col min="152" max="152" width="19.109375" style="47" customWidth="1"/>
+    <col min="153" max="155" width="19.109375" style="4" customWidth="1"/>
+    <col min="156" max="156" width="19.109375" style="47" customWidth="1"/>
+    <col min="157" max="157" width="18.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="158" max="158" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="159" max="159" width="21.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="160" max="160" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="161" max="161" width="22.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="162" max="162" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="163" max="163" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="164" max="164" width="20.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="165" max="165" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="166" max="166" width="22.21875" style="47" bestFit="1" customWidth="1"/>
+    <col min="167" max="167" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="168" max="168" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="169" max="169" width="20.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="170" max="170" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="171" max="171" width="22.21875" style="47" bestFit="1" customWidth="1"/>
+    <col min="172" max="172" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="173" max="173" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="174" max="174" width="20.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="175" max="175" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="176" max="176" width="24.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="177" max="177" width="10.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="178" max="178" width="22.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="179" max="179" width="15.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="180" max="180" width="22.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="181" max="181" width="16.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="182" max="182" width="21.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="183" max="183" width="28.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="184" max="184" width="28.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="185" max="185" width="12.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="186" max="186" width="11.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="187" max="187" width="15.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="188" max="188" width="13.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="189" max="189" width="23.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="190" max="190" width="25.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="191" max="191" width="28.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="192" max="194" width="11.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="195" max="195" width="21.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="196" max="196" width="15" style="5" bestFit="1" customWidth="1"/>
+    <col min="197" max="197" width="17.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="198" max="198" width="6.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="199" max="199" width="9.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="200" max="16384" width="11.44140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:187" s="12" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="91" t="s">
+    <row r="1" spans="1:199" s="12" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="89" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
-      <c r="D1" s="92"/>
-      <c r="E1" s="92"/>
-      <c r="F1" s="92"/>
-      <c r="G1" s="92"/>
-      <c r="H1" s="92"/>
-      <c r="I1" s="92"/>
-      <c r="J1" s="92"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="93"/>
-      <c r="N1" s="88" t="s">
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="90"/>
+      <c r="J1" s="90"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="86" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="89"/>
-      <c r="P1" s="89"/>
-      <c r="Q1" s="89"/>
-      <c r="R1" s="89"/>
-      <c r="S1" s="89"/>
-      <c r="T1" s="89"/>
-      <c r="U1" s="89"/>
-      <c r="V1" s="89"/>
-      <c r="W1" s="89"/>
-      <c r="X1" s="89"/>
-      <c r="Y1" s="89"/>
-      <c r="Z1" s="89"/>
-      <c r="AA1" s="89"/>
-      <c r="AB1" s="89"/>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="113" t="s">
+      <c r="O1" s="87"/>
+      <c r="P1" s="87"/>
+      <c r="Q1" s="87"/>
+      <c r="R1" s="87"/>
+      <c r="S1" s="87"/>
+      <c r="T1" s="87"/>
+      <c r="U1" s="87"/>
+      <c r="V1" s="87"/>
+      <c r="W1" s="87"/>
+      <c r="X1" s="87"/>
+      <c r="Y1" s="87"/>
+      <c r="Z1" s="87"/>
+      <c r="AA1" s="87"/>
+      <c r="AB1" s="87"/>
+      <c r="AC1" s="88"/>
+      <c r="AD1" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="114"/>
-      <c r="AF1" s="114"/>
-      <c r="AG1" s="114"/>
-      <c r="AH1" s="114"/>
-      <c r="AI1" s="114"/>
-      <c r="AJ1" s="114"/>
-      <c r="AK1" s="115"/>
-      <c r="AL1" s="103" t="s">
+      <c r="AE1" s="112"/>
+      <c r="AF1" s="112"/>
+      <c r="AG1" s="112"/>
+      <c r="AH1" s="112"/>
+      <c r="AI1" s="112"/>
+      <c r="AJ1" s="112"/>
+      <c r="AK1" s="113"/>
+      <c r="AL1" s="101" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="104"/>
-      <c r="AN1" s="107" t="s">
+      <c r="AM1" s="102"/>
+      <c r="AN1" s="105" t="s">
         <v>2</v>
       </c>
-      <c r="AO1" s="108"/>
-      <c r="AP1" s="108"/>
-      <c r="AQ1" s="108"/>
-      <c r="AR1" s="109"/>
-      <c r="AS1" s="97" t="s">
+      <c r="AO1" s="106"/>
+      <c r="AP1" s="106"/>
+      <c r="AQ1" s="106"/>
+      <c r="AR1" s="107"/>
+      <c r="AS1" s="95" t="s">
         <v>4</v>
       </c>
-      <c r="AT1" s="99"/>
-      <c r="AU1" s="97" t="s">
+      <c r="AT1" s="97"/>
+      <c r="AU1" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="AV1" s="98"/>
-      <c r="AW1" s="98"/>
-      <c r="AX1" s="98"/>
-      <c r="AY1" s="98"/>
-      <c r="AZ1" s="98"/>
-      <c r="BA1" s="98"/>
-      <c r="BB1" s="98"/>
-      <c r="BC1" s="98"/>
-      <c r="BD1" s="98"/>
-      <c r="BE1" s="98"/>
-      <c r="BF1" s="98"/>
-      <c r="BG1" s="98"/>
-      <c r="BH1" s="98"/>
-      <c r="BI1" s="98"/>
-      <c r="BJ1" s="98"/>
-      <c r="BK1" s="98"/>
-      <c r="BL1" s="98"/>
-      <c r="BM1" s="98"/>
-      <c r="BN1" s="98"/>
-      <c r="BO1" s="98"/>
-      <c r="BP1" s="98"/>
-      <c r="BQ1" s="98"/>
-      <c r="BR1" s="98"/>
-      <c r="BS1" s="98"/>
-      <c r="BT1" s="98"/>
-      <c r="BU1" s="98"/>
-      <c r="BV1" s="98"/>
-      <c r="BW1" s="98"/>
-      <c r="BX1" s="98"/>
-      <c r="BY1" s="98"/>
-      <c r="BZ1" s="98"/>
-      <c r="CA1" s="98"/>
-      <c r="CB1" s="98"/>
-      <c r="CC1" s="98"/>
-      <c r="CD1" s="99"/>
-      <c r="CE1" s="67" t="s">
+      <c r="AV1" s="96"/>
+      <c r="AW1" s="96"/>
+      <c r="AX1" s="96"/>
+      <c r="AY1" s="96"/>
+      <c r="AZ1" s="96"/>
+      <c r="BA1" s="96"/>
+      <c r="BB1" s="96"/>
+      <c r="BC1" s="96"/>
+      <c r="BD1" s="96"/>
+      <c r="BE1" s="96"/>
+      <c r="BF1" s="96"/>
+      <c r="BG1" s="96"/>
+      <c r="BH1" s="96"/>
+      <c r="BI1" s="96"/>
+      <c r="BJ1" s="96"/>
+      <c r="BK1" s="96"/>
+      <c r="BL1" s="96"/>
+      <c r="BM1" s="96"/>
+      <c r="BN1" s="96"/>
+      <c r="BO1" s="96"/>
+      <c r="BP1" s="96"/>
+      <c r="BQ1" s="96"/>
+      <c r="BR1" s="96"/>
+      <c r="BS1" s="96"/>
+      <c r="BT1" s="96"/>
+      <c r="BU1" s="96"/>
+      <c r="BV1" s="96"/>
+      <c r="BW1" s="96"/>
+      <c r="BX1" s="96"/>
+      <c r="BY1" s="96"/>
+      <c r="BZ1" s="96"/>
+      <c r="CA1" s="96"/>
+      <c r="CB1" s="96"/>
+      <c r="CC1" s="96"/>
+      <c r="CD1" s="97"/>
+      <c r="CE1" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="CF1" s="68"/>
-      <c r="CG1" s="68"/>
-      <c r="CH1" s="68"/>
-      <c r="CI1" s="68"/>
-      <c r="CJ1" s="68"/>
-      <c r="CK1" s="68"/>
-      <c r="CL1" s="68"/>
-      <c r="CM1" s="68"/>
-      <c r="CN1" s="68"/>
-      <c r="CO1" s="68"/>
-      <c r="CP1" s="68"/>
-      <c r="CQ1" s="68"/>
-      <c r="CR1" s="68"/>
-      <c r="CS1" s="68"/>
-      <c r="CT1" s="68"/>
-      <c r="CU1" s="68"/>
-      <c r="CV1" s="68"/>
-      <c r="CW1" s="68"/>
-      <c r="CX1" s="68"/>
-      <c r="CY1" s="68"/>
-      <c r="CZ1" s="68"/>
-      <c r="DA1" s="68"/>
-      <c r="DB1" s="68"/>
-      <c r="DC1" s="68"/>
-      <c r="DD1" s="68"/>
-      <c r="DE1" s="68"/>
-      <c r="DF1" s="68"/>
-      <c r="DG1" s="68"/>
-      <c r="DH1" s="68"/>
-      <c r="DI1" s="68"/>
-      <c r="DJ1" s="68"/>
-      <c r="DK1" s="69"/>
-      <c r="DL1" s="73" t="s">
+      <c r="CF1" s="66"/>
+      <c r="CG1" s="66"/>
+      <c r="CH1" s="66"/>
+      <c r="CI1" s="66"/>
+      <c r="CJ1" s="66"/>
+      <c r="CK1" s="66"/>
+      <c r="CL1" s="66"/>
+      <c r="CM1" s="66"/>
+      <c r="CN1" s="66"/>
+      <c r="CO1" s="66"/>
+      <c r="CP1" s="66"/>
+      <c r="CQ1" s="66"/>
+      <c r="CR1" s="66"/>
+      <c r="CS1" s="66"/>
+      <c r="CT1" s="66"/>
+      <c r="CU1" s="66"/>
+      <c r="CV1" s="66"/>
+      <c r="CW1" s="66"/>
+      <c r="CX1" s="66"/>
+      <c r="CY1" s="66"/>
+      <c r="CZ1" s="66"/>
+      <c r="DA1" s="66"/>
+      <c r="DB1" s="66"/>
+      <c r="DC1" s="66"/>
+      <c r="DD1" s="66"/>
+      <c r="DE1" s="66"/>
+      <c r="DF1" s="66"/>
+      <c r="DG1" s="66"/>
+      <c r="DH1" s="66"/>
+      <c r="DI1" s="66"/>
+      <c r="DJ1" s="66"/>
+      <c r="DK1" s="67"/>
+      <c r="DL1" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="DM1" s="74"/>
-      <c r="DN1" s="74"/>
-      <c r="DO1" s="74"/>
-      <c r="DP1" s="74"/>
-      <c r="DQ1" s="74"/>
-      <c r="DR1" s="74"/>
-      <c r="DS1" s="74"/>
-      <c r="DT1" s="74"/>
-      <c r="DU1" s="74"/>
-      <c r="DV1" s="74"/>
-      <c r="DW1" s="74"/>
-      <c r="DX1" s="74"/>
-      <c r="DY1" s="74"/>
-      <c r="DZ1" s="75"/>
-      <c r="EA1" s="79" t="s">
+      <c r="DM1" s="72"/>
+      <c r="DN1" s="72"/>
+      <c r="DO1" s="72"/>
+      <c r="DP1" s="72"/>
+      <c r="DQ1" s="72"/>
+      <c r="DR1" s="72"/>
+      <c r="DS1" s="72"/>
+      <c r="DT1" s="72"/>
+      <c r="DU1" s="72"/>
+      <c r="DV1" s="72"/>
+      <c r="DW1" s="72"/>
+      <c r="DX1" s="72"/>
+      <c r="DY1" s="72"/>
+      <c r="DZ1" s="73"/>
+      <c r="EA1" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="EB1" s="80"/>
-      <c r="EC1" s="80"/>
-      <c r="ED1" s="80"/>
-      <c r="EE1" s="80"/>
-      <c r="EF1" s="80"/>
-      <c r="EG1" s="80"/>
-      <c r="EH1" s="80"/>
-      <c r="EI1" s="80"/>
-      <c r="EJ1" s="80"/>
-      <c r="EK1" s="80"/>
-      <c r="EL1" s="80"/>
-      <c r="EM1" s="80"/>
-      <c r="EN1" s="80"/>
-      <c r="EO1" s="80"/>
-      <c r="EP1" s="80"/>
-      <c r="EQ1" s="80"/>
-      <c r="ER1" s="80"/>
-      <c r="ES1" s="80"/>
-      <c r="ET1" s="80"/>
-      <c r="EU1" s="80"/>
-      <c r="EV1" s="80"/>
-      <c r="EW1" s="80"/>
-      <c r="EX1" s="80"/>
-      <c r="EY1" s="80"/>
-      <c r="EZ1" s="80"/>
-      <c r="FA1" s="80"/>
-      <c r="FB1" s="80"/>
-      <c r="FC1" s="80"/>
-      <c r="FD1" s="80"/>
-      <c r="FE1" s="80"/>
-      <c r="FF1" s="80"/>
-      <c r="FG1" s="80"/>
-      <c r="FH1" s="80"/>
-      <c r="FI1" s="80"/>
-      <c r="FJ1" s="80"/>
-      <c r="FK1" s="80"/>
-      <c r="FL1" s="80"/>
-      <c r="FM1" s="80"/>
-      <c r="FN1" s="80"/>
-      <c r="FO1" s="80"/>
-      <c r="FP1" s="80"/>
-      <c r="FQ1" s="80"/>
-      <c r="FR1" s="80"/>
-      <c r="FS1" s="80"/>
-      <c r="FT1" s="80"/>
-      <c r="FU1" s="80"/>
-      <c r="FV1" s="80"/>
-      <c r="FW1" s="81"/>
-      <c r="FX1" s="91" t="s">
+      <c r="EB1" s="78"/>
+      <c r="EC1" s="78"/>
+      <c r="ED1" s="78"/>
+      <c r="EE1" s="78"/>
+      <c r="EF1" s="78"/>
+      <c r="EG1" s="78"/>
+      <c r="EH1" s="78"/>
+      <c r="EI1" s="78"/>
+      <c r="EJ1" s="78"/>
+      <c r="EK1" s="78"/>
+      <c r="EL1" s="78"/>
+      <c r="EM1" s="78"/>
+      <c r="EN1" s="78"/>
+      <c r="EO1" s="78"/>
+      <c r="EP1" s="78"/>
+      <c r="EQ1" s="78"/>
+      <c r="ER1" s="78"/>
+      <c r="ES1" s="78"/>
+      <c r="ET1" s="78"/>
+      <c r="EU1" s="78"/>
+      <c r="EV1" s="78"/>
+      <c r="EW1" s="78"/>
+      <c r="EX1" s="78"/>
+      <c r="EY1" s="78"/>
+      <c r="EZ1" s="78"/>
+      <c r="FA1" s="78"/>
+      <c r="FB1" s="78"/>
+      <c r="FC1" s="78"/>
+      <c r="FD1" s="78"/>
+      <c r="FE1" s="78"/>
+      <c r="FF1" s="78"/>
+      <c r="FG1" s="78"/>
+      <c r="FH1" s="78"/>
+      <c r="FI1" s="78"/>
+      <c r="FJ1" s="78"/>
+      <c r="FK1" s="78"/>
+      <c r="FL1" s="78"/>
+      <c r="FM1" s="78"/>
+      <c r="FN1" s="78"/>
+      <c r="FO1" s="78"/>
+      <c r="FP1" s="78"/>
+      <c r="FQ1" s="78"/>
+      <c r="FR1" s="78"/>
+      <c r="FS1" s="78"/>
+      <c r="FT1" s="78"/>
+      <c r="FU1" s="78"/>
+      <c r="FV1" s="78"/>
+      <c r="FW1" s="78"/>
+      <c r="FX1" s="78"/>
+      <c r="FY1" s="78"/>
+      <c r="FZ1" s="78"/>
+      <c r="GA1" s="78"/>
+      <c r="GB1" s="78"/>
+      <c r="GC1" s="78"/>
+      <c r="GD1" s="78"/>
+      <c r="GE1" s="78"/>
+      <c r="GF1" s="78"/>
+      <c r="GG1" s="78"/>
+      <c r="GH1" s="78"/>
+      <c r="GI1" s="79"/>
+      <c r="GJ1" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="FY1" s="92"/>
-      <c r="FZ1" s="92"/>
-      <c r="GA1" s="93"/>
-      <c r="GB1" s="82" t="s">
+      <c r="GK1" s="90"/>
+      <c r="GL1" s="90"/>
+      <c r="GM1" s="91"/>
+      <c r="GN1" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="GC1" s="64" t="s">
+      <c r="GO1" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="GD1" s="47" t="s">
+      <c r="GP1" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="GE1" s="47" t="s">
+      <c r="GQ1" s="48" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:187" s="12" customFormat="1" ht="25.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="94"/>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
-      <c r="F2" s="95"/>
-      <c r="G2" s="95"/>
-      <c r="H2" s="95"/>
-      <c r="I2" s="95"/>
-      <c r="J2" s="95"/>
-      <c r="K2" s="95"/>
-      <c r="L2" s="95"/>
-      <c r="M2" s="96"/>
-      <c r="N2" s="50" t="s">
+    <row r="2" spans="1:199" s="12" customFormat="1" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="92"/>
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
+      <c r="I2" s="93"/>
+      <c r="J2" s="93"/>
+      <c r="K2" s="93"/>
+      <c r="L2" s="93"/>
+      <c r="M2" s="94"/>
+      <c r="N2" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="51"/>
-      <c r="P2" s="51"/>
-      <c r="Q2" s="51"/>
-      <c r="R2" s="51"/>
-      <c r="S2" s="51"/>
-      <c r="T2" s="51"/>
-      <c r="U2" s="51"/>
-      <c r="V2" s="85" t="s">
+      <c r="O2" s="52"/>
+      <c r="P2" s="52"/>
+      <c r="Q2" s="52"/>
+      <c r="R2" s="52"/>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+      <c r="U2" s="52"/>
+      <c r="V2" s="83" t="s">
         <v>15</v>
       </c>
-      <c r="W2" s="86"/>
-      <c r="X2" s="86"/>
-      <c r="Y2" s="86"/>
-      <c r="Z2" s="86"/>
-      <c r="AA2" s="86"/>
-      <c r="AB2" s="86"/>
-      <c r="AC2" s="87"/>
-      <c r="AD2" s="116"/>
-      <c r="AE2" s="117"/>
-      <c r="AF2" s="117"/>
-      <c r="AG2" s="117"/>
-      <c r="AH2" s="117"/>
-      <c r="AI2" s="117"/>
-      <c r="AJ2" s="117"/>
-      <c r="AK2" s="118"/>
-      <c r="AL2" s="105"/>
-      <c r="AM2" s="106"/>
-      <c r="AN2" s="110"/>
-      <c r="AO2" s="111"/>
-      <c r="AP2" s="111"/>
-      <c r="AQ2" s="111"/>
-      <c r="AR2" s="112"/>
-      <c r="AS2" s="100"/>
-      <c r="AT2" s="102"/>
-      <c r="AU2" s="100"/>
-      <c r="AV2" s="101"/>
-      <c r="AW2" s="101"/>
-      <c r="AX2" s="101"/>
-      <c r="AY2" s="101"/>
-      <c r="AZ2" s="101"/>
-      <c r="BA2" s="101"/>
-      <c r="BB2" s="101"/>
-      <c r="BC2" s="101"/>
-      <c r="BD2" s="101"/>
-      <c r="BE2" s="101"/>
-      <c r="BF2" s="101"/>
-      <c r="BG2" s="101"/>
-      <c r="BH2" s="101"/>
-      <c r="BI2" s="101"/>
-      <c r="BJ2" s="101"/>
-      <c r="BK2" s="101"/>
-      <c r="BL2" s="101"/>
-      <c r="BM2" s="101"/>
-      <c r="BN2" s="101"/>
-      <c r="BO2" s="101"/>
-      <c r="BP2" s="101"/>
-      <c r="BQ2" s="101"/>
-      <c r="BR2" s="101"/>
-      <c r="BS2" s="101"/>
-      <c r="BT2" s="101"/>
-      <c r="BU2" s="101"/>
-      <c r="BV2" s="101"/>
-      <c r="BW2" s="101"/>
-      <c r="BX2" s="101"/>
-      <c r="BY2" s="101"/>
-      <c r="BZ2" s="101"/>
-      <c r="CA2" s="101"/>
-      <c r="CB2" s="101"/>
-      <c r="CC2" s="101"/>
-      <c r="CD2" s="102"/>
-      <c r="CE2" s="70"/>
-      <c r="CF2" s="71"/>
-      <c r="CG2" s="71"/>
-      <c r="CH2" s="71"/>
-      <c r="CI2" s="71"/>
-      <c r="CJ2" s="71"/>
-      <c r="CK2" s="71"/>
-      <c r="CL2" s="71"/>
-      <c r="CM2" s="71"/>
-      <c r="CN2" s="71"/>
-      <c r="CO2" s="71"/>
-      <c r="CP2" s="71"/>
-      <c r="CQ2" s="71"/>
-      <c r="CR2" s="71"/>
-      <c r="CS2" s="71"/>
-      <c r="CT2" s="71"/>
-      <c r="CU2" s="71"/>
-      <c r="CV2" s="71"/>
-      <c r="CW2" s="71"/>
-      <c r="CX2" s="71"/>
-      <c r="CY2" s="71"/>
-      <c r="CZ2" s="71"/>
-      <c r="DA2" s="71"/>
-      <c r="DB2" s="71"/>
-      <c r="DC2" s="71"/>
-      <c r="DD2" s="71"/>
-      <c r="DE2" s="71"/>
-      <c r="DF2" s="71"/>
-      <c r="DG2" s="71"/>
-      <c r="DH2" s="71"/>
-      <c r="DI2" s="71"/>
-      <c r="DJ2" s="71"/>
-      <c r="DK2" s="72"/>
-      <c r="DL2" s="76"/>
-      <c r="DM2" s="77"/>
-      <c r="DN2" s="77"/>
-      <c r="DO2" s="77"/>
-      <c r="DP2" s="77"/>
-      <c r="DQ2" s="77"/>
-      <c r="DR2" s="77"/>
-      <c r="DS2" s="77"/>
-      <c r="DT2" s="77"/>
-      <c r="DU2" s="77"/>
-      <c r="DV2" s="77"/>
-      <c r="DW2" s="77"/>
-      <c r="DX2" s="77"/>
-      <c r="DY2" s="77"/>
-      <c r="DZ2" s="78"/>
-      <c r="EA2" s="52"/>
-      <c r="EB2" s="53"/>
-      <c r="EC2" s="53"/>
-      <c r="ED2" s="53"/>
-      <c r="EE2" s="53"/>
-      <c r="EF2" s="53"/>
-      <c r="EG2" s="53"/>
-      <c r="EH2" s="53"/>
-      <c r="EI2" s="53"/>
-      <c r="EJ2" s="53"/>
-      <c r="EK2" s="53"/>
-      <c r="EL2" s="53"/>
-      <c r="EM2" s="53"/>
-      <c r="EN2" s="53"/>
-      <c r="EO2" s="54"/>
-      <c r="EP2" s="55" t="s">
+      <c r="W2" s="84"/>
+      <c r="X2" s="84"/>
+      <c r="Y2" s="84"/>
+      <c r="Z2" s="84"/>
+      <c r="AA2" s="84"/>
+      <c r="AB2" s="84"/>
+      <c r="AC2" s="85"/>
+      <c r="AD2" s="114"/>
+      <c r="AE2" s="115"/>
+      <c r="AF2" s="115"/>
+      <c r="AG2" s="115"/>
+      <c r="AH2" s="115"/>
+      <c r="AI2" s="115"/>
+      <c r="AJ2" s="115"/>
+      <c r="AK2" s="116"/>
+      <c r="AL2" s="103"/>
+      <c r="AM2" s="104"/>
+      <c r="AN2" s="108"/>
+      <c r="AO2" s="109"/>
+      <c r="AP2" s="109"/>
+      <c r="AQ2" s="109"/>
+      <c r="AR2" s="110"/>
+      <c r="AS2" s="98"/>
+      <c r="AT2" s="100"/>
+      <c r="AU2" s="98"/>
+      <c r="AV2" s="99"/>
+      <c r="AW2" s="99"/>
+      <c r="AX2" s="99"/>
+      <c r="AY2" s="99"/>
+      <c r="AZ2" s="99"/>
+      <c r="BA2" s="99"/>
+      <c r="BB2" s="99"/>
+      <c r="BC2" s="99"/>
+      <c r="BD2" s="99"/>
+      <c r="BE2" s="99"/>
+      <c r="BF2" s="99"/>
+      <c r="BG2" s="99"/>
+      <c r="BH2" s="99"/>
+      <c r="BI2" s="99"/>
+      <c r="BJ2" s="99"/>
+      <c r="BK2" s="99"/>
+      <c r="BL2" s="99"/>
+      <c r="BM2" s="99"/>
+      <c r="BN2" s="99"/>
+      <c r="BO2" s="99"/>
+      <c r="BP2" s="99"/>
+      <c r="BQ2" s="99"/>
+      <c r="BR2" s="99"/>
+      <c r="BS2" s="99"/>
+      <c r="BT2" s="99"/>
+      <c r="BU2" s="99"/>
+      <c r="BV2" s="99"/>
+      <c r="BW2" s="99"/>
+      <c r="BX2" s="99"/>
+      <c r="BY2" s="99"/>
+      <c r="BZ2" s="99"/>
+      <c r="CA2" s="99"/>
+      <c r="CB2" s="99"/>
+      <c r="CC2" s="99"/>
+      <c r="CD2" s="100"/>
+      <c r="CE2" s="68"/>
+      <c r="CF2" s="69"/>
+      <c r="CG2" s="69"/>
+      <c r="CH2" s="69"/>
+      <c r="CI2" s="69"/>
+      <c r="CJ2" s="69"/>
+      <c r="CK2" s="69"/>
+      <c r="CL2" s="69"/>
+      <c r="CM2" s="69"/>
+      <c r="CN2" s="69"/>
+      <c r="CO2" s="69"/>
+      <c r="CP2" s="69"/>
+      <c r="CQ2" s="69"/>
+      <c r="CR2" s="69"/>
+      <c r="CS2" s="69"/>
+      <c r="CT2" s="69"/>
+      <c r="CU2" s="69"/>
+      <c r="CV2" s="69"/>
+      <c r="CW2" s="69"/>
+      <c r="CX2" s="69"/>
+      <c r="CY2" s="69"/>
+      <c r="CZ2" s="69"/>
+      <c r="DA2" s="69"/>
+      <c r="DB2" s="69"/>
+      <c r="DC2" s="69"/>
+      <c r="DD2" s="69"/>
+      <c r="DE2" s="69"/>
+      <c r="DF2" s="69"/>
+      <c r="DG2" s="69"/>
+      <c r="DH2" s="69"/>
+      <c r="DI2" s="69"/>
+      <c r="DJ2" s="69"/>
+      <c r="DK2" s="70"/>
+      <c r="DL2" s="74"/>
+      <c r="DM2" s="75"/>
+      <c r="DN2" s="75"/>
+      <c r="DO2" s="75"/>
+      <c r="DP2" s="75"/>
+      <c r="DQ2" s="75"/>
+      <c r="DR2" s="75"/>
+      <c r="DS2" s="75"/>
+      <c r="DT2" s="75"/>
+      <c r="DU2" s="75"/>
+      <c r="DV2" s="75"/>
+      <c r="DW2" s="75"/>
+      <c r="DX2" s="75"/>
+      <c r="DY2" s="75"/>
+      <c r="DZ2" s="76"/>
+      <c r="EA2" s="125"/>
+      <c r="EB2" s="117"/>
+      <c r="EC2" s="117"/>
+      <c r="ED2" s="117"/>
+      <c r="EE2" s="117"/>
+      <c r="EF2" s="117"/>
+      <c r="EG2" s="117"/>
+      <c r="EH2" s="117"/>
+      <c r="EI2" s="117"/>
+      <c r="EJ2" s="117"/>
+      <c r="EK2" s="117"/>
+      <c r="EL2" s="117"/>
+      <c r="EM2" s="117"/>
+      <c r="EN2" s="118"/>
+      <c r="EO2" s="122" t="s">
+        <v>242</v>
+      </c>
+      <c r="EP2" s="123"/>
+      <c r="EQ2" s="123"/>
+      <c r="ER2" s="123"/>
+      <c r="ES2" s="123"/>
+      <c r="ET2" s="123"/>
+      <c r="EU2" s="123"/>
+      <c r="EV2" s="123"/>
+      <c r="EW2" s="123"/>
+      <c r="EX2" s="123"/>
+      <c r="EY2" s="123"/>
+      <c r="EZ2" s="123"/>
+      <c r="FA2" s="124"/>
+      <c r="FB2" s="53" t="s">
         <v>16</v>
       </c>
-      <c r="EQ2" s="56"/>
-      <c r="ER2" s="56"/>
-      <c r="ES2" s="56"/>
-      <c r="ET2" s="56"/>
-      <c r="EU2" s="56"/>
-      <c r="EV2" s="56"/>
-      <c r="EW2" s="56"/>
-      <c r="EX2" s="56"/>
-      <c r="EY2" s="56"/>
-      <c r="EZ2" s="56"/>
-      <c r="FA2" s="56"/>
-      <c r="FB2" s="56"/>
-      <c r="FC2" s="56"/>
-      <c r="FD2" s="56"/>
-      <c r="FE2" s="56"/>
-      <c r="FF2" s="57"/>
-      <c r="FG2" s="58" t="s">
+      <c r="FC2" s="54"/>
+      <c r="FD2" s="54"/>
+      <c r="FE2" s="54"/>
+      <c r="FF2" s="54"/>
+      <c r="FG2" s="54"/>
+      <c r="FH2" s="54"/>
+      <c r="FI2" s="54"/>
+      <c r="FJ2" s="54"/>
+      <c r="FK2" s="54"/>
+      <c r="FL2" s="54"/>
+      <c r="FM2" s="54"/>
+      <c r="FN2" s="54"/>
+      <c r="FO2" s="54"/>
+      <c r="FP2" s="54"/>
+      <c r="FQ2" s="54"/>
+      <c r="FR2" s="55"/>
+      <c r="FS2" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="FH2" s="59"/>
-      <c r="FI2" s="59"/>
-      <c r="FJ2" s="59"/>
-      <c r="FK2" s="59"/>
-      <c r="FL2" s="59"/>
-      <c r="FM2" s="59"/>
-      <c r="FN2" s="59"/>
-      <c r="FO2" s="59"/>
-      <c r="FP2" s="60"/>
-      <c r="FQ2" s="61" t="s">
+      <c r="FT2" s="57"/>
+      <c r="FU2" s="57"/>
+      <c r="FV2" s="57"/>
+      <c r="FW2" s="57"/>
+      <c r="FX2" s="57"/>
+      <c r="FY2" s="57"/>
+      <c r="FZ2" s="57"/>
+      <c r="GA2" s="57"/>
+      <c r="GB2" s="58"/>
+      <c r="GC2" s="59" t="s">
         <v>18</v>
       </c>
-      <c r="FR2" s="62"/>
-      <c r="FS2" s="62"/>
-      <c r="FT2" s="62"/>
-      <c r="FU2" s="62"/>
-      <c r="FV2" s="62"/>
-      <c r="FW2" s="63"/>
-      <c r="FX2" s="94"/>
-      <c r="FY2" s="95"/>
-      <c r="FZ2" s="95"/>
-      <c r="GA2" s="96"/>
-      <c r="GB2" s="83"/>
-      <c r="GC2" s="65"/>
-      <c r="GD2" s="48"/>
-      <c r="GE2" s="48"/>
+      <c r="GD2" s="60"/>
+      <c r="GE2" s="60"/>
+      <c r="GF2" s="60"/>
+      <c r="GG2" s="60"/>
+      <c r="GH2" s="60"/>
+      <c r="GI2" s="61"/>
+      <c r="GJ2" s="92"/>
+      <c r="GK2" s="93"/>
+      <c r="GL2" s="93"/>
+      <c r="GM2" s="94"/>
+      <c r="GN2" s="81"/>
+      <c r="GO2" s="63"/>
+      <c r="GP2" s="49"/>
+      <c r="GQ2" s="49"/>
     </row>
-    <row r="3" spans="1:187" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:199" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>204</v>
+        <v>227</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>21</v>
@@ -3492,7 +3682,7 @@
         <v>30</v>
       </c>
       <c r="N3" s="39" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O3" s="22" t="s">
         <v>62</v>
@@ -3507,16 +3697,16 @@
         <v>64</v>
       </c>
       <c r="S3" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="T3" s="22" t="s">
         <v>187</v>
-      </c>
-      <c r="T3" s="22" t="s">
-        <v>188</v>
       </c>
       <c r="U3" s="22" t="s">
         <v>65</v>
       </c>
       <c r="V3" s="23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="W3" s="24" t="s">
         <v>62</v>
@@ -3528,28 +3718,28 @@
         <v>64</v>
       </c>
       <c r="Z3" s="24" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="AA3" s="24" t="s">
         <v>65</v>
       </c>
       <c r="AB3" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="AC3" s="40" t="s">
         <v>187</v>
       </c>
-      <c r="AC3" s="40" t="s">
-        <v>188</v>
-      </c>
       <c r="AD3" s="35" t="s">
+        <v>179</v>
+      </c>
+      <c r="AE3" s="17" t="s">
         <v>180</v>
-      </c>
-      <c r="AE3" s="17" t="s">
-        <v>181</v>
       </c>
       <c r="AF3" s="17" t="s">
         <v>36</v>
       </c>
       <c r="AG3" s="17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AH3" s="17" t="s">
         <v>37</v>
@@ -3558,7 +3748,7 @@
         <v>38</v>
       </c>
       <c r="AJ3" s="17" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="AK3" s="36" t="s">
         <v>39</v>
@@ -3884,129 +4074,165 @@
       <c r="EN3" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="EO3" s="30" t="s">
-        <v>79</v>
-      </c>
-      <c r="EP3" s="41" t="s">
+      <c r="EO3" s="119" t="s">
+        <v>232</v>
+      </c>
+      <c r="EP3" s="120" t="s">
+        <v>51</v>
+      </c>
+      <c r="EQ3" s="120" t="s">
+        <v>233</v>
+      </c>
+      <c r="ER3" s="120" t="s">
+        <v>231</v>
+      </c>
+      <c r="ES3" s="121" t="s">
+        <v>230</v>
+      </c>
+      <c r="ET3" s="120" t="s">
+        <v>51</v>
+      </c>
+      <c r="EU3" s="120" t="s">
+        <v>233</v>
+      </c>
+      <c r="EV3" s="120" t="s">
+        <v>231</v>
+      </c>
+      <c r="EW3" s="121" t="s">
+        <v>230</v>
+      </c>
+      <c r="EX3" s="120" t="s">
+        <v>51</v>
+      </c>
+      <c r="EY3" s="120" t="s">
+        <v>233</v>
+      </c>
+      <c r="EZ3" s="120" t="s">
+        <v>231</v>
+      </c>
+      <c r="FA3" s="121" t="s">
+        <v>230</v>
+      </c>
+      <c r="FB3" s="41" t="s">
         <v>80</v>
       </c>
-      <c r="EQ3" s="14" t="s">
+      <c r="FC3" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="ER3" s="14" t="s">
+      <c r="FD3" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="ES3" s="14" t="s">
+      <c r="FE3" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="ET3" s="15" t="s">
+      <c r="FF3" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="EU3" s="14" t="s">
+      <c r="FG3" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="EV3" s="14" t="s">
+      <c r="FH3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="EW3" s="14" t="s">
+      <c r="FI3" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="EX3" s="14" t="s">
+      <c r="FJ3" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="EY3" s="15" t="s">
+      <c r="FK3" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="EZ3" s="14" t="s">
+      <c r="FL3" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="FA3" s="14" t="s">
+      <c r="FM3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="FB3" s="14" t="s">
+      <c r="FN3" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="FC3" s="14" t="s">
+      <c r="FO3" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="FD3" s="15" t="s">
+      <c r="FP3" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="FE3" s="14" t="s">
+      <c r="FQ3" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="FF3" s="30" t="s">
+      <c r="FR3" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="FG3" s="35" t="s">
+      <c r="FS3" s="35" t="s">
         <v>52</v>
       </c>
-      <c r="FH3" s="17" t="s">
+      <c r="FT3" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="FI3" s="17" t="s">
+      <c r="FU3" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="FJ3" s="17" t="s">
+      <c r="FV3" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="FK3" s="17" t="s">
+      <c r="FW3" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="FL3" s="17" t="s">
+      <c r="FX3" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="FM3" s="17" t="s">
+      <c r="FY3" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="FN3" s="17" t="s">
+      <c r="FZ3" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="FO3" s="17" t="s">
+      <c r="GA3" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="FP3" s="36" t="s">
+      <c r="GB3" s="36" t="s">
         <v>93</v>
       </c>
-      <c r="FQ3" s="42" t="s">
+      <c r="GC3" s="42" t="s">
         <v>94</v>
       </c>
-      <c r="FR3" s="27" t="s">
+      <c r="GD3" s="27" t="s">
         <v>95</v>
       </c>
-      <c r="FS3" s="27" t="s">
+      <c r="GE3" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="FT3" s="27" t="s">
+      <c r="GF3" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="FU3" s="27" t="s">
+      <c r="GG3" s="27" t="s">
         <v>98</v>
       </c>
-      <c r="FV3" s="27" t="s">
+      <c r="GH3" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="FW3" s="43" t="s">
+      <c r="GI3" s="43" t="s">
         <v>100</v>
       </c>
-      <c r="FX3" s="41" t="s">
+      <c r="GJ3" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="FY3" s="14" t="s">
+      <c r="GK3" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="FZ3" s="14" t="s">
+      <c r="GL3" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="GA3" s="44" t="s">
+      <c r="GM3" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="GB3" s="84"/>
-      <c r="GC3" s="66"/>
-      <c r="GD3" s="49"/>
-      <c r="GE3" s="49"/>
+      <c r="GN3" s="82"/>
+      <c r="GO3" s="64"/>
+      <c r="GP3" s="50"/>
+      <c r="GQ3" s="50"/>
     </row>
-    <row r="4" spans="1:187" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>104</v>
       </c>
@@ -4037,20 +4263,20 @@
       <c r="O4" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="P4" s="7">
+      <c r="P4" s="47">
         <v>35626</v>
       </c>
-      <c r="Q4" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="R4" s="5" t="s">
+      <c r="Q4" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="R4" s="47" t="s">
         <v>103</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="U4" s="5" t="s">
         <v>174</v>
@@ -4061,13 +4287,13 @@
       <c r="W4" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="X4" s="45" t="s">
-        <v>103</v>
-      </c>
-      <c r="Y4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="Z4" s="45" t="s">
+      <c r="X4" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y4" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z4" s="47" t="s">
         <v>103</v>
       </c>
       <c r="AA4" s="4" t="s">
@@ -4080,32 +4306,32 @@
         <v>103</v>
       </c>
       <c r="AD4" s="5" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="AE4" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="AF4" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="AG4" s="45">
+        <v>2327.2600000000002</v>
+      </c>
+      <c r="AH4" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="AG4" s="46">
-        <v>2327.2600000000002</v>
-      </c>
-      <c r="AH4" s="5" t="s">
-        <v>208</v>
-      </c>
       <c r="AI4" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AJ4" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AK4" s="6"/>
       <c r="AL4" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="AM4" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="AN4" s="5" t="s">
         <v>103</v>
@@ -4119,136 +4345,318 @@
         <v>12683.75</v>
       </c>
       <c r="AS4" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="AT4" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="EA4" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="EP4" s="5" t="s">
-        <v>218</v>
+        <v>193</v>
+      </c>
+      <c r="EO4" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="EP4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EQ4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="ER4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="ES4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="ET4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EU4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EV4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EW4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EX4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EY4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EZ4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="FA4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="FB4" s="5">
+        <v>4</v>
+      </c>
+      <c r="FD4" s="5">
+        <v>1</v>
+      </c>
+      <c r="FE4" s="7">
+        <v>45300</v>
+      </c>
+      <c r="FF4" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="FG4" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="FH4" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="FI4" s="5">
+        <v>2</v>
+      </c>
+      <c r="FJ4" s="47">
+        <v>44851</v>
+      </c>
+      <c r="FK4" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="FL4" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="FM4" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="FN4" s="5">
+        <v>3</v>
+      </c>
+      <c r="FO4" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="FP4" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="FQ4" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FR4" s="5" t="s">
+        <v>222</v>
       </c>
     </row>
-    <row r="5" spans="1:187" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>106</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>107</v>
       </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G5" s="7">
         <v>26632</v>
       </c>
       <c r="H5" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>193</v>
-      </c>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
       <c r="N5" s="4" t="s">
         <v>107</v>
       </c>
       <c r="O5" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="P5" s="7">
+      <c r="P5" s="47">
         <v>26632</v>
       </c>
-      <c r="Q5" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="R5" s="5" t="s">
+      <c r="Q5" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="R5" s="47" t="s">
         <v>103</v>
       </c>
       <c r="S5" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="U5" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="T5" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="U5" s="5" t="s">
+      <c r="V5" s="4" t="s">
         <v>195</v>
-      </c>
-      <c r="V5" s="4" t="s">
-        <v>196</v>
       </c>
       <c r="W5" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="X5" s="45">
+      <c r="X5" s="47">
         <v>43067</v>
       </c>
-      <c r="Y5" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="Z5" s="45">
+      <c r="Y5" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z5" s="47">
         <v>43273</v>
       </c>
       <c r="AA5" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="AB5" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="AC5" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="AD5" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="AB5" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="AC5" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="AD5" s="5" t="s">
-        <v>200</v>
-      </c>
       <c r="AE5" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AF5" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AG5" s="46">
+      <c r="AG5" s="45">
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="AI5" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="AJ5" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="AK5" s="6"/>
+      <c r="AL5" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="AJ5" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="AL5" s="5" t="s">
-        <v>213</v>
-      </c>
       <c r="AM5" s="5" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="AN5" s="5" t="s">
-        <v>198</v>
-      </c>
+        <v>197</v>
+      </c>
+      <c r="AO5" s="6"/>
+      <c r="AP5" s="6"/>
       <c r="AQ5" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="AR5" s="9">
         <v>0</v>
       </c>
-      <c r="AS5" s="119"/>
-      <c r="AT5" s="119"/>
+      <c r="AS5" s="46"/>
+      <c r="AT5" s="46"/>
       <c r="EA5" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
+      </c>
+      <c r="EO5" s="5">
+        <v>1</v>
+      </c>
+      <c r="EP5" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="EQ5" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="ER5" s="47">
+        <v>46038</v>
+      </c>
+      <c r="ES5" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="ET5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EU5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EV5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EW5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EX5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EY5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EZ5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="FA5" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="FB5" s="5">
+        <v>107</v>
+      </c>
+      <c r="FD5" s="5">
+        <v>1</v>
+      </c>
+      <c r="FE5" s="7">
+        <v>46157</v>
+      </c>
+      <c r="FF5" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="FG5" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="FH5" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="FI5" s="5">
+        <v>2</v>
+      </c>
+      <c r="FJ5" s="47">
+        <v>46090</v>
+      </c>
+      <c r="FK5" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="FL5" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="FM5" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="FN5" s="5">
+        <v>3</v>
+      </c>
+      <c r="FO5" s="47">
+        <v>46051</v>
+      </c>
+      <c r="FP5" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="FQ5" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="FR5" s="5" t="s">
+        <v>222</v>
       </c>
     </row>
-    <row r="6" spans="1:187" ht="78" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>203</v>
-      </c>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="G6" s="7">
         <v>43543</v>
@@ -4259,29 +4667,33 @@
       <c r="I6" s="4" t="s">
         <v>103</v>
       </c>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
       <c r="N6" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="P6" s="7">
+      <c r="P6" s="47">
         <v>43543</v>
       </c>
-      <c r="Q6" s="7">
+      <c r="Q6" s="47">
         <v>44255</v>
       </c>
-      <c r="R6" s="7">
+      <c r="R6" s="47">
         <v>45426</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="V6" s="4" t="s">
         <v>103</v>
@@ -4289,13 +4701,13 @@
       <c r="W6" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="X6" s="45" t="s">
-        <v>103</v>
-      </c>
-      <c r="Y6" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="Z6" s="45" t="s">
+      <c r="X6" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y6" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z6" s="47" t="s">
         <v>103</v>
       </c>
       <c r="AA6" s="4" t="s">
@@ -4308,70 +4720,211 @@
         <v>103</v>
       </c>
       <c r="AD6" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="AE6" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="AE6" s="4" t="s">
-        <v>201</v>
-      </c>
       <c r="AF6" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AG6" s="46">
+      <c r="AG6" s="45">
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="AI6" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AJ6" s="5" t="s">
-        <v>194</v>
-      </c>
+        <v>193</v>
+      </c>
+      <c r="AK6" s="6"/>
       <c r="AL6" s="5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="AM6" s="5" t="s">
         <v>103</v>
       </c>
       <c r="AN6" s="5" t="s">
-        <v>179</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="AO6" s="6"/>
+      <c r="AP6" s="6"/>
       <c r="AQ6" s="5" t="s">
         <v>103</v>
       </c>
       <c r="AR6" s="9">
         <v>0</v>
       </c>
-      <c r="AS6" s="119"/>
-      <c r="AT6" s="119"/>
+      <c r="AS6" s="46"/>
+      <c r="AT6" s="46"/>
       <c r="EA6" s="5" t="s">
-        <v>194</v>
+        <v>193</v>
+      </c>
+      <c r="EO6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="EP6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EQ6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="ER6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="ES6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="ET6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EU6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EV6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EW6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EX6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EY6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="EZ6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="FA6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="FB6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FC6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FD6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FE6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FF6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FG6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FH6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FI6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FJ6" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="FK6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FL6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FM6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FN6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FO6" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="FP6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FQ6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="FR6" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="EO7" s="5">
+        <v>2</v>
+      </c>
+      <c r="EP7" s="4">
+        <v>1</v>
+      </c>
+      <c r="EQ7" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="ER7" s="47" t="s">
+        <v>236</v>
+      </c>
+      <c r="ES7" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="ET7" s="4">
+        <v>2</v>
+      </c>
+      <c r="EU7" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="EV7" s="47">
+        <v>46146</v>
+      </c>
+      <c r="EW7" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="EX7" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="EY7" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="EZ7" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="FA7" s="47" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:GE5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <mergeCells count="21">
+  <autoFilter ref="A3:GQ5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <mergeCells count="22">
+    <mergeCell ref="EO2:FA2"/>
+    <mergeCell ref="EA2:EN2"/>
     <mergeCell ref="AL1:AM2"/>
     <mergeCell ref="AN1:AR2"/>
     <mergeCell ref="AD1:AK2"/>
     <mergeCell ref="AS1:AT2"/>
     <mergeCell ref="A1:M2"/>
-    <mergeCell ref="GD1:GD3"/>
-    <mergeCell ref="GE1:GE3"/>
+    <mergeCell ref="GP1:GP3"/>
+    <mergeCell ref="GQ1:GQ3"/>
     <mergeCell ref="N2:U2"/>
-    <mergeCell ref="EA2:EO2"/>
-    <mergeCell ref="EP2:FF2"/>
-    <mergeCell ref="FG2:FP2"/>
-    <mergeCell ref="FQ2:FW2"/>
-    <mergeCell ref="GC1:GC3"/>
+    <mergeCell ref="FB2:FR2"/>
+    <mergeCell ref="FS2:GB2"/>
+    <mergeCell ref="GC2:GI2"/>
+    <mergeCell ref="GO1:GO3"/>
     <mergeCell ref="CE1:DK2"/>
     <mergeCell ref="DL1:DZ2"/>
-    <mergeCell ref="EA1:FW1"/>
-    <mergeCell ref="GB1:GB3"/>
+    <mergeCell ref="EA1:GI1"/>
+    <mergeCell ref="GN1:GN3"/>
     <mergeCell ref="V2:AC2"/>
     <mergeCell ref="N1:AC1"/>
-    <mergeCell ref="FX1:GA2"/>
+    <mergeCell ref="GJ1:GM2"/>
     <mergeCell ref="AU1:CD2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A7:B1048576 A3:A6">

</xml_diff>

<commit_message>
Cadena de representante legal completa: clasificacion por tercer digito del RUC (persona natural termina cadena, empresa/entidad publica continua), consulta SRI de la persona final encontrada, deteccion de ciclos, limite de 3 niveles - confirmado con INDUAUTO (nivel 1, sin bloqueo)
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11978BAD-3976-4872-9F6B-204F5F872079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC661B8E-97DA-4116-A4CA-0CFD3E47009D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametrizacion" sheetId="3" r:id="rId1"/>
@@ -1894,6 +1894,111 @@
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2017,115 +2122,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3030,7 +3030,7 @@
     <col min="24" max="24" width="20.5546875" style="47" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="16.88671875" style="47" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="19.44140625" style="47" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="140" style="5" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="51.33203125" style="5" customWidth="1"/>
     <col min="28" max="28" width="25.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="29.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="30" max="31" width="27.5546875" style="5" bestFit="1" customWidth="1"/>
@@ -3198,448 +3198,448 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:199" s="12" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="77" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="90"/>
-      <c r="J1" s="90"/>
-      <c r="K1" s="90"/>
-      <c r="L1" s="90"/>
-      <c r="M1" s="91"/>
-      <c r="N1" s="86" t="s">
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="79"/>
+      <c r="N1" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="87"/>
-      <c r="P1" s="87"/>
-      <c r="Q1" s="87"/>
-      <c r="R1" s="87"/>
-      <c r="S1" s="87"/>
-      <c r="T1" s="87"/>
-      <c r="U1" s="87"/>
-      <c r="V1" s="87"/>
-      <c r="W1" s="87"/>
-      <c r="X1" s="87"/>
-      <c r="Y1" s="87"/>
-      <c r="Z1" s="87"/>
-      <c r="AA1" s="87"/>
-      <c r="AB1" s="87"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="111" t="s">
+      <c r="O1" s="122"/>
+      <c r="P1" s="122"/>
+      <c r="Q1" s="122"/>
+      <c r="R1" s="122"/>
+      <c r="S1" s="122"/>
+      <c r="T1" s="122"/>
+      <c r="U1" s="122"/>
+      <c r="V1" s="122"/>
+      <c r="W1" s="122"/>
+      <c r="X1" s="122"/>
+      <c r="Y1" s="122"/>
+      <c r="Z1" s="122"/>
+      <c r="AA1" s="122"/>
+      <c r="AB1" s="122"/>
+      <c r="AC1" s="123"/>
+      <c r="AD1" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="112"/>
-      <c r="AF1" s="112"/>
-      <c r="AG1" s="112"/>
-      <c r="AH1" s="112"/>
-      <c r="AI1" s="112"/>
-      <c r="AJ1" s="112"/>
-      <c r="AK1" s="113"/>
-      <c r="AL1" s="101" t="s">
+      <c r="AE1" s="68"/>
+      <c r="AF1" s="68"/>
+      <c r="AG1" s="68"/>
+      <c r="AH1" s="68"/>
+      <c r="AI1" s="68"/>
+      <c r="AJ1" s="68"/>
+      <c r="AK1" s="69"/>
+      <c r="AL1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="102"/>
-      <c r="AN1" s="105" t="s">
+      <c r="AM1" s="58"/>
+      <c r="AN1" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="AO1" s="106"/>
-      <c r="AP1" s="106"/>
-      <c r="AQ1" s="106"/>
-      <c r="AR1" s="107"/>
-      <c r="AS1" s="95" t="s">
+      <c r="AO1" s="62"/>
+      <c r="AP1" s="62"/>
+      <c r="AQ1" s="62"/>
+      <c r="AR1" s="63"/>
+      <c r="AS1" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="AT1" s="97"/>
-      <c r="AU1" s="95" t="s">
+      <c r="AT1" s="74"/>
+      <c r="AU1" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="AV1" s="96"/>
-      <c r="AW1" s="96"/>
-      <c r="AX1" s="96"/>
-      <c r="AY1" s="96"/>
-      <c r="AZ1" s="96"/>
-      <c r="BA1" s="96"/>
-      <c r="BB1" s="96"/>
-      <c r="BC1" s="96"/>
-      <c r="BD1" s="96"/>
-      <c r="BE1" s="96"/>
-      <c r="BF1" s="96"/>
-      <c r="BG1" s="96"/>
-      <c r="BH1" s="96"/>
-      <c r="BI1" s="96"/>
-      <c r="BJ1" s="96"/>
-      <c r="BK1" s="96"/>
-      <c r="BL1" s="96"/>
-      <c r="BM1" s="96"/>
-      <c r="BN1" s="96"/>
-      <c r="BO1" s="96"/>
-      <c r="BP1" s="96"/>
-      <c r="BQ1" s="96"/>
-      <c r="BR1" s="96"/>
-      <c r="BS1" s="96"/>
-      <c r="BT1" s="96"/>
-      <c r="BU1" s="96"/>
-      <c r="BV1" s="96"/>
-      <c r="BW1" s="96"/>
-      <c r="BX1" s="96"/>
-      <c r="BY1" s="96"/>
-      <c r="BZ1" s="96"/>
-      <c r="CA1" s="96"/>
-      <c r="CB1" s="96"/>
-      <c r="CC1" s="96"/>
-      <c r="CD1" s="97"/>
-      <c r="CE1" s="65" t="s">
+      <c r="AV1" s="124"/>
+      <c r="AW1" s="124"/>
+      <c r="AX1" s="124"/>
+      <c r="AY1" s="124"/>
+      <c r="AZ1" s="124"/>
+      <c r="BA1" s="124"/>
+      <c r="BB1" s="124"/>
+      <c r="BC1" s="124"/>
+      <c r="BD1" s="124"/>
+      <c r="BE1" s="124"/>
+      <c r="BF1" s="124"/>
+      <c r="BG1" s="124"/>
+      <c r="BH1" s="124"/>
+      <c r="BI1" s="124"/>
+      <c r="BJ1" s="124"/>
+      <c r="BK1" s="124"/>
+      <c r="BL1" s="124"/>
+      <c r="BM1" s="124"/>
+      <c r="BN1" s="124"/>
+      <c r="BO1" s="124"/>
+      <c r="BP1" s="124"/>
+      <c r="BQ1" s="124"/>
+      <c r="BR1" s="124"/>
+      <c r="BS1" s="124"/>
+      <c r="BT1" s="124"/>
+      <c r="BU1" s="124"/>
+      <c r="BV1" s="124"/>
+      <c r="BW1" s="124"/>
+      <c r="BX1" s="124"/>
+      <c r="BY1" s="124"/>
+      <c r="BZ1" s="124"/>
+      <c r="CA1" s="124"/>
+      <c r="CB1" s="124"/>
+      <c r="CC1" s="124"/>
+      <c r="CD1" s="74"/>
+      <c r="CE1" s="100" t="s">
         <v>6</v>
       </c>
-      <c r="CF1" s="66"/>
-      <c r="CG1" s="66"/>
-      <c r="CH1" s="66"/>
-      <c r="CI1" s="66"/>
-      <c r="CJ1" s="66"/>
-      <c r="CK1" s="66"/>
-      <c r="CL1" s="66"/>
-      <c r="CM1" s="66"/>
-      <c r="CN1" s="66"/>
-      <c r="CO1" s="66"/>
-      <c r="CP1" s="66"/>
-      <c r="CQ1" s="66"/>
-      <c r="CR1" s="66"/>
-      <c r="CS1" s="66"/>
-      <c r="CT1" s="66"/>
-      <c r="CU1" s="66"/>
-      <c r="CV1" s="66"/>
-      <c r="CW1" s="66"/>
-      <c r="CX1" s="66"/>
-      <c r="CY1" s="66"/>
-      <c r="CZ1" s="66"/>
-      <c r="DA1" s="66"/>
-      <c r="DB1" s="66"/>
-      <c r="DC1" s="66"/>
-      <c r="DD1" s="66"/>
-      <c r="DE1" s="66"/>
-      <c r="DF1" s="66"/>
-      <c r="DG1" s="66"/>
-      <c r="DH1" s="66"/>
-      <c r="DI1" s="66"/>
-      <c r="DJ1" s="66"/>
-      <c r="DK1" s="67"/>
-      <c r="DL1" s="71" t="s">
+      <c r="CF1" s="101"/>
+      <c r="CG1" s="101"/>
+      <c r="CH1" s="101"/>
+      <c r="CI1" s="101"/>
+      <c r="CJ1" s="101"/>
+      <c r="CK1" s="101"/>
+      <c r="CL1" s="101"/>
+      <c r="CM1" s="101"/>
+      <c r="CN1" s="101"/>
+      <c r="CO1" s="101"/>
+      <c r="CP1" s="101"/>
+      <c r="CQ1" s="101"/>
+      <c r="CR1" s="101"/>
+      <c r="CS1" s="101"/>
+      <c r="CT1" s="101"/>
+      <c r="CU1" s="101"/>
+      <c r="CV1" s="101"/>
+      <c r="CW1" s="101"/>
+      <c r="CX1" s="101"/>
+      <c r="CY1" s="101"/>
+      <c r="CZ1" s="101"/>
+      <c r="DA1" s="101"/>
+      <c r="DB1" s="101"/>
+      <c r="DC1" s="101"/>
+      <c r="DD1" s="101"/>
+      <c r="DE1" s="101"/>
+      <c r="DF1" s="101"/>
+      <c r="DG1" s="101"/>
+      <c r="DH1" s="101"/>
+      <c r="DI1" s="101"/>
+      <c r="DJ1" s="101"/>
+      <c r="DK1" s="102"/>
+      <c r="DL1" s="106" t="s">
         <v>7</v>
       </c>
-      <c r="DM1" s="72"/>
-      <c r="DN1" s="72"/>
-      <c r="DO1" s="72"/>
-      <c r="DP1" s="72"/>
-      <c r="DQ1" s="72"/>
-      <c r="DR1" s="72"/>
-      <c r="DS1" s="72"/>
-      <c r="DT1" s="72"/>
-      <c r="DU1" s="72"/>
-      <c r="DV1" s="72"/>
-      <c r="DW1" s="72"/>
-      <c r="DX1" s="72"/>
-      <c r="DY1" s="72"/>
-      <c r="DZ1" s="73"/>
-      <c r="EA1" s="77" t="s">
+      <c r="DM1" s="107"/>
+      <c r="DN1" s="107"/>
+      <c r="DO1" s="107"/>
+      <c r="DP1" s="107"/>
+      <c r="DQ1" s="107"/>
+      <c r="DR1" s="107"/>
+      <c r="DS1" s="107"/>
+      <c r="DT1" s="107"/>
+      <c r="DU1" s="107"/>
+      <c r="DV1" s="107"/>
+      <c r="DW1" s="107"/>
+      <c r="DX1" s="107"/>
+      <c r="DY1" s="107"/>
+      <c r="DZ1" s="108"/>
+      <c r="EA1" s="112" t="s">
         <v>9</v>
       </c>
-      <c r="EB1" s="78"/>
-      <c r="EC1" s="78"/>
-      <c r="ED1" s="78"/>
-      <c r="EE1" s="78"/>
-      <c r="EF1" s="78"/>
-      <c r="EG1" s="78"/>
-      <c r="EH1" s="78"/>
-      <c r="EI1" s="78"/>
-      <c r="EJ1" s="78"/>
-      <c r="EK1" s="78"/>
-      <c r="EL1" s="78"/>
-      <c r="EM1" s="78"/>
-      <c r="EN1" s="78"/>
-      <c r="EO1" s="78"/>
-      <c r="EP1" s="78"/>
-      <c r="EQ1" s="78"/>
-      <c r="ER1" s="78"/>
-      <c r="ES1" s="78"/>
-      <c r="ET1" s="78"/>
-      <c r="EU1" s="78"/>
-      <c r="EV1" s="78"/>
-      <c r="EW1" s="78"/>
-      <c r="EX1" s="78"/>
-      <c r="EY1" s="78"/>
-      <c r="EZ1" s="78"/>
-      <c r="FA1" s="78"/>
-      <c r="FB1" s="78"/>
-      <c r="FC1" s="78"/>
-      <c r="FD1" s="78"/>
-      <c r="FE1" s="78"/>
-      <c r="FF1" s="78"/>
-      <c r="FG1" s="78"/>
-      <c r="FH1" s="78"/>
-      <c r="FI1" s="78"/>
-      <c r="FJ1" s="78"/>
-      <c r="FK1" s="78"/>
-      <c r="FL1" s="78"/>
-      <c r="FM1" s="78"/>
-      <c r="FN1" s="78"/>
-      <c r="FO1" s="78"/>
-      <c r="FP1" s="78"/>
-      <c r="FQ1" s="78"/>
-      <c r="FR1" s="78"/>
-      <c r="FS1" s="78"/>
-      <c r="FT1" s="78"/>
-      <c r="FU1" s="78"/>
-      <c r="FV1" s="78"/>
-      <c r="FW1" s="78"/>
-      <c r="FX1" s="78"/>
-      <c r="FY1" s="78"/>
-      <c r="FZ1" s="78"/>
-      <c r="GA1" s="78"/>
-      <c r="GB1" s="78"/>
-      <c r="GC1" s="78"/>
-      <c r="GD1" s="78"/>
-      <c r="GE1" s="78"/>
-      <c r="GF1" s="78"/>
-      <c r="GG1" s="78"/>
-      <c r="GH1" s="78"/>
-      <c r="GI1" s="79"/>
-      <c r="GJ1" s="89" t="s">
+      <c r="EB1" s="113"/>
+      <c r="EC1" s="113"/>
+      <c r="ED1" s="113"/>
+      <c r="EE1" s="113"/>
+      <c r="EF1" s="113"/>
+      <c r="EG1" s="113"/>
+      <c r="EH1" s="113"/>
+      <c r="EI1" s="113"/>
+      <c r="EJ1" s="113"/>
+      <c r="EK1" s="113"/>
+      <c r="EL1" s="113"/>
+      <c r="EM1" s="113"/>
+      <c r="EN1" s="113"/>
+      <c r="EO1" s="113"/>
+      <c r="EP1" s="113"/>
+      <c r="EQ1" s="113"/>
+      <c r="ER1" s="113"/>
+      <c r="ES1" s="113"/>
+      <c r="ET1" s="113"/>
+      <c r="EU1" s="113"/>
+      <c r="EV1" s="113"/>
+      <c r="EW1" s="113"/>
+      <c r="EX1" s="113"/>
+      <c r="EY1" s="113"/>
+      <c r="EZ1" s="113"/>
+      <c r="FA1" s="113"/>
+      <c r="FB1" s="113"/>
+      <c r="FC1" s="113"/>
+      <c r="FD1" s="113"/>
+      <c r="FE1" s="113"/>
+      <c r="FF1" s="113"/>
+      <c r="FG1" s="113"/>
+      <c r="FH1" s="113"/>
+      <c r="FI1" s="113"/>
+      <c r="FJ1" s="113"/>
+      <c r="FK1" s="113"/>
+      <c r="FL1" s="113"/>
+      <c r="FM1" s="113"/>
+      <c r="FN1" s="113"/>
+      <c r="FO1" s="113"/>
+      <c r="FP1" s="113"/>
+      <c r="FQ1" s="113"/>
+      <c r="FR1" s="113"/>
+      <c r="FS1" s="113"/>
+      <c r="FT1" s="113"/>
+      <c r="FU1" s="113"/>
+      <c r="FV1" s="113"/>
+      <c r="FW1" s="113"/>
+      <c r="FX1" s="113"/>
+      <c r="FY1" s="113"/>
+      <c r="FZ1" s="113"/>
+      <c r="GA1" s="113"/>
+      <c r="GB1" s="113"/>
+      <c r="GC1" s="113"/>
+      <c r="GD1" s="113"/>
+      <c r="GE1" s="113"/>
+      <c r="GF1" s="113"/>
+      <c r="GG1" s="113"/>
+      <c r="GH1" s="113"/>
+      <c r="GI1" s="114"/>
+      <c r="GJ1" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="GK1" s="90"/>
-      <c r="GL1" s="90"/>
-      <c r="GM1" s="91"/>
-      <c r="GN1" s="80" t="s">
+      <c r="GK1" s="78"/>
+      <c r="GL1" s="78"/>
+      <c r="GM1" s="79"/>
+      <c r="GN1" s="115" t="s">
         <v>10</v>
       </c>
-      <c r="GO1" s="62" t="s">
+      <c r="GO1" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="GP1" s="48" t="s">
+      <c r="GP1" s="83" t="s">
         <v>12</v>
       </c>
-      <c r="GQ1" s="48" t="s">
+      <c r="GQ1" s="83" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:199" s="12" customFormat="1" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="92"/>
-      <c r="B2" s="93"/>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93"/>
-      <c r="I2" s="93"/>
-      <c r="J2" s="93"/>
-      <c r="K2" s="93"/>
-      <c r="L2" s="93"/>
-      <c r="M2" s="94"/>
-      <c r="N2" s="51" t="s">
+      <c r="A2" s="80"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="82"/>
+      <c r="N2" s="86" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="52"/>
-      <c r="P2" s="52"/>
-      <c r="Q2" s="52"/>
-      <c r="R2" s="52"/>
-      <c r="S2" s="52"/>
-      <c r="T2" s="52"/>
-      <c r="U2" s="52"/>
-      <c r="V2" s="83" t="s">
+      <c r="O2" s="87"/>
+      <c r="P2" s="87"/>
+      <c r="Q2" s="87"/>
+      <c r="R2" s="87"/>
+      <c r="S2" s="87"/>
+      <c r="T2" s="87"/>
+      <c r="U2" s="87"/>
+      <c r="V2" s="118" t="s">
         <v>15</v>
       </c>
-      <c r="W2" s="84"/>
-      <c r="X2" s="84"/>
-      <c r="Y2" s="84"/>
-      <c r="Z2" s="84"/>
-      <c r="AA2" s="84"/>
-      <c r="AB2" s="84"/>
-      <c r="AC2" s="85"/>
-      <c r="AD2" s="114"/>
-      <c r="AE2" s="115"/>
-      <c r="AF2" s="115"/>
-      <c r="AG2" s="115"/>
-      <c r="AH2" s="115"/>
-      <c r="AI2" s="115"/>
-      <c r="AJ2" s="115"/>
-      <c r="AK2" s="116"/>
-      <c r="AL2" s="103"/>
-      <c r="AM2" s="104"/>
-      <c r="AN2" s="108"/>
-      <c r="AO2" s="109"/>
-      <c r="AP2" s="109"/>
-      <c r="AQ2" s="109"/>
-      <c r="AR2" s="110"/>
-      <c r="AS2" s="98"/>
-      <c r="AT2" s="100"/>
-      <c r="AU2" s="98"/>
-      <c r="AV2" s="99"/>
-      <c r="AW2" s="99"/>
-      <c r="AX2" s="99"/>
-      <c r="AY2" s="99"/>
-      <c r="AZ2" s="99"/>
-      <c r="BA2" s="99"/>
-      <c r="BB2" s="99"/>
-      <c r="BC2" s="99"/>
-      <c r="BD2" s="99"/>
-      <c r="BE2" s="99"/>
-      <c r="BF2" s="99"/>
-      <c r="BG2" s="99"/>
-      <c r="BH2" s="99"/>
-      <c r="BI2" s="99"/>
-      <c r="BJ2" s="99"/>
-      <c r="BK2" s="99"/>
-      <c r="BL2" s="99"/>
-      <c r="BM2" s="99"/>
-      <c r="BN2" s="99"/>
-      <c r="BO2" s="99"/>
-      <c r="BP2" s="99"/>
-      <c r="BQ2" s="99"/>
-      <c r="BR2" s="99"/>
-      <c r="BS2" s="99"/>
-      <c r="BT2" s="99"/>
-      <c r="BU2" s="99"/>
-      <c r="BV2" s="99"/>
-      <c r="BW2" s="99"/>
-      <c r="BX2" s="99"/>
-      <c r="BY2" s="99"/>
-      <c r="BZ2" s="99"/>
-      <c r="CA2" s="99"/>
-      <c r="CB2" s="99"/>
-      <c r="CC2" s="99"/>
-      <c r="CD2" s="100"/>
-      <c r="CE2" s="68"/>
-      <c r="CF2" s="69"/>
-      <c r="CG2" s="69"/>
-      <c r="CH2" s="69"/>
-      <c r="CI2" s="69"/>
-      <c r="CJ2" s="69"/>
-      <c r="CK2" s="69"/>
-      <c r="CL2" s="69"/>
-      <c r="CM2" s="69"/>
-      <c r="CN2" s="69"/>
-      <c r="CO2" s="69"/>
-      <c r="CP2" s="69"/>
-      <c r="CQ2" s="69"/>
-      <c r="CR2" s="69"/>
-      <c r="CS2" s="69"/>
-      <c r="CT2" s="69"/>
-      <c r="CU2" s="69"/>
-      <c r="CV2" s="69"/>
-      <c r="CW2" s="69"/>
-      <c r="CX2" s="69"/>
-      <c r="CY2" s="69"/>
-      <c r="CZ2" s="69"/>
-      <c r="DA2" s="69"/>
-      <c r="DB2" s="69"/>
-      <c r="DC2" s="69"/>
-      <c r="DD2" s="69"/>
-      <c r="DE2" s="69"/>
-      <c r="DF2" s="69"/>
-      <c r="DG2" s="69"/>
-      <c r="DH2" s="69"/>
-      <c r="DI2" s="69"/>
-      <c r="DJ2" s="69"/>
-      <c r="DK2" s="70"/>
-      <c r="DL2" s="74"/>
-      <c r="DM2" s="75"/>
-      <c r="DN2" s="75"/>
-      <c r="DO2" s="75"/>
-      <c r="DP2" s="75"/>
-      <c r="DQ2" s="75"/>
-      <c r="DR2" s="75"/>
-      <c r="DS2" s="75"/>
-      <c r="DT2" s="75"/>
-      <c r="DU2" s="75"/>
-      <c r="DV2" s="75"/>
-      <c r="DW2" s="75"/>
-      <c r="DX2" s="75"/>
-      <c r="DY2" s="75"/>
-      <c r="DZ2" s="76"/>
-      <c r="EA2" s="125"/>
-      <c r="EB2" s="117"/>
-      <c r="EC2" s="117"/>
-      <c r="ED2" s="117"/>
-      <c r="EE2" s="117"/>
-      <c r="EF2" s="117"/>
-      <c r="EG2" s="117"/>
-      <c r="EH2" s="117"/>
-      <c r="EI2" s="117"/>
-      <c r="EJ2" s="117"/>
-      <c r="EK2" s="117"/>
-      <c r="EL2" s="117"/>
-      <c r="EM2" s="117"/>
-      <c r="EN2" s="118"/>
-      <c r="EO2" s="122" t="s">
+      <c r="W2" s="119"/>
+      <c r="X2" s="119"/>
+      <c r="Y2" s="119"/>
+      <c r="Z2" s="119"/>
+      <c r="AA2" s="119"/>
+      <c r="AB2" s="119"/>
+      <c r="AC2" s="120"/>
+      <c r="AD2" s="70"/>
+      <c r="AE2" s="71"/>
+      <c r="AF2" s="71"/>
+      <c r="AG2" s="71"/>
+      <c r="AH2" s="71"/>
+      <c r="AI2" s="71"/>
+      <c r="AJ2" s="71"/>
+      <c r="AK2" s="72"/>
+      <c r="AL2" s="59"/>
+      <c r="AM2" s="60"/>
+      <c r="AN2" s="64"/>
+      <c r="AO2" s="65"/>
+      <c r="AP2" s="65"/>
+      <c r="AQ2" s="65"/>
+      <c r="AR2" s="66"/>
+      <c r="AS2" s="75"/>
+      <c r="AT2" s="76"/>
+      <c r="AU2" s="75"/>
+      <c r="AV2" s="125"/>
+      <c r="AW2" s="125"/>
+      <c r="AX2" s="125"/>
+      <c r="AY2" s="125"/>
+      <c r="AZ2" s="125"/>
+      <c r="BA2" s="125"/>
+      <c r="BB2" s="125"/>
+      <c r="BC2" s="125"/>
+      <c r="BD2" s="125"/>
+      <c r="BE2" s="125"/>
+      <c r="BF2" s="125"/>
+      <c r="BG2" s="125"/>
+      <c r="BH2" s="125"/>
+      <c r="BI2" s="125"/>
+      <c r="BJ2" s="125"/>
+      <c r="BK2" s="125"/>
+      <c r="BL2" s="125"/>
+      <c r="BM2" s="125"/>
+      <c r="BN2" s="125"/>
+      <c r="BO2" s="125"/>
+      <c r="BP2" s="125"/>
+      <c r="BQ2" s="125"/>
+      <c r="BR2" s="125"/>
+      <c r="BS2" s="125"/>
+      <c r="BT2" s="125"/>
+      <c r="BU2" s="125"/>
+      <c r="BV2" s="125"/>
+      <c r="BW2" s="125"/>
+      <c r="BX2" s="125"/>
+      <c r="BY2" s="125"/>
+      <c r="BZ2" s="125"/>
+      <c r="CA2" s="125"/>
+      <c r="CB2" s="125"/>
+      <c r="CC2" s="125"/>
+      <c r="CD2" s="76"/>
+      <c r="CE2" s="103"/>
+      <c r="CF2" s="104"/>
+      <c r="CG2" s="104"/>
+      <c r="CH2" s="104"/>
+      <c r="CI2" s="104"/>
+      <c r="CJ2" s="104"/>
+      <c r="CK2" s="104"/>
+      <c r="CL2" s="104"/>
+      <c r="CM2" s="104"/>
+      <c r="CN2" s="104"/>
+      <c r="CO2" s="104"/>
+      <c r="CP2" s="104"/>
+      <c r="CQ2" s="104"/>
+      <c r="CR2" s="104"/>
+      <c r="CS2" s="104"/>
+      <c r="CT2" s="104"/>
+      <c r="CU2" s="104"/>
+      <c r="CV2" s="104"/>
+      <c r="CW2" s="104"/>
+      <c r="CX2" s="104"/>
+      <c r="CY2" s="104"/>
+      <c r="CZ2" s="104"/>
+      <c r="DA2" s="104"/>
+      <c r="DB2" s="104"/>
+      <c r="DC2" s="104"/>
+      <c r="DD2" s="104"/>
+      <c r="DE2" s="104"/>
+      <c r="DF2" s="104"/>
+      <c r="DG2" s="104"/>
+      <c r="DH2" s="104"/>
+      <c r="DI2" s="104"/>
+      <c r="DJ2" s="104"/>
+      <c r="DK2" s="105"/>
+      <c r="DL2" s="109"/>
+      <c r="DM2" s="110"/>
+      <c r="DN2" s="110"/>
+      <c r="DO2" s="110"/>
+      <c r="DP2" s="110"/>
+      <c r="DQ2" s="110"/>
+      <c r="DR2" s="110"/>
+      <c r="DS2" s="110"/>
+      <c r="DT2" s="110"/>
+      <c r="DU2" s="110"/>
+      <c r="DV2" s="110"/>
+      <c r="DW2" s="110"/>
+      <c r="DX2" s="110"/>
+      <c r="DY2" s="110"/>
+      <c r="DZ2" s="111"/>
+      <c r="EA2" s="54"/>
+      <c r="EB2" s="55"/>
+      <c r="EC2" s="55"/>
+      <c r="ED2" s="55"/>
+      <c r="EE2" s="55"/>
+      <c r="EF2" s="55"/>
+      <c r="EG2" s="55"/>
+      <c r="EH2" s="55"/>
+      <c r="EI2" s="55"/>
+      <c r="EJ2" s="55"/>
+      <c r="EK2" s="55"/>
+      <c r="EL2" s="55"/>
+      <c r="EM2" s="55"/>
+      <c r="EN2" s="56"/>
+      <c r="EO2" s="51" t="s">
         <v>242</v>
       </c>
-      <c r="EP2" s="123"/>
-      <c r="EQ2" s="123"/>
-      <c r="ER2" s="123"/>
-      <c r="ES2" s="123"/>
-      <c r="ET2" s="123"/>
-      <c r="EU2" s="123"/>
-      <c r="EV2" s="123"/>
-      <c r="EW2" s="123"/>
-      <c r="EX2" s="123"/>
-      <c r="EY2" s="123"/>
-      <c r="EZ2" s="123"/>
-      <c r="FA2" s="124"/>
-      <c r="FB2" s="53" t="s">
+      <c r="EP2" s="52"/>
+      <c r="EQ2" s="52"/>
+      <c r="ER2" s="52"/>
+      <c r="ES2" s="52"/>
+      <c r="ET2" s="52"/>
+      <c r="EU2" s="52"/>
+      <c r="EV2" s="52"/>
+      <c r="EW2" s="52"/>
+      <c r="EX2" s="52"/>
+      <c r="EY2" s="52"/>
+      <c r="EZ2" s="52"/>
+      <c r="FA2" s="53"/>
+      <c r="FB2" s="88" t="s">
         <v>16</v>
       </c>
-      <c r="FC2" s="54"/>
-      <c r="FD2" s="54"/>
-      <c r="FE2" s="54"/>
-      <c r="FF2" s="54"/>
-      <c r="FG2" s="54"/>
-      <c r="FH2" s="54"/>
-      <c r="FI2" s="54"/>
-      <c r="FJ2" s="54"/>
-      <c r="FK2" s="54"/>
-      <c r="FL2" s="54"/>
-      <c r="FM2" s="54"/>
-      <c r="FN2" s="54"/>
-      <c r="FO2" s="54"/>
-      <c r="FP2" s="54"/>
-      <c r="FQ2" s="54"/>
-      <c r="FR2" s="55"/>
-      <c r="FS2" s="56" t="s">
+      <c r="FC2" s="89"/>
+      <c r="FD2" s="89"/>
+      <c r="FE2" s="89"/>
+      <c r="FF2" s="89"/>
+      <c r="FG2" s="89"/>
+      <c r="FH2" s="89"/>
+      <c r="FI2" s="89"/>
+      <c r="FJ2" s="89"/>
+      <c r="FK2" s="89"/>
+      <c r="FL2" s="89"/>
+      <c r="FM2" s="89"/>
+      <c r="FN2" s="89"/>
+      <c r="FO2" s="89"/>
+      <c r="FP2" s="89"/>
+      <c r="FQ2" s="89"/>
+      <c r="FR2" s="90"/>
+      <c r="FS2" s="91" t="s">
         <v>17</v>
       </c>
-      <c r="FT2" s="57"/>
-      <c r="FU2" s="57"/>
-      <c r="FV2" s="57"/>
-      <c r="FW2" s="57"/>
-      <c r="FX2" s="57"/>
-      <c r="FY2" s="57"/>
-      <c r="FZ2" s="57"/>
-      <c r="GA2" s="57"/>
-      <c r="GB2" s="58"/>
-      <c r="GC2" s="59" t="s">
+      <c r="FT2" s="92"/>
+      <c r="FU2" s="92"/>
+      <c r="FV2" s="92"/>
+      <c r="FW2" s="92"/>
+      <c r="FX2" s="92"/>
+      <c r="FY2" s="92"/>
+      <c r="FZ2" s="92"/>
+      <c r="GA2" s="92"/>
+      <c r="GB2" s="93"/>
+      <c r="GC2" s="94" t="s">
         <v>18</v>
       </c>
-      <c r="GD2" s="60"/>
-      <c r="GE2" s="60"/>
-      <c r="GF2" s="60"/>
-      <c r="GG2" s="60"/>
-      <c r="GH2" s="60"/>
-      <c r="GI2" s="61"/>
-      <c r="GJ2" s="92"/>
-      <c r="GK2" s="93"/>
-      <c r="GL2" s="93"/>
-      <c r="GM2" s="94"/>
-      <c r="GN2" s="81"/>
-      <c r="GO2" s="63"/>
-      <c r="GP2" s="49"/>
-      <c r="GQ2" s="49"/>
+      <c r="GD2" s="95"/>
+      <c r="GE2" s="95"/>
+      <c r="GF2" s="95"/>
+      <c r="GG2" s="95"/>
+      <c r="GH2" s="95"/>
+      <c r="GI2" s="96"/>
+      <c r="GJ2" s="80"/>
+      <c r="GK2" s="81"/>
+      <c r="GL2" s="81"/>
+      <c r="GM2" s="82"/>
+      <c r="GN2" s="116"/>
+      <c r="GO2" s="98"/>
+      <c r="GP2" s="84"/>
+      <c r="GQ2" s="84"/>
     </row>
     <row r="3" spans="1:199" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
@@ -4074,43 +4074,43 @@
       <c r="EN3" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="EO3" s="119" t="s">
+      <c r="EO3" s="48" t="s">
         <v>232</v>
       </c>
-      <c r="EP3" s="120" t="s">
+      <c r="EP3" s="49" t="s">
         <v>51</v>
       </c>
-      <c r="EQ3" s="120" t="s">
+      <c r="EQ3" s="49" t="s">
         <v>233</v>
       </c>
-      <c r="ER3" s="120" t="s">
+      <c r="ER3" s="49" t="s">
         <v>231</v>
       </c>
-      <c r="ES3" s="121" t="s">
+      <c r="ES3" s="50" t="s">
         <v>230</v>
       </c>
-      <c r="ET3" s="120" t="s">
+      <c r="ET3" s="49" t="s">
         <v>51</v>
       </c>
-      <c r="EU3" s="120" t="s">
+      <c r="EU3" s="49" t="s">
         <v>233</v>
       </c>
-      <c r="EV3" s="120" t="s">
+      <c r="EV3" s="49" t="s">
         <v>231</v>
       </c>
-      <c r="EW3" s="121" t="s">
+      <c r="EW3" s="50" t="s">
         <v>230</v>
       </c>
-      <c r="EX3" s="120" t="s">
+      <c r="EX3" s="49" t="s">
         <v>51</v>
       </c>
-      <c r="EY3" s="120" t="s">
+      <c r="EY3" s="49" t="s">
         <v>233</v>
       </c>
-      <c r="EZ3" s="120" t="s">
+      <c r="EZ3" s="49" t="s">
         <v>231</v>
       </c>
-      <c r="FA3" s="121" t="s">
+      <c r="FA3" s="50" t="s">
         <v>230</v>
       </c>
       <c r="FB3" s="41" t="s">
@@ -4227,10 +4227,10 @@
       <c r="GM3" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="GN3" s="82"/>
-      <c r="GO3" s="64"/>
-      <c r="GP3" s="50"/>
-      <c r="GQ3" s="50"/>
+      <c r="GN3" s="117"/>
+      <c r="GO3" s="99"/>
+      <c r="GP3" s="85"/>
+      <c r="GQ3" s="85"/>
     </row>
     <row r="4" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -4904,12 +4904,6 @@
   </sheetData>
   <autoFilter ref="A3:GQ5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="22">
-    <mergeCell ref="EO2:FA2"/>
-    <mergeCell ref="EA2:EN2"/>
-    <mergeCell ref="AL1:AM2"/>
-    <mergeCell ref="AN1:AR2"/>
-    <mergeCell ref="AD1:AK2"/>
-    <mergeCell ref="AS1:AT2"/>
     <mergeCell ref="A1:M2"/>
     <mergeCell ref="GP1:GP3"/>
     <mergeCell ref="GQ1:GQ3"/>
@@ -4926,6 +4920,12 @@
     <mergeCell ref="N1:AC1"/>
     <mergeCell ref="GJ1:GM2"/>
     <mergeCell ref="AU1:CD2"/>
+    <mergeCell ref="EO2:FA2"/>
+    <mergeCell ref="EA2:EN2"/>
+    <mergeCell ref="AL1:AM2"/>
+    <mergeCell ref="AN1:AR2"/>
+    <mergeCell ref="AD1:AK2"/>
+    <mergeCell ref="AS1:AT2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A7:B1048576 A3:A6">
     <cfRule type="duplicateValues" dxfId="0" priority="142"/>

</xml_diff>

<commit_message>
SRI Consulta de Deudas Firmes: fix del spinner sri-splash persistente - clic sobre el overlay gris (ui-blockui-document) despierta el render atascado, confirmado manualmente. Extraccion de valor de deuda firme funcionando, con manejo de caso sin ningun tipo de deuda
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC661B8E-97DA-4116-A4CA-0CFD3E47009D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB8E6754-2937-4FE8-AF7C-EA74C99B2B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
   </bookViews>
@@ -343,7 +343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="248">
   <si>
     <t>IDENTIFICACIÓN BÁSICA</t>
   </si>
@@ -890,9 +890,6 @@
     <t>SRI OBLIGACIONES TRIBUTARIAS</t>
   </si>
   <si>
-    <t>NO TIENE OBLIGACIONES TRIBUTARIAS PENDIENTES</t>
-  </si>
-  <si>
     <t>DEUDA</t>
   </si>
   <si>
@@ -902,9 +899,6 @@
     <t>Column1</t>
   </si>
   <si>
-    <t>PERIODO + OBLIGACION TRIBUTARIA</t>
-  </si>
-  <si>
     <t>CONTRIBUYENTE FANTASMA</t>
   </si>
   <si>
@@ -956,9 +950,6 @@
     <t>VILLACIS OLIVO ROMMEL JOERICK</t>
   </si>
   <si>
-    <t>Nombre Persona Natural / Juridica</t>
-  </si>
-  <si>
     <t>MUNICIPIO DE QUITO;</t>
   </si>
   <si>
@@ -1074,6 +1065,30 @@
   </si>
   <si>
     <t>SENTENCIADOS</t>
+  </si>
+  <si>
+    <t>Apellidos Y Nombres (P.Natural / P.Juridica)</t>
+  </si>
+  <si>
+    <t>GUAYAS / GUAYAQUIL / XIMENA / LOS RIOS 1301 Y CLEMENTE BALLEN</t>
+  </si>
+  <si>
+    <t>SUSPENDIDO</t>
+  </si>
+  <si>
+    <t>CESE DE ACTIVIDADES</t>
+  </si>
+  <si>
+    <t>No registra deudas firmes</t>
+  </si>
+  <si>
+    <t>ANEXO DECLARACIÓN PATRIMONIAL AÑO 2025</t>
+  </si>
+  <si>
+    <t>AL DIA EN SUS OBLIGACIONES</t>
+  </si>
+  <si>
+    <t>ANEXO TRANSACCIONAL SIMPLIFICADO JUNIO 2026</t>
   </si>
 </sst>
 </file>
@@ -1276,7 +1291,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -1309,30 +1324,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -1508,19 +1499,6 @@
         <color indexed="64"/>
       </right>
       <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
@@ -1748,12 +1726,94 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="126">
+  <cellXfs count="132">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1789,100 +1849,97 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="12" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="12" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="5" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1894,238 +1951,259 @@
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2730,7 +2808,7 @@
         <v>115</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -2887,7 +2965,7 @@
         <v>136</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -3010,7 +3088,7 @@
     <col min="4" max="4" width="17.6640625" style="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.5546875" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="31.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.44140625" style="46" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="25.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="27.44140625" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="22.44140625" style="5" bestFit="1" customWidth="1"/>
@@ -3019,23 +3097,23 @@
     <col min="13" max="13" width="14.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="16.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="24.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.5546875" style="47" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="16.88671875" style="47" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.88671875" style="47" customWidth="1"/>
+    <col min="16" max="16" width="20.5546875" style="46" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.88671875" style="46" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.88671875" style="46" customWidth="1"/>
     <col min="19" max="19" width="24" style="5" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="24.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="46.5546875" style="5" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="16.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="24.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="20.5546875" style="47" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.88671875" style="47" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="19.44140625" style="47" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.5546875" style="46" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.88671875" style="46" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.44140625" style="46" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="51.33203125" style="5" customWidth="1"/>
     <col min="28" max="28" width="25.33203125" style="5" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="29.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="30" max="31" width="27.5546875" style="5" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="24.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14" style="45" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14" style="44" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="24.88671875" style="5" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="29.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="19.6640625" style="5" bestFit="1" customWidth="1"/>
@@ -3148,11 +3226,11 @@
     <col min="144" max="144" width="19.109375" style="5" bestFit="1" customWidth="1"/>
     <col min="145" max="145" width="19.109375" style="5" customWidth="1"/>
     <col min="146" max="147" width="19.109375" style="4" customWidth="1"/>
-    <col min="148" max="148" width="19.109375" style="47" customWidth="1"/>
+    <col min="148" max="148" width="19.109375" style="46" customWidth="1"/>
     <col min="149" max="151" width="19.109375" style="4" customWidth="1"/>
-    <col min="152" max="152" width="19.109375" style="47" customWidth="1"/>
+    <col min="152" max="152" width="19.109375" style="46" customWidth="1"/>
     <col min="153" max="155" width="19.109375" style="4" customWidth="1"/>
-    <col min="156" max="156" width="19.109375" style="47" customWidth="1"/>
+    <col min="156" max="156" width="19.109375" style="46" customWidth="1"/>
     <col min="157" max="157" width="18.88671875" style="4" bestFit="1" customWidth="1"/>
     <col min="158" max="158" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
     <col min="159" max="159" width="21.77734375" style="5" bestFit="1" customWidth="1"/>
@@ -3162,12 +3240,12 @@
     <col min="163" max="163" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
     <col min="164" max="164" width="20.21875" style="5" bestFit="1" customWidth="1"/>
     <col min="165" max="165" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="166" max="166" width="22.21875" style="47" bestFit="1" customWidth="1"/>
+    <col min="166" max="166" width="22.21875" style="46" bestFit="1" customWidth="1"/>
     <col min="167" max="167" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
     <col min="168" max="168" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
     <col min="169" max="169" width="20.21875" style="5" bestFit="1" customWidth="1"/>
     <col min="170" max="170" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="171" max="171" width="22.21875" style="47" bestFit="1" customWidth="1"/>
+    <col min="171" max="171" width="22.21875" style="46" bestFit="1" customWidth="1"/>
     <col min="172" max="172" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
     <col min="173" max="173" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
     <col min="174" max="174" width="20.21875" style="5" bestFit="1" customWidth="1"/>
@@ -3198,458 +3276,458 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:199" s="12" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="79"/>
-      <c r="N1" s="121" t="s">
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="E1" s="50"/>
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="I1" s="50"/>
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="M1" s="51"/>
+      <c r="N1" s="119" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="122"/>
-      <c r="P1" s="122"/>
-      <c r="Q1" s="122"/>
-      <c r="R1" s="122"/>
-      <c r="S1" s="122"/>
-      <c r="T1" s="122"/>
-      <c r="U1" s="122"/>
-      <c r="V1" s="122"/>
-      <c r="W1" s="122"/>
-      <c r="X1" s="122"/>
-      <c r="Y1" s="122"/>
-      <c r="Z1" s="122"/>
-      <c r="AA1" s="122"/>
-      <c r="AB1" s="122"/>
-      <c r="AC1" s="123"/>
-      <c r="AD1" s="67" t="s">
+      <c r="O1" s="113"/>
+      <c r="P1" s="113"/>
+      <c r="Q1" s="113"/>
+      <c r="R1" s="113"/>
+      <c r="S1" s="113"/>
+      <c r="T1" s="113"/>
+      <c r="U1" s="113"/>
+      <c r="V1" s="113"/>
+      <c r="W1" s="113"/>
+      <c r="X1" s="113"/>
+      <c r="Y1" s="113"/>
+      <c r="Z1" s="113"/>
+      <c r="AA1" s="113"/>
+      <c r="AB1" s="113"/>
+      <c r="AC1" s="114"/>
+      <c r="AD1" s="107" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="68"/>
-      <c r="AF1" s="68"/>
-      <c r="AG1" s="68"/>
-      <c r="AH1" s="68"/>
-      <c r="AI1" s="68"/>
-      <c r="AJ1" s="68"/>
-      <c r="AK1" s="69"/>
-      <c r="AL1" s="57" t="s">
+      <c r="AE1" s="108"/>
+      <c r="AF1" s="108"/>
+      <c r="AG1" s="108"/>
+      <c r="AH1" s="108"/>
+      <c r="AI1" s="108"/>
+      <c r="AJ1" s="108"/>
+      <c r="AK1" s="109"/>
+      <c r="AL1" s="97" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="58"/>
-      <c r="AN1" s="61" t="s">
+      <c r="AM1" s="98"/>
+      <c r="AN1" s="101" t="s">
         <v>2</v>
       </c>
-      <c r="AO1" s="62"/>
-      <c r="AP1" s="62"/>
-      <c r="AQ1" s="62"/>
-      <c r="AR1" s="63"/>
-      <c r="AS1" s="73" t="s">
+      <c r="AO1" s="102"/>
+      <c r="AP1" s="102"/>
+      <c r="AQ1" s="102"/>
+      <c r="AR1" s="103"/>
+      <c r="AS1" s="85" t="s">
         <v>4</v>
       </c>
-      <c r="AT1" s="74"/>
-      <c r="AU1" s="73" t="s">
+      <c r="AT1" s="87"/>
+      <c r="AU1" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="AV1" s="124"/>
-      <c r="AW1" s="124"/>
-      <c r="AX1" s="124"/>
-      <c r="AY1" s="124"/>
-      <c r="AZ1" s="124"/>
-      <c r="BA1" s="124"/>
-      <c r="BB1" s="124"/>
-      <c r="BC1" s="124"/>
-      <c r="BD1" s="124"/>
-      <c r="BE1" s="124"/>
-      <c r="BF1" s="124"/>
-      <c r="BG1" s="124"/>
-      <c r="BH1" s="124"/>
-      <c r="BI1" s="124"/>
-      <c r="BJ1" s="124"/>
-      <c r="BK1" s="124"/>
-      <c r="BL1" s="124"/>
-      <c r="BM1" s="124"/>
-      <c r="BN1" s="124"/>
-      <c r="BO1" s="124"/>
-      <c r="BP1" s="124"/>
-      <c r="BQ1" s="124"/>
-      <c r="BR1" s="124"/>
-      <c r="BS1" s="124"/>
-      <c r="BT1" s="124"/>
-      <c r="BU1" s="124"/>
-      <c r="BV1" s="124"/>
-      <c r="BW1" s="124"/>
-      <c r="BX1" s="124"/>
-      <c r="BY1" s="124"/>
-      <c r="BZ1" s="124"/>
-      <c r="CA1" s="124"/>
-      <c r="CB1" s="124"/>
-      <c r="CC1" s="124"/>
-      <c r="CD1" s="74"/>
-      <c r="CE1" s="100" t="s">
+      <c r="AV1" s="86"/>
+      <c r="AW1" s="86"/>
+      <c r="AX1" s="86"/>
+      <c r="AY1" s="86"/>
+      <c r="AZ1" s="86"/>
+      <c r="BA1" s="86"/>
+      <c r="BB1" s="86"/>
+      <c r="BC1" s="86"/>
+      <c r="BD1" s="86"/>
+      <c r="BE1" s="86"/>
+      <c r="BF1" s="86"/>
+      <c r="BG1" s="86"/>
+      <c r="BH1" s="86"/>
+      <c r="BI1" s="86"/>
+      <c r="BJ1" s="86"/>
+      <c r="BK1" s="86"/>
+      <c r="BL1" s="86"/>
+      <c r="BM1" s="86"/>
+      <c r="BN1" s="86"/>
+      <c r="BO1" s="86"/>
+      <c r="BP1" s="86"/>
+      <c r="BQ1" s="86"/>
+      <c r="BR1" s="86"/>
+      <c r="BS1" s="86"/>
+      <c r="BT1" s="86"/>
+      <c r="BU1" s="86"/>
+      <c r="BV1" s="86"/>
+      <c r="BW1" s="86"/>
+      <c r="BX1" s="86"/>
+      <c r="BY1" s="86"/>
+      <c r="BZ1" s="86"/>
+      <c r="CA1" s="86"/>
+      <c r="CB1" s="86"/>
+      <c r="CC1" s="86"/>
+      <c r="CD1" s="87"/>
+      <c r="CE1" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="CF1" s="101"/>
-      <c r="CG1" s="101"/>
-      <c r="CH1" s="101"/>
-      <c r="CI1" s="101"/>
-      <c r="CJ1" s="101"/>
-      <c r="CK1" s="101"/>
-      <c r="CL1" s="101"/>
-      <c r="CM1" s="101"/>
-      <c r="CN1" s="101"/>
-      <c r="CO1" s="101"/>
-      <c r="CP1" s="101"/>
-      <c r="CQ1" s="101"/>
-      <c r="CR1" s="101"/>
-      <c r="CS1" s="101"/>
-      <c r="CT1" s="101"/>
-      <c r="CU1" s="101"/>
-      <c r="CV1" s="101"/>
-      <c r="CW1" s="101"/>
-      <c r="CX1" s="101"/>
-      <c r="CY1" s="101"/>
-      <c r="CZ1" s="101"/>
-      <c r="DA1" s="101"/>
-      <c r="DB1" s="101"/>
-      <c r="DC1" s="101"/>
-      <c r="DD1" s="101"/>
-      <c r="DE1" s="101"/>
-      <c r="DF1" s="101"/>
-      <c r="DG1" s="101"/>
-      <c r="DH1" s="101"/>
-      <c r="DI1" s="101"/>
-      <c r="DJ1" s="101"/>
-      <c r="DK1" s="102"/>
-      <c r="DL1" s="106" t="s">
+      <c r="CF1" s="68"/>
+      <c r="CG1" s="68"/>
+      <c r="CH1" s="68"/>
+      <c r="CI1" s="68"/>
+      <c r="CJ1" s="68"/>
+      <c r="CK1" s="68"/>
+      <c r="CL1" s="68"/>
+      <c r="CM1" s="68"/>
+      <c r="CN1" s="68"/>
+      <c r="CO1" s="68"/>
+      <c r="CP1" s="68"/>
+      <c r="CQ1" s="68"/>
+      <c r="CR1" s="68"/>
+      <c r="CS1" s="68"/>
+      <c r="CT1" s="68"/>
+      <c r="CU1" s="68"/>
+      <c r="CV1" s="68"/>
+      <c r="CW1" s="68"/>
+      <c r="CX1" s="68"/>
+      <c r="CY1" s="68"/>
+      <c r="CZ1" s="68"/>
+      <c r="DA1" s="68"/>
+      <c r="DB1" s="68"/>
+      <c r="DC1" s="68"/>
+      <c r="DD1" s="68"/>
+      <c r="DE1" s="68"/>
+      <c r="DF1" s="68"/>
+      <c r="DG1" s="68"/>
+      <c r="DH1" s="68"/>
+      <c r="DI1" s="68"/>
+      <c r="DJ1" s="68"/>
+      <c r="DK1" s="69"/>
+      <c r="DL1" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="DM1" s="107"/>
-      <c r="DN1" s="107"/>
-      <c r="DO1" s="107"/>
-      <c r="DP1" s="107"/>
-      <c r="DQ1" s="107"/>
-      <c r="DR1" s="107"/>
-      <c r="DS1" s="107"/>
-      <c r="DT1" s="107"/>
-      <c r="DU1" s="107"/>
-      <c r="DV1" s="107"/>
-      <c r="DW1" s="107"/>
-      <c r="DX1" s="107"/>
-      <c r="DY1" s="107"/>
-      <c r="DZ1" s="108"/>
-      <c r="EA1" s="112" t="s">
+      <c r="DM1" s="74"/>
+      <c r="DN1" s="74"/>
+      <c r="DO1" s="74"/>
+      <c r="DP1" s="74"/>
+      <c r="DQ1" s="74"/>
+      <c r="DR1" s="74"/>
+      <c r="DS1" s="74"/>
+      <c r="DT1" s="74"/>
+      <c r="DU1" s="74"/>
+      <c r="DV1" s="74"/>
+      <c r="DW1" s="74"/>
+      <c r="DX1" s="74"/>
+      <c r="DY1" s="74"/>
+      <c r="DZ1" s="75"/>
+      <c r="EA1" s="79" t="s">
         <v>9</v>
       </c>
-      <c r="EB1" s="113"/>
-      <c r="EC1" s="113"/>
-      <c r="ED1" s="113"/>
-      <c r="EE1" s="113"/>
-      <c r="EF1" s="113"/>
-      <c r="EG1" s="113"/>
-      <c r="EH1" s="113"/>
-      <c r="EI1" s="113"/>
-      <c r="EJ1" s="113"/>
-      <c r="EK1" s="113"/>
-      <c r="EL1" s="113"/>
-      <c r="EM1" s="113"/>
-      <c r="EN1" s="113"/>
-      <c r="EO1" s="113"/>
-      <c r="EP1" s="113"/>
-      <c r="EQ1" s="113"/>
-      <c r="ER1" s="113"/>
-      <c r="ES1" s="113"/>
-      <c r="ET1" s="113"/>
-      <c r="EU1" s="113"/>
-      <c r="EV1" s="113"/>
-      <c r="EW1" s="113"/>
-      <c r="EX1" s="113"/>
-      <c r="EY1" s="113"/>
-      <c r="EZ1" s="113"/>
-      <c r="FA1" s="113"/>
-      <c r="FB1" s="113"/>
-      <c r="FC1" s="113"/>
-      <c r="FD1" s="113"/>
-      <c r="FE1" s="113"/>
-      <c r="FF1" s="113"/>
-      <c r="FG1" s="113"/>
-      <c r="FH1" s="113"/>
-      <c r="FI1" s="113"/>
-      <c r="FJ1" s="113"/>
-      <c r="FK1" s="113"/>
-      <c r="FL1" s="113"/>
-      <c r="FM1" s="113"/>
-      <c r="FN1" s="113"/>
-      <c r="FO1" s="113"/>
-      <c r="FP1" s="113"/>
-      <c r="FQ1" s="113"/>
-      <c r="FR1" s="113"/>
-      <c r="FS1" s="113"/>
-      <c r="FT1" s="113"/>
-      <c r="FU1" s="113"/>
-      <c r="FV1" s="113"/>
-      <c r="FW1" s="113"/>
-      <c r="FX1" s="113"/>
-      <c r="FY1" s="113"/>
-      <c r="FZ1" s="113"/>
-      <c r="GA1" s="113"/>
-      <c r="GB1" s="113"/>
-      <c r="GC1" s="113"/>
-      <c r="GD1" s="113"/>
-      <c r="GE1" s="113"/>
-      <c r="GF1" s="113"/>
-      <c r="GG1" s="113"/>
-      <c r="GH1" s="113"/>
-      <c r="GI1" s="114"/>
-      <c r="GJ1" s="77" t="s">
+      <c r="EB1" s="80"/>
+      <c r="EC1" s="80"/>
+      <c r="ED1" s="80"/>
+      <c r="EE1" s="80"/>
+      <c r="EF1" s="80"/>
+      <c r="EG1" s="80"/>
+      <c r="EH1" s="80"/>
+      <c r="EI1" s="80"/>
+      <c r="EJ1" s="80"/>
+      <c r="EK1" s="80"/>
+      <c r="EL1" s="80"/>
+      <c r="EM1" s="80"/>
+      <c r="EN1" s="80"/>
+      <c r="EO1" s="80"/>
+      <c r="EP1" s="80"/>
+      <c r="EQ1" s="80"/>
+      <c r="ER1" s="80"/>
+      <c r="ES1" s="80"/>
+      <c r="ET1" s="80"/>
+      <c r="EU1" s="80"/>
+      <c r="EV1" s="80"/>
+      <c r="EW1" s="80"/>
+      <c r="EX1" s="80"/>
+      <c r="EY1" s="80"/>
+      <c r="EZ1" s="80"/>
+      <c r="FA1" s="80"/>
+      <c r="FB1" s="80"/>
+      <c r="FC1" s="80"/>
+      <c r="FD1" s="80"/>
+      <c r="FE1" s="80"/>
+      <c r="FF1" s="80"/>
+      <c r="FG1" s="80"/>
+      <c r="FH1" s="80"/>
+      <c r="FI1" s="80"/>
+      <c r="FJ1" s="80"/>
+      <c r="FK1" s="80"/>
+      <c r="FL1" s="80"/>
+      <c r="FM1" s="80"/>
+      <c r="FN1" s="80"/>
+      <c r="FO1" s="80"/>
+      <c r="FP1" s="80"/>
+      <c r="FQ1" s="80"/>
+      <c r="FR1" s="80"/>
+      <c r="FS1" s="80"/>
+      <c r="FT1" s="80"/>
+      <c r="FU1" s="80"/>
+      <c r="FV1" s="80"/>
+      <c r="FW1" s="80"/>
+      <c r="FX1" s="80"/>
+      <c r="FY1" s="80"/>
+      <c r="FZ1" s="80"/>
+      <c r="GA1" s="80"/>
+      <c r="GB1" s="80"/>
+      <c r="GC1" s="80"/>
+      <c r="GD1" s="80"/>
+      <c r="GE1" s="80"/>
+      <c r="GF1" s="80"/>
+      <c r="GG1" s="80"/>
+      <c r="GH1" s="80"/>
+      <c r="GI1" s="81"/>
+      <c r="GJ1" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="GK1" s="78"/>
-      <c r="GL1" s="78"/>
-      <c r="GM1" s="79"/>
-      <c r="GN1" s="115" t="s">
+      <c r="GK1" s="50"/>
+      <c r="GL1" s="50"/>
+      <c r="GM1" s="51"/>
+      <c r="GN1" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="GO1" s="97" t="s">
+      <c r="GO1" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="GP1" s="83" t="s">
+      <c r="GP1" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="GQ1" s="83" t="s">
+      <c r="GQ1" s="55" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:199" s="12" customFormat="1" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="80"/>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="81"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
-      <c r="G2" s="81"/>
-      <c r="H2" s="81"/>
-      <c r="I2" s="81"/>
-      <c r="J2" s="81"/>
-      <c r="K2" s="81"/>
-      <c r="L2" s="81"/>
-      <c r="M2" s="82"/>
-      <c r="N2" s="86" t="s">
+      <c r="A2" s="52"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="53"/>
+      <c r="M2" s="54"/>
+      <c r="N2" s="120" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="87"/>
-      <c r="P2" s="87"/>
-      <c r="Q2" s="87"/>
-      <c r="R2" s="87"/>
-      <c r="S2" s="87"/>
-      <c r="T2" s="87"/>
-      <c r="U2" s="87"/>
-      <c r="V2" s="118" t="s">
+      <c r="O2" s="121"/>
+      <c r="P2" s="121"/>
+      <c r="Q2" s="121"/>
+      <c r="R2" s="121"/>
+      <c r="S2" s="121"/>
+      <c r="T2" s="121"/>
+      <c r="U2" s="122"/>
+      <c r="V2" s="115" t="s">
         <v>15</v>
       </c>
-      <c r="W2" s="119"/>
-      <c r="X2" s="119"/>
-      <c r="Y2" s="119"/>
-      <c r="Z2" s="119"/>
-      <c r="AA2" s="119"/>
-      <c r="AB2" s="119"/>
-      <c r="AC2" s="120"/>
-      <c r="AD2" s="70"/>
-      <c r="AE2" s="71"/>
-      <c r="AF2" s="71"/>
-      <c r="AG2" s="71"/>
-      <c r="AH2" s="71"/>
-      <c r="AI2" s="71"/>
-      <c r="AJ2" s="71"/>
-      <c r="AK2" s="72"/>
-      <c r="AL2" s="59"/>
-      <c r="AM2" s="60"/>
-      <c r="AN2" s="64"/>
-      <c r="AO2" s="65"/>
-      <c r="AP2" s="65"/>
-      <c r="AQ2" s="65"/>
-      <c r="AR2" s="66"/>
-      <c r="AS2" s="75"/>
-      <c r="AT2" s="76"/>
-      <c r="AU2" s="75"/>
-      <c r="AV2" s="125"/>
-      <c r="AW2" s="125"/>
-      <c r="AX2" s="125"/>
-      <c r="AY2" s="125"/>
-      <c r="AZ2" s="125"/>
-      <c r="BA2" s="125"/>
-      <c r="BB2" s="125"/>
-      <c r="BC2" s="125"/>
-      <c r="BD2" s="125"/>
-      <c r="BE2" s="125"/>
-      <c r="BF2" s="125"/>
-      <c r="BG2" s="125"/>
-      <c r="BH2" s="125"/>
-      <c r="BI2" s="125"/>
-      <c r="BJ2" s="125"/>
-      <c r="BK2" s="125"/>
-      <c r="BL2" s="125"/>
-      <c r="BM2" s="125"/>
-      <c r="BN2" s="125"/>
-      <c r="BO2" s="125"/>
-      <c r="BP2" s="125"/>
-      <c r="BQ2" s="125"/>
-      <c r="BR2" s="125"/>
-      <c r="BS2" s="125"/>
-      <c r="BT2" s="125"/>
-      <c r="BU2" s="125"/>
-      <c r="BV2" s="125"/>
-      <c r="BW2" s="125"/>
-      <c r="BX2" s="125"/>
-      <c r="BY2" s="125"/>
-      <c r="BZ2" s="125"/>
-      <c r="CA2" s="125"/>
-      <c r="CB2" s="125"/>
-      <c r="CC2" s="125"/>
-      <c r="CD2" s="76"/>
-      <c r="CE2" s="103"/>
-      <c r="CF2" s="104"/>
-      <c r="CG2" s="104"/>
-      <c r="CH2" s="104"/>
-      <c r="CI2" s="104"/>
-      <c r="CJ2" s="104"/>
-      <c r="CK2" s="104"/>
-      <c r="CL2" s="104"/>
-      <c r="CM2" s="104"/>
-      <c r="CN2" s="104"/>
-      <c r="CO2" s="104"/>
-      <c r="CP2" s="104"/>
-      <c r="CQ2" s="104"/>
-      <c r="CR2" s="104"/>
-      <c r="CS2" s="104"/>
-      <c r="CT2" s="104"/>
-      <c r="CU2" s="104"/>
-      <c r="CV2" s="104"/>
-      <c r="CW2" s="104"/>
-      <c r="CX2" s="104"/>
-      <c r="CY2" s="104"/>
-      <c r="CZ2" s="104"/>
-      <c r="DA2" s="104"/>
-      <c r="DB2" s="104"/>
-      <c r="DC2" s="104"/>
-      <c r="DD2" s="104"/>
-      <c r="DE2" s="104"/>
-      <c r="DF2" s="104"/>
-      <c r="DG2" s="104"/>
-      <c r="DH2" s="104"/>
-      <c r="DI2" s="104"/>
-      <c r="DJ2" s="104"/>
-      <c r="DK2" s="105"/>
-      <c r="DL2" s="109"/>
-      <c r="DM2" s="110"/>
-      <c r="DN2" s="110"/>
-      <c r="DO2" s="110"/>
-      <c r="DP2" s="110"/>
-      <c r="DQ2" s="110"/>
-      <c r="DR2" s="110"/>
-      <c r="DS2" s="110"/>
-      <c r="DT2" s="110"/>
-      <c r="DU2" s="110"/>
-      <c r="DV2" s="110"/>
-      <c r="DW2" s="110"/>
-      <c r="DX2" s="110"/>
-      <c r="DY2" s="110"/>
-      <c r="DZ2" s="111"/>
-      <c r="EA2" s="54"/>
-      <c r="EB2" s="55"/>
-      <c r="EC2" s="55"/>
-      <c r="ED2" s="55"/>
-      <c r="EE2" s="55"/>
-      <c r="EF2" s="55"/>
-      <c r="EG2" s="55"/>
-      <c r="EH2" s="55"/>
-      <c r="EI2" s="55"/>
-      <c r="EJ2" s="55"/>
-      <c r="EK2" s="55"/>
-      <c r="EL2" s="55"/>
-      <c r="EM2" s="55"/>
-      <c r="EN2" s="56"/>
-      <c r="EO2" s="51" t="s">
-        <v>242</v>
-      </c>
-      <c r="EP2" s="52"/>
-      <c r="EQ2" s="52"/>
-      <c r="ER2" s="52"/>
-      <c r="ES2" s="52"/>
-      <c r="ET2" s="52"/>
-      <c r="EU2" s="52"/>
-      <c r="EV2" s="52"/>
-      <c r="EW2" s="52"/>
-      <c r="EX2" s="52"/>
-      <c r="EY2" s="52"/>
-      <c r="EZ2" s="52"/>
-      <c r="FA2" s="53"/>
-      <c r="FB2" s="88" t="s">
+      <c r="W2" s="116"/>
+      <c r="X2" s="116"/>
+      <c r="Y2" s="116"/>
+      <c r="Z2" s="116"/>
+      <c r="AA2" s="116"/>
+      <c r="AB2" s="116"/>
+      <c r="AC2" s="117"/>
+      <c r="AD2" s="110"/>
+      <c r="AE2" s="111"/>
+      <c r="AF2" s="111"/>
+      <c r="AG2" s="111"/>
+      <c r="AH2" s="111"/>
+      <c r="AI2" s="111"/>
+      <c r="AJ2" s="111"/>
+      <c r="AK2" s="112"/>
+      <c r="AL2" s="99"/>
+      <c r="AM2" s="100"/>
+      <c r="AN2" s="104"/>
+      <c r="AO2" s="105"/>
+      <c r="AP2" s="105"/>
+      <c r="AQ2" s="105"/>
+      <c r="AR2" s="106"/>
+      <c r="AS2" s="88"/>
+      <c r="AT2" s="90"/>
+      <c r="AU2" s="88"/>
+      <c r="AV2" s="89"/>
+      <c r="AW2" s="89"/>
+      <c r="AX2" s="89"/>
+      <c r="AY2" s="89"/>
+      <c r="AZ2" s="89"/>
+      <c r="BA2" s="89"/>
+      <c r="BB2" s="89"/>
+      <c r="BC2" s="89"/>
+      <c r="BD2" s="89"/>
+      <c r="BE2" s="89"/>
+      <c r="BF2" s="89"/>
+      <c r="BG2" s="89"/>
+      <c r="BH2" s="89"/>
+      <c r="BI2" s="89"/>
+      <c r="BJ2" s="89"/>
+      <c r="BK2" s="89"/>
+      <c r="BL2" s="89"/>
+      <c r="BM2" s="89"/>
+      <c r="BN2" s="89"/>
+      <c r="BO2" s="89"/>
+      <c r="BP2" s="89"/>
+      <c r="BQ2" s="89"/>
+      <c r="BR2" s="89"/>
+      <c r="BS2" s="89"/>
+      <c r="BT2" s="89"/>
+      <c r="BU2" s="89"/>
+      <c r="BV2" s="89"/>
+      <c r="BW2" s="89"/>
+      <c r="BX2" s="89"/>
+      <c r="BY2" s="89"/>
+      <c r="BZ2" s="89"/>
+      <c r="CA2" s="89"/>
+      <c r="CB2" s="89"/>
+      <c r="CC2" s="89"/>
+      <c r="CD2" s="90"/>
+      <c r="CE2" s="70"/>
+      <c r="CF2" s="71"/>
+      <c r="CG2" s="71"/>
+      <c r="CH2" s="71"/>
+      <c r="CI2" s="71"/>
+      <c r="CJ2" s="71"/>
+      <c r="CK2" s="71"/>
+      <c r="CL2" s="71"/>
+      <c r="CM2" s="71"/>
+      <c r="CN2" s="71"/>
+      <c r="CO2" s="71"/>
+      <c r="CP2" s="71"/>
+      <c r="CQ2" s="71"/>
+      <c r="CR2" s="71"/>
+      <c r="CS2" s="71"/>
+      <c r="CT2" s="71"/>
+      <c r="CU2" s="71"/>
+      <c r="CV2" s="71"/>
+      <c r="CW2" s="71"/>
+      <c r="CX2" s="71"/>
+      <c r="CY2" s="71"/>
+      <c r="CZ2" s="71"/>
+      <c r="DA2" s="71"/>
+      <c r="DB2" s="71"/>
+      <c r="DC2" s="71"/>
+      <c r="DD2" s="71"/>
+      <c r="DE2" s="71"/>
+      <c r="DF2" s="71"/>
+      <c r="DG2" s="71"/>
+      <c r="DH2" s="71"/>
+      <c r="DI2" s="71"/>
+      <c r="DJ2" s="71"/>
+      <c r="DK2" s="72"/>
+      <c r="DL2" s="76"/>
+      <c r="DM2" s="77"/>
+      <c r="DN2" s="77"/>
+      <c r="DO2" s="77"/>
+      <c r="DP2" s="77"/>
+      <c r="DQ2" s="77"/>
+      <c r="DR2" s="77"/>
+      <c r="DS2" s="77"/>
+      <c r="DT2" s="77"/>
+      <c r="DU2" s="77"/>
+      <c r="DV2" s="77"/>
+      <c r="DW2" s="77"/>
+      <c r="DX2" s="77"/>
+      <c r="DY2" s="77"/>
+      <c r="DZ2" s="78"/>
+      <c r="EA2" s="94"/>
+      <c r="EB2" s="95"/>
+      <c r="EC2" s="95"/>
+      <c r="ED2" s="95"/>
+      <c r="EE2" s="95"/>
+      <c r="EF2" s="95"/>
+      <c r="EG2" s="95"/>
+      <c r="EH2" s="95"/>
+      <c r="EI2" s="95"/>
+      <c r="EJ2" s="95"/>
+      <c r="EK2" s="95"/>
+      <c r="EL2" s="95"/>
+      <c r="EM2" s="95"/>
+      <c r="EN2" s="96"/>
+      <c r="EO2" s="91" t="s">
+        <v>239</v>
+      </c>
+      <c r="EP2" s="92"/>
+      <c r="EQ2" s="92"/>
+      <c r="ER2" s="92"/>
+      <c r="ES2" s="92"/>
+      <c r="ET2" s="92"/>
+      <c r="EU2" s="92"/>
+      <c r="EV2" s="92"/>
+      <c r="EW2" s="92"/>
+      <c r="EX2" s="92"/>
+      <c r="EY2" s="92"/>
+      <c r="EZ2" s="92"/>
+      <c r="FA2" s="93"/>
+      <c r="FB2" s="129" t="s">
         <v>16</v>
       </c>
-      <c r="FC2" s="89"/>
-      <c r="FD2" s="89"/>
-      <c r="FE2" s="89"/>
-      <c r="FF2" s="89"/>
-      <c r="FG2" s="89"/>
-      <c r="FH2" s="89"/>
-      <c r="FI2" s="89"/>
-      <c r="FJ2" s="89"/>
-      <c r="FK2" s="89"/>
-      <c r="FL2" s="89"/>
-      <c r="FM2" s="89"/>
-      <c r="FN2" s="89"/>
-      <c r="FO2" s="89"/>
-      <c r="FP2" s="89"/>
-      <c r="FQ2" s="89"/>
-      <c r="FR2" s="90"/>
-      <c r="FS2" s="91" t="s">
+      <c r="FC2" s="130"/>
+      <c r="FD2" s="130"/>
+      <c r="FE2" s="130"/>
+      <c r="FF2" s="130"/>
+      <c r="FG2" s="130"/>
+      <c r="FH2" s="130"/>
+      <c r="FI2" s="130"/>
+      <c r="FJ2" s="130"/>
+      <c r="FK2" s="130"/>
+      <c r="FL2" s="130"/>
+      <c r="FM2" s="130"/>
+      <c r="FN2" s="130"/>
+      <c r="FO2" s="130"/>
+      <c r="FP2" s="130"/>
+      <c r="FQ2" s="130"/>
+      <c r="FR2" s="131"/>
+      <c r="FS2" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="FT2" s="92"/>
-      <c r="FU2" s="92"/>
-      <c r="FV2" s="92"/>
-      <c r="FW2" s="92"/>
-      <c r="FX2" s="92"/>
-      <c r="FY2" s="92"/>
-      <c r="FZ2" s="92"/>
-      <c r="GA2" s="92"/>
-      <c r="GB2" s="93"/>
-      <c r="GC2" s="94" t="s">
+      <c r="FT2" s="59"/>
+      <c r="FU2" s="59"/>
+      <c r="FV2" s="59"/>
+      <c r="FW2" s="59"/>
+      <c r="FX2" s="59"/>
+      <c r="FY2" s="59"/>
+      <c r="FZ2" s="59"/>
+      <c r="GA2" s="59"/>
+      <c r="GB2" s="60"/>
+      <c r="GC2" s="61" t="s">
         <v>18</v>
       </c>
-      <c r="GD2" s="95"/>
-      <c r="GE2" s="95"/>
-      <c r="GF2" s="95"/>
-      <c r="GG2" s="95"/>
-      <c r="GH2" s="95"/>
-      <c r="GI2" s="96"/>
-      <c r="GJ2" s="80"/>
-      <c r="GK2" s="81"/>
-      <c r="GL2" s="81"/>
-      <c r="GM2" s="82"/>
-      <c r="GN2" s="116"/>
-      <c r="GO2" s="98"/>
-      <c r="GP2" s="84"/>
-      <c r="GQ2" s="84"/>
+      <c r="GD2" s="62"/>
+      <c r="GE2" s="62"/>
+      <c r="GF2" s="62"/>
+      <c r="GG2" s="62"/>
+      <c r="GH2" s="62"/>
+      <c r="GI2" s="63"/>
+      <c r="GJ2" s="52"/>
+      <c r="GK2" s="53"/>
+      <c r="GL2" s="53"/>
+      <c r="GM2" s="54"/>
+      <c r="GN2" s="83"/>
+      <c r="GO2" s="65"/>
+      <c r="GP2" s="56"/>
+      <c r="GQ2" s="56"/>
     </row>
     <row r="3" spans="1:199" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>203</v>
+        <v>240</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>21</v>
@@ -3678,11 +3756,11 @@
       <c r="L3" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="M3" s="30" t="s">
+      <c r="M3" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="N3" s="39" t="s">
-        <v>189</v>
+      <c r="N3" s="38" t="s">
+        <v>187</v>
       </c>
       <c r="O3" s="22" t="s">
         <v>62</v>
@@ -3694,42 +3772,42 @@
         <v>64</v>
       </c>
       <c r="R3" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="S3" s="22" t="s">
+        <v>184</v>
+      </c>
+      <c r="T3" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="U3" s="123" t="s">
+        <v>65</v>
+      </c>
+      <c r="V3" s="118" t="s">
+        <v>187</v>
+      </c>
+      <c r="W3" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="X3" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y3" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="S3" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="T3" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="U3" s="22" t="s">
+      <c r="Z3" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="AA3" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="V3" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="W3" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="X3" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="Y3" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="Z3" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="AA3" s="24" t="s">
-        <v>65</v>
-      </c>
-      <c r="AB3" s="24" t="s">
-        <v>186</v>
-      </c>
-      <c r="AC3" s="40" t="s">
-        <v>187</v>
-      </c>
-      <c r="AD3" s="35" t="s">
+      <c r="AB3" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="AC3" s="39" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD3" s="34" t="s">
         <v>179</v>
       </c>
       <c r="AE3" s="17" t="s">
@@ -3739,7 +3817,7 @@
         <v>36</v>
       </c>
       <c r="AG3" s="17" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AH3" s="17" t="s">
         <v>37</v>
@@ -3748,18 +3826,18 @@
         <v>38</v>
       </c>
       <c r="AJ3" s="17" t="s">
-        <v>210</v>
-      </c>
-      <c r="AK3" s="36" t="s">
+        <v>207</v>
+      </c>
+      <c r="AK3" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="AL3" s="31" t="s">
+      <c r="AL3" s="30" t="s">
         <v>31</v>
       </c>
-      <c r="AM3" s="32" t="s">
+      <c r="AM3" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="AN3" s="33" t="s">
+      <c r="AN3" s="32" t="s">
         <v>178</v>
       </c>
       <c r="AO3" s="16" t="s">
@@ -3771,16 +3849,16 @@
       <c r="AQ3" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="AR3" s="34" t="s">
+      <c r="AR3" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="AS3" s="37" t="s">
+      <c r="AS3" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="AT3" s="29" t="s">
+      <c r="AT3" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="AU3" s="28" t="s">
+      <c r="AU3" s="27" t="s">
         <v>42</v>
       </c>
       <c r="AV3" s="18" t="s">
@@ -3885,10 +3963,10 @@
       <c r="CC3" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="CD3" s="38" t="s">
+      <c r="CD3" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="CE3" s="28" t="s">
+      <c r="CE3" s="27" t="s">
         <v>50</v>
       </c>
       <c r="CF3" s="19" t="s">
@@ -3984,10 +4062,10 @@
       <c r="DJ3" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="DK3" s="29" t="s">
+      <c r="DK3" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="DL3" s="28" t="s">
+      <c r="DL3" s="27" t="s">
         <v>59</v>
       </c>
       <c r="DM3" s="18" t="s">
@@ -4029,37 +4107,37 @@
       <c r="DY3" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="DZ3" s="29" t="s">
+      <c r="DZ3" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="EA3" s="41" t="s">
+      <c r="EA3" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="EB3" s="25" t="s">
+      <c r="EB3" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="EC3" s="25" t="s">
+      <c r="EC3" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="ED3" s="25" t="s">
+      <c r="ED3" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="EE3" s="25" t="s">
+      <c r="EE3" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="EF3" s="25" t="s">
+      <c r="EF3" s="24" t="s">
         <v>70</v>
       </c>
-      <c r="EG3" s="25" t="s">
+      <c r="EG3" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="EH3" s="26" t="s">
+      <c r="EH3" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="EI3" s="25" t="s">
+      <c r="EI3" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="EJ3" s="25" t="s">
+      <c r="EJ3" s="24" t="s">
         <v>74</v>
       </c>
       <c r="EK3" s="14" t="s">
@@ -4071,100 +4149,100 @@
       <c r="EM3" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="EN3" s="14" t="s">
+      <c r="EN3" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="EO3" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="EP3" s="49" t="s">
+      <c r="EO3" s="124" t="s">
+        <v>229</v>
+      </c>
+      <c r="EP3" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="EQ3" s="49" t="s">
-        <v>233</v>
-      </c>
-      <c r="ER3" s="49" t="s">
-        <v>231</v>
-      </c>
-      <c r="ES3" s="50" t="s">
+      <c r="EQ3" s="47" t="s">
         <v>230</v>
       </c>
-      <c r="ET3" s="49" t="s">
+      <c r="ER3" s="47" t="s">
+        <v>228</v>
+      </c>
+      <c r="ES3" s="48" t="s">
+        <v>227</v>
+      </c>
+      <c r="ET3" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="EU3" s="49" t="s">
-        <v>233</v>
-      </c>
-      <c r="EV3" s="49" t="s">
-        <v>231</v>
-      </c>
-      <c r="EW3" s="50" t="s">
+      <c r="EU3" s="47" t="s">
         <v>230</v>
       </c>
-      <c r="EX3" s="49" t="s">
+      <c r="EV3" s="47" t="s">
+        <v>228</v>
+      </c>
+      <c r="EW3" s="48" t="s">
+        <v>227</v>
+      </c>
+      <c r="EX3" s="47" t="s">
         <v>51</v>
       </c>
-      <c r="EY3" s="49" t="s">
-        <v>233</v>
-      </c>
-      <c r="EZ3" s="49" t="s">
-        <v>231</v>
-      </c>
-      <c r="FA3" s="50" t="s">
+      <c r="EY3" s="47" t="s">
         <v>230</v>
       </c>
-      <c r="FB3" s="41" t="s">
+      <c r="EZ3" s="47" t="s">
+        <v>228</v>
+      </c>
+      <c r="FA3" s="48" t="s">
+        <v>227</v>
+      </c>
+      <c r="FB3" s="125" t="s">
         <v>80</v>
       </c>
-      <c r="FC3" s="14" t="s">
+      <c r="FC3" s="126" t="s">
         <v>81</v>
       </c>
-      <c r="FD3" s="14" t="s">
+      <c r="FD3" s="126" t="s">
         <v>51</v>
       </c>
-      <c r="FE3" s="14" t="s">
+      <c r="FE3" s="126" t="s">
         <v>82</v>
       </c>
-      <c r="FF3" s="15" t="s">
+      <c r="FF3" s="127" t="s">
         <v>83</v>
       </c>
-      <c r="FG3" s="14" t="s">
+      <c r="FG3" s="126" t="s">
         <v>84</v>
       </c>
-      <c r="FH3" s="14" t="s">
+      <c r="FH3" s="126" t="s">
         <v>10</v>
       </c>
-      <c r="FI3" s="14" t="s">
+      <c r="FI3" s="126" t="s">
         <v>51</v>
       </c>
-      <c r="FJ3" s="14" t="s">
+      <c r="FJ3" s="126" t="s">
         <v>82</v>
       </c>
-      <c r="FK3" s="15" t="s">
+      <c r="FK3" s="127" t="s">
         <v>83</v>
       </c>
-      <c r="FL3" s="14" t="s">
+      <c r="FL3" s="126" t="s">
         <v>84</v>
       </c>
-      <c r="FM3" s="14" t="s">
+      <c r="FM3" s="126" t="s">
         <v>10</v>
       </c>
-      <c r="FN3" s="14" t="s">
+      <c r="FN3" s="126" t="s">
         <v>51</v>
       </c>
-      <c r="FO3" s="14" t="s">
+      <c r="FO3" s="126" t="s">
         <v>82</v>
       </c>
-      <c r="FP3" s="15" t="s">
+      <c r="FP3" s="127" t="s">
         <v>83</v>
       </c>
-      <c r="FQ3" s="14" t="s">
+      <c r="FQ3" s="126" t="s">
         <v>84</v>
       </c>
-      <c r="FR3" s="30" t="s">
+      <c r="FR3" s="128" t="s">
         <v>10</v>
       </c>
-      <c r="FS3" s="35" t="s">
+      <c r="FS3" s="34" t="s">
         <v>52</v>
       </c>
       <c r="FT3" s="17" t="s">
@@ -4191,31 +4269,31 @@
       <c r="GA3" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="GB3" s="36" t="s">
+      <c r="GB3" s="35" t="s">
         <v>93</v>
       </c>
-      <c r="GC3" s="42" t="s">
+      <c r="GC3" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="GD3" s="27" t="s">
+      <c r="GD3" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="GE3" s="27" t="s">
+      <c r="GE3" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="GF3" s="27" t="s">
+      <c r="GF3" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="GG3" s="27" t="s">
+      <c r="GG3" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="GH3" s="27" t="s">
+      <c r="GH3" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="GI3" s="43" t="s">
+      <c r="GI3" s="42" t="s">
         <v>100</v>
       </c>
-      <c r="GJ3" s="41" t="s">
+      <c r="GJ3" s="40" t="s">
         <v>101</v>
       </c>
       <c r="GK3" s="14" t="s">
@@ -4224,13 +4302,13 @@
       <c r="GL3" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="GM3" s="44" t="s">
+      <c r="GM3" s="43" t="s">
         <v>102</v>
       </c>
-      <c r="GN3" s="117"/>
-      <c r="GO3" s="99"/>
-      <c r="GP3" s="85"/>
-      <c r="GQ3" s="85"/>
+      <c r="GN3" s="84"/>
+      <c r="GO3" s="66"/>
+      <c r="GP3" s="57"/>
+      <c r="GQ3" s="57"/>
     </row>
     <row r="4" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -4244,7 +4322,7 @@
       <c r="F4" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="46">
         <v>35626</v>
       </c>
       <c r="H4" s="5" t="s">
@@ -4263,20 +4341,20 @@
       <c r="O4" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="P4" s="47">
+      <c r="P4" s="46">
         <v>35626</v>
       </c>
-      <c r="Q4" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="R4" s="47" t="s">
+      <c r="Q4" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="R4" s="46" t="s">
         <v>103</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U4" s="5" t="s">
         <v>174</v>
@@ -4287,13 +4365,13 @@
       <c r="W4" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="X4" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="Y4" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="Z4" s="47" t="s">
+      <c r="X4" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y4" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z4" s="46" t="s">
         <v>103</v>
       </c>
       <c r="AA4" s="4" t="s">
@@ -4306,32 +4384,32 @@
         <v>103</v>
       </c>
       <c r="AD4" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="AE4" s="5" t="s">
-        <v>185</v>
+        <v>247</v>
       </c>
       <c r="AF4" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="AG4" s="45">
+        <v>201</v>
+      </c>
+      <c r="AG4" s="44">
         <v>2327.2600000000002</v>
       </c>
       <c r="AH4" s="5" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="AI4" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AJ4" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AK4" s="6"/>
       <c r="AL4" s="5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="AM4" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="AN4" s="5" t="s">
         <v>103</v>
@@ -4345,13 +4423,13 @@
         <v>12683.75</v>
       </c>
       <c r="AS4" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AT4" s="5" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="EA4" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="EO4" s="5" t="s">
         <v>103</v>
@@ -4402,33 +4480,33 @@
         <v>45300</v>
       </c>
       <c r="FF4" s="4" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="FG4" s="5" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="FH4" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="FI4" s="5">
         <v>2</v>
       </c>
-      <c r="FJ4" s="47">
+      <c r="FJ4" s="46">
         <v>44851</v>
       </c>
       <c r="FK4" s="4" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="FL4" s="5" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="FM4" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="FN4" s="5">
         <v>3</v>
       </c>
-      <c r="FO4" s="47" t="s">
+      <c r="FO4" s="46" t="s">
         <v>103</v>
       </c>
       <c r="FP4" s="4" t="s">
@@ -4438,7 +4516,7 @@
         <v>103</v>
       </c>
       <c r="FR4" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4451,16 +4529,16 @@
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="G5" s="46">
+        <v>26632</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>190</v>
-      </c>
-      <c r="G5" s="7">
-        <v>26632</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>192</v>
       </c>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
@@ -4472,106 +4550,106 @@
       <c r="O5" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="P5" s="47">
+      <c r="P5" s="46">
         <v>26632</v>
       </c>
-      <c r="Q5" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="R5" s="47" t="s">
+      <c r="Q5" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="R5" s="46" t="s">
         <v>103</v>
       </c>
       <c r="S5" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="T5" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="U5" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="V5" s="4" t="s">
         <v>193</v>
-      </c>
-      <c r="T5" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="U5" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="V5" s="4" t="s">
-        <v>195</v>
       </c>
       <c r="W5" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="X5" s="47">
+      <c r="X5" s="46">
         <v>43067</v>
       </c>
-      <c r="Y5" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="Z5" s="47">
+      <c r="Y5" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z5" s="46">
         <v>43273</v>
       </c>
       <c r="AA5" s="5" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AC5" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AD5" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="AE5" s="5" t="s">
-        <v>181</v>
+        <v>246</v>
       </c>
       <c r="AF5" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AG5" s="45">
+      <c r="AG5" s="44">
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="AI5" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="AI5" s="5" t="s">
-        <v>209</v>
-      </c>
       <c r="AJ5" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AK5" s="6"/>
       <c r="AL5" s="5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="AM5" s="5" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="AN5" s="5" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
       <c r="AQ5" s="5" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="AR5" s="9">
         <v>0</v>
       </c>
-      <c r="AS5" s="46"/>
-      <c r="AT5" s="46"/>
+      <c r="AS5" s="45"/>
+      <c r="AT5" s="45"/>
       <c r="EA5" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="EO5" s="5">
         <v>1</v>
       </c>
       <c r="EP5" s="4" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="EQ5" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="ER5" s="47">
+        <v>237</v>
+      </c>
+      <c r="ER5" s="46">
         <v>46038</v>
       </c>
       <c r="ES5" s="4" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="ET5" s="4" t="s">
         <v>103</v>
@@ -4607,58 +4685,58 @@
         <v>46157</v>
       </c>
       <c r="FF5" s="4" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="FG5" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="FH5" s="5" t="s">
         <v>219</v>
-      </c>
-      <c r="FH5" s="5" t="s">
-        <v>222</v>
       </c>
       <c r="FI5" s="5">
         <v>2</v>
       </c>
-      <c r="FJ5" s="47">
+      <c r="FJ5" s="46">
         <v>46090</v>
       </c>
       <c r="FK5" s="4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="FL5" s="5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="FM5" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="FN5" s="5">
         <v>3</v>
       </c>
-      <c r="FO5" s="47">
+      <c r="FO5" s="46">
         <v>46051</v>
       </c>
       <c r="FP5" s="4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="FQ5" s="5" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="FR5" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="G6" s="7">
+        <v>204</v>
+      </c>
+      <c r="G6" s="46">
         <v>43543</v>
       </c>
       <c r="H6" s="5" t="s">
@@ -4672,28 +4750,28 @@
       <c r="L6" s="6"/>
       <c r="M6" s="6"/>
       <c r="N6" s="5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="O6" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="P6" s="47">
+      <c r="P6" s="46">
         <v>43543</v>
       </c>
-      <c r="Q6" s="47">
+      <c r="Q6" s="46">
         <v>44255</v>
       </c>
-      <c r="R6" s="47">
+      <c r="R6" s="46">
         <v>45426</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="V6" s="4" t="s">
         <v>103</v>
@@ -4701,13 +4779,13 @@
       <c r="W6" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="X6" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="Y6" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="Z6" s="47" t="s">
+      <c r="X6" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y6" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z6" s="46" t="s">
         <v>103</v>
       </c>
       <c r="AA6" s="4" t="s">
@@ -4720,29 +4798,29 @@
         <v>103</v>
       </c>
       <c r="AD6" s="5" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="AE6" s="4" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="AF6" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="AG6" s="45">
+      <c r="AG6" s="44">
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="AI6" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AJ6" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="AK6" s="6"/>
       <c r="AL6" s="5" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="AM6" s="5" t="s">
         <v>103</v>
@@ -4758,10 +4836,10 @@
       <c r="AR6" s="9">
         <v>0</v>
       </c>
-      <c r="AS6" s="46"/>
-      <c r="AT6" s="46"/>
+      <c r="AS6" s="45"/>
+      <c r="AT6" s="45"/>
       <c r="EA6" s="5" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="EO6" s="5" t="s">
         <v>103</v>
@@ -4826,7 +4904,7 @@
       <c r="FI6" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="FJ6" s="47" t="s">
+      <c r="FJ6" s="46" t="s">
         <v>103</v>
       </c>
       <c r="FK6" s="5" t="s">
@@ -4841,7 +4919,7 @@
       <c r="FN6" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="FO6" s="47" t="s">
+      <c r="FO6" s="46" t="s">
         <v>103</v>
       </c>
       <c r="FP6" s="5" t="s">
@@ -4856,10 +4934,76 @@
     </row>
     <row r="7" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>228</v>
+        <v>225</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="G7" s="46">
+        <v>39694</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="P7" s="46">
+        <v>39694</v>
+      </c>
+      <c r="Q7" s="46">
+        <v>45139</v>
+      </c>
+      <c r="R7" s="46">
+        <v>43469</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="T7" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="U7" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="V7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="W7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="X7" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y7" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z7" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="AA7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="AB7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="AC7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="AD7" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="AE7" s="5" t="s">
+        <v>245</v>
       </c>
       <c r="EO7" s="5">
         <v>2</v>
@@ -4868,42 +5012,48 @@
         <v>1</v>
       </c>
       <c r="EQ7" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="ER7" s="46" t="s">
+        <v>233</v>
+      </c>
+      <c r="ES7" s="4" t="s">
         <v>234</v>
-      </c>
-      <c r="ER7" s="47" t="s">
-        <v>236</v>
-      </c>
-      <c r="ES7" s="4" t="s">
-        <v>237</v>
       </c>
       <c r="ET7" s="4">
         <v>2</v>
       </c>
       <c r="EU7" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="EV7" s="46">
+        <v>46146</v>
+      </c>
+      <c r="EW7" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="EV7" s="47">
-        <v>46146</v>
-      </c>
-      <c r="EW7" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="EX7" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="EY7" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="EZ7" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="FA7" s="47" t="s">
+      <c r="EX7" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="EY7" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="EZ7" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="FA7" s="46" t="s">
         <v>103</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:GQ5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="22">
+    <mergeCell ref="EO2:FA2"/>
+    <mergeCell ref="EA2:EN2"/>
+    <mergeCell ref="AL1:AM2"/>
+    <mergeCell ref="AN1:AR2"/>
+    <mergeCell ref="AD1:AK2"/>
+    <mergeCell ref="AS1:AT2"/>
     <mergeCell ref="A1:M2"/>
     <mergeCell ref="GP1:GP3"/>
     <mergeCell ref="GQ1:GQ3"/>
@@ -4920,12 +5070,6 @@
     <mergeCell ref="N1:AC1"/>
     <mergeCell ref="GJ1:GM2"/>
     <mergeCell ref="AU1:CD2"/>
-    <mergeCell ref="EO2:FA2"/>
-    <mergeCell ref="EA2:EN2"/>
-    <mergeCell ref="AL1:AM2"/>
-    <mergeCell ref="AN1:AR2"/>
-    <mergeCell ref="AD1:AK2"/>
-    <mergeCell ref="AS1:AT2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A7:B1048576 A3:A6">
     <cfRule type="duplicateValues" dxfId="0" priority="142"/>

</xml_diff>

<commit_message>
SRI Estado Tributario completo: fix acordeon colapsado (mat-expansion-panel) que ocultaba la tabla de obligaciones pendientes, agregar captura de evidencia. Fix dato de prueba incorrecto en script (RUC en vez de cedula) que causaba carpeta de evidencia duplicada
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB8E6754-2937-4FE8-AF7C-EA74C99B2B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F26087E-CA5B-4C71-A6E6-D14CAD21DE55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Revision" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Revision!$A$3:$GQ$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Revision!$A$3:$GN$5</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -284,7 +284,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="FW3" authorId="1" shapeId="0" xr:uid="{4B658DD9-EA7C-4527-82E1-C9110A8EA055}">
+    <comment ref="FT3" authorId="1" shapeId="0" xr:uid="{4B658DD9-EA7C-4527-82E1-C9110A8EA055}">
       <text>
         <r>
           <rPr>
@@ -343,7 +343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="252">
   <si>
     <t>IDENTIFICACIÓN BÁSICA</t>
   </si>
@@ -563,9 +563,6 @@
     <t>Último año en el cargo</t>
   </si>
   <si>
-    <t>Remuneración</t>
-  </si>
-  <si>
     <t>Es PEP</t>
   </si>
   <si>
@@ -578,12 +575,6 @@
     <t>Impedimento salida del país</t>
   </si>
   <si>
-    <t>Empresas Fantasmas</t>
-  </si>
-  <si>
-    <t>Empresas Fantasmas Relacionados</t>
-  </si>
-  <si>
     <t>Sentenciados</t>
   </si>
   <si>
@@ -605,9 +596,6 @@
     <t>REGISTRO CIVIL</t>
   </si>
   <si>
-    <t>CNT</t>
-  </si>
-  <si>
     <t>CNE (Residencia Extranjera)</t>
   </si>
   <si>
@@ -1089,6 +1077,30 @@
   </si>
   <si>
     <t>ANEXO TRANSACCIONAL SIMPLIFICADO JUNIO 2026</t>
+  </si>
+  <si>
+    <t>Vigente Actual - 3 (2026 - 2024) !Desactualizados</t>
+  </si>
+  <si>
+    <t>Si esta dentro de la categoria es PEPS</t>
+  </si>
+  <si>
+    <t>Registro SI/NO</t>
+  </si>
+  <si>
+    <t>TIEMPO QUE HA EJERCIDO EL ULTIMO CARGO</t>
+  </si>
+  <si>
+    <t>ULTIMO DE LA LISTA</t>
+  </si>
+  <si>
+    <t>CARGO + ENTIDAD</t>
+  </si>
+  <si>
+    <t>Remuneración APROX.</t>
+  </si>
+  <si>
+    <t>resumene AI</t>
   </si>
 </sst>
 </file>
@@ -1813,7 +1825,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2098,9 +2110,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2204,6 +2213,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2799,250 +2817,250 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C2" t="s">
         <v>108</v>
-      </c>
-      <c r="C2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" t="s">
         <v>109</v>
-      </c>
-      <c r="C3" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" t="s">
         <v>110</v>
-      </c>
-      <c r="C4" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C5" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C8" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C9" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C10" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C11" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C13" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C14" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C15" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C17" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C18" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C21" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C22" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -3079,7 +3097,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3838F483-03F0-4F1D-B50C-3B9C5206BD2F}">
-  <dimension ref="A1:GQ7"/>
+  <dimension ref="A1:GN7"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="70.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" style="4" bestFit="1" customWidth="1"/>
@@ -3222,60 +3240,57 @@
     <col min="140" max="140" width="25.5546875" style="5" bestFit="1" customWidth="1"/>
     <col min="141" max="141" width="22.5546875" style="5" bestFit="1" customWidth="1"/>
     <col min="142" max="142" width="24.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="143" max="143" width="16.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="144" max="144" width="19.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="145" max="145" width="19.109375" style="5" customWidth="1"/>
-    <col min="146" max="147" width="19.109375" style="4" customWidth="1"/>
-    <col min="148" max="148" width="19.109375" style="46" customWidth="1"/>
-    <col min="149" max="151" width="19.109375" style="4" customWidth="1"/>
-    <col min="152" max="152" width="19.109375" style="46" customWidth="1"/>
-    <col min="153" max="155" width="19.109375" style="4" customWidth="1"/>
-    <col min="156" max="156" width="19.109375" style="46" customWidth="1"/>
-    <col min="157" max="157" width="18.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="158" max="158" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="159" max="159" width="21.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="160" max="160" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="161" max="161" width="22.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="162" max="162" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="163" max="163" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="164" max="164" width="20.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="165" max="165" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="166" max="166" width="22.21875" style="46" bestFit="1" customWidth="1"/>
-    <col min="167" max="167" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="168" max="168" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="169" max="169" width="20.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="170" max="170" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="171" max="171" width="22.21875" style="46" bestFit="1" customWidth="1"/>
-    <col min="172" max="172" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="173" max="173" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="174" max="174" width="20.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="175" max="175" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="176" max="176" width="24.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="177" max="177" width="10.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="178" max="178" width="22.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="179" max="179" width="15.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="180" max="180" width="22.77734375" style="5" bestFit="1" customWidth="1"/>
-    <col min="181" max="181" width="16.21875" style="5" bestFit="1" customWidth="1"/>
-    <col min="182" max="182" width="21.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="183" max="183" width="28.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="184" max="184" width="28.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="185" max="185" width="12.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="186" max="186" width="11.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="187" max="187" width="15.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="188" max="188" width="13.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="189" max="189" width="23.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="190" max="190" width="25.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="191" max="191" width="28.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="192" max="194" width="11.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="195" max="195" width="21.109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="196" max="196" width="15" style="5" bestFit="1" customWidth="1"/>
-    <col min="197" max="197" width="17.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="198" max="198" width="6.88671875" style="11" bestFit="1" customWidth="1"/>
-    <col min="199" max="199" width="9.88671875" style="11" bestFit="1" customWidth="1"/>
-    <col min="200" max="16384" width="11.44140625" style="5"/>
+    <col min="143" max="143" width="19.109375" style="5" customWidth="1"/>
+    <col min="144" max="145" width="19.109375" style="4" customWidth="1"/>
+    <col min="146" max="146" width="19.109375" style="46" customWidth="1"/>
+    <col min="147" max="149" width="19.109375" style="4" customWidth="1"/>
+    <col min="150" max="150" width="19.109375" style="46" customWidth="1"/>
+    <col min="151" max="153" width="19.109375" style="4" customWidth="1"/>
+    <col min="154" max="154" width="19.109375" style="46" customWidth="1"/>
+    <col min="155" max="155" width="18.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="156" max="156" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="157" max="157" width="21.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="158" max="158" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="159" max="159" width="22.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="160" max="160" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="161" max="161" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="162" max="162" width="20.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="163" max="163" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="164" max="164" width="22.21875" style="46" bestFit="1" customWidth="1"/>
+    <col min="165" max="165" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="166" max="166" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="167" max="167" width="20.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="168" max="168" width="9.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="169" max="169" width="22.21875" style="46" bestFit="1" customWidth="1"/>
+    <col min="170" max="170" width="17.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="171" max="171" width="23.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="172" max="172" width="20.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="173" max="173" width="19.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="174" max="174" width="24.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="175" max="175" width="22.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="176" max="176" width="15.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="177" max="177" width="22.77734375" style="5" bestFit="1" customWidth="1"/>
+    <col min="178" max="178" width="16.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="179" max="179" width="21.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="180" max="180" width="28.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="181" max="181" width="28.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="182" max="182" width="12.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="183" max="183" width="11.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="184" max="184" width="15.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="185" max="185" width="13.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="186" max="186" width="23.33203125" style="5" bestFit="1" customWidth="1"/>
+    <col min="187" max="187" width="25.5546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="188" max="188" width="28.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="189" max="191" width="11.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="192" max="192" width="21.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="193" max="193" width="15" style="5" bestFit="1" customWidth="1"/>
+    <col min="194" max="194" width="17.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="195" max="195" width="6.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="196" max="196" width="9.88671875" style="11" bestFit="1" customWidth="1"/>
+    <col min="197" max="16384" width="11.44140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:199" s="12" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:196" s="12" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
@@ -3291,45 +3306,45 @@
       <c r="K1" s="50"/>
       <c r="L1" s="50"/>
       <c r="M1" s="51"/>
-      <c r="N1" s="119" t="s">
+      <c r="N1" s="118" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="113"/>
-      <c r="P1" s="113"/>
-      <c r="Q1" s="113"/>
-      <c r="R1" s="113"/>
-      <c r="S1" s="113"/>
-      <c r="T1" s="113"/>
-      <c r="U1" s="113"/>
-      <c r="V1" s="113"/>
-      <c r="W1" s="113"/>
-      <c r="X1" s="113"/>
-      <c r="Y1" s="113"/>
-      <c r="Z1" s="113"/>
-      <c r="AA1" s="113"/>
-      <c r="AB1" s="113"/>
-      <c r="AC1" s="114"/>
-      <c r="AD1" s="107" t="s">
+      <c r="O1" s="112"/>
+      <c r="P1" s="112"/>
+      <c r="Q1" s="112"/>
+      <c r="R1" s="112"/>
+      <c r="S1" s="112"/>
+      <c r="T1" s="112"/>
+      <c r="U1" s="112"/>
+      <c r="V1" s="112"/>
+      <c r="W1" s="112"/>
+      <c r="X1" s="112"/>
+      <c r="Y1" s="112"/>
+      <c r="Z1" s="112"/>
+      <c r="AA1" s="112"/>
+      <c r="AB1" s="112"/>
+      <c r="AC1" s="113"/>
+      <c r="AD1" s="106" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="108"/>
-      <c r="AF1" s="108"/>
-      <c r="AG1" s="108"/>
-      <c r="AH1" s="108"/>
-      <c r="AI1" s="108"/>
-      <c r="AJ1" s="108"/>
-      <c r="AK1" s="109"/>
-      <c r="AL1" s="97" t="s">
+      <c r="AE1" s="107"/>
+      <c r="AF1" s="107"/>
+      <c r="AG1" s="107"/>
+      <c r="AH1" s="107"/>
+      <c r="AI1" s="107"/>
+      <c r="AJ1" s="107"/>
+      <c r="AK1" s="108"/>
+      <c r="AL1" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="98"/>
-      <c r="AN1" s="101" t="s">
+      <c r="AM1" s="97"/>
+      <c r="AN1" s="100" t="s">
         <v>2</v>
       </c>
-      <c r="AO1" s="102"/>
-      <c r="AP1" s="102"/>
-      <c r="AQ1" s="102"/>
-      <c r="AR1" s="103"/>
+      <c r="AO1" s="101"/>
+      <c r="AP1" s="101"/>
+      <c r="AQ1" s="101"/>
+      <c r="AR1" s="102"/>
       <c r="AS1" s="85" t="s">
         <v>4</v>
       </c>
@@ -3483,30 +3498,27 @@
       <c r="GC1" s="80"/>
       <c r="GD1" s="80"/>
       <c r="GE1" s="80"/>
-      <c r="GF1" s="80"/>
-      <c r="GG1" s="80"/>
-      <c r="GH1" s="80"/>
-      <c r="GI1" s="81"/>
-      <c r="GJ1" s="49" t="s">
+      <c r="GF1" s="81"/>
+      <c r="GG1" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="GK1" s="50"/>
-      <c r="GL1" s="50"/>
-      <c r="GM1" s="51"/>
-      <c r="GN1" s="82" t="s">
+      <c r="GH1" s="50"/>
+      <c r="GI1" s="50"/>
+      <c r="GJ1" s="51"/>
+      <c r="GK1" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="GO1" s="64" t="s">
+      <c r="GL1" s="64" t="s">
         <v>11</v>
       </c>
-      <c r="GP1" s="55" t="s">
+      <c r="GM1" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="GQ1" s="55" t="s">
+      <c r="GN1" s="55" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:199" s="12" customFormat="1" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:196" s="12" customFormat="1" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="52"/>
       <c r="B2" s="53"/>
       <c r="C2" s="53"/>
@@ -3520,41 +3532,41 @@
       <c r="K2" s="53"/>
       <c r="L2" s="53"/>
       <c r="M2" s="54"/>
-      <c r="N2" s="120" t="s">
+      <c r="N2" s="119" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="121"/>
-      <c r="P2" s="121"/>
-      <c r="Q2" s="121"/>
-      <c r="R2" s="121"/>
-      <c r="S2" s="121"/>
-      <c r="T2" s="121"/>
-      <c r="U2" s="122"/>
-      <c r="V2" s="115" t="s">
+      <c r="O2" s="120"/>
+      <c r="P2" s="120"/>
+      <c r="Q2" s="120"/>
+      <c r="R2" s="120"/>
+      <c r="S2" s="120"/>
+      <c r="T2" s="120"/>
+      <c r="U2" s="121"/>
+      <c r="V2" s="114" t="s">
         <v>15</v>
       </c>
-      <c r="W2" s="116"/>
-      <c r="X2" s="116"/>
-      <c r="Y2" s="116"/>
-      <c r="Z2" s="116"/>
-      <c r="AA2" s="116"/>
-      <c r="AB2" s="116"/>
-      <c r="AC2" s="117"/>
-      <c r="AD2" s="110"/>
-      <c r="AE2" s="111"/>
-      <c r="AF2" s="111"/>
-      <c r="AG2" s="111"/>
-      <c r="AH2" s="111"/>
-      <c r="AI2" s="111"/>
-      <c r="AJ2" s="111"/>
-      <c r="AK2" s="112"/>
-      <c r="AL2" s="99"/>
-      <c r="AM2" s="100"/>
-      <c r="AN2" s="104"/>
-      <c r="AO2" s="105"/>
-      <c r="AP2" s="105"/>
-      <c r="AQ2" s="105"/>
-      <c r="AR2" s="106"/>
+      <c r="W2" s="115"/>
+      <c r="X2" s="115"/>
+      <c r="Y2" s="115"/>
+      <c r="Z2" s="115"/>
+      <c r="AA2" s="115"/>
+      <c r="AB2" s="115"/>
+      <c r="AC2" s="116"/>
+      <c r="AD2" s="109"/>
+      <c r="AE2" s="110"/>
+      <c r="AF2" s="110"/>
+      <c r="AG2" s="110"/>
+      <c r="AH2" s="110"/>
+      <c r="AI2" s="110"/>
+      <c r="AJ2" s="110"/>
+      <c r="AK2" s="111"/>
+      <c r="AL2" s="98"/>
+      <c r="AM2" s="99"/>
+      <c r="AN2" s="103"/>
+      <c r="AO2" s="104"/>
+      <c r="AP2" s="104"/>
+      <c r="AQ2" s="104"/>
+      <c r="AR2" s="105"/>
       <c r="AS2" s="88"/>
       <c r="AT2" s="90"/>
       <c r="AU2" s="88"/>
@@ -3653,11 +3665,11 @@
       <c r="EJ2" s="95"/>
       <c r="EK2" s="95"/>
       <c r="EL2" s="95"/>
-      <c r="EM2" s="95"/>
-      <c r="EN2" s="96"/>
-      <c r="EO2" s="91" t="s">
-        <v>239</v>
-      </c>
+      <c r="EM2" s="91" t="s">
+        <v>235</v>
+      </c>
+      <c r="EN2" s="92"/>
+      <c r="EO2" s="92"/>
       <c r="EP2" s="92"/>
       <c r="EQ2" s="92"/>
       <c r="ER2" s="92"/>
@@ -3667,67 +3679,64 @@
       <c r="EV2" s="92"/>
       <c r="EW2" s="92"/>
       <c r="EX2" s="92"/>
-      <c r="EY2" s="92"/>
-      <c r="EZ2" s="92"/>
-      <c r="FA2" s="93"/>
-      <c r="FB2" s="129" t="s">
+      <c r="EY2" s="93"/>
+      <c r="EZ2" s="128" t="s">
         <v>16</v>
       </c>
-      <c r="FC2" s="130"/>
-      <c r="FD2" s="130"/>
-      <c r="FE2" s="130"/>
-      <c r="FF2" s="130"/>
-      <c r="FG2" s="130"/>
-      <c r="FH2" s="130"/>
-      <c r="FI2" s="130"/>
-      <c r="FJ2" s="130"/>
-      <c r="FK2" s="130"/>
-      <c r="FL2" s="130"/>
-      <c r="FM2" s="130"/>
-      <c r="FN2" s="130"/>
-      <c r="FO2" s="130"/>
+      <c r="FA2" s="129"/>
+      <c r="FB2" s="129"/>
+      <c r="FC2" s="129"/>
+      <c r="FD2" s="129"/>
+      <c r="FE2" s="129"/>
+      <c r="FF2" s="129"/>
+      <c r="FG2" s="129"/>
+      <c r="FH2" s="129"/>
+      <c r="FI2" s="129"/>
+      <c r="FJ2" s="129"/>
+      <c r="FK2" s="129"/>
+      <c r="FL2" s="129"/>
+      <c r="FM2" s="129"/>
+      <c r="FN2" s="129"/>
+      <c r="FO2" s="129"/>
       <c r="FP2" s="130"/>
-      <c r="FQ2" s="130"/>
-      <c r="FR2" s="131"/>
-      <c r="FS2" s="58" t="s">
+      <c r="FQ2" s="58" t="s">
         <v>17</v>
       </c>
+      <c r="FR2" s="59"/>
+      <c r="FS2" s="59"/>
       <c r="FT2" s="59"/>
       <c r="FU2" s="59"/>
       <c r="FV2" s="59"/>
       <c r="FW2" s="59"/>
       <c r="FX2" s="59"/>
-      <c r="FY2" s="59"/>
-      <c r="FZ2" s="59"/>
-      <c r="GA2" s="59"/>
-      <c r="GB2" s="60"/>
-      <c r="GC2" s="61" t="s">
+      <c r="FY2" s="60"/>
+      <c r="FZ2" s="61" t="s">
         <v>18</v>
       </c>
+      <c r="GA2" s="62"/>
+      <c r="GB2" s="62"/>
+      <c r="GC2" s="62"/>
       <c r="GD2" s="62"/>
       <c r="GE2" s="62"/>
-      <c r="GF2" s="62"/>
-      <c r="GG2" s="62"/>
-      <c r="GH2" s="62"/>
-      <c r="GI2" s="63"/>
-      <c r="GJ2" s="52"/>
-      <c r="GK2" s="53"/>
-      <c r="GL2" s="53"/>
-      <c r="GM2" s="54"/>
-      <c r="GN2" s="83"/>
-      <c r="GO2" s="65"/>
-      <c r="GP2" s="56"/>
-      <c r="GQ2" s="56"/>
+      <c r="GF2" s="63"/>
+      <c r="GG2" s="52"/>
+      <c r="GH2" s="53"/>
+      <c r="GI2" s="53"/>
+      <c r="GJ2" s="54"/>
+      <c r="GK2" s="83"/>
+      <c r="GL2" s="65"/>
+      <c r="GM2" s="56"/>
+      <c r="GN2" s="56"/>
     </row>
-    <row r="3" spans="1:199" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:196" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>21</v>
@@ -3760,7 +3769,7 @@
         <v>30</v>
       </c>
       <c r="N3" s="38" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="O3" s="22" t="s">
         <v>62</v>
@@ -3772,19 +3781,19 @@
         <v>64</v>
       </c>
       <c r="R3" s="22" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="S3" s="22" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="T3" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="U3" s="123" t="s">
+        <v>181</v>
+      </c>
+      <c r="U3" s="122" t="s">
         <v>65</v>
       </c>
-      <c r="V3" s="118" t="s">
-        <v>187</v>
+      <c r="V3" s="117" t="s">
+        <v>183</v>
       </c>
       <c r="W3" s="23" t="s">
         <v>62</v>
@@ -3796,28 +3805,28 @@
         <v>64</v>
       </c>
       <c r="Z3" s="23" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="AA3" s="23" t="s">
         <v>65</v>
       </c>
       <c r="AB3" s="23" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="AC3" s="39" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="AD3" s="34" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="AE3" s="17" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="AF3" s="17" t="s">
         <v>36</v>
       </c>
       <c r="AG3" s="17" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="AH3" s="17" t="s">
         <v>37</v>
@@ -3826,7 +3835,7 @@
         <v>38</v>
       </c>
       <c r="AJ3" s="17" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="AK3" s="35" t="s">
         <v>39</v>
@@ -3838,10 +3847,10 @@
         <v>32</v>
       </c>
       <c r="AN3" s="32" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="AO3" s="16" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="AP3" s="16" t="s">
         <v>33</v>
@@ -4132,501 +4141,537 @@
         <v>71</v>
       </c>
       <c r="EH3" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="EI3" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="EI3" s="24" t="s">
+      <c r="EJ3" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="EJ3" s="24" t="s">
+      <c r="EK3" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="EK3" s="14" t="s">
+      <c r="EL3" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="EL3" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="EM3" s="14" t="s">
+      <c r="EM3" s="123" t="s">
+        <v>225</v>
+      </c>
+      <c r="EN3" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="EO3" s="47" t="s">
+        <v>226</v>
+      </c>
+      <c r="EP3" s="47" t="s">
+        <v>224</v>
+      </c>
+      <c r="EQ3" s="48" t="s">
+        <v>223</v>
+      </c>
+      <c r="ER3" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="ES3" s="47" t="s">
+        <v>226</v>
+      </c>
+      <c r="ET3" s="47" t="s">
+        <v>224</v>
+      </c>
+      <c r="EU3" s="48" t="s">
+        <v>223</v>
+      </c>
+      <c r="EV3" s="47" t="s">
+        <v>51</v>
+      </c>
+      <c r="EW3" s="47" t="s">
+        <v>226</v>
+      </c>
+      <c r="EX3" s="47" t="s">
+        <v>224</v>
+      </c>
+      <c r="EY3" s="48" t="s">
+        <v>223</v>
+      </c>
+      <c r="EZ3" s="124" t="s">
         <v>77</v>
       </c>
-      <c r="EN3" s="29" t="s">
+      <c r="FA3" s="125" t="s">
         <v>78</v>
       </c>
-      <c r="EO3" s="124" t="s">
-        <v>229</v>
-      </c>
-      <c r="EP3" s="47" t="s">
+      <c r="FB3" s="125" t="s">
         <v>51</v>
       </c>
-      <c r="EQ3" s="47" t="s">
-        <v>230</v>
-      </c>
-      <c r="ER3" s="47" t="s">
-        <v>228</v>
-      </c>
-      <c r="ES3" s="48" t="s">
-        <v>227</v>
-      </c>
-      <c r="ET3" s="47" t="s">
+      <c r="FC3" s="125" t="s">
+        <v>79</v>
+      </c>
+      <c r="FD3" s="126" t="s">
+        <v>80</v>
+      </c>
+      <c r="FE3" s="125" t="s">
+        <v>81</v>
+      </c>
+      <c r="FF3" s="125" t="s">
+        <v>10</v>
+      </c>
+      <c r="FG3" s="125" t="s">
         <v>51</v>
       </c>
-      <c r="EU3" s="47" t="s">
-        <v>230</v>
-      </c>
-      <c r="EV3" s="47" t="s">
-        <v>228</v>
-      </c>
-      <c r="EW3" s="48" t="s">
-        <v>227</v>
-      </c>
-      <c r="EX3" s="47" t="s">
+      <c r="FH3" s="125" t="s">
+        <v>79</v>
+      </c>
+      <c r="FI3" s="126" t="s">
+        <v>80</v>
+      </c>
+      <c r="FJ3" s="125" t="s">
+        <v>81</v>
+      </c>
+      <c r="FK3" s="125" t="s">
+        <v>10</v>
+      </c>
+      <c r="FL3" s="125" t="s">
         <v>51</v>
       </c>
-      <c r="EY3" s="47" t="s">
-        <v>230</v>
-      </c>
-      <c r="EZ3" s="47" t="s">
-        <v>228</v>
-      </c>
-      <c r="FA3" s="48" t="s">
-        <v>227</v>
-      </c>
-      <c r="FB3" s="125" t="s">
+      <c r="FM3" s="125" t="s">
+        <v>79</v>
+      </c>
+      <c r="FN3" s="126" t="s">
         <v>80</v>
       </c>
-      <c r="FC3" s="126" t="s">
+      <c r="FO3" s="125" t="s">
         <v>81</v>
       </c>
-      <c r="FD3" s="126" t="s">
-        <v>51</v>
-      </c>
-      <c r="FE3" s="126" t="s">
+      <c r="FP3" s="127" t="s">
+        <v>10</v>
+      </c>
+      <c r="FQ3" s="34" t="s">
+        <v>52</v>
+      </c>
+      <c r="FR3" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="FF3" s="127" t="s">
+      <c r="FS3" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="FG3" s="126" t="s">
+      <c r="FT3" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="FH3" s="126" t="s">
-        <v>10</v>
-      </c>
-      <c r="FI3" s="126" t="s">
-        <v>51</v>
-      </c>
-      <c r="FJ3" s="126" t="s">
-        <v>82</v>
-      </c>
-      <c r="FK3" s="127" t="s">
-        <v>83</v>
-      </c>
-      <c r="FL3" s="126" t="s">
-        <v>84</v>
-      </c>
-      <c r="FM3" s="126" t="s">
-        <v>10</v>
-      </c>
-      <c r="FN3" s="126" t="s">
-        <v>51</v>
-      </c>
-      <c r="FO3" s="126" t="s">
-        <v>82</v>
-      </c>
-      <c r="FP3" s="127" t="s">
-        <v>83</v>
-      </c>
-      <c r="FQ3" s="126" t="s">
-        <v>84</v>
-      </c>
-      <c r="FR3" s="128" t="s">
-        <v>10</v>
-      </c>
-      <c r="FS3" s="34" t="s">
-        <v>52</v>
-      </c>
-      <c r="FT3" s="17" t="s">
+      <c r="FU3" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="FU3" s="17" t="s">
+      <c r="FV3" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="FV3" s="17" t="s">
+      <c r="FW3" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="FW3" s="17" t="s">
+      <c r="FX3" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="FX3" s="17" t="s">
+      <c r="FY3" s="35" t="s">
         <v>89</v>
       </c>
-      <c r="FY3" s="17" t="s">
+      <c r="FZ3" s="41" t="s">
         <v>90</v>
       </c>
-      <c r="FZ3" s="17" t="s">
+      <c r="GA3" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="GA3" s="17" t="s">
+      <c r="GB3" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="GB3" s="35" t="s">
+      <c r="GC3" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="GC3" s="41" t="s">
+      <c r="GD3" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="GD3" s="26" t="s">
+      <c r="GE3" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="GE3" s="26" t="s">
+      <c r="GF3" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="GF3" s="26" t="s">
+      <c r="GG3" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="GG3" s="26" t="s">
+      <c r="GH3" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="GI3" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="GJ3" s="43" t="s">
         <v>98</v>
       </c>
-      <c r="GH3" s="26" t="s">
-        <v>99</v>
-      </c>
-      <c r="GI3" s="42" t="s">
+      <c r="GK3" s="84"/>
+      <c r="GL3" s="66"/>
+      <c r="GM3" s="57"/>
+      <c r="GN3" s="57"/>
+    </row>
+    <row r="4" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="GJ3" s="40" t="s">
+      <c r="B4" s="5" t="s">
         <v>101</v>
-      </c>
-      <c r="GK3" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="GL3" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="GM3" s="43" t="s">
-        <v>102</v>
-      </c>
-      <c r="GN3" s="84"/>
-      <c r="GO3" s="66"/>
-      <c r="GP3" s="57"/>
-      <c r="GQ3" s="57"/>
-    </row>
-    <row r="4" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>105</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="5" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="G4" s="46">
         <v>35626</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="J4" s="8"/>
       <c r="K4" s="8"/>
       <c r="L4" s="8"/>
       <c r="M4" s="8"/>
       <c r="N4" s="5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="P4" s="46">
         <v>35626</v>
       </c>
       <c r="Q4" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="R4" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="W4" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="X4" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="Y4" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="Z4" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AA4" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AB4" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AC4" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AD4" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="AE4" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="AF4" s="5" t="s">
         <v>197</v>
-      </c>
-      <c r="AE4" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="AF4" s="5" t="s">
-        <v>201</v>
       </c>
       <c r="AG4" s="44">
         <v>2327.2600000000002</v>
       </c>
       <c r="AH4" s="5" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="AI4" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="AJ4" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="AK4" s="6"/>
       <c r="AL4" s="5" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="AM4" s="5" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="AN4" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AO4" s="6"/>
       <c r="AP4" s="6"/>
       <c r="AQ4" s="5" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="AR4" s="9">
         <v>12683.75</v>
       </c>
       <c r="AS4" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="AT4" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="EA4" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="EO4" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="EB4" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="EC4" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="ED4" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="EE4" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="EF4" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="EG4" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="EH4" s="133"/>
+      <c r="EJ4" s="6"/>
+      <c r="EK4" s="6"/>
+      <c r="EL4" s="6"/>
+      <c r="EM4" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="EN4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EO4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EP4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EQ4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="ER4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="ES4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="ET4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EU4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EV4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EW4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EX4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EY4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EZ4" s="5">
+        <v>4</v>
+      </c>
+      <c r="FB4" s="5">
+        <v>1</v>
+      </c>
+      <c r="FC4" s="7">
+        <v>45300</v>
+      </c>
+      <c r="FD4" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="FE4" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="FF4" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="FG4" s="5">
+        <v>2</v>
+      </c>
+      <c r="FH4" s="46">
+        <v>44851</v>
+      </c>
+      <c r="FI4" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="FJ4" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="FK4" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="FL4" s="5">
+        <v>3</v>
+      </c>
+      <c r="FM4" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="FN4" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="FO4" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="FP4" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="FS4" s="6"/>
+      <c r="FT4" s="6"/>
+      <c r="FU4" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="FW4" s="6"/>
+      <c r="FX4" s="6"/>
+      <c r="FY4" s="6"/>
+      <c r="FZ4" s="6"/>
+      <c r="GA4" s="6"/>
+      <c r="GB4" s="6"/>
+      <c r="GC4" s="6"/>
+      <c r="GD4" s="45"/>
+      <c r="GE4" s="6"/>
+      <c r="GF4" s="6"/>
+      <c r="GG4" s="6"/>
+      <c r="GH4" s="6"/>
+      <c r="GI4" s="6"/>
+      <c r="GJ4" s="6"/>
+      <c r="GK4" s="6"/>
+      <c r="GL4" s="131"/>
+      <c r="GM4" s="132"/>
+      <c r="GN4" s="132"/>
+    </row>
+    <row r="5" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>103</v>
-      </c>
-      <c r="EP4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EQ4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="ER4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="ES4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="ET4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EU4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EV4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EW4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EX4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EY4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EZ4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="FA4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="FB4" s="5">
-        <v>4</v>
-      </c>
-      <c r="FD4" s="5">
-        <v>1</v>
-      </c>
-      <c r="FE4" s="7">
-        <v>45300</v>
-      </c>
-      <c r="FF4" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="FG4" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="FH4" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="FI4" s="5">
-        <v>2</v>
-      </c>
-      <c r="FJ4" s="46">
-        <v>44851</v>
-      </c>
-      <c r="FK4" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="FL4" s="5" t="s">
-        <v>223</v>
-      </c>
-      <c r="FM4" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="FN4" s="5">
-        <v>3</v>
-      </c>
-      <c r="FO4" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="FP4" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="FQ4" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="FR4" s="5" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="5" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="5" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="G5" s="46">
         <v>26632</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
       <c r="N5" s="4" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="P5" s="46">
         <v>26632</v>
       </c>
       <c r="Q5" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="R5" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="X5" s="46">
         <v>43067</v>
       </c>
       <c r="Y5" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="Z5" s="46">
         <v>43273</v>
       </c>
       <c r="AA5" s="5" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="AC5" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="AD5" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="AE5" s="5" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="AF5" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AG5" s="44">
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="AI5" s="5" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="AJ5" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="AK5" s="6"/>
       <c r="AL5" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="AM5" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="AM5" s="5" t="s">
-        <v>212</v>
-      </c>
       <c r="AN5" s="5" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
       <c r="AQ5" s="5" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="AR5" s="9">
         <v>0</v>
@@ -4634,126 +4679,126 @@
       <c r="AS5" s="45"/>
       <c r="AT5" s="45"/>
       <c r="EA5" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="EO5" s="5">
+        <v>187</v>
+      </c>
+      <c r="EM5" s="5">
         <v>1</v>
       </c>
-      <c r="EP5" s="4" t="s">
-        <v>236</v>
+      <c r="EN5" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="EO5" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="EP5" s="46">
+        <v>46038</v>
       </c>
       <c r="EQ5" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="ER5" s="46">
-        <v>46038</v>
+        <v>234</v>
+      </c>
+      <c r="ER5" s="4" t="s">
+        <v>99</v>
       </c>
       <c r="ES5" s="4" t="s">
-        <v>238</v>
+        <v>99</v>
       </c>
       <c r="ET5" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EU5" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EV5" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EW5" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EX5" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EY5" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EZ5" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="FA5" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="EZ5" s="5">
+        <v>107</v>
       </c>
       <c r="FB5" s="5">
-        <v>107</v>
-      </c>
-      <c r="FD5" s="5">
         <v>1</v>
       </c>
-      <c r="FE5" s="7">
+      <c r="FC5" s="7">
         <v>46157</v>
       </c>
-      <c r="FF5" s="4" t="s">
+      <c r="FD5" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="FE5" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="FF5" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="FG5" s="5" t="s">
+      <c r="FG5" s="5">
+        <v>2</v>
+      </c>
+      <c r="FH5" s="46">
+        <v>46090</v>
+      </c>
+      <c r="FI5" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="FJ5" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="FK5" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="FL5" s="5">
+        <v>3</v>
+      </c>
+      <c r="FM5" s="46">
+        <v>46051</v>
+      </c>
+      <c r="FN5" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="FH5" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="FI5" s="5">
-        <v>2</v>
-      </c>
-      <c r="FJ5" s="46">
-        <v>46090</v>
-      </c>
-      <c r="FK5" s="4" t="s">
+      <c r="FO5" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="FL5" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="FM5" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="FN5" s="5">
-        <v>3</v>
-      </c>
-      <c r="FO5" s="46">
-        <v>46051</v>
-      </c>
-      <c r="FP5" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="FQ5" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="FR5" s="5" t="s">
-        <v>219</v>
+      <c r="FP5" s="5" t="s">
+        <v>215</v>
       </c>
     </row>
-    <row r="6" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="5" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="G6" s="46">
         <v>43543</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
       <c r="M6" s="6"/>
       <c r="N6" s="5" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="P6" s="46">
         <v>43543</v>
@@ -4765,73 +4810,73 @@
         <v>45426</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="V6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="W6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="X6" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="Y6" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="Z6" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AA6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AB6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AC6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AD6" s="5" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="AE6" s="4" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="AF6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AG6" s="44">
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="AI6" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="AJ6" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="AK6" s="6"/>
       <c r="AL6" s="5" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="AM6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AN6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AO6" s="6"/>
       <c r="AP6" s="6"/>
       <c r="AQ6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AR6" s="9">
         <v>0</v>
@@ -4839,123 +4884,123 @@
       <c r="AS6" s="45"/>
       <c r="AT6" s="45"/>
       <c r="EA6" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="EO6" s="5" t="s">
-        <v>103</v>
+        <v>187</v>
+      </c>
+      <c r="EM6" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="EN6" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="EO6" s="4" t="s">
+        <v>99</v>
       </c>
       <c r="EP6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EQ6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="ER6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="ES6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="ET6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EU6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EV6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EW6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EX6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EY6" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="EZ6" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="FA6" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="EZ6" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="FA6" s="5" t="s">
+        <v>99</v>
       </c>
       <c r="FB6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="FC6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="FD6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="FE6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="FF6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="FG6" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="FH6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="FH6" s="46" t="s">
+        <v>99</v>
       </c>
       <c r="FI6" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="FJ6" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="FJ6" s="5" t="s">
+        <v>99</v>
       </c>
       <c r="FK6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="FL6" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="FM6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="FM6" s="46" t="s">
+        <v>99</v>
       </c>
       <c r="FN6" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="FO6" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
+      </c>
+      <c r="FO6" s="5" t="s">
+        <v>99</v>
       </c>
       <c r="FP6" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="FQ6" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="FR6" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:199" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="G7" s="46">
         <v>39694</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="P7" s="46">
         <v>39694</v>
@@ -4967,108 +5012,108 @@
         <v>43469</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="T7" s="5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="V7" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="W7" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="X7" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="Y7" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="Z7" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AA7" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AB7" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AC7" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="AD7" s="5" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="AE7" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="EO7" s="5">
+        <v>241</v>
+      </c>
+      <c r="EM7" s="5">
         <v>2</v>
       </c>
-      <c r="EP7" s="4">
+      <c r="EN7" s="4">
         <v>1</v>
       </c>
+      <c r="EO7" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="EP7" s="46" t="s">
+        <v>229</v>
+      </c>
       <c r="EQ7" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="ER7" s="4">
+        <v>2</v>
+      </c>
+      <c r="ES7" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="ET7" s="46">
+        <v>46146</v>
+      </c>
+      <c r="EU7" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="ER7" s="46" t="s">
-        <v>233</v>
-      </c>
-      <c r="ES7" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="ET7" s="4">
-        <v>2</v>
-      </c>
-      <c r="EU7" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="EV7" s="46">
-        <v>46146</v>
-      </c>
-      <c r="EW7" s="4" t="s">
-        <v>235</v>
+      <c r="EV7" s="46" t="s">
+        <v>99</v>
+      </c>
+      <c r="EW7" s="46" t="s">
+        <v>99</v>
       </c>
       <c r="EX7" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="EY7" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="EZ7" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="FA7" s="46" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:GQ5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A3:GN5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="22">
-    <mergeCell ref="EO2:FA2"/>
-    <mergeCell ref="EA2:EN2"/>
+    <mergeCell ref="EM2:EY2"/>
+    <mergeCell ref="EA2:EL2"/>
     <mergeCell ref="AL1:AM2"/>
     <mergeCell ref="AN1:AR2"/>
     <mergeCell ref="AD1:AK2"/>
     <mergeCell ref="AS1:AT2"/>
     <mergeCell ref="A1:M2"/>
-    <mergeCell ref="GP1:GP3"/>
-    <mergeCell ref="GQ1:GQ3"/>
+    <mergeCell ref="GM1:GM3"/>
+    <mergeCell ref="GN1:GN3"/>
     <mergeCell ref="N2:U2"/>
-    <mergeCell ref="FB2:FR2"/>
-    <mergeCell ref="FS2:GB2"/>
-    <mergeCell ref="GC2:GI2"/>
-    <mergeCell ref="GO1:GO3"/>
+    <mergeCell ref="EZ2:FP2"/>
+    <mergeCell ref="FQ2:FY2"/>
+    <mergeCell ref="FZ2:GF2"/>
+    <mergeCell ref="GL1:GL3"/>
     <mergeCell ref="CE1:DK2"/>
     <mergeCell ref="DL1:DZ2"/>
-    <mergeCell ref="EA1:GI1"/>
-    <mergeCell ref="GN1:GN3"/>
+    <mergeCell ref="EA1:GF1"/>
+    <mergeCell ref="GK1:GK3"/>
     <mergeCell ref="V2:AC2"/>
     <mergeCell ref="N1:AC1"/>
-    <mergeCell ref="GJ1:GM2"/>
+    <mergeCell ref="GG1:GJ2"/>
     <mergeCell ref="AU1:CD2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A7:B1048576 A3:A6">

</xml_diff>

<commit_message>
Municipio de Manta completo: reCAPTCHA v2 con resolucion manual, doble validacion cedula/RUC (confirmado que SI pueden dar resultados distintos, contrario a lo esperado inicialmente), Portoviejo excluido del proyecto (sin campo de consulta disponible)
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F26087E-CA5B-4C71-A6E6-D14CAD21DE55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{136BE5D1-CF25-4616-B3E4-751BD1FAFA8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
   </bookViews>
@@ -1969,6 +1969,111 @@
     <xf numFmtId="49" fontId="5" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1996,6 +2101,24 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2077,151 +2200,28 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3291,442 +3291,442 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:196" s="12" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
-      <c r="E1" s="50"/>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="51"/>
-      <c r="N1" s="118" t="s">
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="E1" s="85"/>
+      <c r="F1" s="85"/>
+      <c r="G1" s="85"/>
+      <c r="H1" s="85"/>
+      <c r="I1" s="85"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="85"/>
+      <c r="L1" s="85"/>
+      <c r="M1" s="86"/>
+      <c r="N1" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="112"/>
-      <c r="P1" s="112"/>
-      <c r="Q1" s="112"/>
-      <c r="R1" s="112"/>
-      <c r="S1" s="112"/>
-      <c r="T1" s="112"/>
-      <c r="U1" s="112"/>
-      <c r="V1" s="112"/>
-      <c r="W1" s="112"/>
-      <c r="X1" s="112"/>
-      <c r="Y1" s="112"/>
-      <c r="Z1" s="112"/>
-      <c r="AA1" s="112"/>
-      <c r="AB1" s="112"/>
-      <c r="AC1" s="113"/>
-      <c r="AD1" s="106" t="s">
+      <c r="O1" s="130"/>
+      <c r="P1" s="130"/>
+      <c r="Q1" s="130"/>
+      <c r="R1" s="130"/>
+      <c r="S1" s="130"/>
+      <c r="T1" s="130"/>
+      <c r="U1" s="130"/>
+      <c r="V1" s="130"/>
+      <c r="W1" s="130"/>
+      <c r="X1" s="130"/>
+      <c r="Y1" s="130"/>
+      <c r="Z1" s="130"/>
+      <c r="AA1" s="130"/>
+      <c r="AB1" s="130"/>
+      <c r="AC1" s="131"/>
+      <c r="AD1" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="107"/>
-      <c r="AF1" s="107"/>
-      <c r="AG1" s="107"/>
-      <c r="AH1" s="107"/>
-      <c r="AI1" s="107"/>
-      <c r="AJ1" s="107"/>
-      <c r="AK1" s="108"/>
-      <c r="AL1" s="96" t="s">
+      <c r="AE1" s="75"/>
+      <c r="AF1" s="75"/>
+      <c r="AG1" s="75"/>
+      <c r="AH1" s="75"/>
+      <c r="AI1" s="75"/>
+      <c r="AJ1" s="75"/>
+      <c r="AK1" s="76"/>
+      <c r="AL1" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="97"/>
-      <c r="AN1" s="100" t="s">
+      <c r="AM1" s="65"/>
+      <c r="AN1" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="AO1" s="101"/>
-      <c r="AP1" s="101"/>
-      <c r="AQ1" s="101"/>
-      <c r="AR1" s="102"/>
-      <c r="AS1" s="85" t="s">
+      <c r="AO1" s="69"/>
+      <c r="AP1" s="69"/>
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="70"/>
+      <c r="AS1" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="AT1" s="87"/>
-      <c r="AU1" s="85" t="s">
+      <c r="AT1" s="81"/>
+      <c r="AU1" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="AV1" s="86"/>
-      <c r="AW1" s="86"/>
-      <c r="AX1" s="86"/>
-      <c r="AY1" s="86"/>
-      <c r="AZ1" s="86"/>
-      <c r="BA1" s="86"/>
-      <c r="BB1" s="86"/>
-      <c r="BC1" s="86"/>
-      <c r="BD1" s="86"/>
-      <c r="BE1" s="86"/>
-      <c r="BF1" s="86"/>
-      <c r="BG1" s="86"/>
-      <c r="BH1" s="86"/>
-      <c r="BI1" s="86"/>
-      <c r="BJ1" s="86"/>
-      <c r="BK1" s="86"/>
-      <c r="BL1" s="86"/>
-      <c r="BM1" s="86"/>
-      <c r="BN1" s="86"/>
-      <c r="BO1" s="86"/>
-      <c r="BP1" s="86"/>
-      <c r="BQ1" s="86"/>
-      <c r="BR1" s="86"/>
-      <c r="BS1" s="86"/>
-      <c r="BT1" s="86"/>
-      <c r="BU1" s="86"/>
-      <c r="BV1" s="86"/>
-      <c r="BW1" s="86"/>
-      <c r="BX1" s="86"/>
-      <c r="BY1" s="86"/>
-      <c r="BZ1" s="86"/>
-      <c r="CA1" s="86"/>
-      <c r="CB1" s="86"/>
-      <c r="CC1" s="86"/>
-      <c r="CD1" s="87"/>
-      <c r="CE1" s="67" t="s">
+      <c r="AV1" s="132"/>
+      <c r="AW1" s="132"/>
+      <c r="AX1" s="132"/>
+      <c r="AY1" s="132"/>
+      <c r="AZ1" s="132"/>
+      <c r="BA1" s="132"/>
+      <c r="BB1" s="132"/>
+      <c r="BC1" s="132"/>
+      <c r="BD1" s="132"/>
+      <c r="BE1" s="132"/>
+      <c r="BF1" s="132"/>
+      <c r="BG1" s="132"/>
+      <c r="BH1" s="132"/>
+      <c r="BI1" s="132"/>
+      <c r="BJ1" s="132"/>
+      <c r="BK1" s="132"/>
+      <c r="BL1" s="132"/>
+      <c r="BM1" s="132"/>
+      <c r="BN1" s="132"/>
+      <c r="BO1" s="132"/>
+      <c r="BP1" s="132"/>
+      <c r="BQ1" s="132"/>
+      <c r="BR1" s="132"/>
+      <c r="BS1" s="132"/>
+      <c r="BT1" s="132"/>
+      <c r="BU1" s="132"/>
+      <c r="BV1" s="132"/>
+      <c r="BW1" s="132"/>
+      <c r="BX1" s="132"/>
+      <c r="BY1" s="132"/>
+      <c r="BZ1" s="132"/>
+      <c r="CA1" s="132"/>
+      <c r="CB1" s="132"/>
+      <c r="CC1" s="132"/>
+      <c r="CD1" s="81"/>
+      <c r="CE1" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="CF1" s="68"/>
-      <c r="CG1" s="68"/>
-      <c r="CH1" s="68"/>
-      <c r="CI1" s="68"/>
-      <c r="CJ1" s="68"/>
-      <c r="CK1" s="68"/>
-      <c r="CL1" s="68"/>
-      <c r="CM1" s="68"/>
-      <c r="CN1" s="68"/>
-      <c r="CO1" s="68"/>
-      <c r="CP1" s="68"/>
-      <c r="CQ1" s="68"/>
-      <c r="CR1" s="68"/>
-      <c r="CS1" s="68"/>
-      <c r="CT1" s="68"/>
-      <c r="CU1" s="68"/>
-      <c r="CV1" s="68"/>
-      <c r="CW1" s="68"/>
-      <c r="CX1" s="68"/>
-      <c r="CY1" s="68"/>
-      <c r="CZ1" s="68"/>
-      <c r="DA1" s="68"/>
-      <c r="DB1" s="68"/>
-      <c r="DC1" s="68"/>
-      <c r="DD1" s="68"/>
-      <c r="DE1" s="68"/>
-      <c r="DF1" s="68"/>
-      <c r="DG1" s="68"/>
-      <c r="DH1" s="68"/>
-      <c r="DI1" s="68"/>
-      <c r="DJ1" s="68"/>
-      <c r="DK1" s="69"/>
-      <c r="DL1" s="73" t="s">
+      <c r="CF1" s="109"/>
+      <c r="CG1" s="109"/>
+      <c r="CH1" s="109"/>
+      <c r="CI1" s="109"/>
+      <c r="CJ1" s="109"/>
+      <c r="CK1" s="109"/>
+      <c r="CL1" s="109"/>
+      <c r="CM1" s="109"/>
+      <c r="CN1" s="109"/>
+      <c r="CO1" s="109"/>
+      <c r="CP1" s="109"/>
+      <c r="CQ1" s="109"/>
+      <c r="CR1" s="109"/>
+      <c r="CS1" s="109"/>
+      <c r="CT1" s="109"/>
+      <c r="CU1" s="109"/>
+      <c r="CV1" s="109"/>
+      <c r="CW1" s="109"/>
+      <c r="CX1" s="109"/>
+      <c r="CY1" s="109"/>
+      <c r="CZ1" s="109"/>
+      <c r="DA1" s="109"/>
+      <c r="DB1" s="109"/>
+      <c r="DC1" s="109"/>
+      <c r="DD1" s="109"/>
+      <c r="DE1" s="109"/>
+      <c r="DF1" s="109"/>
+      <c r="DG1" s="109"/>
+      <c r="DH1" s="109"/>
+      <c r="DI1" s="109"/>
+      <c r="DJ1" s="109"/>
+      <c r="DK1" s="110"/>
+      <c r="DL1" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="DM1" s="74"/>
-      <c r="DN1" s="74"/>
-      <c r="DO1" s="74"/>
-      <c r="DP1" s="74"/>
-      <c r="DQ1" s="74"/>
-      <c r="DR1" s="74"/>
-      <c r="DS1" s="74"/>
-      <c r="DT1" s="74"/>
-      <c r="DU1" s="74"/>
-      <c r="DV1" s="74"/>
-      <c r="DW1" s="74"/>
-      <c r="DX1" s="74"/>
-      <c r="DY1" s="74"/>
-      <c r="DZ1" s="75"/>
-      <c r="EA1" s="79" t="s">
+      <c r="DM1" s="115"/>
+      <c r="DN1" s="115"/>
+      <c r="DO1" s="115"/>
+      <c r="DP1" s="115"/>
+      <c r="DQ1" s="115"/>
+      <c r="DR1" s="115"/>
+      <c r="DS1" s="115"/>
+      <c r="DT1" s="115"/>
+      <c r="DU1" s="115"/>
+      <c r="DV1" s="115"/>
+      <c r="DW1" s="115"/>
+      <c r="DX1" s="115"/>
+      <c r="DY1" s="115"/>
+      <c r="DZ1" s="116"/>
+      <c r="EA1" s="120" t="s">
         <v>9</v>
       </c>
-      <c r="EB1" s="80"/>
-      <c r="EC1" s="80"/>
-      <c r="ED1" s="80"/>
-      <c r="EE1" s="80"/>
-      <c r="EF1" s="80"/>
-      <c r="EG1" s="80"/>
-      <c r="EH1" s="80"/>
-      <c r="EI1" s="80"/>
-      <c r="EJ1" s="80"/>
-      <c r="EK1" s="80"/>
-      <c r="EL1" s="80"/>
-      <c r="EM1" s="80"/>
-      <c r="EN1" s="80"/>
-      <c r="EO1" s="80"/>
-      <c r="EP1" s="80"/>
-      <c r="EQ1" s="80"/>
-      <c r="ER1" s="80"/>
-      <c r="ES1" s="80"/>
-      <c r="ET1" s="80"/>
-      <c r="EU1" s="80"/>
-      <c r="EV1" s="80"/>
-      <c r="EW1" s="80"/>
-      <c r="EX1" s="80"/>
-      <c r="EY1" s="80"/>
-      <c r="EZ1" s="80"/>
-      <c r="FA1" s="80"/>
-      <c r="FB1" s="80"/>
-      <c r="FC1" s="80"/>
-      <c r="FD1" s="80"/>
-      <c r="FE1" s="80"/>
-      <c r="FF1" s="80"/>
-      <c r="FG1" s="80"/>
-      <c r="FH1" s="80"/>
-      <c r="FI1" s="80"/>
-      <c r="FJ1" s="80"/>
-      <c r="FK1" s="80"/>
-      <c r="FL1" s="80"/>
-      <c r="FM1" s="80"/>
-      <c r="FN1" s="80"/>
-      <c r="FO1" s="80"/>
-      <c r="FP1" s="80"/>
-      <c r="FQ1" s="80"/>
-      <c r="FR1" s="80"/>
-      <c r="FS1" s="80"/>
-      <c r="FT1" s="80"/>
-      <c r="FU1" s="80"/>
-      <c r="FV1" s="80"/>
-      <c r="FW1" s="80"/>
-      <c r="FX1" s="80"/>
-      <c r="FY1" s="80"/>
-      <c r="FZ1" s="80"/>
-      <c r="GA1" s="80"/>
-      <c r="GB1" s="80"/>
-      <c r="GC1" s="80"/>
-      <c r="GD1" s="80"/>
-      <c r="GE1" s="80"/>
-      <c r="GF1" s="81"/>
-      <c r="GG1" s="49" t="s">
+      <c r="EB1" s="121"/>
+      <c r="EC1" s="121"/>
+      <c r="ED1" s="121"/>
+      <c r="EE1" s="121"/>
+      <c r="EF1" s="121"/>
+      <c r="EG1" s="121"/>
+      <c r="EH1" s="121"/>
+      <c r="EI1" s="121"/>
+      <c r="EJ1" s="121"/>
+      <c r="EK1" s="121"/>
+      <c r="EL1" s="121"/>
+      <c r="EM1" s="121"/>
+      <c r="EN1" s="121"/>
+      <c r="EO1" s="121"/>
+      <c r="EP1" s="121"/>
+      <c r="EQ1" s="121"/>
+      <c r="ER1" s="121"/>
+      <c r="ES1" s="121"/>
+      <c r="ET1" s="121"/>
+      <c r="EU1" s="121"/>
+      <c r="EV1" s="121"/>
+      <c r="EW1" s="121"/>
+      <c r="EX1" s="121"/>
+      <c r="EY1" s="121"/>
+      <c r="EZ1" s="121"/>
+      <c r="FA1" s="121"/>
+      <c r="FB1" s="121"/>
+      <c r="FC1" s="121"/>
+      <c r="FD1" s="121"/>
+      <c r="FE1" s="121"/>
+      <c r="FF1" s="121"/>
+      <c r="FG1" s="121"/>
+      <c r="FH1" s="121"/>
+      <c r="FI1" s="121"/>
+      <c r="FJ1" s="121"/>
+      <c r="FK1" s="121"/>
+      <c r="FL1" s="121"/>
+      <c r="FM1" s="121"/>
+      <c r="FN1" s="121"/>
+      <c r="FO1" s="121"/>
+      <c r="FP1" s="121"/>
+      <c r="FQ1" s="121"/>
+      <c r="FR1" s="121"/>
+      <c r="FS1" s="121"/>
+      <c r="FT1" s="121"/>
+      <c r="FU1" s="121"/>
+      <c r="FV1" s="121"/>
+      <c r="FW1" s="121"/>
+      <c r="FX1" s="121"/>
+      <c r="FY1" s="121"/>
+      <c r="FZ1" s="121"/>
+      <c r="GA1" s="121"/>
+      <c r="GB1" s="121"/>
+      <c r="GC1" s="121"/>
+      <c r="GD1" s="121"/>
+      <c r="GE1" s="121"/>
+      <c r="GF1" s="122"/>
+      <c r="GG1" s="84" t="s">
         <v>19</v>
       </c>
-      <c r="GH1" s="50"/>
-      <c r="GI1" s="50"/>
-      <c r="GJ1" s="51"/>
-      <c r="GK1" s="82" t="s">
+      <c r="GH1" s="85"/>
+      <c r="GI1" s="85"/>
+      <c r="GJ1" s="86"/>
+      <c r="GK1" s="123" t="s">
         <v>10</v>
       </c>
-      <c r="GL1" s="64" t="s">
+      <c r="GL1" s="105" t="s">
         <v>11</v>
       </c>
-      <c r="GM1" s="55" t="s">
+      <c r="GM1" s="90" t="s">
         <v>12</v>
       </c>
-      <c r="GN1" s="55" t="s">
+      <c r="GN1" s="90" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:196" s="12" customFormat="1" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="52"/>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="54"/>
-      <c r="N2" s="119" t="s">
+      <c r="A2" s="87"/>
+      <c r="B2" s="88"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="88"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="88"/>
+      <c r="H2" s="88"/>
+      <c r="I2" s="88"/>
+      <c r="J2" s="88"/>
+      <c r="K2" s="88"/>
+      <c r="L2" s="88"/>
+      <c r="M2" s="89"/>
+      <c r="N2" s="93" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="120"/>
-      <c r="P2" s="120"/>
-      <c r="Q2" s="120"/>
-      <c r="R2" s="120"/>
-      <c r="S2" s="120"/>
-      <c r="T2" s="120"/>
-      <c r="U2" s="121"/>
-      <c r="V2" s="114" t="s">
+      <c r="O2" s="94"/>
+      <c r="P2" s="94"/>
+      <c r="Q2" s="94"/>
+      <c r="R2" s="94"/>
+      <c r="S2" s="94"/>
+      <c r="T2" s="94"/>
+      <c r="U2" s="95"/>
+      <c r="V2" s="126" t="s">
         <v>15</v>
       </c>
-      <c r="W2" s="115"/>
-      <c r="X2" s="115"/>
-      <c r="Y2" s="115"/>
-      <c r="Z2" s="115"/>
-      <c r="AA2" s="115"/>
-      <c r="AB2" s="115"/>
-      <c r="AC2" s="116"/>
-      <c r="AD2" s="109"/>
-      <c r="AE2" s="110"/>
-      <c r="AF2" s="110"/>
-      <c r="AG2" s="110"/>
-      <c r="AH2" s="110"/>
-      <c r="AI2" s="110"/>
-      <c r="AJ2" s="110"/>
-      <c r="AK2" s="111"/>
-      <c r="AL2" s="98"/>
-      <c r="AM2" s="99"/>
-      <c r="AN2" s="103"/>
-      <c r="AO2" s="104"/>
-      <c r="AP2" s="104"/>
-      <c r="AQ2" s="104"/>
-      <c r="AR2" s="105"/>
-      <c r="AS2" s="88"/>
-      <c r="AT2" s="90"/>
-      <c r="AU2" s="88"/>
-      <c r="AV2" s="89"/>
-      <c r="AW2" s="89"/>
-      <c r="AX2" s="89"/>
-      <c r="AY2" s="89"/>
-      <c r="AZ2" s="89"/>
-      <c r="BA2" s="89"/>
-      <c r="BB2" s="89"/>
-      <c r="BC2" s="89"/>
-      <c r="BD2" s="89"/>
-      <c r="BE2" s="89"/>
-      <c r="BF2" s="89"/>
-      <c r="BG2" s="89"/>
-      <c r="BH2" s="89"/>
-      <c r="BI2" s="89"/>
-      <c r="BJ2" s="89"/>
-      <c r="BK2" s="89"/>
-      <c r="BL2" s="89"/>
-      <c r="BM2" s="89"/>
-      <c r="BN2" s="89"/>
-      <c r="BO2" s="89"/>
-      <c r="BP2" s="89"/>
-      <c r="BQ2" s="89"/>
-      <c r="BR2" s="89"/>
-      <c r="BS2" s="89"/>
-      <c r="BT2" s="89"/>
-      <c r="BU2" s="89"/>
-      <c r="BV2" s="89"/>
-      <c r="BW2" s="89"/>
-      <c r="BX2" s="89"/>
-      <c r="BY2" s="89"/>
-      <c r="BZ2" s="89"/>
-      <c r="CA2" s="89"/>
-      <c r="CB2" s="89"/>
-      <c r="CC2" s="89"/>
-      <c r="CD2" s="90"/>
-      <c r="CE2" s="70"/>
-      <c r="CF2" s="71"/>
-      <c r="CG2" s="71"/>
-      <c r="CH2" s="71"/>
-      <c r="CI2" s="71"/>
-      <c r="CJ2" s="71"/>
-      <c r="CK2" s="71"/>
-      <c r="CL2" s="71"/>
-      <c r="CM2" s="71"/>
-      <c r="CN2" s="71"/>
-      <c r="CO2" s="71"/>
-      <c r="CP2" s="71"/>
-      <c r="CQ2" s="71"/>
-      <c r="CR2" s="71"/>
-      <c r="CS2" s="71"/>
-      <c r="CT2" s="71"/>
-      <c r="CU2" s="71"/>
-      <c r="CV2" s="71"/>
-      <c r="CW2" s="71"/>
-      <c r="CX2" s="71"/>
-      <c r="CY2" s="71"/>
-      <c r="CZ2" s="71"/>
-      <c r="DA2" s="71"/>
-      <c r="DB2" s="71"/>
-      <c r="DC2" s="71"/>
-      <c r="DD2" s="71"/>
-      <c r="DE2" s="71"/>
-      <c r="DF2" s="71"/>
-      <c r="DG2" s="71"/>
-      <c r="DH2" s="71"/>
-      <c r="DI2" s="71"/>
-      <c r="DJ2" s="71"/>
-      <c r="DK2" s="72"/>
-      <c r="DL2" s="76"/>
-      <c r="DM2" s="77"/>
-      <c r="DN2" s="77"/>
-      <c r="DO2" s="77"/>
-      <c r="DP2" s="77"/>
-      <c r="DQ2" s="77"/>
-      <c r="DR2" s="77"/>
-      <c r="DS2" s="77"/>
-      <c r="DT2" s="77"/>
-      <c r="DU2" s="77"/>
-      <c r="DV2" s="77"/>
-      <c r="DW2" s="77"/>
-      <c r="DX2" s="77"/>
-      <c r="DY2" s="77"/>
-      <c r="DZ2" s="78"/>
-      <c r="EA2" s="94"/>
-      <c r="EB2" s="95"/>
-      <c r="EC2" s="95"/>
-      <c r="ED2" s="95"/>
-      <c r="EE2" s="95"/>
-      <c r="EF2" s="95"/>
-      <c r="EG2" s="95"/>
-      <c r="EH2" s="95"/>
-      <c r="EI2" s="95"/>
-      <c r="EJ2" s="95"/>
-      <c r="EK2" s="95"/>
-      <c r="EL2" s="95"/>
-      <c r="EM2" s="91" t="s">
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
+      <c r="Z2" s="127"/>
+      <c r="AA2" s="127"/>
+      <c r="AB2" s="127"/>
+      <c r="AC2" s="128"/>
+      <c r="AD2" s="77"/>
+      <c r="AE2" s="78"/>
+      <c r="AF2" s="78"/>
+      <c r="AG2" s="78"/>
+      <c r="AH2" s="78"/>
+      <c r="AI2" s="78"/>
+      <c r="AJ2" s="78"/>
+      <c r="AK2" s="79"/>
+      <c r="AL2" s="66"/>
+      <c r="AM2" s="67"/>
+      <c r="AN2" s="71"/>
+      <c r="AO2" s="72"/>
+      <c r="AP2" s="72"/>
+      <c r="AQ2" s="72"/>
+      <c r="AR2" s="73"/>
+      <c r="AS2" s="82"/>
+      <c r="AT2" s="83"/>
+      <c r="AU2" s="82"/>
+      <c r="AV2" s="133"/>
+      <c r="AW2" s="133"/>
+      <c r="AX2" s="133"/>
+      <c r="AY2" s="133"/>
+      <c r="AZ2" s="133"/>
+      <c r="BA2" s="133"/>
+      <c r="BB2" s="133"/>
+      <c r="BC2" s="133"/>
+      <c r="BD2" s="133"/>
+      <c r="BE2" s="133"/>
+      <c r="BF2" s="133"/>
+      <c r="BG2" s="133"/>
+      <c r="BH2" s="133"/>
+      <c r="BI2" s="133"/>
+      <c r="BJ2" s="133"/>
+      <c r="BK2" s="133"/>
+      <c r="BL2" s="133"/>
+      <c r="BM2" s="133"/>
+      <c r="BN2" s="133"/>
+      <c r="BO2" s="133"/>
+      <c r="BP2" s="133"/>
+      <c r="BQ2" s="133"/>
+      <c r="BR2" s="133"/>
+      <c r="BS2" s="133"/>
+      <c r="BT2" s="133"/>
+      <c r="BU2" s="133"/>
+      <c r="BV2" s="133"/>
+      <c r="BW2" s="133"/>
+      <c r="BX2" s="133"/>
+      <c r="BY2" s="133"/>
+      <c r="BZ2" s="133"/>
+      <c r="CA2" s="133"/>
+      <c r="CB2" s="133"/>
+      <c r="CC2" s="133"/>
+      <c r="CD2" s="83"/>
+      <c r="CE2" s="111"/>
+      <c r="CF2" s="112"/>
+      <c r="CG2" s="112"/>
+      <c r="CH2" s="112"/>
+      <c r="CI2" s="112"/>
+      <c r="CJ2" s="112"/>
+      <c r="CK2" s="112"/>
+      <c r="CL2" s="112"/>
+      <c r="CM2" s="112"/>
+      <c r="CN2" s="112"/>
+      <c r="CO2" s="112"/>
+      <c r="CP2" s="112"/>
+      <c r="CQ2" s="112"/>
+      <c r="CR2" s="112"/>
+      <c r="CS2" s="112"/>
+      <c r="CT2" s="112"/>
+      <c r="CU2" s="112"/>
+      <c r="CV2" s="112"/>
+      <c r="CW2" s="112"/>
+      <c r="CX2" s="112"/>
+      <c r="CY2" s="112"/>
+      <c r="CZ2" s="112"/>
+      <c r="DA2" s="112"/>
+      <c r="DB2" s="112"/>
+      <c r="DC2" s="112"/>
+      <c r="DD2" s="112"/>
+      <c r="DE2" s="112"/>
+      <c r="DF2" s="112"/>
+      <c r="DG2" s="112"/>
+      <c r="DH2" s="112"/>
+      <c r="DI2" s="112"/>
+      <c r="DJ2" s="112"/>
+      <c r="DK2" s="113"/>
+      <c r="DL2" s="117"/>
+      <c r="DM2" s="118"/>
+      <c r="DN2" s="118"/>
+      <c r="DO2" s="118"/>
+      <c r="DP2" s="118"/>
+      <c r="DQ2" s="118"/>
+      <c r="DR2" s="118"/>
+      <c r="DS2" s="118"/>
+      <c r="DT2" s="118"/>
+      <c r="DU2" s="118"/>
+      <c r="DV2" s="118"/>
+      <c r="DW2" s="118"/>
+      <c r="DX2" s="118"/>
+      <c r="DY2" s="118"/>
+      <c r="DZ2" s="119"/>
+      <c r="EA2" s="62"/>
+      <c r="EB2" s="63"/>
+      <c r="EC2" s="63"/>
+      <c r="ED2" s="63"/>
+      <c r="EE2" s="63"/>
+      <c r="EF2" s="63"/>
+      <c r="EG2" s="63"/>
+      <c r="EH2" s="63"/>
+      <c r="EI2" s="63"/>
+      <c r="EJ2" s="63"/>
+      <c r="EK2" s="63"/>
+      <c r="EL2" s="63"/>
+      <c r="EM2" s="59" t="s">
         <v>235</v>
       </c>
-      <c r="EN2" s="92"/>
-      <c r="EO2" s="92"/>
-      <c r="EP2" s="92"/>
-      <c r="EQ2" s="92"/>
-      <c r="ER2" s="92"/>
-      <c r="ES2" s="92"/>
-      <c r="ET2" s="92"/>
-      <c r="EU2" s="92"/>
-      <c r="EV2" s="92"/>
-      <c r="EW2" s="92"/>
-      <c r="EX2" s="92"/>
-      <c r="EY2" s="93"/>
-      <c r="EZ2" s="128" t="s">
+      <c r="EN2" s="60"/>
+      <c r="EO2" s="60"/>
+      <c r="EP2" s="60"/>
+      <c r="EQ2" s="60"/>
+      <c r="ER2" s="60"/>
+      <c r="ES2" s="60"/>
+      <c r="ET2" s="60"/>
+      <c r="EU2" s="60"/>
+      <c r="EV2" s="60"/>
+      <c r="EW2" s="60"/>
+      <c r="EX2" s="60"/>
+      <c r="EY2" s="61"/>
+      <c r="EZ2" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="FA2" s="129"/>
-      <c r="FB2" s="129"/>
-      <c r="FC2" s="129"/>
-      <c r="FD2" s="129"/>
-      <c r="FE2" s="129"/>
-      <c r="FF2" s="129"/>
-      <c r="FG2" s="129"/>
-      <c r="FH2" s="129"/>
-      <c r="FI2" s="129"/>
-      <c r="FJ2" s="129"/>
-      <c r="FK2" s="129"/>
-      <c r="FL2" s="129"/>
-      <c r="FM2" s="129"/>
-      <c r="FN2" s="129"/>
-      <c r="FO2" s="129"/>
-      <c r="FP2" s="130"/>
-      <c r="FQ2" s="58" t="s">
+      <c r="FA2" s="97"/>
+      <c r="FB2" s="97"/>
+      <c r="FC2" s="97"/>
+      <c r="FD2" s="97"/>
+      <c r="FE2" s="97"/>
+      <c r="FF2" s="97"/>
+      <c r="FG2" s="97"/>
+      <c r="FH2" s="97"/>
+      <c r="FI2" s="97"/>
+      <c r="FJ2" s="97"/>
+      <c r="FK2" s="97"/>
+      <c r="FL2" s="97"/>
+      <c r="FM2" s="97"/>
+      <c r="FN2" s="97"/>
+      <c r="FO2" s="97"/>
+      <c r="FP2" s="98"/>
+      <c r="FQ2" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="FR2" s="59"/>
-      <c r="FS2" s="59"/>
-      <c r="FT2" s="59"/>
-      <c r="FU2" s="59"/>
-      <c r="FV2" s="59"/>
-      <c r="FW2" s="59"/>
-      <c r="FX2" s="59"/>
-      <c r="FY2" s="60"/>
-      <c r="FZ2" s="61" t="s">
+      <c r="FR2" s="100"/>
+      <c r="FS2" s="100"/>
+      <c r="FT2" s="100"/>
+      <c r="FU2" s="100"/>
+      <c r="FV2" s="100"/>
+      <c r="FW2" s="100"/>
+      <c r="FX2" s="100"/>
+      <c r="FY2" s="101"/>
+      <c r="FZ2" s="102" t="s">
         <v>18</v>
       </c>
-      <c r="GA2" s="62"/>
-      <c r="GB2" s="62"/>
-      <c r="GC2" s="62"/>
-      <c r="GD2" s="62"/>
-      <c r="GE2" s="62"/>
-      <c r="GF2" s="63"/>
-      <c r="GG2" s="52"/>
-      <c r="GH2" s="53"/>
-      <c r="GI2" s="53"/>
-      <c r="GJ2" s="54"/>
-      <c r="GK2" s="83"/>
-      <c r="GL2" s="65"/>
-      <c r="GM2" s="56"/>
-      <c r="GN2" s="56"/>
+      <c r="GA2" s="103"/>
+      <c r="GB2" s="103"/>
+      <c r="GC2" s="103"/>
+      <c r="GD2" s="103"/>
+      <c r="GE2" s="103"/>
+      <c r="GF2" s="104"/>
+      <c r="GG2" s="87"/>
+      <c r="GH2" s="88"/>
+      <c r="GI2" s="88"/>
+      <c r="GJ2" s="89"/>
+      <c r="GK2" s="124"/>
+      <c r="GL2" s="106"/>
+      <c r="GM2" s="91"/>
+      <c r="GN2" s="91"/>
     </row>
     <row r="3" spans="1:196" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
@@ -3789,10 +3789,10 @@
       <c r="T3" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="U3" s="122" t="s">
+      <c r="U3" s="50" t="s">
         <v>65</v>
       </c>
-      <c r="V3" s="117" t="s">
+      <c r="V3" s="49" t="s">
         <v>183</v>
       </c>
       <c r="W3" s="23" t="s">
@@ -4155,7 +4155,7 @@
       <c r="EL3" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="EM3" s="123" t="s">
+      <c r="EM3" s="51" t="s">
         <v>225</v>
       </c>
       <c r="EN3" s="47" t="s">
@@ -4194,55 +4194,55 @@
       <c r="EY3" s="48" t="s">
         <v>223</v>
       </c>
-      <c r="EZ3" s="124" t="s">
+      <c r="EZ3" s="52" t="s">
         <v>77</v>
       </c>
-      <c r="FA3" s="125" t="s">
+      <c r="FA3" s="53" t="s">
         <v>78</v>
       </c>
-      <c r="FB3" s="125" t="s">
+      <c r="FB3" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="FC3" s="125" t="s">
+      <c r="FC3" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="FD3" s="126" t="s">
+      <c r="FD3" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="FE3" s="125" t="s">
+      <c r="FE3" s="53" t="s">
         <v>81</v>
       </c>
-      <c r="FF3" s="125" t="s">
+      <c r="FF3" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="FG3" s="125" t="s">
+      <c r="FG3" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="FH3" s="125" t="s">
+      <c r="FH3" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="FI3" s="126" t="s">
+      <c r="FI3" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="FJ3" s="125" t="s">
+      <c r="FJ3" s="53" t="s">
         <v>81</v>
       </c>
-      <c r="FK3" s="125" t="s">
+      <c r="FK3" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="FL3" s="125" t="s">
+      <c r="FL3" s="53" t="s">
         <v>51</v>
       </c>
-      <c r="FM3" s="125" t="s">
+      <c r="FM3" s="53" t="s">
         <v>79</v>
       </c>
-      <c r="FN3" s="126" t="s">
+      <c r="FN3" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="FO3" s="125" t="s">
+      <c r="FO3" s="53" t="s">
         <v>81</v>
       </c>
-      <c r="FP3" s="127" t="s">
+      <c r="FP3" s="55" t="s">
         <v>10</v>
       </c>
       <c r="FQ3" s="34" t="s">
@@ -4305,10 +4305,10 @@
       <c r="GJ3" s="43" t="s">
         <v>98</v>
       </c>
-      <c r="GK3" s="84"/>
-      <c r="GL3" s="66"/>
-      <c r="GM3" s="57"/>
-      <c r="GN3" s="57"/>
+      <c r="GK3" s="125"/>
+      <c r="GL3" s="107"/>
+      <c r="GM3" s="92"/>
+      <c r="GN3" s="92"/>
     </row>
     <row r="4" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -4449,7 +4449,7 @@
       <c r="EG4" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="EH4" s="133"/>
+      <c r="EH4" s="58"/>
       <c r="EJ4" s="6"/>
       <c r="EK4" s="6"/>
       <c r="EL4" s="6"/>
@@ -4560,9 +4560,9 @@
       <c r="GI4" s="6"/>
       <c r="GJ4" s="6"/>
       <c r="GK4" s="6"/>
-      <c r="GL4" s="131"/>
-      <c r="GM4" s="132"/>
-      <c r="GN4" s="132"/>
+      <c r="GL4" s="56"/>
+      <c r="GM4" s="57"/>
+      <c r="GN4" s="57"/>
     </row>
     <row r="5" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
@@ -5093,12 +5093,6 @@
   </sheetData>
   <autoFilter ref="A3:GN5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="22">
-    <mergeCell ref="EM2:EY2"/>
-    <mergeCell ref="EA2:EL2"/>
-    <mergeCell ref="AL1:AM2"/>
-    <mergeCell ref="AN1:AR2"/>
-    <mergeCell ref="AD1:AK2"/>
-    <mergeCell ref="AS1:AT2"/>
     <mergeCell ref="A1:M2"/>
     <mergeCell ref="GM1:GM3"/>
     <mergeCell ref="GN1:GN3"/>
@@ -5115,6 +5109,12 @@
     <mergeCell ref="N1:AC1"/>
     <mergeCell ref="GG1:GJ2"/>
     <mergeCell ref="AU1:CD2"/>
+    <mergeCell ref="EM2:EY2"/>
+    <mergeCell ref="EA2:EL2"/>
+    <mergeCell ref="AL1:AM2"/>
+    <mergeCell ref="AN1:AR2"/>
+    <mergeCell ref="AD1:AK2"/>
+    <mergeCell ref="AS1:AT2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A7:B1048576 A3:A6">
     <cfRule type="duplicateValues" dxfId="0" priority="142"/>

</xml_diff>

<commit_message>
SERCOP Certificados: confirmar descarga real de PDF funcionando (certificado_sercop_6902.pdf generado correctamente)
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF258E6-6A0E-4FAF-9175-46EA2F8BFF35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930963E8-97F7-46BB-8DBB-E1C264FDDCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
   </bookViews>
@@ -343,7 +343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="250">
   <si>
     <t>IDENTIFICACIÓN BÁSICA</t>
   </si>
@@ -716,9 +716,6 @@
     <t>Municipio de Esmeraldas</t>
   </si>
   <si>
-    <t>Municipio de Portoviejo</t>
-  </si>
-  <si>
     <t>Municipio de Manta</t>
   </si>
   <si>
@@ -734,9 +731,6 @@
     <t>https://consulta.esmeraldas.gob.ec/index.jsp</t>
   </si>
   <si>
-    <t>https://online.portoviejo.gob.ec/consultas/deudas.aspx</t>
-  </si>
-  <si>
     <t>https://portalciudadano.manta.gob.ec/consulta</t>
   </si>
   <si>
@@ -746,9 +740,6 @@
     <t>SERCOP / INCOP - Para determinar si es contratista del estado</t>
   </si>
   <si>
-    <t>SERCOP / INCOP - Descargar los certificados de contratos pendientes e incumplimientos</t>
-  </si>
-  <si>
     <t>Contraloría General del Estado</t>
   </si>
   <si>
@@ -824,9 +815,6 @@
     <t>URL_MUNICIPIO_ESMERALDAS</t>
   </si>
   <si>
-    <t>URL_MUNICIPIO_PORTOVIEJO</t>
-  </si>
-  <si>
     <t>URL_MUNICIPIO_MANTA</t>
   </si>
   <si>
@@ -884,9 +872,6 @@
     <t>https://www.compraspublicas.gob.ec/ProcesoContratacion/compras/EP/EmpReporteIncumplidos.cpe</t>
   </si>
   <si>
-    <t>Column1</t>
-  </si>
-  <si>
     <t>CONTRIBUYENTE FANTASMA</t>
   </si>
   <si>
@@ -1101,6 +1086,15 @@
   </si>
   <si>
     <t>resumene AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SERCOP / INCOP - Descargar los certificados de contratos pendientes </t>
+  </si>
+  <si>
+    <t>SERCOP / INCOP - Descargar los certificados de proveedores Incumplidos</t>
+  </si>
+  <si>
+    <t>URL_SERCOP_CER_INCUMPLIDOS</t>
   </si>
 </sst>
 </file>
@@ -1999,6 +1993,168 @@
     <xf numFmtId="44" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2060,168 +2216,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2477,13 +2471,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73BF0AB6-137A-4C16-B7EA-A0F9ABB400D1}" name="Table1" displayName="Table1" ref="A1:D22" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:D22" xr:uid="{73BF0AB6-137A-4C16-B7EA-A0F9ABB400D1}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73BF0AB6-137A-4C16-B7EA-A0F9ABB400D1}" name="Table1" displayName="Table1" ref="A1:C22" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:C22" xr:uid="{73BF0AB6-137A-4C16-B7EA-A0F9ABB400D1}"/>
+  <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{4D888731-8D4A-4AEE-A379-E92B20CE92EB}" name="Parametro" dataCellStyle="Hyperlink"/>
     <tableColumn id="2" xr3:uid="{C53BB495-EF99-4F05-98C6-92F765BE3CC6}" name="URL" dataCellStyle="Hyperlink"/>
     <tableColumn id="3" xr3:uid="{B9420EBC-919E-4A06-95AE-ECF311B7E39E}" name="Descripcion"/>
-    <tableColumn id="4" xr3:uid="{908A75CE-E1AA-4C96-AE91-1A8BCD32DBD2}" name="Column1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2806,16 +2799,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB3E01D9-B2C1-48D3-B1F2-810A5BB9689D}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="114.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="73" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="85.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>112</v>
       </c>
@@ -2825,13 +2817,10 @@
       <c r="C1" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>179</v>
-      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>104</v>
@@ -2840,9 +2829,9 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>105</v>
@@ -2851,9 +2840,9 @@
         <v>109</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>106</v>
@@ -2862,191 +2851,188 @@
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C6" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C7" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C9" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C13" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>157</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C14" t="s">
         <v>130</v>
       </c>
-      <c r="C10" t="s">
-        <v>124</v>
-      </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>151</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="C11" t="s">
-        <v>145</v>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>158</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C15" t="s">
+        <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>152</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>153</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C13" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>154</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C14" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>161</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="C15" t="s">
-        <v>132</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>162</v>
+        <v>249</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="C16" t="s">
-        <v>133</v>
+        <v>248</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>107</v>
       </c>
       <c r="C17" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C18" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C21" t="s">
         <v>76</v>
@@ -3054,13 +3040,13 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C22" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -3068,27 +3054,27 @@
     <hyperlink ref="B2" r:id="rId1" xr:uid="{7E3E4823-4E67-447B-A1CC-923292E28BEE}"/>
     <hyperlink ref="B4" r:id="rId2" xr:uid="{51FF7CBE-A5B0-4AFA-980F-9F0A965A2D3D}"/>
     <hyperlink ref="B3" r:id="rId3" xr:uid="{7B15B4D3-7801-415F-85E3-318FF67A9386}"/>
-    <hyperlink ref="B11" r:id="rId4" xr:uid="{84130E50-C138-4463-8D42-258C21BABAB5}"/>
-    <hyperlink ref="B12" r:id="rId5" display="https://appscvs1.supercias.gob.ec/consultaPersona/consulta_cia_param.zul" xr:uid="{0418C6EA-900E-455C-BB8A-E13404EDF68A}"/>
-    <hyperlink ref="B13" r:id="rId6" xr:uid="{7951AC72-1FC0-4DB7-91E0-CFFFBF7D5F43}"/>
-    <hyperlink ref="B14" r:id="rId7" xr:uid="{1F1654F3-293E-47F5-9D8C-67194E8A8F9F}"/>
+    <hyperlink ref="B10" r:id="rId4" xr:uid="{84130E50-C138-4463-8D42-258C21BABAB5}"/>
+    <hyperlink ref="B11" r:id="rId5" display="https://appscvs1.supercias.gob.ec/consultaPersona/consulta_cia_param.zul" xr:uid="{0418C6EA-900E-455C-BB8A-E13404EDF68A}"/>
+    <hyperlink ref="B12" r:id="rId6" xr:uid="{7951AC72-1FC0-4DB7-91E0-CFFFBF7D5F43}"/>
+    <hyperlink ref="B13" r:id="rId7" xr:uid="{1F1654F3-293E-47F5-9D8C-67194E8A8F9F}"/>
     <hyperlink ref="B5" r:id="rId8" xr:uid="{3699A5F2-8B4A-43CE-80A0-921A93B535BF}"/>
     <hyperlink ref="B6" r:id="rId9" location="/impuestos" xr:uid="{6E5A712C-0E27-416A-B914-68378D39DF2A}"/>
     <hyperlink ref="B7" r:id="rId10" xr:uid="{5412E673-E978-4804-8B65-D342B8D18386}"/>
     <hyperlink ref="B8" r:id="rId11" xr:uid="{792F2547-5678-4113-938A-8D2D57D01640}"/>
-    <hyperlink ref="B9" r:id="rId12" xr:uid="{A05BF404-98E7-4F23-89F7-A1A12A5DEC31}"/>
-    <hyperlink ref="B10" r:id="rId13" xr:uid="{463932E4-F449-4134-BFD7-E7A0C7286ECA}"/>
-    <hyperlink ref="B15" r:id="rId14" xr:uid="{495EDC15-68A7-4BE8-927E-BBB2578DE476}"/>
-    <hyperlink ref="B16" r:id="rId15" xr:uid="{3E6ED92F-8DD2-4B8C-95B0-4AA438BAADDB}"/>
-    <hyperlink ref="B17" r:id="rId16" xr:uid="{3A7B0726-F844-45E6-93AD-1931F90CF7E3}"/>
-    <hyperlink ref="B18" r:id="rId17" xr:uid="{057C59D7-61DF-4DFE-AAB9-51379F9D4E9A}"/>
-    <hyperlink ref="B19" r:id="rId18" xr:uid="{7A19A534-3F06-458B-80C6-6487E63D744D}"/>
-    <hyperlink ref="B20" r:id="rId19" xr:uid="{202C7379-4017-4D51-8DB5-D98D00C3F830}"/>
-    <hyperlink ref="B22" r:id="rId20" xr:uid="{C453A5E9-477A-4E66-96B1-EE76A90ED6E2}"/>
-    <hyperlink ref="B21" r:id="rId21" location="!/" xr:uid="{7DF53A54-D175-45A6-AB86-9F8D80DE0845}"/>
-    <hyperlink ref="D15" r:id="rId22" tooltip="https://www.compraspublicas.gob.ec/procesocontratacion/compras/ep/empreporteincumplidos.cpe" xr:uid="{16F119B6-E73C-4E08-A079-B80EA25C38B9}"/>
+    <hyperlink ref="B9" r:id="rId12" xr:uid="{463932E4-F449-4134-BFD7-E7A0C7286ECA}"/>
+    <hyperlink ref="B14" r:id="rId13" xr:uid="{495EDC15-68A7-4BE8-927E-BBB2578DE476}"/>
+    <hyperlink ref="B15" r:id="rId14" xr:uid="{3E6ED92F-8DD2-4B8C-95B0-4AA438BAADDB}"/>
+    <hyperlink ref="B17" r:id="rId15" xr:uid="{3A7B0726-F844-45E6-93AD-1931F90CF7E3}"/>
+    <hyperlink ref="B18" r:id="rId16" xr:uid="{057C59D7-61DF-4DFE-AAB9-51379F9D4E9A}"/>
+    <hyperlink ref="B19" r:id="rId17" xr:uid="{7A19A534-3F06-458B-80C6-6487E63D744D}"/>
+    <hyperlink ref="B20" r:id="rId18" xr:uid="{202C7379-4017-4D51-8DB5-D98D00C3F830}"/>
+    <hyperlink ref="B22" r:id="rId19" xr:uid="{C453A5E9-477A-4E66-96B1-EE76A90ED6E2}"/>
+    <hyperlink ref="B21" r:id="rId20" location="!/" xr:uid="{7DF53A54-D175-45A6-AB86-9F8D80DE0845}"/>
+    <hyperlink ref="B16" r:id="rId21" tooltip="https://www.compraspublicas.gob.ec/procesocontratacion/compras/ep/empreporteincumplidos.cpe" xr:uid="{16F119B6-E73C-4E08-A079-B80EA25C38B9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId22"/>
   <tableParts count="1">
     <tablePart r:id="rId23"/>
   </tableParts>
@@ -3291,452 +3277,452 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:196" s="12" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="59" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="85"/>
-      <c r="C1" s="85"/>
-      <c r="D1" s="85"/>
-      <c r="E1" s="85"/>
-      <c r="F1" s="85"/>
-      <c r="G1" s="85"/>
-      <c r="H1" s="85"/>
-      <c r="I1" s="85"/>
-      <c r="J1" s="85"/>
-      <c r="K1" s="85"/>
-      <c r="L1" s="85"/>
-      <c r="M1" s="86"/>
-      <c r="N1" s="129" t="s">
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="61"/>
+      <c r="N1" s="104" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="130"/>
-      <c r="P1" s="130"/>
-      <c r="Q1" s="130"/>
-      <c r="R1" s="130"/>
-      <c r="S1" s="130"/>
-      <c r="T1" s="130"/>
-      <c r="U1" s="130"/>
-      <c r="V1" s="130"/>
-      <c r="W1" s="130"/>
-      <c r="X1" s="130"/>
-      <c r="Y1" s="130"/>
-      <c r="Z1" s="130"/>
-      <c r="AA1" s="130"/>
-      <c r="AB1" s="130"/>
-      <c r="AC1" s="131"/>
-      <c r="AD1" s="74" t="s">
+      <c r="O1" s="105"/>
+      <c r="P1" s="105"/>
+      <c r="Q1" s="105"/>
+      <c r="R1" s="105"/>
+      <c r="S1" s="105"/>
+      <c r="T1" s="105"/>
+      <c r="U1" s="105"/>
+      <c r="V1" s="105"/>
+      <c r="W1" s="105"/>
+      <c r="X1" s="105"/>
+      <c r="Y1" s="105"/>
+      <c r="Z1" s="105"/>
+      <c r="AA1" s="105"/>
+      <c r="AB1" s="105"/>
+      <c r="AC1" s="106"/>
+      <c r="AD1" s="128" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="75"/>
-      <c r="AF1" s="75"/>
-      <c r="AG1" s="75"/>
-      <c r="AH1" s="75"/>
-      <c r="AI1" s="75"/>
-      <c r="AJ1" s="75"/>
-      <c r="AK1" s="76"/>
-      <c r="AL1" s="64" t="s">
+      <c r="AE1" s="129"/>
+      <c r="AF1" s="129"/>
+      <c r="AG1" s="129"/>
+      <c r="AH1" s="129"/>
+      <c r="AI1" s="129"/>
+      <c r="AJ1" s="129"/>
+      <c r="AK1" s="130"/>
+      <c r="AL1" s="118" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="65"/>
-      <c r="AN1" s="68" t="s">
+      <c r="AM1" s="119"/>
+      <c r="AN1" s="122" t="s">
         <v>2</v>
       </c>
-      <c r="AO1" s="69"/>
-      <c r="AP1" s="69"/>
-      <c r="AQ1" s="69"/>
-      <c r="AR1" s="70"/>
-      <c r="AS1" s="80" t="s">
+      <c r="AO1" s="123"/>
+      <c r="AP1" s="123"/>
+      <c r="AQ1" s="123"/>
+      <c r="AR1" s="124"/>
+      <c r="AS1" s="107" t="s">
         <v>4</v>
       </c>
-      <c r="AT1" s="81"/>
-      <c r="AU1" s="80" t="s">
+      <c r="AT1" s="109"/>
+      <c r="AU1" s="107" t="s">
         <v>5</v>
       </c>
-      <c r="AV1" s="132"/>
-      <c r="AW1" s="132"/>
-      <c r="AX1" s="132"/>
-      <c r="AY1" s="132"/>
-      <c r="AZ1" s="132"/>
-      <c r="BA1" s="132"/>
-      <c r="BB1" s="132"/>
-      <c r="BC1" s="132"/>
-      <c r="BD1" s="132"/>
-      <c r="BE1" s="132"/>
-      <c r="BF1" s="132"/>
-      <c r="BG1" s="132"/>
-      <c r="BH1" s="132"/>
-      <c r="BI1" s="132"/>
-      <c r="BJ1" s="132"/>
-      <c r="BK1" s="132"/>
-      <c r="BL1" s="132"/>
-      <c r="BM1" s="132"/>
-      <c r="BN1" s="132"/>
-      <c r="BO1" s="132"/>
-      <c r="BP1" s="132"/>
-      <c r="BQ1" s="132"/>
-      <c r="BR1" s="132"/>
-      <c r="BS1" s="132"/>
-      <c r="BT1" s="132"/>
-      <c r="BU1" s="132"/>
-      <c r="BV1" s="132"/>
-      <c r="BW1" s="132"/>
-      <c r="BX1" s="132"/>
-      <c r="BY1" s="132"/>
-      <c r="BZ1" s="132"/>
-      <c r="CA1" s="132"/>
-      <c r="CB1" s="132"/>
-      <c r="CC1" s="132"/>
-      <c r="CD1" s="81"/>
-      <c r="CE1" s="108" t="s">
+      <c r="AV1" s="108"/>
+      <c r="AW1" s="108"/>
+      <c r="AX1" s="108"/>
+      <c r="AY1" s="108"/>
+      <c r="AZ1" s="108"/>
+      <c r="BA1" s="108"/>
+      <c r="BB1" s="108"/>
+      <c r="BC1" s="108"/>
+      <c r="BD1" s="108"/>
+      <c r="BE1" s="108"/>
+      <c r="BF1" s="108"/>
+      <c r="BG1" s="108"/>
+      <c r="BH1" s="108"/>
+      <c r="BI1" s="108"/>
+      <c r="BJ1" s="108"/>
+      <c r="BK1" s="108"/>
+      <c r="BL1" s="108"/>
+      <c r="BM1" s="108"/>
+      <c r="BN1" s="108"/>
+      <c r="BO1" s="108"/>
+      <c r="BP1" s="108"/>
+      <c r="BQ1" s="108"/>
+      <c r="BR1" s="108"/>
+      <c r="BS1" s="108"/>
+      <c r="BT1" s="108"/>
+      <c r="BU1" s="108"/>
+      <c r="BV1" s="108"/>
+      <c r="BW1" s="108"/>
+      <c r="BX1" s="108"/>
+      <c r="BY1" s="108"/>
+      <c r="BZ1" s="108"/>
+      <c r="CA1" s="108"/>
+      <c r="CB1" s="108"/>
+      <c r="CC1" s="108"/>
+      <c r="CD1" s="109"/>
+      <c r="CE1" s="83" t="s">
         <v>6</v>
       </c>
-      <c r="CF1" s="109"/>
-      <c r="CG1" s="109"/>
-      <c r="CH1" s="109"/>
-      <c r="CI1" s="109"/>
-      <c r="CJ1" s="109"/>
-      <c r="CK1" s="109"/>
-      <c r="CL1" s="109"/>
-      <c r="CM1" s="109"/>
-      <c r="CN1" s="109"/>
-      <c r="CO1" s="109"/>
-      <c r="CP1" s="109"/>
-      <c r="CQ1" s="109"/>
-      <c r="CR1" s="109"/>
-      <c r="CS1" s="109"/>
-      <c r="CT1" s="109"/>
-      <c r="CU1" s="109"/>
-      <c r="CV1" s="109"/>
-      <c r="CW1" s="109"/>
-      <c r="CX1" s="109"/>
-      <c r="CY1" s="109"/>
-      <c r="CZ1" s="109"/>
-      <c r="DA1" s="109"/>
-      <c r="DB1" s="109"/>
-      <c r="DC1" s="109"/>
-      <c r="DD1" s="109"/>
-      <c r="DE1" s="109"/>
-      <c r="DF1" s="109"/>
-      <c r="DG1" s="109"/>
-      <c r="DH1" s="109"/>
-      <c r="DI1" s="109"/>
-      <c r="DJ1" s="109"/>
-      <c r="DK1" s="110"/>
-      <c r="DL1" s="114" t="s">
+      <c r="CF1" s="84"/>
+      <c r="CG1" s="84"/>
+      <c r="CH1" s="84"/>
+      <c r="CI1" s="84"/>
+      <c r="CJ1" s="84"/>
+      <c r="CK1" s="84"/>
+      <c r="CL1" s="84"/>
+      <c r="CM1" s="84"/>
+      <c r="CN1" s="84"/>
+      <c r="CO1" s="84"/>
+      <c r="CP1" s="84"/>
+      <c r="CQ1" s="84"/>
+      <c r="CR1" s="84"/>
+      <c r="CS1" s="84"/>
+      <c r="CT1" s="84"/>
+      <c r="CU1" s="84"/>
+      <c r="CV1" s="84"/>
+      <c r="CW1" s="84"/>
+      <c r="CX1" s="84"/>
+      <c r="CY1" s="84"/>
+      <c r="CZ1" s="84"/>
+      <c r="DA1" s="84"/>
+      <c r="DB1" s="84"/>
+      <c r="DC1" s="84"/>
+      <c r="DD1" s="84"/>
+      <c r="DE1" s="84"/>
+      <c r="DF1" s="84"/>
+      <c r="DG1" s="84"/>
+      <c r="DH1" s="84"/>
+      <c r="DI1" s="84"/>
+      <c r="DJ1" s="84"/>
+      <c r="DK1" s="85"/>
+      <c r="DL1" s="89" t="s">
         <v>7</v>
       </c>
-      <c r="DM1" s="115"/>
-      <c r="DN1" s="115"/>
-      <c r="DO1" s="115"/>
-      <c r="DP1" s="115"/>
-      <c r="DQ1" s="115"/>
-      <c r="DR1" s="115"/>
-      <c r="DS1" s="115"/>
-      <c r="DT1" s="115"/>
-      <c r="DU1" s="115"/>
-      <c r="DV1" s="115"/>
-      <c r="DW1" s="115"/>
-      <c r="DX1" s="115"/>
-      <c r="DY1" s="115"/>
-      <c r="DZ1" s="116"/>
-      <c r="EA1" s="120" t="s">
+      <c r="DM1" s="90"/>
+      <c r="DN1" s="90"/>
+      <c r="DO1" s="90"/>
+      <c r="DP1" s="90"/>
+      <c r="DQ1" s="90"/>
+      <c r="DR1" s="90"/>
+      <c r="DS1" s="90"/>
+      <c r="DT1" s="90"/>
+      <c r="DU1" s="90"/>
+      <c r="DV1" s="90"/>
+      <c r="DW1" s="90"/>
+      <c r="DX1" s="90"/>
+      <c r="DY1" s="90"/>
+      <c r="DZ1" s="91"/>
+      <c r="EA1" s="95" t="s">
         <v>9</v>
       </c>
-      <c r="EB1" s="121"/>
-      <c r="EC1" s="121"/>
-      <c r="ED1" s="121"/>
-      <c r="EE1" s="121"/>
-      <c r="EF1" s="121"/>
-      <c r="EG1" s="121"/>
-      <c r="EH1" s="121"/>
-      <c r="EI1" s="121"/>
-      <c r="EJ1" s="121"/>
-      <c r="EK1" s="121"/>
-      <c r="EL1" s="121"/>
-      <c r="EM1" s="121"/>
-      <c r="EN1" s="121"/>
-      <c r="EO1" s="121"/>
-      <c r="EP1" s="121"/>
-      <c r="EQ1" s="121"/>
-      <c r="ER1" s="121"/>
-      <c r="ES1" s="121"/>
-      <c r="ET1" s="121"/>
-      <c r="EU1" s="121"/>
-      <c r="EV1" s="121"/>
-      <c r="EW1" s="121"/>
-      <c r="EX1" s="121"/>
-      <c r="EY1" s="121"/>
-      <c r="EZ1" s="121"/>
-      <c r="FA1" s="121"/>
-      <c r="FB1" s="121"/>
-      <c r="FC1" s="121"/>
-      <c r="FD1" s="121"/>
-      <c r="FE1" s="121"/>
-      <c r="FF1" s="121"/>
-      <c r="FG1" s="121"/>
-      <c r="FH1" s="121"/>
-      <c r="FI1" s="121"/>
-      <c r="FJ1" s="121"/>
-      <c r="FK1" s="121"/>
-      <c r="FL1" s="121"/>
-      <c r="FM1" s="121"/>
-      <c r="FN1" s="121"/>
-      <c r="FO1" s="121"/>
-      <c r="FP1" s="121"/>
-      <c r="FQ1" s="121"/>
-      <c r="FR1" s="121"/>
-      <c r="FS1" s="121"/>
-      <c r="FT1" s="121"/>
-      <c r="FU1" s="121"/>
-      <c r="FV1" s="121"/>
-      <c r="FW1" s="121"/>
-      <c r="FX1" s="121"/>
-      <c r="FY1" s="121"/>
-      <c r="FZ1" s="121"/>
-      <c r="GA1" s="121"/>
-      <c r="GB1" s="121"/>
-      <c r="GC1" s="121"/>
-      <c r="GD1" s="121"/>
-      <c r="GE1" s="121"/>
-      <c r="GF1" s="122"/>
-      <c r="GG1" s="84" t="s">
+      <c r="EB1" s="96"/>
+      <c r="EC1" s="96"/>
+      <c r="ED1" s="96"/>
+      <c r="EE1" s="96"/>
+      <c r="EF1" s="96"/>
+      <c r="EG1" s="96"/>
+      <c r="EH1" s="96"/>
+      <c r="EI1" s="96"/>
+      <c r="EJ1" s="96"/>
+      <c r="EK1" s="96"/>
+      <c r="EL1" s="96"/>
+      <c r="EM1" s="96"/>
+      <c r="EN1" s="96"/>
+      <c r="EO1" s="96"/>
+      <c r="EP1" s="96"/>
+      <c r="EQ1" s="96"/>
+      <c r="ER1" s="96"/>
+      <c r="ES1" s="96"/>
+      <c r="ET1" s="96"/>
+      <c r="EU1" s="96"/>
+      <c r="EV1" s="96"/>
+      <c r="EW1" s="96"/>
+      <c r="EX1" s="96"/>
+      <c r="EY1" s="96"/>
+      <c r="EZ1" s="96"/>
+      <c r="FA1" s="96"/>
+      <c r="FB1" s="96"/>
+      <c r="FC1" s="96"/>
+      <c r="FD1" s="96"/>
+      <c r="FE1" s="96"/>
+      <c r="FF1" s="96"/>
+      <c r="FG1" s="96"/>
+      <c r="FH1" s="96"/>
+      <c r="FI1" s="96"/>
+      <c r="FJ1" s="96"/>
+      <c r="FK1" s="96"/>
+      <c r="FL1" s="96"/>
+      <c r="FM1" s="96"/>
+      <c r="FN1" s="96"/>
+      <c r="FO1" s="96"/>
+      <c r="FP1" s="96"/>
+      <c r="FQ1" s="96"/>
+      <c r="FR1" s="96"/>
+      <c r="FS1" s="96"/>
+      <c r="FT1" s="96"/>
+      <c r="FU1" s="96"/>
+      <c r="FV1" s="96"/>
+      <c r="FW1" s="96"/>
+      <c r="FX1" s="96"/>
+      <c r="FY1" s="96"/>
+      <c r="FZ1" s="96"/>
+      <c r="GA1" s="96"/>
+      <c r="GB1" s="96"/>
+      <c r="GC1" s="96"/>
+      <c r="GD1" s="96"/>
+      <c r="GE1" s="96"/>
+      <c r="GF1" s="97"/>
+      <c r="GG1" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="GH1" s="85"/>
-      <c r="GI1" s="85"/>
-      <c r="GJ1" s="86"/>
-      <c r="GK1" s="123" t="s">
+      <c r="GH1" s="60"/>
+      <c r="GI1" s="60"/>
+      <c r="GJ1" s="61"/>
+      <c r="GK1" s="98" t="s">
         <v>10</v>
       </c>
-      <c r="GL1" s="105" t="s">
+      <c r="GL1" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="GM1" s="90" t="s">
+      <c r="GM1" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="GN1" s="90" t="s">
+      <c r="GN1" s="65" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:196" s="12" customFormat="1" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="87"/>
-      <c r="B2" s="88"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="88"/>
-      <c r="E2" s="88"/>
-      <c r="F2" s="88"/>
-      <c r="G2" s="88"/>
-      <c r="H2" s="88"/>
-      <c r="I2" s="88"/>
-      <c r="J2" s="88"/>
-      <c r="K2" s="88"/>
-      <c r="L2" s="88"/>
-      <c r="M2" s="89"/>
-      <c r="N2" s="93" t="s">
+      <c r="A2" s="62"/>
+      <c r="B2" s="63"/>
+      <c r="C2" s="63"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="63"/>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="63"/>
+      <c r="M2" s="64"/>
+      <c r="N2" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="94"/>
-      <c r="P2" s="94"/>
-      <c r="Q2" s="94"/>
-      <c r="R2" s="94"/>
-      <c r="S2" s="94"/>
-      <c r="T2" s="94"/>
-      <c r="U2" s="95"/>
-      <c r="V2" s="126" t="s">
+      <c r="O2" s="69"/>
+      <c r="P2" s="69"/>
+      <c r="Q2" s="69"/>
+      <c r="R2" s="69"/>
+      <c r="S2" s="69"/>
+      <c r="T2" s="69"/>
+      <c r="U2" s="70"/>
+      <c r="V2" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="W2" s="127"/>
-      <c r="X2" s="127"/>
-      <c r="Y2" s="127"/>
-      <c r="Z2" s="127"/>
-      <c r="AA2" s="127"/>
-      <c r="AB2" s="127"/>
-      <c r="AC2" s="128"/>
-      <c r="AD2" s="77"/>
-      <c r="AE2" s="78"/>
-      <c r="AF2" s="78"/>
-      <c r="AG2" s="78"/>
-      <c r="AH2" s="78"/>
-      <c r="AI2" s="78"/>
-      <c r="AJ2" s="78"/>
-      <c r="AK2" s="79"/>
-      <c r="AL2" s="66"/>
-      <c r="AM2" s="67"/>
-      <c r="AN2" s="71"/>
-      <c r="AO2" s="72"/>
-      <c r="AP2" s="72"/>
-      <c r="AQ2" s="72"/>
-      <c r="AR2" s="73"/>
-      <c r="AS2" s="82"/>
-      <c r="AT2" s="83"/>
-      <c r="AU2" s="82"/>
-      <c r="AV2" s="133"/>
-      <c r="AW2" s="133"/>
-      <c r="AX2" s="133"/>
-      <c r="AY2" s="133"/>
-      <c r="AZ2" s="133"/>
-      <c r="BA2" s="133"/>
-      <c r="BB2" s="133"/>
-      <c r="BC2" s="133"/>
-      <c r="BD2" s="133"/>
-      <c r="BE2" s="133"/>
-      <c r="BF2" s="133"/>
-      <c r="BG2" s="133"/>
-      <c r="BH2" s="133"/>
-      <c r="BI2" s="133"/>
-      <c r="BJ2" s="133"/>
-      <c r="BK2" s="133"/>
-      <c r="BL2" s="133"/>
-      <c r="BM2" s="133"/>
-      <c r="BN2" s="133"/>
-      <c r="BO2" s="133"/>
-      <c r="BP2" s="133"/>
-      <c r="BQ2" s="133"/>
-      <c r="BR2" s="133"/>
-      <c r="BS2" s="133"/>
-      <c r="BT2" s="133"/>
-      <c r="BU2" s="133"/>
-      <c r="BV2" s="133"/>
-      <c r="BW2" s="133"/>
-      <c r="BX2" s="133"/>
-      <c r="BY2" s="133"/>
-      <c r="BZ2" s="133"/>
-      <c r="CA2" s="133"/>
-      <c r="CB2" s="133"/>
-      <c r="CC2" s="133"/>
-      <c r="CD2" s="83"/>
-      <c r="CE2" s="111"/>
-      <c r="CF2" s="112"/>
-      <c r="CG2" s="112"/>
-      <c r="CH2" s="112"/>
-      <c r="CI2" s="112"/>
-      <c r="CJ2" s="112"/>
-      <c r="CK2" s="112"/>
-      <c r="CL2" s="112"/>
-      <c r="CM2" s="112"/>
-      <c r="CN2" s="112"/>
-      <c r="CO2" s="112"/>
-      <c r="CP2" s="112"/>
-      <c r="CQ2" s="112"/>
-      <c r="CR2" s="112"/>
-      <c r="CS2" s="112"/>
-      <c r="CT2" s="112"/>
-      <c r="CU2" s="112"/>
-      <c r="CV2" s="112"/>
-      <c r="CW2" s="112"/>
-      <c r="CX2" s="112"/>
-      <c r="CY2" s="112"/>
-      <c r="CZ2" s="112"/>
-      <c r="DA2" s="112"/>
-      <c r="DB2" s="112"/>
-      <c r="DC2" s="112"/>
-      <c r="DD2" s="112"/>
-      <c r="DE2" s="112"/>
-      <c r="DF2" s="112"/>
-      <c r="DG2" s="112"/>
-      <c r="DH2" s="112"/>
-      <c r="DI2" s="112"/>
-      <c r="DJ2" s="112"/>
-      <c r="DK2" s="113"/>
-      <c r="DL2" s="117"/>
-      <c r="DM2" s="118"/>
-      <c r="DN2" s="118"/>
-      <c r="DO2" s="118"/>
-      <c r="DP2" s="118"/>
-      <c r="DQ2" s="118"/>
-      <c r="DR2" s="118"/>
-      <c r="DS2" s="118"/>
-      <c r="DT2" s="118"/>
-      <c r="DU2" s="118"/>
-      <c r="DV2" s="118"/>
-      <c r="DW2" s="118"/>
-      <c r="DX2" s="118"/>
-      <c r="DY2" s="118"/>
-      <c r="DZ2" s="119"/>
-      <c r="EA2" s="62"/>
-      <c r="EB2" s="63"/>
-      <c r="EC2" s="63"/>
-      <c r="ED2" s="63"/>
-      <c r="EE2" s="63"/>
-      <c r="EF2" s="63"/>
-      <c r="EG2" s="63"/>
-      <c r="EH2" s="63"/>
-      <c r="EI2" s="63"/>
-      <c r="EJ2" s="63"/>
-      <c r="EK2" s="63"/>
-      <c r="EL2" s="63"/>
-      <c r="EM2" s="59" t="s">
-        <v>235</v>
-      </c>
-      <c r="EN2" s="60"/>
-      <c r="EO2" s="60"/>
-      <c r="EP2" s="60"/>
-      <c r="EQ2" s="60"/>
-      <c r="ER2" s="60"/>
-      <c r="ES2" s="60"/>
-      <c r="ET2" s="60"/>
-      <c r="EU2" s="60"/>
-      <c r="EV2" s="60"/>
-      <c r="EW2" s="60"/>
-      <c r="EX2" s="60"/>
-      <c r="EY2" s="61"/>
-      <c r="EZ2" s="96" t="s">
+      <c r="W2" s="102"/>
+      <c r="X2" s="102"/>
+      <c r="Y2" s="102"/>
+      <c r="Z2" s="102"/>
+      <c r="AA2" s="102"/>
+      <c r="AB2" s="102"/>
+      <c r="AC2" s="103"/>
+      <c r="AD2" s="131"/>
+      <c r="AE2" s="132"/>
+      <c r="AF2" s="132"/>
+      <c r="AG2" s="132"/>
+      <c r="AH2" s="132"/>
+      <c r="AI2" s="132"/>
+      <c r="AJ2" s="132"/>
+      <c r="AK2" s="133"/>
+      <c r="AL2" s="120"/>
+      <c r="AM2" s="121"/>
+      <c r="AN2" s="125"/>
+      <c r="AO2" s="126"/>
+      <c r="AP2" s="126"/>
+      <c r="AQ2" s="126"/>
+      <c r="AR2" s="127"/>
+      <c r="AS2" s="110"/>
+      <c r="AT2" s="112"/>
+      <c r="AU2" s="110"/>
+      <c r="AV2" s="111"/>
+      <c r="AW2" s="111"/>
+      <c r="AX2" s="111"/>
+      <c r="AY2" s="111"/>
+      <c r="AZ2" s="111"/>
+      <c r="BA2" s="111"/>
+      <c r="BB2" s="111"/>
+      <c r="BC2" s="111"/>
+      <c r="BD2" s="111"/>
+      <c r="BE2" s="111"/>
+      <c r="BF2" s="111"/>
+      <c r="BG2" s="111"/>
+      <c r="BH2" s="111"/>
+      <c r="BI2" s="111"/>
+      <c r="BJ2" s="111"/>
+      <c r="BK2" s="111"/>
+      <c r="BL2" s="111"/>
+      <c r="BM2" s="111"/>
+      <c r="BN2" s="111"/>
+      <c r="BO2" s="111"/>
+      <c r="BP2" s="111"/>
+      <c r="BQ2" s="111"/>
+      <c r="BR2" s="111"/>
+      <c r="BS2" s="111"/>
+      <c r="BT2" s="111"/>
+      <c r="BU2" s="111"/>
+      <c r="BV2" s="111"/>
+      <c r="BW2" s="111"/>
+      <c r="BX2" s="111"/>
+      <c r="BY2" s="111"/>
+      <c r="BZ2" s="111"/>
+      <c r="CA2" s="111"/>
+      <c r="CB2" s="111"/>
+      <c r="CC2" s="111"/>
+      <c r="CD2" s="112"/>
+      <c r="CE2" s="86"/>
+      <c r="CF2" s="87"/>
+      <c r="CG2" s="87"/>
+      <c r="CH2" s="87"/>
+      <c r="CI2" s="87"/>
+      <c r="CJ2" s="87"/>
+      <c r="CK2" s="87"/>
+      <c r="CL2" s="87"/>
+      <c r="CM2" s="87"/>
+      <c r="CN2" s="87"/>
+      <c r="CO2" s="87"/>
+      <c r="CP2" s="87"/>
+      <c r="CQ2" s="87"/>
+      <c r="CR2" s="87"/>
+      <c r="CS2" s="87"/>
+      <c r="CT2" s="87"/>
+      <c r="CU2" s="87"/>
+      <c r="CV2" s="87"/>
+      <c r="CW2" s="87"/>
+      <c r="CX2" s="87"/>
+      <c r="CY2" s="87"/>
+      <c r="CZ2" s="87"/>
+      <c r="DA2" s="87"/>
+      <c r="DB2" s="87"/>
+      <c r="DC2" s="87"/>
+      <c r="DD2" s="87"/>
+      <c r="DE2" s="87"/>
+      <c r="DF2" s="87"/>
+      <c r="DG2" s="87"/>
+      <c r="DH2" s="87"/>
+      <c r="DI2" s="87"/>
+      <c r="DJ2" s="87"/>
+      <c r="DK2" s="88"/>
+      <c r="DL2" s="92"/>
+      <c r="DM2" s="93"/>
+      <c r="DN2" s="93"/>
+      <c r="DO2" s="93"/>
+      <c r="DP2" s="93"/>
+      <c r="DQ2" s="93"/>
+      <c r="DR2" s="93"/>
+      <c r="DS2" s="93"/>
+      <c r="DT2" s="93"/>
+      <c r="DU2" s="93"/>
+      <c r="DV2" s="93"/>
+      <c r="DW2" s="93"/>
+      <c r="DX2" s="93"/>
+      <c r="DY2" s="93"/>
+      <c r="DZ2" s="94"/>
+      <c r="EA2" s="116"/>
+      <c r="EB2" s="117"/>
+      <c r="EC2" s="117"/>
+      <c r="ED2" s="117"/>
+      <c r="EE2" s="117"/>
+      <c r="EF2" s="117"/>
+      <c r="EG2" s="117"/>
+      <c r="EH2" s="117"/>
+      <c r="EI2" s="117"/>
+      <c r="EJ2" s="117"/>
+      <c r="EK2" s="117"/>
+      <c r="EL2" s="117"/>
+      <c r="EM2" s="113" t="s">
+        <v>230</v>
+      </c>
+      <c r="EN2" s="114"/>
+      <c r="EO2" s="114"/>
+      <c r="EP2" s="114"/>
+      <c r="EQ2" s="114"/>
+      <c r="ER2" s="114"/>
+      <c r="ES2" s="114"/>
+      <c r="ET2" s="114"/>
+      <c r="EU2" s="114"/>
+      <c r="EV2" s="114"/>
+      <c r="EW2" s="114"/>
+      <c r="EX2" s="114"/>
+      <c r="EY2" s="115"/>
+      <c r="EZ2" s="71" t="s">
         <v>16</v>
       </c>
-      <c r="FA2" s="97"/>
-      <c r="FB2" s="97"/>
-      <c r="FC2" s="97"/>
-      <c r="FD2" s="97"/>
-      <c r="FE2" s="97"/>
-      <c r="FF2" s="97"/>
-      <c r="FG2" s="97"/>
-      <c r="FH2" s="97"/>
-      <c r="FI2" s="97"/>
-      <c r="FJ2" s="97"/>
-      <c r="FK2" s="97"/>
-      <c r="FL2" s="97"/>
-      <c r="FM2" s="97"/>
-      <c r="FN2" s="97"/>
-      <c r="FO2" s="97"/>
-      <c r="FP2" s="98"/>
-      <c r="FQ2" s="99" t="s">
+      <c r="FA2" s="72"/>
+      <c r="FB2" s="72"/>
+      <c r="FC2" s="72"/>
+      <c r="FD2" s="72"/>
+      <c r="FE2" s="72"/>
+      <c r="FF2" s="72"/>
+      <c r="FG2" s="72"/>
+      <c r="FH2" s="72"/>
+      <c r="FI2" s="72"/>
+      <c r="FJ2" s="72"/>
+      <c r="FK2" s="72"/>
+      <c r="FL2" s="72"/>
+      <c r="FM2" s="72"/>
+      <c r="FN2" s="72"/>
+      <c r="FO2" s="72"/>
+      <c r="FP2" s="73"/>
+      <c r="FQ2" s="74" t="s">
         <v>17</v>
       </c>
-      <c r="FR2" s="100"/>
-      <c r="FS2" s="100"/>
-      <c r="FT2" s="100"/>
-      <c r="FU2" s="100"/>
-      <c r="FV2" s="100"/>
-      <c r="FW2" s="100"/>
-      <c r="FX2" s="100"/>
-      <c r="FY2" s="101"/>
-      <c r="FZ2" s="102" t="s">
+      <c r="FR2" s="75"/>
+      <c r="FS2" s="75"/>
+      <c r="FT2" s="75"/>
+      <c r="FU2" s="75"/>
+      <c r="FV2" s="75"/>
+      <c r="FW2" s="75"/>
+      <c r="FX2" s="75"/>
+      <c r="FY2" s="76"/>
+      <c r="FZ2" s="77" t="s">
         <v>18</v>
       </c>
-      <c r="GA2" s="103"/>
-      <c r="GB2" s="103"/>
-      <c r="GC2" s="103"/>
-      <c r="GD2" s="103"/>
-      <c r="GE2" s="103"/>
-      <c r="GF2" s="104"/>
-      <c r="GG2" s="87"/>
-      <c r="GH2" s="88"/>
-      <c r="GI2" s="88"/>
-      <c r="GJ2" s="89"/>
-      <c r="GK2" s="124"/>
-      <c r="GL2" s="106"/>
-      <c r="GM2" s="91"/>
-      <c r="GN2" s="91"/>
+      <c r="GA2" s="78"/>
+      <c r="GB2" s="78"/>
+      <c r="GC2" s="78"/>
+      <c r="GD2" s="78"/>
+      <c r="GE2" s="78"/>
+      <c r="GF2" s="79"/>
+      <c r="GG2" s="62"/>
+      <c r="GH2" s="63"/>
+      <c r="GI2" s="63"/>
+      <c r="GJ2" s="64"/>
+      <c r="GK2" s="99"/>
+      <c r="GL2" s="81"/>
+      <c r="GM2" s="66"/>
+      <c r="GN2" s="66"/>
     </row>
     <row r="3" spans="1:196" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="D3" s="14" t="s">
         <v>21</v>
@@ -3769,7 +3755,7 @@
         <v>30</v>
       </c>
       <c r="N3" s="38" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="O3" s="22" t="s">
         <v>62</v>
@@ -3781,19 +3767,19 @@
         <v>64</v>
       </c>
       <c r="R3" s="22" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="S3" s="22" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="T3" s="22" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="U3" s="50" t="s">
         <v>65</v>
       </c>
       <c r="V3" s="49" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="W3" s="23" t="s">
         <v>62</v>
@@ -3805,28 +3791,28 @@
         <v>64</v>
       </c>
       <c r="Z3" s="23" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="AA3" s="23" t="s">
         <v>65</v>
       </c>
       <c r="AB3" s="23" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="AC3" s="39" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="AD3" s="34" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="AE3" s="17" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="AF3" s="17" t="s">
         <v>36</v>
       </c>
       <c r="AG3" s="17" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="AH3" s="17" t="s">
         <v>37</v>
@@ -3835,7 +3821,7 @@
         <v>38</v>
       </c>
       <c r="AJ3" s="17" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="AK3" s="35" t="s">
         <v>39</v>
@@ -3847,10 +3833,10 @@
         <v>32</v>
       </c>
       <c r="AN3" s="32" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="AO3" s="16" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="AP3" s="16" t="s">
         <v>33</v>
@@ -4141,7 +4127,7 @@
         <v>71</v>
       </c>
       <c r="EH3" s="25" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="EI3" s="24" t="s">
         <v>72</v>
@@ -4156,43 +4142,43 @@
         <v>75</v>
       </c>
       <c r="EM3" s="51" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="EN3" s="47" t="s">
         <v>51</v>
       </c>
       <c r="EO3" s="47" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="EP3" s="47" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="EQ3" s="48" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="ER3" s="47" t="s">
         <v>51</v>
       </c>
       <c r="ES3" s="47" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="ET3" s="47" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="EU3" s="48" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="EV3" s="47" t="s">
         <v>51</v>
       </c>
       <c r="EW3" s="47" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="EX3" s="47" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="EY3" s="48" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="EZ3" s="52" t="s">
         <v>77</v>
@@ -4305,10 +4291,10 @@
       <c r="GJ3" s="43" t="s">
         <v>98</v>
       </c>
-      <c r="GK3" s="125"/>
-      <c r="GL3" s="107"/>
-      <c r="GM3" s="92"/>
-      <c r="GN3" s="92"/>
+      <c r="GK3" s="100"/>
+      <c r="GL3" s="82"/>
+      <c r="GM3" s="67"/>
+      <c r="GN3" s="67"/>
     </row>
     <row r="4" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -4320,7 +4306,7 @@
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
       <c r="F4" s="5" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="G4" s="46">
         <v>35626</v>
@@ -4339,7 +4325,7 @@
         <v>101</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="P4" s="46">
         <v>35626</v>
@@ -4351,13 +4337,13 @@
         <v>99</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="V4" s="4" t="s">
         <v>99</v>
@@ -4384,32 +4370,32 @@
         <v>99</v>
       </c>
       <c r="AD4" s="5" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="AE4" s="5" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="AF4" s="5" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="AG4" s="44">
         <v>2327.2600000000002</v>
       </c>
       <c r="AH4" s="5" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="AI4" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="AJ4" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="AK4" s="6"/>
       <c r="AL4" s="5" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="AM4" s="5" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="AN4" s="5" t="s">
         <v>99</v>
@@ -4417,37 +4403,37 @@
       <c r="AO4" s="6"/>
       <c r="AP4" s="6"/>
       <c r="AQ4" s="5" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="AR4" s="9">
         <v>12683.75</v>
       </c>
       <c r="AS4" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="AT4" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="EA4" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="AT4" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="EA4" s="5" t="s">
-        <v>187</v>
-      </c>
       <c r="EB4" s="5" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="EC4" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="ED4" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="EE4" s="5" t="s">
         <v>244</v>
       </c>
-      <c r="ED4" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="EE4" s="5" t="s">
-        <v>249</v>
-      </c>
       <c r="EF4" s="5" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="EG4" s="5" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="EH4" s="58"/>
       <c r="EJ4" s="6"/>
@@ -4502,13 +4488,13 @@
         <v>45300</v>
       </c>
       <c r="FD4" s="4" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="FE4" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="FF4" s="5" t="s">
         <v>210</v>
-      </c>
-      <c r="FF4" s="5" t="s">
-        <v>215</v>
       </c>
       <c r="FG4" s="5">
         <v>2</v>
@@ -4517,13 +4503,13 @@
         <v>44851</v>
       </c>
       <c r="FI4" s="4" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="FJ4" s="5" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="FK4" s="5" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="FL4" s="5">
         <v>3</v>
@@ -4538,12 +4524,12 @@
         <v>99</v>
       </c>
       <c r="FP4" s="5" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="FS4" s="6"/>
       <c r="FT4" s="6"/>
       <c r="FU4" s="5" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="FW4" s="6"/>
       <c r="FX4" s="6"/>
@@ -4574,16 +4560,16 @@
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="5" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="G5" s="46">
         <v>26632</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
@@ -4593,7 +4579,7 @@
         <v>103</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="P5" s="46">
         <v>26632</v>
@@ -4605,19 +4591,19 @@
         <v>99</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="V5" s="4" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="X5" s="46">
         <v>43067</v>
@@ -4629,19 +4615,19 @@
         <v>43273</v>
       </c>
       <c r="AA5" s="5" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="AC5" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="AD5" s="5" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="AE5" s="5" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="AF5" s="5" t="s">
         <v>99</v>
@@ -4650,28 +4636,28 @@
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="AI5" s="5" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="AJ5" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="AK5" s="6"/>
       <c r="AL5" s="5" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="AM5" s="5" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="AN5" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="AO5" s="6"/>
       <c r="AP5" s="6"/>
       <c r="AQ5" s="5" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="AR5" s="9">
         <v>0</v>
@@ -4679,22 +4665,22 @@
       <c r="AS5" s="45"/>
       <c r="AT5" s="45"/>
       <c r="EA5" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="EM5" s="5">
         <v>1</v>
       </c>
       <c r="EN5" s="4" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="EO5" s="4" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="EP5" s="46">
         <v>46038</v>
       </c>
       <c r="EQ5" s="4" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="ER5" s="4" t="s">
         <v>99</v>
@@ -4730,13 +4716,13 @@
         <v>46157</v>
       </c>
       <c r="FD5" s="4" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="FE5" s="5" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="FF5" s="5" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="FG5" s="5">
         <v>2</v>
@@ -4745,13 +4731,13 @@
         <v>46090</v>
       </c>
       <c r="FI5" s="4" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="FJ5" s="5" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="FK5" s="5" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="FL5" s="5">
         <v>3</v>
@@ -4760,26 +4746,26 @@
         <v>46051</v>
       </c>
       <c r="FN5" s="4" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="FO5" s="5" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="FP5" s="5" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="5" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="G6" s="46">
         <v>43543</v>
@@ -4795,10 +4781,10 @@
       <c r="L6" s="6"/>
       <c r="M6" s="6"/>
       <c r="N6" s="5" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="P6" s="46">
         <v>43543</v>
@@ -4810,13 +4796,13 @@
         <v>45426</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="V6" s="4" t="s">
         <v>99</v>
@@ -4843,10 +4829,10 @@
         <v>99</v>
       </c>
       <c r="AD6" s="5" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="AE6" s="4" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="AF6" s="5" t="s">
         <v>99</v>
@@ -4855,17 +4841,17 @@
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="AI6" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="AJ6" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="AK6" s="6"/>
       <c r="AL6" s="5" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="AM6" s="5" t="s">
         <v>99</v>
@@ -4884,7 +4870,7 @@
       <c r="AS6" s="45"/>
       <c r="AT6" s="45"/>
       <c r="EA6" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="EM6" s="5" t="s">
         <v>99</v>
@@ -4979,13 +4965,13 @@
     </row>
     <row r="7" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="G7" s="46">
         <v>39694</v>
@@ -4997,10 +4983,10 @@
         <v>99</v>
       </c>
       <c r="N7" s="5" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="O7" s="5" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="P7" s="46">
         <v>39694</v>
@@ -5012,13 +4998,13 @@
         <v>43469</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="T7" s="5" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="V7" s="4" t="s">
         <v>99</v>
@@ -5045,10 +5031,10 @@
         <v>99</v>
       </c>
       <c r="AD7" s="5" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="AE7" s="5" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="EM7" s="5">
         <v>2</v>
@@ -5057,25 +5043,25 @@
         <v>1</v>
       </c>
       <c r="EO7" s="4" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="EP7" s="46" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="EQ7" s="4" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="ER7" s="4">
         <v>2</v>
       </c>
       <c r="ES7" s="4" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="ET7" s="46">
         <v>46146</v>
       </c>
       <c r="EU7" s="4" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="EV7" s="46" t="s">
         <v>99</v>
@@ -5093,6 +5079,12 @@
   </sheetData>
   <autoFilter ref="A3:GN5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="22">
+    <mergeCell ref="EM2:EY2"/>
+    <mergeCell ref="EA2:EL2"/>
+    <mergeCell ref="AL1:AM2"/>
+    <mergeCell ref="AN1:AR2"/>
+    <mergeCell ref="AD1:AK2"/>
+    <mergeCell ref="AS1:AT2"/>
     <mergeCell ref="A1:M2"/>
     <mergeCell ref="GM1:GM3"/>
     <mergeCell ref="GN1:GN3"/>
@@ -5109,12 +5101,6 @@
     <mergeCell ref="N1:AC1"/>
     <mergeCell ref="GG1:GJ2"/>
     <mergeCell ref="AU1:CD2"/>
-    <mergeCell ref="EM2:EY2"/>
-    <mergeCell ref="EA2:EL2"/>
-    <mergeCell ref="AL1:AM2"/>
-    <mergeCell ref="AN1:AR2"/>
-    <mergeCell ref="AD1:AK2"/>
-    <mergeCell ref="AS1:AT2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A7:B1048576 A3:A6">
     <cfRule type="duplicateValues" dxfId="0" priority="142"/>

</xml_diff>

<commit_message>
Fix evidencia.py: forzar scroll al inicio (scrollY=0) antes de capturar full_page - resuelve inconsistencia donde la barra de navegacion fija (position:sticky/fixed) a veces quedaba superpuesta a mitad del contenido en vez de arriba, confirmado con multiples pruebas
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930963E8-97F7-46BB-8DBB-E1C264FDDCDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3B647E-FA78-4767-8194-F76E9532DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametrizacion" sheetId="3" r:id="rId1"/>
@@ -343,7 +343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="252">
   <si>
     <t>IDENTIFICACIÓN BÁSICA</t>
   </si>
@@ -1095,6 +1095,12 @@
   </si>
   <si>
     <t>URL_SERCOP_CER_INCUMPLIDOS</t>
+  </si>
+  <si>
+    <t>AMBACAR CIA. LTDA.</t>
+  </si>
+  <si>
+    <t>1890010705001</t>
   </si>
 </sst>
 </file>
@@ -1993,6 +1999,81 @@
     <xf numFmtId="44" fontId="9" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2137,85 +2218,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2974,79 +2980,79 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>249</v>
+        <v>159</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>174</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
-        <v>248</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>107</v>
+        <v>133</v>
       </c>
       <c r="C17" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C18" t="s">
-        <v>135</v>
+        <v>134</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
+      </c>
+      <c r="C20" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C21" t="s">
-        <v>76</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>164</v>
+        <v>249</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>139</v>
+        <v>174</v>
       </c>
       <c r="C22" t="s">
-        <v>141</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>
@@ -3065,13 +3071,13 @@
     <hyperlink ref="B9" r:id="rId12" xr:uid="{463932E4-F449-4134-BFD7-E7A0C7286ECA}"/>
     <hyperlink ref="B14" r:id="rId13" xr:uid="{495EDC15-68A7-4BE8-927E-BBB2578DE476}"/>
     <hyperlink ref="B15" r:id="rId14" xr:uid="{3E6ED92F-8DD2-4B8C-95B0-4AA438BAADDB}"/>
-    <hyperlink ref="B17" r:id="rId15" xr:uid="{3A7B0726-F844-45E6-93AD-1931F90CF7E3}"/>
-    <hyperlink ref="B18" r:id="rId16" xr:uid="{057C59D7-61DF-4DFE-AAB9-51379F9D4E9A}"/>
-    <hyperlink ref="B19" r:id="rId17" xr:uid="{7A19A534-3F06-458B-80C6-6487E63D744D}"/>
-    <hyperlink ref="B20" r:id="rId18" xr:uid="{202C7379-4017-4D51-8DB5-D98D00C3F830}"/>
-    <hyperlink ref="B22" r:id="rId19" xr:uid="{C453A5E9-477A-4E66-96B1-EE76A90ED6E2}"/>
-    <hyperlink ref="B21" r:id="rId20" location="!/" xr:uid="{7DF53A54-D175-45A6-AB86-9F8D80DE0845}"/>
-    <hyperlink ref="B16" r:id="rId21" tooltip="https://www.compraspublicas.gob.ec/procesocontratacion/compras/ep/empreporteincumplidos.cpe" xr:uid="{16F119B6-E73C-4E08-A079-B80EA25C38B9}"/>
+    <hyperlink ref="B16" r:id="rId15" xr:uid="{3A7B0726-F844-45E6-93AD-1931F90CF7E3}"/>
+    <hyperlink ref="B17" r:id="rId16" xr:uid="{057C59D7-61DF-4DFE-AAB9-51379F9D4E9A}"/>
+    <hyperlink ref="B18" r:id="rId17" xr:uid="{7A19A534-3F06-458B-80C6-6487E63D744D}"/>
+    <hyperlink ref="B19" r:id="rId18" xr:uid="{202C7379-4017-4D51-8DB5-D98D00C3F830}"/>
+    <hyperlink ref="B21" r:id="rId19" xr:uid="{C453A5E9-477A-4E66-96B1-EE76A90ED6E2}"/>
+    <hyperlink ref="B20" r:id="rId20" location="!/" xr:uid="{7DF53A54-D175-45A6-AB86-9F8D80DE0845}"/>
+    <hyperlink ref="B22" r:id="rId21" tooltip="https://www.compraspublicas.gob.ec/procesocontratacion/compras/ep/empreporteincumplidos.cpe" xr:uid="{16F119B6-E73C-4E08-A079-B80EA25C38B9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId22"/>
@@ -3083,7 +3089,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3838F483-03F0-4F1D-B50C-3B9C5206BD2F}">
-  <dimension ref="A1:GN7"/>
+  <dimension ref="A1:GN8"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="70.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" style="4" bestFit="1" customWidth="1"/>
@@ -3277,442 +3283,442 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:196" s="12" customFormat="1" ht="24" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="61"/>
-      <c r="N1" s="104" t="s">
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="E1" s="85"/>
+      <c r="F1" s="85"/>
+      <c r="G1" s="85"/>
+      <c r="H1" s="85"/>
+      <c r="I1" s="85"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="85"/>
+      <c r="L1" s="85"/>
+      <c r="M1" s="86"/>
+      <c r="N1" s="129" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="105"/>
-      <c r="P1" s="105"/>
-      <c r="Q1" s="105"/>
-      <c r="R1" s="105"/>
-      <c r="S1" s="105"/>
-      <c r="T1" s="105"/>
-      <c r="U1" s="105"/>
-      <c r="V1" s="105"/>
-      <c r="W1" s="105"/>
-      <c r="X1" s="105"/>
-      <c r="Y1" s="105"/>
-      <c r="Z1" s="105"/>
-      <c r="AA1" s="105"/>
-      <c r="AB1" s="105"/>
-      <c r="AC1" s="106"/>
-      <c r="AD1" s="128" t="s">
+      <c r="O1" s="130"/>
+      <c r="P1" s="130"/>
+      <c r="Q1" s="130"/>
+      <c r="R1" s="130"/>
+      <c r="S1" s="130"/>
+      <c r="T1" s="130"/>
+      <c r="U1" s="130"/>
+      <c r="V1" s="130"/>
+      <c r="W1" s="130"/>
+      <c r="X1" s="130"/>
+      <c r="Y1" s="130"/>
+      <c r="Z1" s="130"/>
+      <c r="AA1" s="130"/>
+      <c r="AB1" s="130"/>
+      <c r="AC1" s="131"/>
+      <c r="AD1" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="AE1" s="129"/>
-      <c r="AF1" s="129"/>
-      <c r="AG1" s="129"/>
-      <c r="AH1" s="129"/>
-      <c r="AI1" s="129"/>
-      <c r="AJ1" s="129"/>
-      <c r="AK1" s="130"/>
-      <c r="AL1" s="118" t="s">
+      <c r="AE1" s="75"/>
+      <c r="AF1" s="75"/>
+      <c r="AG1" s="75"/>
+      <c r="AH1" s="75"/>
+      <c r="AI1" s="75"/>
+      <c r="AJ1" s="75"/>
+      <c r="AK1" s="76"/>
+      <c r="AL1" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="AM1" s="119"/>
-      <c r="AN1" s="122" t="s">
+      <c r="AM1" s="65"/>
+      <c r="AN1" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="AO1" s="123"/>
-      <c r="AP1" s="123"/>
-      <c r="AQ1" s="123"/>
-      <c r="AR1" s="124"/>
-      <c r="AS1" s="107" t="s">
+      <c r="AO1" s="69"/>
+      <c r="AP1" s="69"/>
+      <c r="AQ1" s="69"/>
+      <c r="AR1" s="70"/>
+      <c r="AS1" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="AT1" s="109"/>
-      <c r="AU1" s="107" t="s">
+      <c r="AT1" s="81"/>
+      <c r="AU1" s="80" t="s">
         <v>5</v>
       </c>
-      <c r="AV1" s="108"/>
-      <c r="AW1" s="108"/>
-      <c r="AX1" s="108"/>
-      <c r="AY1" s="108"/>
-      <c r="AZ1" s="108"/>
-      <c r="BA1" s="108"/>
-      <c r="BB1" s="108"/>
-      <c r="BC1" s="108"/>
-      <c r="BD1" s="108"/>
-      <c r="BE1" s="108"/>
-      <c r="BF1" s="108"/>
-      <c r="BG1" s="108"/>
-      <c r="BH1" s="108"/>
-      <c r="BI1" s="108"/>
-      <c r="BJ1" s="108"/>
-      <c r="BK1" s="108"/>
-      <c r="BL1" s="108"/>
-      <c r="BM1" s="108"/>
-      <c r="BN1" s="108"/>
-      <c r="BO1" s="108"/>
-      <c r="BP1" s="108"/>
-      <c r="BQ1" s="108"/>
-      <c r="BR1" s="108"/>
-      <c r="BS1" s="108"/>
-      <c r="BT1" s="108"/>
-      <c r="BU1" s="108"/>
-      <c r="BV1" s="108"/>
-      <c r="BW1" s="108"/>
-      <c r="BX1" s="108"/>
-      <c r="BY1" s="108"/>
-      <c r="BZ1" s="108"/>
-      <c r="CA1" s="108"/>
-      <c r="CB1" s="108"/>
-      <c r="CC1" s="108"/>
-      <c r="CD1" s="109"/>
-      <c r="CE1" s="83" t="s">
+      <c r="AV1" s="132"/>
+      <c r="AW1" s="132"/>
+      <c r="AX1" s="132"/>
+      <c r="AY1" s="132"/>
+      <c r="AZ1" s="132"/>
+      <c r="BA1" s="132"/>
+      <c r="BB1" s="132"/>
+      <c r="BC1" s="132"/>
+      <c r="BD1" s="132"/>
+      <c r="BE1" s="132"/>
+      <c r="BF1" s="132"/>
+      <c r="BG1" s="132"/>
+      <c r="BH1" s="132"/>
+      <c r="BI1" s="132"/>
+      <c r="BJ1" s="132"/>
+      <c r="BK1" s="132"/>
+      <c r="BL1" s="132"/>
+      <c r="BM1" s="132"/>
+      <c r="BN1" s="132"/>
+      <c r="BO1" s="132"/>
+      <c r="BP1" s="132"/>
+      <c r="BQ1" s="132"/>
+      <c r="BR1" s="132"/>
+      <c r="BS1" s="132"/>
+      <c r="BT1" s="132"/>
+      <c r="BU1" s="132"/>
+      <c r="BV1" s="132"/>
+      <c r="BW1" s="132"/>
+      <c r="BX1" s="132"/>
+      <c r="BY1" s="132"/>
+      <c r="BZ1" s="132"/>
+      <c r="CA1" s="132"/>
+      <c r="CB1" s="132"/>
+      <c r="CC1" s="132"/>
+      <c r="CD1" s="81"/>
+      <c r="CE1" s="108" t="s">
         <v>6</v>
       </c>
-      <c r="CF1" s="84"/>
-      <c r="CG1" s="84"/>
-      <c r="CH1" s="84"/>
-      <c r="CI1" s="84"/>
-      <c r="CJ1" s="84"/>
-      <c r="CK1" s="84"/>
-      <c r="CL1" s="84"/>
-      <c r="CM1" s="84"/>
-      <c r="CN1" s="84"/>
-      <c r="CO1" s="84"/>
-      <c r="CP1" s="84"/>
-      <c r="CQ1" s="84"/>
-      <c r="CR1" s="84"/>
-      <c r="CS1" s="84"/>
-      <c r="CT1" s="84"/>
-      <c r="CU1" s="84"/>
-      <c r="CV1" s="84"/>
-      <c r="CW1" s="84"/>
-      <c r="CX1" s="84"/>
-      <c r="CY1" s="84"/>
-      <c r="CZ1" s="84"/>
-      <c r="DA1" s="84"/>
-      <c r="DB1" s="84"/>
-      <c r="DC1" s="84"/>
-      <c r="DD1" s="84"/>
-      <c r="DE1" s="84"/>
-      <c r="DF1" s="84"/>
-      <c r="DG1" s="84"/>
-      <c r="DH1" s="84"/>
-      <c r="DI1" s="84"/>
-      <c r="DJ1" s="84"/>
-      <c r="DK1" s="85"/>
-      <c r="DL1" s="89" t="s">
+      <c r="CF1" s="109"/>
+      <c r="CG1" s="109"/>
+      <c r="CH1" s="109"/>
+      <c r="CI1" s="109"/>
+      <c r="CJ1" s="109"/>
+      <c r="CK1" s="109"/>
+      <c r="CL1" s="109"/>
+      <c r="CM1" s="109"/>
+      <c r="CN1" s="109"/>
+      <c r="CO1" s="109"/>
+      <c r="CP1" s="109"/>
+      <c r="CQ1" s="109"/>
+      <c r="CR1" s="109"/>
+      <c r="CS1" s="109"/>
+      <c r="CT1" s="109"/>
+      <c r="CU1" s="109"/>
+      <c r="CV1" s="109"/>
+      <c r="CW1" s="109"/>
+      <c r="CX1" s="109"/>
+      <c r="CY1" s="109"/>
+      <c r="CZ1" s="109"/>
+      <c r="DA1" s="109"/>
+      <c r="DB1" s="109"/>
+      <c r="DC1" s="109"/>
+      <c r="DD1" s="109"/>
+      <c r="DE1" s="109"/>
+      <c r="DF1" s="109"/>
+      <c r="DG1" s="109"/>
+      <c r="DH1" s="109"/>
+      <c r="DI1" s="109"/>
+      <c r="DJ1" s="109"/>
+      <c r="DK1" s="110"/>
+      <c r="DL1" s="114" t="s">
         <v>7</v>
       </c>
-      <c r="DM1" s="90"/>
-      <c r="DN1" s="90"/>
-      <c r="DO1" s="90"/>
-      <c r="DP1" s="90"/>
-      <c r="DQ1" s="90"/>
-      <c r="DR1" s="90"/>
-      <c r="DS1" s="90"/>
-      <c r="DT1" s="90"/>
-      <c r="DU1" s="90"/>
-      <c r="DV1" s="90"/>
-      <c r="DW1" s="90"/>
-      <c r="DX1" s="90"/>
-      <c r="DY1" s="90"/>
-      <c r="DZ1" s="91"/>
-      <c r="EA1" s="95" t="s">
+      <c r="DM1" s="115"/>
+      <c r="DN1" s="115"/>
+      <c r="DO1" s="115"/>
+      <c r="DP1" s="115"/>
+      <c r="DQ1" s="115"/>
+      <c r="DR1" s="115"/>
+      <c r="DS1" s="115"/>
+      <c r="DT1" s="115"/>
+      <c r="DU1" s="115"/>
+      <c r="DV1" s="115"/>
+      <c r="DW1" s="115"/>
+      <c r="DX1" s="115"/>
+      <c r="DY1" s="115"/>
+      <c r="DZ1" s="116"/>
+      <c r="EA1" s="120" t="s">
         <v>9</v>
       </c>
-      <c r="EB1" s="96"/>
-      <c r="EC1" s="96"/>
-      <c r="ED1" s="96"/>
-      <c r="EE1" s="96"/>
-      <c r="EF1" s="96"/>
-      <c r="EG1" s="96"/>
-      <c r="EH1" s="96"/>
-      <c r="EI1" s="96"/>
-      <c r="EJ1" s="96"/>
-      <c r="EK1" s="96"/>
-      <c r="EL1" s="96"/>
-      <c r="EM1" s="96"/>
-      <c r="EN1" s="96"/>
-      <c r="EO1" s="96"/>
-      <c r="EP1" s="96"/>
-      <c r="EQ1" s="96"/>
-      <c r="ER1" s="96"/>
-      <c r="ES1" s="96"/>
-      <c r="ET1" s="96"/>
-      <c r="EU1" s="96"/>
-      <c r="EV1" s="96"/>
-      <c r="EW1" s="96"/>
-      <c r="EX1" s="96"/>
-      <c r="EY1" s="96"/>
-      <c r="EZ1" s="96"/>
-      <c r="FA1" s="96"/>
-      <c r="FB1" s="96"/>
-      <c r="FC1" s="96"/>
-      <c r="FD1" s="96"/>
-      <c r="FE1" s="96"/>
-      <c r="FF1" s="96"/>
-      <c r="FG1" s="96"/>
-      <c r="FH1" s="96"/>
-      <c r="FI1" s="96"/>
-      <c r="FJ1" s="96"/>
-      <c r="FK1" s="96"/>
-      <c r="FL1" s="96"/>
-      <c r="FM1" s="96"/>
-      <c r="FN1" s="96"/>
-      <c r="FO1" s="96"/>
-      <c r="FP1" s="96"/>
-      <c r="FQ1" s="96"/>
-      <c r="FR1" s="96"/>
-      <c r="FS1" s="96"/>
-      <c r="FT1" s="96"/>
-      <c r="FU1" s="96"/>
-      <c r="FV1" s="96"/>
-      <c r="FW1" s="96"/>
-      <c r="FX1" s="96"/>
-      <c r="FY1" s="96"/>
-      <c r="FZ1" s="96"/>
-      <c r="GA1" s="96"/>
-      <c r="GB1" s="96"/>
-      <c r="GC1" s="96"/>
-      <c r="GD1" s="96"/>
-      <c r="GE1" s="96"/>
-      <c r="GF1" s="97"/>
-      <c r="GG1" s="59" t="s">
+      <c r="EB1" s="121"/>
+      <c r="EC1" s="121"/>
+      <c r="ED1" s="121"/>
+      <c r="EE1" s="121"/>
+      <c r="EF1" s="121"/>
+      <c r="EG1" s="121"/>
+      <c r="EH1" s="121"/>
+      <c r="EI1" s="121"/>
+      <c r="EJ1" s="121"/>
+      <c r="EK1" s="121"/>
+      <c r="EL1" s="121"/>
+      <c r="EM1" s="121"/>
+      <c r="EN1" s="121"/>
+      <c r="EO1" s="121"/>
+      <c r="EP1" s="121"/>
+      <c r="EQ1" s="121"/>
+      <c r="ER1" s="121"/>
+      <c r="ES1" s="121"/>
+      <c r="ET1" s="121"/>
+      <c r="EU1" s="121"/>
+      <c r="EV1" s="121"/>
+      <c r="EW1" s="121"/>
+      <c r="EX1" s="121"/>
+      <c r="EY1" s="121"/>
+      <c r="EZ1" s="121"/>
+      <c r="FA1" s="121"/>
+      <c r="FB1" s="121"/>
+      <c r="FC1" s="121"/>
+      <c r="FD1" s="121"/>
+      <c r="FE1" s="121"/>
+      <c r="FF1" s="121"/>
+      <c r="FG1" s="121"/>
+      <c r="FH1" s="121"/>
+      <c r="FI1" s="121"/>
+      <c r="FJ1" s="121"/>
+      <c r="FK1" s="121"/>
+      <c r="FL1" s="121"/>
+      <c r="FM1" s="121"/>
+      <c r="FN1" s="121"/>
+      <c r="FO1" s="121"/>
+      <c r="FP1" s="121"/>
+      <c r="FQ1" s="121"/>
+      <c r="FR1" s="121"/>
+      <c r="FS1" s="121"/>
+      <c r="FT1" s="121"/>
+      <c r="FU1" s="121"/>
+      <c r="FV1" s="121"/>
+      <c r="FW1" s="121"/>
+      <c r="FX1" s="121"/>
+      <c r="FY1" s="121"/>
+      <c r="FZ1" s="121"/>
+      <c r="GA1" s="121"/>
+      <c r="GB1" s="121"/>
+      <c r="GC1" s="121"/>
+      <c r="GD1" s="121"/>
+      <c r="GE1" s="121"/>
+      <c r="GF1" s="122"/>
+      <c r="GG1" s="84" t="s">
         <v>19</v>
       </c>
-      <c r="GH1" s="60"/>
-      <c r="GI1" s="60"/>
-      <c r="GJ1" s="61"/>
-      <c r="GK1" s="98" t="s">
+      <c r="GH1" s="85"/>
+      <c r="GI1" s="85"/>
+      <c r="GJ1" s="86"/>
+      <c r="GK1" s="123" t="s">
         <v>10</v>
       </c>
-      <c r="GL1" s="80" t="s">
+      <c r="GL1" s="105" t="s">
         <v>11</v>
       </c>
-      <c r="GM1" s="65" t="s">
+      <c r="GM1" s="90" t="s">
         <v>12</v>
       </c>
-      <c r="GN1" s="65" t="s">
+      <c r="GN1" s="90" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:196" s="12" customFormat="1" ht="25.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="62"/>
-      <c r="B2" s="63"/>
-      <c r="C2" s="63"/>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="63"/>
-      <c r="I2" s="63"/>
-      <c r="J2" s="63"/>
-      <c r="K2" s="63"/>
-      <c r="L2" s="63"/>
-      <c r="M2" s="64"/>
-      <c r="N2" s="68" t="s">
+      <c r="A2" s="87"/>
+      <c r="B2" s="88"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="88"/>
+      <c r="E2" s="88"/>
+      <c r="F2" s="88"/>
+      <c r="G2" s="88"/>
+      <c r="H2" s="88"/>
+      <c r="I2" s="88"/>
+      <c r="J2" s="88"/>
+      <c r="K2" s="88"/>
+      <c r="L2" s="88"/>
+      <c r="M2" s="89"/>
+      <c r="N2" s="93" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="69"/>
-      <c r="P2" s="69"/>
-      <c r="Q2" s="69"/>
-      <c r="R2" s="69"/>
-      <c r="S2" s="69"/>
-      <c r="T2" s="69"/>
-      <c r="U2" s="70"/>
-      <c r="V2" s="101" t="s">
+      <c r="O2" s="94"/>
+      <c r="P2" s="94"/>
+      <c r="Q2" s="94"/>
+      <c r="R2" s="94"/>
+      <c r="S2" s="94"/>
+      <c r="T2" s="94"/>
+      <c r="U2" s="95"/>
+      <c r="V2" s="126" t="s">
         <v>15</v>
       </c>
-      <c r="W2" s="102"/>
-      <c r="X2" s="102"/>
-      <c r="Y2" s="102"/>
-      <c r="Z2" s="102"/>
-      <c r="AA2" s="102"/>
-      <c r="AB2" s="102"/>
-      <c r="AC2" s="103"/>
-      <c r="AD2" s="131"/>
-      <c r="AE2" s="132"/>
-      <c r="AF2" s="132"/>
-      <c r="AG2" s="132"/>
-      <c r="AH2" s="132"/>
-      <c r="AI2" s="132"/>
-      <c r="AJ2" s="132"/>
-      <c r="AK2" s="133"/>
-      <c r="AL2" s="120"/>
-      <c r="AM2" s="121"/>
-      <c r="AN2" s="125"/>
-      <c r="AO2" s="126"/>
-      <c r="AP2" s="126"/>
-      <c r="AQ2" s="126"/>
-      <c r="AR2" s="127"/>
-      <c r="AS2" s="110"/>
-      <c r="AT2" s="112"/>
-      <c r="AU2" s="110"/>
-      <c r="AV2" s="111"/>
-      <c r="AW2" s="111"/>
-      <c r="AX2" s="111"/>
-      <c r="AY2" s="111"/>
-      <c r="AZ2" s="111"/>
-      <c r="BA2" s="111"/>
-      <c r="BB2" s="111"/>
-      <c r="BC2" s="111"/>
-      <c r="BD2" s="111"/>
-      <c r="BE2" s="111"/>
-      <c r="BF2" s="111"/>
-      <c r="BG2" s="111"/>
-      <c r="BH2" s="111"/>
-      <c r="BI2" s="111"/>
-      <c r="BJ2" s="111"/>
-      <c r="BK2" s="111"/>
-      <c r="BL2" s="111"/>
-      <c r="BM2" s="111"/>
-      <c r="BN2" s="111"/>
-      <c r="BO2" s="111"/>
-      <c r="BP2" s="111"/>
-      <c r="BQ2" s="111"/>
-      <c r="BR2" s="111"/>
-      <c r="BS2" s="111"/>
-      <c r="BT2" s="111"/>
-      <c r="BU2" s="111"/>
-      <c r="BV2" s="111"/>
-      <c r="BW2" s="111"/>
-      <c r="BX2" s="111"/>
-      <c r="BY2" s="111"/>
-      <c r="BZ2" s="111"/>
-      <c r="CA2" s="111"/>
-      <c r="CB2" s="111"/>
-      <c r="CC2" s="111"/>
-      <c r="CD2" s="112"/>
-      <c r="CE2" s="86"/>
-      <c r="CF2" s="87"/>
-      <c r="CG2" s="87"/>
-      <c r="CH2" s="87"/>
-      <c r="CI2" s="87"/>
-      <c r="CJ2" s="87"/>
-      <c r="CK2" s="87"/>
-      <c r="CL2" s="87"/>
-      <c r="CM2" s="87"/>
-      <c r="CN2" s="87"/>
-      <c r="CO2" s="87"/>
-      <c r="CP2" s="87"/>
-      <c r="CQ2" s="87"/>
-      <c r="CR2" s="87"/>
-      <c r="CS2" s="87"/>
-      <c r="CT2" s="87"/>
-      <c r="CU2" s="87"/>
-      <c r="CV2" s="87"/>
-      <c r="CW2" s="87"/>
-      <c r="CX2" s="87"/>
-      <c r="CY2" s="87"/>
-      <c r="CZ2" s="87"/>
-      <c r="DA2" s="87"/>
-      <c r="DB2" s="87"/>
-      <c r="DC2" s="87"/>
-      <c r="DD2" s="87"/>
-      <c r="DE2" s="87"/>
-      <c r="DF2" s="87"/>
-      <c r="DG2" s="87"/>
-      <c r="DH2" s="87"/>
-      <c r="DI2" s="87"/>
-      <c r="DJ2" s="87"/>
-      <c r="DK2" s="88"/>
-      <c r="DL2" s="92"/>
-      <c r="DM2" s="93"/>
-      <c r="DN2" s="93"/>
-      <c r="DO2" s="93"/>
-      <c r="DP2" s="93"/>
-      <c r="DQ2" s="93"/>
-      <c r="DR2" s="93"/>
-      <c r="DS2" s="93"/>
-      <c r="DT2" s="93"/>
-      <c r="DU2" s="93"/>
-      <c r="DV2" s="93"/>
-      <c r="DW2" s="93"/>
-      <c r="DX2" s="93"/>
-      <c r="DY2" s="93"/>
-      <c r="DZ2" s="94"/>
-      <c r="EA2" s="116"/>
-      <c r="EB2" s="117"/>
-      <c r="EC2" s="117"/>
-      <c r="ED2" s="117"/>
-      <c r="EE2" s="117"/>
-      <c r="EF2" s="117"/>
-      <c r="EG2" s="117"/>
-      <c r="EH2" s="117"/>
-      <c r="EI2" s="117"/>
-      <c r="EJ2" s="117"/>
-      <c r="EK2" s="117"/>
-      <c r="EL2" s="117"/>
-      <c r="EM2" s="113" t="s">
+      <c r="W2" s="127"/>
+      <c r="X2" s="127"/>
+      <c r="Y2" s="127"/>
+      <c r="Z2" s="127"/>
+      <c r="AA2" s="127"/>
+      <c r="AB2" s="127"/>
+      <c r="AC2" s="128"/>
+      <c r="AD2" s="77"/>
+      <c r="AE2" s="78"/>
+      <c r="AF2" s="78"/>
+      <c r="AG2" s="78"/>
+      <c r="AH2" s="78"/>
+      <c r="AI2" s="78"/>
+      <c r="AJ2" s="78"/>
+      <c r="AK2" s="79"/>
+      <c r="AL2" s="66"/>
+      <c r="AM2" s="67"/>
+      <c r="AN2" s="71"/>
+      <c r="AO2" s="72"/>
+      <c r="AP2" s="72"/>
+      <c r="AQ2" s="72"/>
+      <c r="AR2" s="73"/>
+      <c r="AS2" s="82"/>
+      <c r="AT2" s="83"/>
+      <c r="AU2" s="82"/>
+      <c r="AV2" s="133"/>
+      <c r="AW2" s="133"/>
+      <c r="AX2" s="133"/>
+      <c r="AY2" s="133"/>
+      <c r="AZ2" s="133"/>
+      <c r="BA2" s="133"/>
+      <c r="BB2" s="133"/>
+      <c r="BC2" s="133"/>
+      <c r="BD2" s="133"/>
+      <c r="BE2" s="133"/>
+      <c r="BF2" s="133"/>
+      <c r="BG2" s="133"/>
+      <c r="BH2" s="133"/>
+      <c r="BI2" s="133"/>
+      <c r="BJ2" s="133"/>
+      <c r="BK2" s="133"/>
+      <c r="BL2" s="133"/>
+      <c r="BM2" s="133"/>
+      <c r="BN2" s="133"/>
+      <c r="BO2" s="133"/>
+      <c r="BP2" s="133"/>
+      <c r="BQ2" s="133"/>
+      <c r="BR2" s="133"/>
+      <c r="BS2" s="133"/>
+      <c r="BT2" s="133"/>
+      <c r="BU2" s="133"/>
+      <c r="BV2" s="133"/>
+      <c r="BW2" s="133"/>
+      <c r="BX2" s="133"/>
+      <c r="BY2" s="133"/>
+      <c r="BZ2" s="133"/>
+      <c r="CA2" s="133"/>
+      <c r="CB2" s="133"/>
+      <c r="CC2" s="133"/>
+      <c r="CD2" s="83"/>
+      <c r="CE2" s="111"/>
+      <c r="CF2" s="112"/>
+      <c r="CG2" s="112"/>
+      <c r="CH2" s="112"/>
+      <c r="CI2" s="112"/>
+      <c r="CJ2" s="112"/>
+      <c r="CK2" s="112"/>
+      <c r="CL2" s="112"/>
+      <c r="CM2" s="112"/>
+      <c r="CN2" s="112"/>
+      <c r="CO2" s="112"/>
+      <c r="CP2" s="112"/>
+      <c r="CQ2" s="112"/>
+      <c r="CR2" s="112"/>
+      <c r="CS2" s="112"/>
+      <c r="CT2" s="112"/>
+      <c r="CU2" s="112"/>
+      <c r="CV2" s="112"/>
+      <c r="CW2" s="112"/>
+      <c r="CX2" s="112"/>
+      <c r="CY2" s="112"/>
+      <c r="CZ2" s="112"/>
+      <c r="DA2" s="112"/>
+      <c r="DB2" s="112"/>
+      <c r="DC2" s="112"/>
+      <c r="DD2" s="112"/>
+      <c r="DE2" s="112"/>
+      <c r="DF2" s="112"/>
+      <c r="DG2" s="112"/>
+      <c r="DH2" s="112"/>
+      <c r="DI2" s="112"/>
+      <c r="DJ2" s="112"/>
+      <c r="DK2" s="113"/>
+      <c r="DL2" s="117"/>
+      <c r="DM2" s="118"/>
+      <c r="DN2" s="118"/>
+      <c r="DO2" s="118"/>
+      <c r="DP2" s="118"/>
+      <c r="DQ2" s="118"/>
+      <c r="DR2" s="118"/>
+      <c r="DS2" s="118"/>
+      <c r="DT2" s="118"/>
+      <c r="DU2" s="118"/>
+      <c r="DV2" s="118"/>
+      <c r="DW2" s="118"/>
+      <c r="DX2" s="118"/>
+      <c r="DY2" s="118"/>
+      <c r="DZ2" s="119"/>
+      <c r="EA2" s="62"/>
+      <c r="EB2" s="63"/>
+      <c r="EC2" s="63"/>
+      <c r="ED2" s="63"/>
+      <c r="EE2" s="63"/>
+      <c r="EF2" s="63"/>
+      <c r="EG2" s="63"/>
+      <c r="EH2" s="63"/>
+      <c r="EI2" s="63"/>
+      <c r="EJ2" s="63"/>
+      <c r="EK2" s="63"/>
+      <c r="EL2" s="63"/>
+      <c r="EM2" s="59" t="s">
         <v>230</v>
       </c>
-      <c r="EN2" s="114"/>
-      <c r="EO2" s="114"/>
-      <c r="EP2" s="114"/>
-      <c r="EQ2" s="114"/>
-      <c r="ER2" s="114"/>
-      <c r="ES2" s="114"/>
-      <c r="ET2" s="114"/>
-      <c r="EU2" s="114"/>
-      <c r="EV2" s="114"/>
-      <c r="EW2" s="114"/>
-      <c r="EX2" s="114"/>
-      <c r="EY2" s="115"/>
-      <c r="EZ2" s="71" t="s">
+      <c r="EN2" s="60"/>
+      <c r="EO2" s="60"/>
+      <c r="EP2" s="60"/>
+      <c r="EQ2" s="60"/>
+      <c r="ER2" s="60"/>
+      <c r="ES2" s="60"/>
+      <c r="ET2" s="60"/>
+      <c r="EU2" s="60"/>
+      <c r="EV2" s="60"/>
+      <c r="EW2" s="60"/>
+      <c r="EX2" s="60"/>
+      <c r="EY2" s="61"/>
+      <c r="EZ2" s="96" t="s">
         <v>16</v>
       </c>
-      <c r="FA2" s="72"/>
-      <c r="FB2" s="72"/>
-      <c r="FC2" s="72"/>
-      <c r="FD2" s="72"/>
-      <c r="FE2" s="72"/>
-      <c r="FF2" s="72"/>
-      <c r="FG2" s="72"/>
-      <c r="FH2" s="72"/>
-      <c r="FI2" s="72"/>
-      <c r="FJ2" s="72"/>
-      <c r="FK2" s="72"/>
-      <c r="FL2" s="72"/>
-      <c r="FM2" s="72"/>
-      <c r="FN2" s="72"/>
-      <c r="FO2" s="72"/>
-      <c r="FP2" s="73"/>
-      <c r="FQ2" s="74" t="s">
+      <c r="FA2" s="97"/>
+      <c r="FB2" s="97"/>
+      <c r="FC2" s="97"/>
+      <c r="FD2" s="97"/>
+      <c r="FE2" s="97"/>
+      <c r="FF2" s="97"/>
+      <c r="FG2" s="97"/>
+      <c r="FH2" s="97"/>
+      <c r="FI2" s="97"/>
+      <c r="FJ2" s="97"/>
+      <c r="FK2" s="97"/>
+      <c r="FL2" s="97"/>
+      <c r="FM2" s="97"/>
+      <c r="FN2" s="97"/>
+      <c r="FO2" s="97"/>
+      <c r="FP2" s="98"/>
+      <c r="FQ2" s="99" t="s">
         <v>17</v>
       </c>
-      <c r="FR2" s="75"/>
-      <c r="FS2" s="75"/>
-      <c r="FT2" s="75"/>
-      <c r="FU2" s="75"/>
-      <c r="FV2" s="75"/>
-      <c r="FW2" s="75"/>
-      <c r="FX2" s="75"/>
-      <c r="FY2" s="76"/>
-      <c r="FZ2" s="77" t="s">
+      <c r="FR2" s="100"/>
+      <c r="FS2" s="100"/>
+      <c r="FT2" s="100"/>
+      <c r="FU2" s="100"/>
+      <c r="FV2" s="100"/>
+      <c r="FW2" s="100"/>
+      <c r="FX2" s="100"/>
+      <c r="FY2" s="101"/>
+      <c r="FZ2" s="102" t="s">
         <v>18</v>
       </c>
-      <c r="GA2" s="78"/>
-      <c r="GB2" s="78"/>
-      <c r="GC2" s="78"/>
-      <c r="GD2" s="78"/>
-      <c r="GE2" s="78"/>
-      <c r="GF2" s="79"/>
-      <c r="GG2" s="62"/>
-      <c r="GH2" s="63"/>
-      <c r="GI2" s="63"/>
-      <c r="GJ2" s="64"/>
-      <c r="GK2" s="99"/>
-      <c r="GL2" s="81"/>
-      <c r="GM2" s="66"/>
-      <c r="GN2" s="66"/>
+      <c r="GA2" s="103"/>
+      <c r="GB2" s="103"/>
+      <c r="GC2" s="103"/>
+      <c r="GD2" s="103"/>
+      <c r="GE2" s="103"/>
+      <c r="GF2" s="104"/>
+      <c r="GG2" s="87"/>
+      <c r="GH2" s="88"/>
+      <c r="GI2" s="88"/>
+      <c r="GJ2" s="89"/>
+      <c r="GK2" s="124"/>
+      <c r="GL2" s="106"/>
+      <c r="GM2" s="91"/>
+      <c r="GN2" s="91"/>
     </row>
     <row r="3" spans="1:196" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="13" t="s">
@@ -4291,10 +4297,10 @@
       <c r="GJ3" s="43" t="s">
         <v>98</v>
       </c>
-      <c r="GK3" s="100"/>
-      <c r="GL3" s="82"/>
-      <c r="GM3" s="67"/>
-      <c r="GN3" s="67"/>
+      <c r="GK3" s="125"/>
+      <c r="GL3" s="107"/>
+      <c r="GM3" s="92"/>
+      <c r="GN3" s="92"/>
     </row>
     <row r="4" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -5076,15 +5082,17 @@
         <v>99</v>
       </c>
     </row>
+    <row r="8" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>250</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:GN5" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="22">
-    <mergeCell ref="EM2:EY2"/>
-    <mergeCell ref="EA2:EL2"/>
-    <mergeCell ref="AL1:AM2"/>
-    <mergeCell ref="AN1:AR2"/>
-    <mergeCell ref="AD1:AK2"/>
-    <mergeCell ref="AS1:AT2"/>
     <mergeCell ref="A1:M2"/>
     <mergeCell ref="GM1:GM3"/>
     <mergeCell ref="GN1:GN3"/>
@@ -5101,6 +5109,12 @@
     <mergeCell ref="N1:AC1"/>
     <mergeCell ref="GG1:GJ2"/>
     <mergeCell ref="AU1:CD2"/>
+    <mergeCell ref="EM2:EY2"/>
+    <mergeCell ref="EA2:EL2"/>
+    <mergeCell ref="AL1:AM2"/>
+    <mergeCell ref="AN1:AR2"/>
+    <mergeCell ref="AD1:AK2"/>
+    <mergeCell ref="AS1:AT2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A7:B1048576 A3:A6">
     <cfRule type="duplicateValues" dxfId="0" priority="142"/>

</xml_diff>

<commit_message>
Reordenar main.py segun secuencia de ejecucion confirmada: SRI, Municipios, SERCOP, Salud, IESS, SCVS, Antecedentes Penales, Sentenciados, Funcion Judicial + Fiscalia, Contraloria
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3B647E-FA78-4767-8194-F76E9532DD08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9985CA12-2C74-4AC1-9120-1EA073B75CEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" activeTab="1" xr2:uid="{5FC7DFE8-7D61-4367-A58E-059126CAAC7E}"/>
   </bookViews>
@@ -253,7 +253,22 @@
         </r>
       </text>
     </comment>
-    <comment ref="AN3" authorId="0" shapeId="0" xr:uid="{D0A9EAAD-4334-404B-86F8-6183FC999B8A}">
+    <comment ref="AN3" authorId="0" shapeId="0" xr:uid="{55E42DED-5D92-47C5-B21F-2B310DA734C9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>SI registra y no registra
+NO posee registro en el sitio web</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AR3" authorId="0" shapeId="0" xr:uid="{D0A9EAAD-4334-404B-86F8-6183FC999B8A}">
       <text>
         <r>
           <rPr>
@@ -266,21 +281,6 @@
           <t>Compañias
 SI Cumple con sis obligaciones
 NO Cumple con sis obligaciones</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AQ3" authorId="0" shapeId="0" xr:uid="{55E42DED-5D92-47C5-B21F-2B310DA734C9}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>SI registra y no registra
-NO posee registro en el sitio web</t>
         </r>
       </text>
     </comment>
@@ -3838,20 +3838,20 @@
       <c r="AM3" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="AN3" s="32" t="s">
+      <c r="AN3" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="AO3" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="AP3" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="AQ3" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="AR3" s="32" t="s">
         <v>170</v>
-      </c>
-      <c r="AO3" s="16" t="s">
-        <v>169</v>
-      </c>
-      <c r="AP3" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="AQ3" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="AR3" s="33" t="s">
-        <v>35</v>
       </c>
       <c r="AS3" s="36" t="s">
         <v>40</v>
@@ -4404,15 +4404,15 @@
         <v>200</v>
       </c>
       <c r="AN4" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="AO4" s="6"/>
+        <v>168</v>
+      </c>
+      <c r="AO4" s="9">
+        <v>12683.75</v>
+      </c>
       <c r="AP4" s="6"/>
-      <c r="AQ4" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="AR4" s="9">
-        <v>12683.75</v>
+      <c r="AQ4" s="6"/>
+      <c r="AR4" s="5" t="s">
+        <v>99</v>
       </c>
       <c r="AS4" s="5" t="s">
         <v>177</v>
@@ -4658,15 +4658,15 @@
         <v>203</v>
       </c>
       <c r="AN5" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="AO5" s="9">
+        <v>0</v>
+      </c>
+      <c r="AP5" s="6"/>
+      <c r="AQ5" s="6"/>
+      <c r="AR5" s="5" t="s">
         <v>186</v>
-      </c>
-      <c r="AO5" s="6"/>
-      <c r="AP5" s="6"/>
-      <c r="AQ5" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="AR5" s="9">
-        <v>0</v>
       </c>
       <c r="AS5" s="45"/>
       <c r="AT5" s="45"/>
@@ -4865,13 +4865,13 @@
       <c r="AN6" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="AO6" s="6"/>
+      <c r="AO6" s="9">
+        <v>0</v>
+      </c>
       <c r="AP6" s="6"/>
-      <c r="AQ6" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="AR6" s="9">
-        <v>0</v>
+      <c r="AQ6" s="6"/>
+      <c r="AR6" s="5" t="s">
+        <v>99</v>
       </c>
       <c r="AS6" s="45"/>
       <c r="AT6" s="45"/>

</xml_diff>

<commit_message>
feat(excel): mapeo de Municipios, SERCOP (proveedor + certificados), Salud, IESS, SCVS Companias
- escribir_municipios: consolida los 5 municipios en 2 columnas
  (AF nombres con deuda separados por '/', AG suma total). Caso borde:
  si no esta registrado en ninguno, mensaje especial en vez de 'Ninguno'.
- escribir_sercop_proveedor: columna AH (INCOP), texto directo del
  scraper.
- escribir_sercop_certificados: columnas AI/AJ, un valor por cada uno
  de los 2 tipos de certificado (contratos pendientes / incumplimientos).
- escribir_salud: columnas AL/AM (situacion laboral, tipo afiliacion).
- escribir_iess: columnas AN/AO (texto mora + deuda en formato \$,
  normalizado a \.00 cuando no hay mora).
- escribir_scvs_companias: columna AR (Supercias), mapea el texto
  crudo del scraper a las 3 opciones exactas (SI/NO cumple/NA).
- Todos probados con datos de ejemplo en tests/prueba_manual_excel_writer.py.
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="259" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="259" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametrizacion" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Revision'!$A$3:$GN$5</definedName>
   </definedNames>
-  <calcPr calcId="191028" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -24,7 +24,7 @@
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="13">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -92,26 +92,6 @@
       <family val="1"/>
       <color theme="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color indexed="81"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Tahoma"/>
-      <family val="2"/>
-      <color indexed="81"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-      <b val="1"/>
-      <color indexed="81"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
@@ -218,7 +198,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="53">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -227,21 +207,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -266,36 +231,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -330,53 +265,10 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -434,9 +326,7 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -448,39 +338,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top style="medium">
         <color indexed="64"/>
@@ -525,69 +382,13 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -611,19 +412,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -695,36 +483,6 @@
         <color indexed="64"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
@@ -755,15 +513,6 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -844,6 +593,45 @@
         <color indexed="64"/>
       </right>
       <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -853,47 +641,17 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="171">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -912,7 +670,7 @@
     <xf numFmtId="14" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -927,437 +685,263 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="28" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1512,8 +1096,9 @@
     </comment>
     <comment ref="AH3" authorId="0" shapeId="0">
       <text>
-        <t>PROVEDOR DEL ESTADO
-SI / NO</t>
+        <t xml:space="preserve">PROVEEDOR DEL ESTADO/
+NO ES PROVEEDOR DEL ESTADO
+</t>
       </text>
     </comment>
     <comment ref="AI3" authorId="0" shapeId="0">
@@ -2418,7 +2003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:GN8"/>
+  <dimension ref="A1:GN10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.44140625" defaultRowHeight="70.05" customHeight="1" outlineLevelCol="0"/>
   <cols>
     <col width="14.6640625" bestFit="1" customWidth="1" style="4" min="1" max="1"/>
@@ -2427,7 +2012,7 @@
     <col width="17.6640625" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
     <col width="27.5546875" bestFit="1" customWidth="1" style="5" min="5" max="5"/>
     <col width="31.21875" bestFit="1" customWidth="1" style="5" min="6" max="6"/>
-    <col width="18.44140625" bestFit="1" customWidth="1" style="134" min="7" max="7"/>
+    <col width="18.44140625" bestFit="1" customWidth="1" style="100" min="7" max="7"/>
     <col width="25.88671875" bestFit="1" customWidth="1" style="5" min="8" max="8"/>
     <col width="27.44140625" bestFit="1" customWidth="1" style="4" min="9" max="9"/>
     <col width="22.44140625" bestFit="1" customWidth="1" style="5" min="10" max="10"/>
@@ -2436,23 +2021,24 @@
     <col width="14.44140625" bestFit="1" customWidth="1" style="5" min="13" max="13"/>
     <col width="16.44140625" bestFit="1" customWidth="1" style="5" min="14" max="14"/>
     <col width="24.77734375" bestFit="1" customWidth="1" style="5" min="15" max="15"/>
-    <col width="20.5546875" bestFit="1" customWidth="1" style="134" min="16" max="16"/>
-    <col width="16.88671875" bestFit="1" customWidth="1" style="134" min="17" max="17"/>
-    <col width="16.88671875" customWidth="1" style="134" min="18" max="18"/>
+    <col width="20.5546875" bestFit="1" customWidth="1" style="100" min="16" max="16"/>
+    <col width="16.88671875" bestFit="1" customWidth="1" style="100" min="17" max="17"/>
+    <col width="16.88671875" customWidth="1" style="100" min="18" max="18"/>
     <col width="24" bestFit="1" customWidth="1" style="5" min="19" max="19"/>
     <col width="24.109375" bestFit="1" customWidth="1" style="5" min="20" max="20"/>
     <col width="46.5546875" bestFit="1" customWidth="1" style="5" min="21" max="21"/>
     <col width="16.44140625" bestFit="1" customWidth="1" style="5" min="22" max="22"/>
     <col width="24.77734375" bestFit="1" customWidth="1" style="5" min="23" max="23"/>
-    <col width="20.5546875" bestFit="1" customWidth="1" style="134" min="24" max="24"/>
-    <col width="16.88671875" bestFit="1" customWidth="1" style="134" min="25" max="25"/>
-    <col width="19.44140625" bestFit="1" customWidth="1" style="134" min="26" max="26"/>
+    <col width="20.5546875" bestFit="1" customWidth="1" style="100" min="24" max="24"/>
+    <col width="16.88671875" bestFit="1" customWidth="1" style="100" min="25" max="25"/>
+    <col width="19.44140625" bestFit="1" customWidth="1" style="100" min="26" max="26"/>
     <col width="51.33203125" customWidth="1" style="5" min="27" max="27"/>
     <col width="25.33203125" bestFit="1" customWidth="1" style="5" min="28" max="28"/>
     <col width="29.109375" bestFit="1" customWidth="1" style="5" min="29" max="29"/>
-    <col width="27.5546875" bestFit="1" customWidth="1" style="5" min="30" max="31"/>
+    <col width="27.5546875" bestFit="1" customWidth="1" style="5" min="30" max="30"/>
+    <col width="29.88671875" customWidth="1" style="5" min="31" max="31"/>
     <col width="24.33203125" bestFit="1" customWidth="1" style="5" min="32" max="32"/>
-    <col width="14" bestFit="1" customWidth="1" style="135" min="33" max="33"/>
+    <col width="14" bestFit="1" customWidth="1" style="101" min="33" max="33"/>
     <col width="24.88671875" bestFit="1" customWidth="1" style="5" min="34" max="34"/>
     <col width="29.44140625" bestFit="1" customWidth="1" style="5" min="35" max="35"/>
     <col width="19.6640625" bestFit="1" customWidth="1" style="5" min="36" max="36"/>
@@ -2460,54 +2046,54 @@
     <col width="23.21875" bestFit="1" customWidth="1" style="5" min="38" max="38"/>
     <col width="23.77734375" bestFit="1" customWidth="1" style="5" min="39" max="39"/>
     <col width="28.88671875" bestFit="1" customWidth="1" style="5" min="40" max="40"/>
-    <col width="11.33203125" bestFit="1" customWidth="1" style="5" min="41" max="41"/>
+    <col width="15.33203125" customWidth="1" style="101" min="41" max="41"/>
     <col width="23.109375" bestFit="1" customWidth="1" style="5" min="42" max="42"/>
     <col width="22.88671875" bestFit="1" customWidth="1" style="5" min="43" max="43"/>
-    <col width="25.88671875" bestFit="1" customWidth="1" style="136" min="44" max="44"/>
+    <col width="25.88671875" bestFit="1" customWidth="1" style="102" min="44" max="44"/>
     <col width="34.6640625" bestFit="1" customWidth="1" style="5" min="45" max="46"/>
     <col width="27.21875" bestFit="1" customWidth="1" style="5" min="47" max="47"/>
     <col width="26.88671875" bestFit="1" customWidth="1" style="5" min="48" max="48"/>
     <col width="10.77734375" bestFit="1" customWidth="1" style="4" min="49" max="49"/>
     <col width="11.88671875" bestFit="1" customWidth="1" style="5" min="50" max="50"/>
-    <col width="23.21875" bestFit="1" customWidth="1" style="136" min="51" max="51"/>
+    <col width="23.21875" bestFit="1" customWidth="1" style="102" min="51" max="51"/>
     <col width="21" bestFit="1" customWidth="1" style="5" min="52" max="52"/>
     <col width="27.6640625" bestFit="1" customWidth="1" style="5" min="53" max="53"/>
     <col width="20.21875" bestFit="1" customWidth="1" style="5" min="54" max="54"/>
-    <col width="30" bestFit="1" customWidth="1" style="136" min="55" max="55"/>
+    <col width="30" bestFit="1" customWidth="1" style="102" min="55" max="55"/>
     <col width="27.21875" bestFit="1" customWidth="1" style="5" min="56" max="56"/>
     <col width="26.88671875" bestFit="1" customWidth="1" style="5" min="57" max="57"/>
     <col width="10.77734375" bestFit="1" customWidth="1" style="4" min="58" max="58"/>
     <col width="11.88671875" bestFit="1" customWidth="1" style="5" min="59" max="59"/>
-    <col width="23.21875" bestFit="1" customWidth="1" style="136" min="60" max="60"/>
+    <col width="23.21875" bestFit="1" customWidth="1" style="102" min="60" max="60"/>
     <col width="21" bestFit="1" customWidth="1" style="5" min="61" max="61"/>
     <col width="18.44140625" bestFit="1" customWidth="1" style="5" min="62" max="62"/>
     <col width="20.21875" bestFit="1" customWidth="1" style="5" min="63" max="63"/>
-    <col width="30" bestFit="1" customWidth="1" style="136" min="64" max="64"/>
+    <col width="30" bestFit="1" customWidth="1" style="102" min="64" max="64"/>
     <col width="27.21875" bestFit="1" customWidth="1" style="5" min="65" max="65"/>
     <col width="26.88671875" bestFit="1" customWidth="1" style="5" min="66" max="66"/>
     <col width="10.77734375" bestFit="1" customWidth="1" style="4" min="67" max="67"/>
     <col width="11.88671875" bestFit="1" customWidth="1" style="5" min="68" max="68"/>
-    <col width="23.21875" bestFit="1" customWidth="1" style="136" min="69" max="69"/>
+    <col width="23.21875" bestFit="1" customWidth="1" style="102" min="69" max="69"/>
     <col width="21" bestFit="1" customWidth="1" style="5" min="70" max="70"/>
     <col width="18.44140625" bestFit="1" customWidth="1" style="5" min="71" max="71"/>
     <col width="20.21875" bestFit="1" customWidth="1" style="5" min="72" max="72"/>
-    <col width="30" bestFit="1" customWidth="1" style="136" min="73" max="73"/>
+    <col width="30" bestFit="1" customWidth="1" style="102" min="73" max="73"/>
     <col width="39.109375" bestFit="1" customWidth="1" style="5" min="74" max="74"/>
     <col width="26.88671875" bestFit="1" customWidth="1" style="5" min="75" max="75"/>
     <col width="10.77734375" bestFit="1" customWidth="1" style="4" min="76" max="76"/>
     <col width="11.88671875" bestFit="1" customWidth="1" style="5" min="77" max="77"/>
-    <col width="23.21875" bestFit="1" customWidth="1" style="136" min="78" max="78"/>
+    <col width="23.21875" bestFit="1" customWidth="1" style="102" min="78" max="78"/>
     <col width="21" bestFit="1" customWidth="1" style="5" min="79" max="79"/>
     <col width="27.6640625" bestFit="1" customWidth="1" style="5" min="80" max="80"/>
     <col width="20.21875" bestFit="1" customWidth="1" style="5" min="81" max="81"/>
-    <col width="30" bestFit="1" customWidth="1" style="136" min="82" max="82"/>
+    <col width="30" bestFit="1" customWidth="1" style="102" min="82" max="82"/>
     <col width="27" customWidth="1" style="5" min="83" max="83"/>
     <col width="9.5546875" bestFit="1" customWidth="1" style="5" min="84" max="84"/>
     <col width="19.44140625" bestFit="1" customWidth="1" style="4" min="85" max="85"/>
     <col width="14" bestFit="1" customWidth="1" style="5" min="86" max="86"/>
     <col width="19.109375" bestFit="1" customWidth="1" style="5" min="87" max="87"/>
     <col width="20.33203125" bestFit="1" customWidth="1" style="5" min="88" max="88"/>
-    <col width="11.88671875" bestFit="1" customWidth="1" style="136" min="89" max="89"/>
+    <col width="11.88671875" bestFit="1" customWidth="1" style="102" min="89" max="89"/>
     <col width="16.6640625" bestFit="1" customWidth="1" style="5" min="90" max="90"/>
     <col width="25.33203125" bestFit="1" customWidth="1" style="5" min="91" max="91"/>
     <col width="9.5546875" bestFit="1" customWidth="1" style="5" min="92" max="92"/>
@@ -2515,7 +2101,7 @@
     <col width="14" bestFit="1" customWidth="1" style="5" min="94" max="94"/>
     <col width="19.109375" bestFit="1" customWidth="1" style="5" min="95" max="95"/>
     <col width="20.33203125" bestFit="1" customWidth="1" style="5" min="96" max="96"/>
-    <col width="11.88671875" bestFit="1" customWidth="1" style="136" min="97" max="97"/>
+    <col width="11.88671875" bestFit="1" customWidth="1" style="102" min="97" max="97"/>
     <col width="16.6640625" bestFit="1" customWidth="1" style="5" min="98" max="98"/>
     <col width="25.33203125" bestFit="1" customWidth="1" style="5" min="99" max="99"/>
     <col width="9.5546875" bestFit="1" customWidth="1" style="5" min="100" max="100"/>
@@ -2523,7 +2109,7 @@
     <col width="14" bestFit="1" customWidth="1" style="5" min="102" max="102"/>
     <col width="19.109375" bestFit="1" customWidth="1" style="5" min="103" max="103"/>
     <col width="20.33203125" bestFit="1" customWidth="1" style="5" min="104" max="104"/>
-    <col width="11.88671875" bestFit="1" customWidth="1" style="136" min="105" max="105"/>
+    <col width="11.88671875" bestFit="1" customWidth="1" style="102" min="105" max="105"/>
     <col width="16.6640625" bestFit="1" customWidth="1" style="5" min="106" max="106"/>
     <col width="25.33203125" bestFit="1" customWidth="1" style="5" min="107" max="107"/>
     <col width="9.5546875" bestFit="1" customWidth="1" style="5" min="108" max="108"/>
@@ -2531,7 +2117,7 @@
     <col width="14" bestFit="1" customWidth="1" style="5" min="110" max="110"/>
     <col width="19.109375" bestFit="1" customWidth="1" style="5" min="111" max="111"/>
     <col width="20.33203125" bestFit="1" customWidth="1" style="5" min="112" max="112"/>
-    <col width="11.88671875" bestFit="1" customWidth="1" style="136" min="113" max="113"/>
+    <col width="11.88671875" bestFit="1" customWidth="1" style="102" min="113" max="113"/>
     <col width="16.6640625" bestFit="1" customWidth="1" style="5" min="114" max="114"/>
     <col width="25.33203125" bestFit="1" customWidth="1" style="5" min="115" max="115"/>
     <col width="22.77734375" bestFit="1" customWidth="1" style="5" min="116" max="116"/>
@@ -2556,18 +2142,18 @@
     <col width="11.88671875" bestFit="1" customWidth="1" style="5" min="135" max="135"/>
     <col width="20" bestFit="1" customWidth="1" style="5" min="136" max="136"/>
     <col width="21.88671875" bestFit="1" customWidth="1" style="5" min="137" max="137"/>
-    <col width="20.77734375" bestFit="1" customWidth="1" style="136" min="138" max="138"/>
+    <col width="20.77734375" bestFit="1" customWidth="1" style="102" min="138" max="138"/>
     <col width="12.77734375" bestFit="1" customWidth="1" style="5" min="139" max="139"/>
     <col width="25.5546875" bestFit="1" customWidth="1" style="5" min="140" max="140"/>
     <col width="22.5546875" bestFit="1" customWidth="1" style="5" min="141" max="141"/>
     <col width="24.109375" bestFit="1" customWidth="1" style="5" min="142" max="142"/>
     <col width="19.109375" customWidth="1" style="5" min="143" max="143"/>
     <col width="19.109375" customWidth="1" style="4" min="144" max="145"/>
-    <col width="19.109375" customWidth="1" style="134" min="146" max="146"/>
+    <col width="19.109375" customWidth="1" style="100" min="146" max="146"/>
     <col width="19.109375" customWidth="1" style="4" min="147" max="149"/>
-    <col width="19.109375" customWidth="1" style="134" min="150" max="150"/>
+    <col width="19.109375" customWidth="1" style="100" min="150" max="150"/>
     <col width="19.109375" customWidth="1" style="4" min="151" max="153"/>
-    <col width="19.109375" customWidth="1" style="134" min="154" max="154"/>
+    <col width="19.109375" customWidth="1" style="100" min="154" max="154"/>
     <col width="18.88671875" bestFit="1" customWidth="1" style="4" min="155" max="155"/>
     <col width="19.44140625" bestFit="1" customWidth="1" style="5" min="156" max="156"/>
     <col width="21.77734375" bestFit="1" customWidth="1" style="5" min="157" max="157"/>
@@ -2577,12 +2163,12 @@
     <col width="23.77734375" bestFit="1" customWidth="1" style="5" min="161" max="161"/>
     <col width="20.21875" bestFit="1" customWidth="1" style="5" min="162" max="162"/>
     <col width="9.5546875" bestFit="1" customWidth="1" style="5" min="163" max="163"/>
-    <col width="22.21875" bestFit="1" customWidth="1" style="134" min="164" max="164"/>
+    <col width="22.21875" bestFit="1" customWidth="1" style="100" min="164" max="164"/>
     <col width="17.33203125" bestFit="1" customWidth="1" style="4" min="165" max="165"/>
     <col width="23.77734375" bestFit="1" customWidth="1" style="5" min="166" max="166"/>
     <col width="20.21875" bestFit="1" customWidth="1" style="5" min="167" max="167"/>
     <col width="9.5546875" bestFit="1" customWidth="1" style="5" min="168" max="168"/>
-    <col width="22.21875" bestFit="1" customWidth="1" style="134" min="169" max="169"/>
+    <col width="22.21875" bestFit="1" customWidth="1" style="100" min="169" max="169"/>
     <col width="17.33203125" bestFit="1" customWidth="1" style="4" min="170" max="170"/>
     <col width="23.77734375" bestFit="1" customWidth="1" style="5" min="171" max="171"/>
     <col width="20.21875" bestFit="1" customWidth="1" style="5" min="172" max="172"/>
@@ -2605,491 +2191,492 @@
     <col width="11.109375" bestFit="1" customWidth="1" style="5" min="189" max="191"/>
     <col width="21.109375" bestFit="1" customWidth="1" style="5" min="192" max="192"/>
     <col width="15" bestFit="1" customWidth="1" style="5" min="193" max="193"/>
-    <col width="17.6640625" bestFit="1" customWidth="1" style="137" min="194" max="194"/>
+    <col width="17.6640625" bestFit="1" customWidth="1" style="103" min="194" max="194"/>
     <col width="6.88671875" bestFit="1" customWidth="1" style="11" min="195" max="195"/>
     <col width="9.88671875" bestFit="1" customWidth="1" style="11" min="196" max="196"/>
-    <col width="11.44140625" customWidth="1" style="5" min="197" max="16384"/>
+    <col width="11.44140625" customWidth="1" style="5" min="197" max="210"/>
+    <col width="11.44140625" customWidth="1" style="5" min="211" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customFormat="1" customHeight="1" s="12" thickBot="1">
-      <c r="A1" s="138" t="inlineStr">
+      <c r="A1" s="66" t="inlineStr">
         <is>
           <t>IDENTIFICACIÓN BÁSICA</t>
         </is>
       </c>
-      <c r="B1" s="139" t="n"/>
-      <c r="C1" s="139" t="n"/>
-      <c r="D1" s="139" t="n"/>
-      <c r="E1" s="139" t="n"/>
-      <c r="F1" s="139" t="n"/>
-      <c r="G1" s="139" t="n"/>
-      <c r="H1" s="139" t="n"/>
-      <c r="I1" s="139" t="n"/>
-      <c r="J1" s="139" t="n"/>
-      <c r="K1" s="139" t="n"/>
-      <c r="L1" s="139" t="n"/>
-      <c r="M1" s="140" t="n"/>
-      <c r="N1" s="141" t="inlineStr">
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="67" t="n"/>
+      <c r="G1" s="67" t="n"/>
+      <c r="H1" s="67" t="n"/>
+      <c r="I1" s="67" t="n"/>
+      <c r="J1" s="67" t="n"/>
+      <c r="K1" s="67" t="n"/>
+      <c r="L1" s="67" t="n"/>
+      <c r="M1" s="68" t="n"/>
+      <c r="N1" s="98" t="inlineStr">
         <is>
           <t>Situación Fiscal</t>
         </is>
       </c>
-      <c r="O1" s="139" t="n"/>
-      <c r="P1" s="139" t="n"/>
-      <c r="Q1" s="139" t="n"/>
-      <c r="R1" s="139" t="n"/>
-      <c r="S1" s="139" t="n"/>
-      <c r="T1" s="139" t="n"/>
-      <c r="U1" s="139" t="n"/>
-      <c r="V1" s="139" t="n"/>
-      <c r="W1" s="139" t="n"/>
-      <c r="X1" s="139" t="n"/>
-      <c r="Y1" s="139" t="n"/>
-      <c r="Z1" s="139" t="n"/>
-      <c r="AA1" s="139" t="n"/>
-      <c r="AB1" s="139" t="n"/>
-      <c r="AC1" s="140" t="n"/>
-      <c r="AD1" s="142" t="inlineStr">
+      <c r="O1" s="67" t="n"/>
+      <c r="P1" s="67" t="n"/>
+      <c r="Q1" s="67" t="n"/>
+      <c r="R1" s="67" t="n"/>
+      <c r="S1" s="67" t="n"/>
+      <c r="T1" s="67" t="n"/>
+      <c r="U1" s="67" t="n"/>
+      <c r="V1" s="67" t="n"/>
+      <c r="W1" s="67" t="n"/>
+      <c r="X1" s="67" t="n"/>
+      <c r="Y1" s="67" t="n"/>
+      <c r="Z1" s="67" t="n"/>
+      <c r="AA1" s="67" t="n"/>
+      <c r="AB1" s="67" t="n"/>
+      <c r="AC1" s="68" t="n"/>
+      <c r="AD1" s="93" t="inlineStr">
         <is>
           <t>CERTIFICADOS INCOP / SRI / MUNICIPIO</t>
         </is>
       </c>
-      <c r="AE1" s="139" t="n"/>
-      <c r="AF1" s="139" t="n"/>
-      <c r="AG1" s="139" t="n"/>
-      <c r="AH1" s="139" t="n"/>
-      <c r="AI1" s="139" t="n"/>
-      <c r="AJ1" s="139" t="n"/>
-      <c r="AK1" s="140" t="n"/>
-      <c r="AL1" s="143" t="inlineStr">
+      <c r="AE1" s="67" t="n"/>
+      <c r="AF1" s="67" t="n"/>
+      <c r="AG1" s="67" t="n"/>
+      <c r="AH1" s="67" t="n"/>
+      <c r="AI1" s="67" t="n"/>
+      <c r="AJ1" s="67" t="n"/>
+      <c r="AK1" s="68" t="n"/>
+      <c r="AL1" s="86" t="inlineStr">
         <is>
           <t>SITUACION LABORAL</t>
         </is>
       </c>
-      <c r="AM1" s="140" t="n"/>
-      <c r="AN1" s="144" t="inlineStr">
+      <c r="AM1" s="68" t="n"/>
+      <c r="AN1" s="99" t="inlineStr">
         <is>
           <t>CERTIFICADOS CCO</t>
         </is>
       </c>
-      <c r="AO1" s="139" t="n"/>
-      <c r="AP1" s="139" t="n"/>
-      <c r="AQ1" s="139" t="n"/>
-      <c r="AR1" s="140" t="n"/>
-      <c r="AS1" s="80" t="inlineStr">
+      <c r="AO1" s="67" t="n"/>
+      <c r="AP1" s="67" t="n"/>
+      <c r="AQ1" s="67" t="n"/>
+      <c r="AR1" s="68" t="n"/>
+      <c r="AS1" s="92" t="inlineStr">
         <is>
           <t>SUPERCIAS</t>
         </is>
       </c>
-      <c r="AT1" s="145" t="n"/>
-      <c r="AU1" s="80" t="inlineStr">
+      <c r="AT1" s="82" t="n"/>
+      <c r="AU1" s="92" t="inlineStr">
         <is>
           <t xml:space="preserve">Empresas Relacionadas </t>
         </is>
       </c>
-      <c r="AV1" s="139" t="n"/>
-      <c r="AW1" s="139" t="n"/>
-      <c r="AX1" s="139" t="n"/>
-      <c r="AY1" s="139" t="n"/>
-      <c r="AZ1" s="139" t="n"/>
-      <c r="BA1" s="139" t="n"/>
-      <c r="BB1" s="139" t="n"/>
-      <c r="BC1" s="139" t="n"/>
-      <c r="BD1" s="139" t="n"/>
-      <c r="BE1" s="139" t="n"/>
-      <c r="BF1" s="139" t="n"/>
-      <c r="BG1" s="139" t="n"/>
-      <c r="BH1" s="139" t="n"/>
-      <c r="BI1" s="139" t="n"/>
-      <c r="BJ1" s="139" t="n"/>
-      <c r="BK1" s="139" t="n"/>
-      <c r="BL1" s="139" t="n"/>
-      <c r="BM1" s="139" t="n"/>
-      <c r="BN1" s="139" t="n"/>
-      <c r="BO1" s="139" t="n"/>
-      <c r="BP1" s="139" t="n"/>
-      <c r="BQ1" s="139" t="n"/>
-      <c r="BR1" s="139" t="n"/>
-      <c r="BS1" s="139" t="n"/>
-      <c r="BT1" s="139" t="n"/>
-      <c r="BU1" s="139" t="n"/>
-      <c r="BV1" s="139" t="n"/>
-      <c r="BW1" s="139" t="n"/>
-      <c r="BX1" s="139" t="n"/>
-      <c r="BY1" s="139" t="n"/>
-      <c r="BZ1" s="139" t="n"/>
-      <c r="CA1" s="139" t="n"/>
-      <c r="CB1" s="139" t="n"/>
-      <c r="CC1" s="139" t="n"/>
-      <c r="CD1" s="145" t="n"/>
-      <c r="CE1" s="108" t="inlineStr">
+      <c r="AV1" s="67" t="n"/>
+      <c r="AW1" s="67" t="n"/>
+      <c r="AX1" s="67" t="n"/>
+      <c r="AY1" s="67" t="n"/>
+      <c r="AZ1" s="67" t="n"/>
+      <c r="BA1" s="67" t="n"/>
+      <c r="BB1" s="67" t="n"/>
+      <c r="BC1" s="67" t="n"/>
+      <c r="BD1" s="67" t="n"/>
+      <c r="BE1" s="67" t="n"/>
+      <c r="BF1" s="67" t="n"/>
+      <c r="BG1" s="67" t="n"/>
+      <c r="BH1" s="67" t="n"/>
+      <c r="BI1" s="67" t="n"/>
+      <c r="BJ1" s="67" t="n"/>
+      <c r="BK1" s="67" t="n"/>
+      <c r="BL1" s="67" t="n"/>
+      <c r="BM1" s="67" t="n"/>
+      <c r="BN1" s="67" t="n"/>
+      <c r="BO1" s="67" t="n"/>
+      <c r="BP1" s="67" t="n"/>
+      <c r="BQ1" s="67" t="n"/>
+      <c r="BR1" s="67" t="n"/>
+      <c r="BS1" s="67" t="n"/>
+      <c r="BT1" s="67" t="n"/>
+      <c r="BU1" s="67" t="n"/>
+      <c r="BV1" s="67" t="n"/>
+      <c r="BW1" s="67" t="n"/>
+      <c r="BX1" s="67" t="n"/>
+      <c r="BY1" s="67" t="n"/>
+      <c r="BZ1" s="67" t="n"/>
+      <c r="CA1" s="67" t="n"/>
+      <c r="CB1" s="67" t="n"/>
+      <c r="CC1" s="67" t="n"/>
+      <c r="CD1" s="82" t="n"/>
+      <c r="CE1" s="94" t="inlineStr">
         <is>
           <t>BENEFICIARIOS FINALES</t>
         </is>
       </c>
-      <c r="CF1" s="139" t="n"/>
-      <c r="CG1" s="139" t="n"/>
-      <c r="CH1" s="139" t="n"/>
-      <c r="CI1" s="139" t="n"/>
-      <c r="CJ1" s="139" t="n"/>
-      <c r="CK1" s="139" t="n"/>
-      <c r="CL1" s="139" t="n"/>
-      <c r="CM1" s="139" t="n"/>
-      <c r="CN1" s="139" t="n"/>
-      <c r="CO1" s="139" t="n"/>
-      <c r="CP1" s="139" t="n"/>
-      <c r="CQ1" s="139" t="n"/>
-      <c r="CR1" s="139" t="n"/>
-      <c r="CS1" s="139" t="n"/>
-      <c r="CT1" s="139" t="n"/>
-      <c r="CU1" s="139" t="n"/>
-      <c r="CV1" s="139" t="n"/>
-      <c r="CW1" s="139" t="n"/>
-      <c r="CX1" s="139" t="n"/>
-      <c r="CY1" s="139" t="n"/>
-      <c r="CZ1" s="139" t="n"/>
-      <c r="DA1" s="139" t="n"/>
-      <c r="DB1" s="139" t="n"/>
-      <c r="DC1" s="139" t="n"/>
-      <c r="DD1" s="139" t="n"/>
-      <c r="DE1" s="139" t="n"/>
-      <c r="DF1" s="139" t="n"/>
-      <c r="DG1" s="139" t="n"/>
-      <c r="DH1" s="139" t="n"/>
-      <c r="DI1" s="139" t="n"/>
-      <c r="DJ1" s="139" t="n"/>
-      <c r="DK1" s="145" t="n"/>
-      <c r="DL1" s="114" t="inlineStr">
+      <c r="CF1" s="67" t="n"/>
+      <c r="CG1" s="67" t="n"/>
+      <c r="CH1" s="67" t="n"/>
+      <c r="CI1" s="67" t="n"/>
+      <c r="CJ1" s="67" t="n"/>
+      <c r="CK1" s="67" t="n"/>
+      <c r="CL1" s="67" t="n"/>
+      <c r="CM1" s="67" t="n"/>
+      <c r="CN1" s="67" t="n"/>
+      <c r="CO1" s="67" t="n"/>
+      <c r="CP1" s="67" t="n"/>
+      <c r="CQ1" s="67" t="n"/>
+      <c r="CR1" s="67" t="n"/>
+      <c r="CS1" s="67" t="n"/>
+      <c r="CT1" s="67" t="n"/>
+      <c r="CU1" s="67" t="n"/>
+      <c r="CV1" s="67" t="n"/>
+      <c r="CW1" s="67" t="n"/>
+      <c r="CX1" s="67" t="n"/>
+      <c r="CY1" s="67" t="n"/>
+      <c r="CZ1" s="67" t="n"/>
+      <c r="DA1" s="67" t="n"/>
+      <c r="DB1" s="67" t="n"/>
+      <c r="DC1" s="67" t="n"/>
+      <c r="DD1" s="67" t="n"/>
+      <c r="DE1" s="67" t="n"/>
+      <c r="DF1" s="67" t="n"/>
+      <c r="DG1" s="67" t="n"/>
+      <c r="DH1" s="67" t="n"/>
+      <c r="DI1" s="67" t="n"/>
+      <c r="DJ1" s="67" t="n"/>
+      <c r="DK1" s="82" t="n"/>
+      <c r="DL1" s="89" t="inlineStr">
         <is>
           <t>Empresas Extranjeras</t>
         </is>
       </c>
-      <c r="DM1" s="139" t="n"/>
-      <c r="DN1" s="139" t="n"/>
-      <c r="DO1" s="139" t="n"/>
-      <c r="DP1" s="139" t="n"/>
-      <c r="DQ1" s="139" t="n"/>
-      <c r="DR1" s="139" t="n"/>
-      <c r="DS1" s="139" t="n"/>
-      <c r="DT1" s="139" t="n"/>
-      <c r="DU1" s="139" t="n"/>
-      <c r="DV1" s="139" t="n"/>
-      <c r="DW1" s="139" t="n"/>
-      <c r="DX1" s="139" t="n"/>
-      <c r="DY1" s="139" t="n"/>
-      <c r="DZ1" s="145" t="n"/>
-      <c r="EA1" s="120" t="inlineStr">
+      <c r="DM1" s="67" t="n"/>
+      <c r="DN1" s="67" t="n"/>
+      <c r="DO1" s="67" t="n"/>
+      <c r="DP1" s="67" t="n"/>
+      <c r="DQ1" s="67" t="n"/>
+      <c r="DR1" s="67" t="n"/>
+      <c r="DS1" s="67" t="n"/>
+      <c r="DT1" s="67" t="n"/>
+      <c r="DU1" s="67" t="n"/>
+      <c r="DV1" s="67" t="n"/>
+      <c r="DW1" s="67" t="n"/>
+      <c r="DX1" s="67" t="n"/>
+      <c r="DY1" s="67" t="n"/>
+      <c r="DZ1" s="82" t="n"/>
+      <c r="EA1" s="81" t="inlineStr">
         <is>
           <t>Antecedentes Legales LA/FT</t>
         </is>
       </c>
-      <c r="EB1" s="139" t="n"/>
-      <c r="EC1" s="139" t="n"/>
-      <c r="ED1" s="139" t="n"/>
-      <c r="EE1" s="139" t="n"/>
-      <c r="EF1" s="139" t="n"/>
-      <c r="EG1" s="139" t="n"/>
-      <c r="EH1" s="139" t="n"/>
-      <c r="EI1" s="139" t="n"/>
-      <c r="EJ1" s="139" t="n"/>
-      <c r="EK1" s="139" t="n"/>
-      <c r="EL1" s="139" t="n"/>
-      <c r="EM1" s="139" t="n"/>
-      <c r="EN1" s="139" t="n"/>
-      <c r="EO1" s="139" t="n"/>
-      <c r="EP1" s="139" t="n"/>
-      <c r="EQ1" s="139" t="n"/>
-      <c r="ER1" s="139" t="n"/>
-      <c r="ES1" s="139" t="n"/>
-      <c r="ET1" s="139" t="n"/>
-      <c r="EU1" s="139" t="n"/>
-      <c r="EV1" s="139" t="n"/>
-      <c r="EW1" s="139" t="n"/>
-      <c r="EX1" s="139" t="n"/>
-      <c r="EY1" s="139" t="n"/>
-      <c r="EZ1" s="139" t="n"/>
-      <c r="FA1" s="139" t="n"/>
-      <c r="FB1" s="139" t="n"/>
-      <c r="FC1" s="139" t="n"/>
-      <c r="FD1" s="139" t="n"/>
-      <c r="FE1" s="139" t="n"/>
-      <c r="FF1" s="139" t="n"/>
-      <c r="FG1" s="139" t="n"/>
-      <c r="FH1" s="139" t="n"/>
-      <c r="FI1" s="139" t="n"/>
-      <c r="FJ1" s="139" t="n"/>
-      <c r="FK1" s="139" t="n"/>
-      <c r="FL1" s="139" t="n"/>
-      <c r="FM1" s="139" t="n"/>
-      <c r="FN1" s="139" t="n"/>
-      <c r="FO1" s="139" t="n"/>
-      <c r="FP1" s="139" t="n"/>
-      <c r="FQ1" s="139" t="n"/>
-      <c r="FR1" s="139" t="n"/>
-      <c r="FS1" s="139" t="n"/>
-      <c r="FT1" s="139" t="n"/>
-      <c r="FU1" s="139" t="n"/>
-      <c r="FV1" s="139" t="n"/>
-      <c r="FW1" s="139" t="n"/>
-      <c r="FX1" s="139" t="n"/>
-      <c r="FY1" s="139" t="n"/>
-      <c r="FZ1" s="139" t="n"/>
-      <c r="GA1" s="139" t="n"/>
-      <c r="GB1" s="139" t="n"/>
-      <c r="GC1" s="139" t="n"/>
-      <c r="GD1" s="139" t="n"/>
-      <c r="GE1" s="139" t="n"/>
-      <c r="GF1" s="145" t="n"/>
-      <c r="GG1" s="138" t="inlineStr">
+      <c r="EB1" s="67" t="n"/>
+      <c r="EC1" s="67" t="n"/>
+      <c r="ED1" s="67" t="n"/>
+      <c r="EE1" s="67" t="n"/>
+      <c r="EF1" s="67" t="n"/>
+      <c r="EG1" s="67" t="n"/>
+      <c r="EH1" s="67" t="n"/>
+      <c r="EI1" s="67" t="n"/>
+      <c r="EJ1" s="67" t="n"/>
+      <c r="EK1" s="67" t="n"/>
+      <c r="EL1" s="67" t="n"/>
+      <c r="EM1" s="67" t="n"/>
+      <c r="EN1" s="67" t="n"/>
+      <c r="EO1" s="67" t="n"/>
+      <c r="EP1" s="67" t="n"/>
+      <c r="EQ1" s="67" t="n"/>
+      <c r="ER1" s="67" t="n"/>
+      <c r="ES1" s="67" t="n"/>
+      <c r="ET1" s="67" t="n"/>
+      <c r="EU1" s="67" t="n"/>
+      <c r="EV1" s="67" t="n"/>
+      <c r="EW1" s="67" t="n"/>
+      <c r="EX1" s="67" t="n"/>
+      <c r="EY1" s="67" t="n"/>
+      <c r="EZ1" s="67" t="n"/>
+      <c r="FA1" s="67" t="n"/>
+      <c r="FB1" s="67" t="n"/>
+      <c r="FC1" s="67" t="n"/>
+      <c r="FD1" s="67" t="n"/>
+      <c r="FE1" s="67" t="n"/>
+      <c r="FF1" s="67" t="n"/>
+      <c r="FG1" s="67" t="n"/>
+      <c r="FH1" s="67" t="n"/>
+      <c r="FI1" s="67" t="n"/>
+      <c r="FJ1" s="67" t="n"/>
+      <c r="FK1" s="67" t="n"/>
+      <c r="FL1" s="67" t="n"/>
+      <c r="FM1" s="67" t="n"/>
+      <c r="FN1" s="67" t="n"/>
+      <c r="FO1" s="67" t="n"/>
+      <c r="FP1" s="67" t="n"/>
+      <c r="FQ1" s="67" t="n"/>
+      <c r="FR1" s="67" t="n"/>
+      <c r="FS1" s="67" t="n"/>
+      <c r="FT1" s="67" t="n"/>
+      <c r="FU1" s="67" t="n"/>
+      <c r="FV1" s="67" t="n"/>
+      <c r="FW1" s="67" t="n"/>
+      <c r="FX1" s="67" t="n"/>
+      <c r="FY1" s="67" t="n"/>
+      <c r="FZ1" s="67" t="n"/>
+      <c r="GA1" s="67" t="n"/>
+      <c r="GB1" s="67" t="n"/>
+      <c r="GC1" s="67" t="n"/>
+      <c r="GD1" s="67" t="n"/>
+      <c r="GE1" s="67" t="n"/>
+      <c r="GF1" s="82" t="n"/>
+      <c r="GG1" s="66" t="inlineStr">
         <is>
           <t>Determinación del perfil</t>
         </is>
       </c>
-      <c r="GH1" s="139" t="n"/>
-      <c r="GI1" s="139" t="n"/>
-      <c r="GJ1" s="140" t="n"/>
-      <c r="GK1" s="123" t="inlineStr">
+      <c r="GH1" s="67" t="n"/>
+      <c r="GI1" s="67" t="n"/>
+      <c r="GJ1" s="68" t="n"/>
+      <c r="GK1" s="74" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="GL1" s="146" t="inlineStr">
+      <c r="GL1" s="104" t="inlineStr">
         <is>
           <t xml:space="preserve">Fecha de revision </t>
         </is>
       </c>
-      <c r="GM1" s="90" t="inlineStr">
+      <c r="GM1" s="77" t="inlineStr">
         <is>
           <t>ÁREA</t>
         </is>
       </c>
-      <c r="GN1" s="90" t="inlineStr">
+      <c r="GN1" s="77" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
     </row>
     <row r="2" ht="25.8" customFormat="1" customHeight="1" s="12" thickBot="1">
-      <c r="A2" s="147" t="n"/>
-      <c r="B2" s="148" t="n"/>
-      <c r="C2" s="148" t="n"/>
-      <c r="D2" s="148" t="n"/>
-      <c r="E2" s="148" t="n"/>
-      <c r="F2" s="148" t="n"/>
-      <c r="G2" s="148" t="n"/>
-      <c r="H2" s="148" t="n"/>
-      <c r="I2" s="148" t="n"/>
-      <c r="J2" s="148" t="n"/>
-      <c r="K2" s="148" t="n"/>
-      <c r="L2" s="148" t="n"/>
-      <c r="M2" s="149" t="n"/>
-      <c r="N2" s="93" t="inlineStr">
+      <c r="A2" s="69" t="n"/>
+      <c r="B2" s="70" t="n"/>
+      <c r="C2" s="70" t="n"/>
+      <c r="D2" s="70" t="n"/>
+      <c r="E2" s="70" t="n"/>
+      <c r="F2" s="70" t="n"/>
+      <c r="G2" s="70" t="n"/>
+      <c r="H2" s="70" t="n"/>
+      <c r="I2" s="70" t="n"/>
+      <c r="J2" s="70" t="n"/>
+      <c r="K2" s="70" t="n"/>
+      <c r="L2" s="70" t="n"/>
+      <c r="M2" s="71" t="n"/>
+      <c r="N2" s="88" t="inlineStr">
         <is>
           <t>PERSONA NATURAL / JURIDICA</t>
         </is>
       </c>
-      <c r="O2" s="150" t="n"/>
-      <c r="P2" s="150" t="n"/>
-      <c r="Q2" s="150" t="n"/>
-      <c r="R2" s="150" t="n"/>
-      <c r="S2" s="150" t="n"/>
-      <c r="T2" s="150" t="n"/>
-      <c r="U2" s="151" t="n"/>
-      <c r="V2" s="152" t="inlineStr">
+      <c r="O2" s="64" t="n"/>
+      <c r="P2" s="64" t="n"/>
+      <c r="Q2" s="64" t="n"/>
+      <c r="R2" s="64" t="n"/>
+      <c r="S2" s="64" t="n"/>
+      <c r="T2" s="64" t="n"/>
+      <c r="U2" s="65" t="n"/>
+      <c r="V2" s="72" t="inlineStr">
         <is>
           <t>REPRESENTANTE LEGAL</t>
         </is>
       </c>
-      <c r="W2" s="150" t="n"/>
-      <c r="X2" s="150" t="n"/>
-      <c r="Y2" s="150" t="n"/>
-      <c r="Z2" s="150" t="n"/>
-      <c r="AA2" s="150" t="n"/>
-      <c r="AB2" s="150" t="n"/>
-      <c r="AC2" s="153" t="n"/>
-      <c r="AD2" s="147" t="n"/>
-      <c r="AE2" s="148" t="n"/>
-      <c r="AF2" s="148" t="n"/>
-      <c r="AG2" s="148" t="n"/>
-      <c r="AH2" s="148" t="n"/>
-      <c r="AI2" s="148" t="n"/>
-      <c r="AJ2" s="148" t="n"/>
-      <c r="AK2" s="149" t="n"/>
-      <c r="AL2" s="147" t="n"/>
-      <c r="AM2" s="149" t="n"/>
-      <c r="AN2" s="147" t="n"/>
-      <c r="AO2" s="148" t="n"/>
-      <c r="AP2" s="148" t="n"/>
-      <c r="AQ2" s="148" t="n"/>
-      <c r="AR2" s="149" t="n"/>
-      <c r="AS2" s="154" t="n"/>
-      <c r="AT2" s="155" t="n"/>
-      <c r="AU2" s="154" t="n"/>
-      <c r="AV2" s="156" t="n"/>
-      <c r="AW2" s="156" t="n"/>
-      <c r="AX2" s="156" t="n"/>
-      <c r="AY2" s="156" t="n"/>
-      <c r="AZ2" s="156" t="n"/>
-      <c r="BA2" s="156" t="n"/>
-      <c r="BB2" s="156" t="n"/>
-      <c r="BC2" s="156" t="n"/>
-      <c r="BD2" s="156" t="n"/>
-      <c r="BE2" s="156" t="n"/>
-      <c r="BF2" s="156" t="n"/>
-      <c r="BG2" s="156" t="n"/>
-      <c r="BH2" s="156" t="n"/>
-      <c r="BI2" s="156" t="n"/>
-      <c r="BJ2" s="156" t="n"/>
-      <c r="BK2" s="156" t="n"/>
-      <c r="BL2" s="156" t="n"/>
-      <c r="BM2" s="156" t="n"/>
-      <c r="BN2" s="156" t="n"/>
-      <c r="BO2" s="156" t="n"/>
-      <c r="BP2" s="156" t="n"/>
-      <c r="BQ2" s="156" t="n"/>
-      <c r="BR2" s="156" t="n"/>
-      <c r="BS2" s="156" t="n"/>
-      <c r="BT2" s="156" t="n"/>
-      <c r="BU2" s="156" t="n"/>
-      <c r="BV2" s="156" t="n"/>
-      <c r="BW2" s="156" t="n"/>
-      <c r="BX2" s="156" t="n"/>
-      <c r="BY2" s="156" t="n"/>
-      <c r="BZ2" s="156" t="n"/>
-      <c r="CA2" s="156" t="n"/>
-      <c r="CB2" s="156" t="n"/>
-      <c r="CC2" s="156" t="n"/>
-      <c r="CD2" s="155" t="n"/>
-      <c r="CE2" s="154" t="n"/>
-      <c r="CF2" s="156" t="n"/>
-      <c r="CG2" s="156" t="n"/>
-      <c r="CH2" s="156" t="n"/>
-      <c r="CI2" s="156" t="n"/>
-      <c r="CJ2" s="156" t="n"/>
-      <c r="CK2" s="156" t="n"/>
-      <c r="CL2" s="156" t="n"/>
-      <c r="CM2" s="156" t="n"/>
-      <c r="CN2" s="156" t="n"/>
-      <c r="CO2" s="156" t="n"/>
-      <c r="CP2" s="156" t="n"/>
-      <c r="CQ2" s="156" t="n"/>
-      <c r="CR2" s="156" t="n"/>
-      <c r="CS2" s="156" t="n"/>
-      <c r="CT2" s="156" t="n"/>
-      <c r="CU2" s="156" t="n"/>
-      <c r="CV2" s="156" t="n"/>
-      <c r="CW2" s="156" t="n"/>
-      <c r="CX2" s="156" t="n"/>
-      <c r="CY2" s="156" t="n"/>
-      <c r="CZ2" s="156" t="n"/>
-      <c r="DA2" s="156" t="n"/>
-      <c r="DB2" s="156" t="n"/>
-      <c r="DC2" s="156" t="n"/>
-      <c r="DD2" s="156" t="n"/>
-      <c r="DE2" s="156" t="n"/>
-      <c r="DF2" s="156" t="n"/>
-      <c r="DG2" s="156" t="n"/>
-      <c r="DH2" s="156" t="n"/>
-      <c r="DI2" s="156" t="n"/>
-      <c r="DJ2" s="156" t="n"/>
-      <c r="DK2" s="155" t="n"/>
-      <c r="DL2" s="154" t="n"/>
-      <c r="DM2" s="156" t="n"/>
-      <c r="DN2" s="156" t="n"/>
-      <c r="DO2" s="156" t="n"/>
-      <c r="DP2" s="156" t="n"/>
-      <c r="DQ2" s="156" t="n"/>
-      <c r="DR2" s="156" t="n"/>
-      <c r="DS2" s="156" t="n"/>
-      <c r="DT2" s="156" t="n"/>
-      <c r="DU2" s="156" t="n"/>
-      <c r="DV2" s="156" t="n"/>
-      <c r="DW2" s="156" t="n"/>
-      <c r="DX2" s="156" t="n"/>
-      <c r="DY2" s="156" t="n"/>
-      <c r="DZ2" s="155" t="n"/>
-      <c r="EA2" s="62" t="n"/>
-      <c r="EB2" s="150" t="n"/>
-      <c r="EC2" s="150" t="n"/>
-      <c r="ED2" s="150" t="n"/>
-      <c r="EE2" s="150" t="n"/>
-      <c r="EF2" s="150" t="n"/>
-      <c r="EG2" s="150" t="n"/>
-      <c r="EH2" s="150" t="n"/>
-      <c r="EI2" s="150" t="n"/>
-      <c r="EJ2" s="150" t="n"/>
-      <c r="EK2" s="150" t="n"/>
-      <c r="EL2" s="150" t="n"/>
-      <c r="EM2" s="157" t="inlineStr">
+      <c r="W2" s="64" t="n"/>
+      <c r="X2" s="64" t="n"/>
+      <c r="Y2" s="64" t="n"/>
+      <c r="Z2" s="64" t="n"/>
+      <c r="AA2" s="64" t="n"/>
+      <c r="AB2" s="64" t="n"/>
+      <c r="AC2" s="73" t="n"/>
+      <c r="AD2" s="69" t="n"/>
+      <c r="AE2" s="70" t="n"/>
+      <c r="AF2" s="70" t="n"/>
+      <c r="AG2" s="70" t="n"/>
+      <c r="AH2" s="70" t="n"/>
+      <c r="AI2" s="70" t="n"/>
+      <c r="AJ2" s="70" t="n"/>
+      <c r="AK2" s="71" t="n"/>
+      <c r="AL2" s="69" t="n"/>
+      <c r="AM2" s="71" t="n"/>
+      <c r="AN2" s="69" t="n"/>
+      <c r="AO2" s="70" t="n"/>
+      <c r="AP2" s="70" t="n"/>
+      <c r="AQ2" s="70" t="n"/>
+      <c r="AR2" s="71" t="n"/>
+      <c r="AS2" s="76" t="n"/>
+      <c r="AT2" s="91" t="n"/>
+      <c r="AU2" s="76" t="n"/>
+      <c r="AV2" s="90" t="n"/>
+      <c r="AW2" s="90" t="n"/>
+      <c r="AX2" s="90" t="n"/>
+      <c r="AY2" s="90" t="n"/>
+      <c r="AZ2" s="90" t="n"/>
+      <c r="BA2" s="90" t="n"/>
+      <c r="BB2" s="90" t="n"/>
+      <c r="BC2" s="90" t="n"/>
+      <c r="BD2" s="90" t="n"/>
+      <c r="BE2" s="90" t="n"/>
+      <c r="BF2" s="90" t="n"/>
+      <c r="BG2" s="90" t="n"/>
+      <c r="BH2" s="90" t="n"/>
+      <c r="BI2" s="90" t="n"/>
+      <c r="BJ2" s="90" t="n"/>
+      <c r="BK2" s="90" t="n"/>
+      <c r="BL2" s="90" t="n"/>
+      <c r="BM2" s="90" t="n"/>
+      <c r="BN2" s="90" t="n"/>
+      <c r="BO2" s="90" t="n"/>
+      <c r="BP2" s="90" t="n"/>
+      <c r="BQ2" s="90" t="n"/>
+      <c r="BR2" s="90" t="n"/>
+      <c r="BS2" s="90" t="n"/>
+      <c r="BT2" s="90" t="n"/>
+      <c r="BU2" s="90" t="n"/>
+      <c r="BV2" s="90" t="n"/>
+      <c r="BW2" s="90" t="n"/>
+      <c r="BX2" s="90" t="n"/>
+      <c r="BY2" s="90" t="n"/>
+      <c r="BZ2" s="90" t="n"/>
+      <c r="CA2" s="90" t="n"/>
+      <c r="CB2" s="90" t="n"/>
+      <c r="CC2" s="90" t="n"/>
+      <c r="CD2" s="91" t="n"/>
+      <c r="CE2" s="76" t="n"/>
+      <c r="CF2" s="90" t="n"/>
+      <c r="CG2" s="90" t="n"/>
+      <c r="CH2" s="90" t="n"/>
+      <c r="CI2" s="90" t="n"/>
+      <c r="CJ2" s="90" t="n"/>
+      <c r="CK2" s="90" t="n"/>
+      <c r="CL2" s="90" t="n"/>
+      <c r="CM2" s="90" t="n"/>
+      <c r="CN2" s="90" t="n"/>
+      <c r="CO2" s="90" t="n"/>
+      <c r="CP2" s="90" t="n"/>
+      <c r="CQ2" s="90" t="n"/>
+      <c r="CR2" s="90" t="n"/>
+      <c r="CS2" s="90" t="n"/>
+      <c r="CT2" s="90" t="n"/>
+      <c r="CU2" s="90" t="n"/>
+      <c r="CV2" s="90" t="n"/>
+      <c r="CW2" s="90" t="n"/>
+      <c r="CX2" s="90" t="n"/>
+      <c r="CY2" s="90" t="n"/>
+      <c r="CZ2" s="90" t="n"/>
+      <c r="DA2" s="90" t="n"/>
+      <c r="DB2" s="90" t="n"/>
+      <c r="DC2" s="90" t="n"/>
+      <c r="DD2" s="90" t="n"/>
+      <c r="DE2" s="90" t="n"/>
+      <c r="DF2" s="90" t="n"/>
+      <c r="DG2" s="90" t="n"/>
+      <c r="DH2" s="90" t="n"/>
+      <c r="DI2" s="90" t="n"/>
+      <c r="DJ2" s="90" t="n"/>
+      <c r="DK2" s="91" t="n"/>
+      <c r="DL2" s="76" t="n"/>
+      <c r="DM2" s="90" t="n"/>
+      <c r="DN2" s="90" t="n"/>
+      <c r="DO2" s="90" t="n"/>
+      <c r="DP2" s="90" t="n"/>
+      <c r="DQ2" s="90" t="n"/>
+      <c r="DR2" s="90" t="n"/>
+      <c r="DS2" s="90" t="n"/>
+      <c r="DT2" s="90" t="n"/>
+      <c r="DU2" s="90" t="n"/>
+      <c r="DV2" s="90" t="n"/>
+      <c r="DW2" s="90" t="n"/>
+      <c r="DX2" s="90" t="n"/>
+      <c r="DY2" s="90" t="n"/>
+      <c r="DZ2" s="91" t="n"/>
+      <c r="EA2" s="80" t="n"/>
+      <c r="EB2" s="64" t="n"/>
+      <c r="EC2" s="64" t="n"/>
+      <c r="ED2" s="64" t="n"/>
+      <c r="EE2" s="64" t="n"/>
+      <c r="EF2" s="64" t="n"/>
+      <c r="EG2" s="64" t="n"/>
+      <c r="EH2" s="64" t="n"/>
+      <c r="EI2" s="64" t="n"/>
+      <c r="EJ2" s="64" t="n"/>
+      <c r="EK2" s="64" t="n"/>
+      <c r="EL2" s="64" t="n"/>
+      <c r="EM2" s="95" t="inlineStr">
         <is>
           <t>SENTENCIADOS</t>
         </is>
       </c>
-      <c r="EN2" s="158" t="n"/>
-      <c r="EO2" s="158" t="n"/>
-      <c r="EP2" s="158" t="n"/>
-      <c r="EQ2" s="158" t="n"/>
-      <c r="ER2" s="158" t="n"/>
-      <c r="ES2" s="158" t="n"/>
-      <c r="ET2" s="158" t="n"/>
-      <c r="EU2" s="158" t="n"/>
-      <c r="EV2" s="158" t="n"/>
-      <c r="EW2" s="158" t="n"/>
-      <c r="EX2" s="158" t="n"/>
-      <c r="EY2" s="159" t="n"/>
-      <c r="EZ2" s="96" t="inlineStr">
+      <c r="EN2" s="84" t="n"/>
+      <c r="EO2" s="84" t="n"/>
+      <c r="EP2" s="84" t="n"/>
+      <c r="EQ2" s="84" t="n"/>
+      <c r="ER2" s="84" t="n"/>
+      <c r="ES2" s="84" t="n"/>
+      <c r="ET2" s="84" t="n"/>
+      <c r="EU2" s="84" t="n"/>
+      <c r="EV2" s="84" t="n"/>
+      <c r="EW2" s="84" t="n"/>
+      <c r="EX2" s="84" t="n"/>
+      <c r="EY2" s="96" t="n"/>
+      <c r="EZ2" s="83" t="inlineStr">
         <is>
           <t>CNJ</t>
         </is>
       </c>
-      <c r="FA2" s="158" t="n"/>
-      <c r="FB2" s="158" t="n"/>
-      <c r="FC2" s="158" t="n"/>
-      <c r="FD2" s="158" t="n"/>
-      <c r="FE2" s="158" t="n"/>
-      <c r="FF2" s="158" t="n"/>
-      <c r="FG2" s="158" t="n"/>
-      <c r="FH2" s="158" t="n"/>
-      <c r="FI2" s="158" t="n"/>
-      <c r="FJ2" s="158" t="n"/>
-      <c r="FK2" s="158" t="n"/>
-      <c r="FL2" s="158" t="n"/>
-      <c r="FM2" s="158" t="n"/>
-      <c r="FN2" s="158" t="n"/>
-      <c r="FO2" s="158" t="n"/>
-      <c r="FP2" s="160" t="n"/>
-      <c r="FQ2" s="99" t="inlineStr">
+      <c r="FA2" s="84" t="n"/>
+      <c r="FB2" s="84" t="n"/>
+      <c r="FC2" s="84" t="n"/>
+      <c r="FD2" s="84" t="n"/>
+      <c r="FE2" s="84" t="n"/>
+      <c r="FF2" s="84" t="n"/>
+      <c r="FG2" s="84" t="n"/>
+      <c r="FH2" s="84" t="n"/>
+      <c r="FI2" s="84" t="n"/>
+      <c r="FJ2" s="84" t="n"/>
+      <c r="FK2" s="84" t="n"/>
+      <c r="FL2" s="84" t="n"/>
+      <c r="FM2" s="84" t="n"/>
+      <c r="FN2" s="84" t="n"/>
+      <c r="FO2" s="84" t="n"/>
+      <c r="FP2" s="85" t="n"/>
+      <c r="FQ2" s="63" t="inlineStr">
         <is>
           <t>Revisión bases de datos públicas</t>
         </is>
       </c>
-      <c r="FR2" s="150" t="n"/>
-      <c r="FS2" s="150" t="n"/>
-      <c r="FT2" s="150" t="n"/>
-      <c r="FU2" s="150" t="n"/>
-      <c r="FV2" s="150" t="n"/>
-      <c r="FW2" s="150" t="n"/>
-      <c r="FX2" s="150" t="n"/>
-      <c r="FY2" s="151" t="n"/>
-      <c r="FZ2" s="102" t="inlineStr">
+      <c r="FR2" s="64" t="n"/>
+      <c r="FS2" s="64" t="n"/>
+      <c r="FT2" s="64" t="n"/>
+      <c r="FU2" s="64" t="n"/>
+      <c r="FV2" s="64" t="n"/>
+      <c r="FW2" s="64" t="n"/>
+      <c r="FX2" s="64" t="n"/>
+      <c r="FY2" s="65" t="n"/>
+      <c r="FZ2" s="97" t="inlineStr">
         <is>
           <t xml:space="preserve">Revisión en listas Internacionales </t>
         </is>
       </c>
-      <c r="GA2" s="150" t="n"/>
-      <c r="GB2" s="150" t="n"/>
-      <c r="GC2" s="150" t="n"/>
-      <c r="GD2" s="150" t="n"/>
-      <c r="GE2" s="150" t="n"/>
-      <c r="GF2" s="151" t="n"/>
-      <c r="GG2" s="147" t="n"/>
-      <c r="GH2" s="148" t="n"/>
-      <c r="GI2" s="148" t="n"/>
-      <c r="GJ2" s="149" t="n"/>
-      <c r="GK2" s="161" t="n"/>
-      <c r="GL2" s="162" t="n"/>
-      <c r="GM2" s="162" t="n"/>
-      <c r="GN2" s="162" t="n"/>
+      <c r="GA2" s="64" t="n"/>
+      <c r="GB2" s="64" t="n"/>
+      <c r="GC2" s="64" t="n"/>
+      <c r="GD2" s="64" t="n"/>
+      <c r="GE2" s="64" t="n"/>
+      <c r="GF2" s="65" t="n"/>
+      <c r="GG2" s="69" t="n"/>
+      <c r="GH2" s="70" t="n"/>
+      <c r="GI2" s="70" t="n"/>
+      <c r="GJ2" s="71" t="n"/>
+      <c r="GK2" s="75" t="n"/>
+      <c r="GL2" s="78" t="n"/>
+      <c r="GM2" s="78" t="n"/>
+      <c r="GN2" s="78" t="n"/>
     </row>
     <row r="3" ht="58.2" customHeight="1" thickBot="1">
       <c r="A3" s="13" t="inlineStr">
@@ -3292,7 +2879,7 @@
           <t>IESS</t>
         </is>
       </c>
-      <c r="AO3" s="163" t="inlineStr">
+      <c r="AO3" s="105" t="inlineStr">
         <is>
           <t>Deuda obligaciones patronales</t>
         </is>
@@ -3343,7 +2930,7 @@
           <t>Cargo</t>
         </is>
       </c>
-      <c r="AY3" s="164" t="inlineStr">
+      <c r="AY3" s="106" t="inlineStr">
         <is>
           <t>Capital Invertido</t>
         </is>
@@ -3363,7 +2950,7 @@
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="BC3" s="164" t="inlineStr">
+      <c r="BC3" s="106" t="inlineStr">
         <is>
           <t>Patrimonio (Último año)
 BG - 3</t>
@@ -3389,7 +2976,7 @@
           <t>Cargo</t>
         </is>
       </c>
-      <c r="BH3" s="164" t="inlineStr">
+      <c r="BH3" s="106" t="inlineStr">
         <is>
           <t>Capital Invertido</t>
         </is>
@@ -3409,7 +2996,7 @@
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="BL3" s="164" t="inlineStr">
+      <c r="BL3" s="106" t="inlineStr">
         <is>
           <t>Patrimonio (Último año)
 BG - 3</t>
@@ -3435,7 +3022,7 @@
           <t>Cargo</t>
         </is>
       </c>
-      <c r="BQ3" s="164" t="inlineStr">
+      <c r="BQ3" s="106" t="inlineStr">
         <is>
           <t>Capital Invertido</t>
         </is>
@@ -3455,7 +3042,7 @@
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="BU3" s="164" t="inlineStr">
+      <c r="BU3" s="106" t="inlineStr">
         <is>
           <t>Patrimonio (Último año)
 BG - 3</t>
@@ -3481,7 +3068,7 @@
           <t>Cargo</t>
         </is>
       </c>
-      <c r="BZ3" s="164" t="inlineStr">
+      <c r="BZ3" s="106" t="inlineStr">
         <is>
           <t>Capital Invertido</t>
         </is>
@@ -3501,7 +3088,7 @@
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="CD3" s="165" t="inlineStr">
+      <c r="CD3" s="107" t="inlineStr">
         <is>
           <t>Patrimonio (Último año)
 BG - 3</t>
@@ -3537,7 +3124,7 @@
           <t>Tipo inversión</t>
         </is>
       </c>
-      <c r="CK3" s="164" t="inlineStr">
+      <c r="CK3" s="106" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
@@ -3577,7 +3164,7 @@
           <t>Tipo inversión</t>
         </is>
       </c>
-      <c r="CS3" s="164" t="inlineStr">
+      <c r="CS3" s="106" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
@@ -3617,7 +3204,7 @@
           <t>Tipo inversión</t>
         </is>
       </c>
-      <c r="DA3" s="164" t="inlineStr">
+      <c r="DA3" s="106" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
@@ -3657,7 +3244,7 @@
           <t>Tipo inversión</t>
         </is>
       </c>
-      <c r="DI3" s="164" t="inlineStr">
+      <c r="DI3" s="106" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
@@ -3782,7 +3369,7 @@
           <t>Último año en el cargo</t>
         </is>
       </c>
-      <c r="EH3" s="166" t="inlineStr">
+      <c r="EH3" s="108" t="inlineStr">
         <is>
           <t>Remuneración APROX.</t>
         </is>
@@ -4057,10 +3644,10 @@
           <t xml:space="preserve">Perfil de Riesgo </t>
         </is>
       </c>
-      <c r="GK3" s="154" t="n"/>
-      <c r="GL3" s="167" t="n"/>
-      <c r="GM3" s="167" t="n"/>
-      <c r="GN3" s="167" t="n"/>
+      <c r="GK3" s="76" t="n"/>
+      <c r="GL3" s="79" t="n"/>
+      <c r="GM3" s="79" t="n"/>
+      <c r="GN3" s="79" t="n"/>
     </row>
     <row r="4" ht="70.05" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -4075,163 +3662,153 @@
       </c>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>001/PICHINCHA / QUITO / IÑAQUITO / AV REPUIBLICA DEL SALVADOR N35-82 Y PORTUGAL; 002</t>
-        </is>
-      </c>
-      <c r="G4" s="134" t="n">
+      <c r="F4" s="59" t="inlineStr">
+        <is>
+          <t>QUITO - PICHINCHA</t>
+        </is>
+      </c>
+      <c r="G4" s="100" t="n">
         <v>35626</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
+      <c r="H4" s="59" t="inlineStr"/>
+      <c r="I4" s="60" t="inlineStr"/>
       <c r="J4" s="8" t="n"/>
       <c r="K4" s="8" t="n"/>
       <c r="L4" s="8" t="n"/>
       <c r="M4" s="8" t="n"/>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="59" t="inlineStr">
         <is>
           <t>TORRES GORDILLO DIEGO PATRICIO</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="59" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="P4" s="134" t="n">
-        <v>35626</v>
-      </c>
-      <c r="Q4" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="R4" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="P4" s="109" t="inlineStr">
+        <is>
+          <t>01/01/2015</t>
+        </is>
+      </c>
+      <c r="Q4" s="109" t="inlineStr"/>
+      <c r="R4" s="109" t="inlineStr"/>
+      <c r="S4" s="59" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="T4" s="5" t="inlineStr">
+      <c r="T4" s="59" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
-        <is>
-          <t>ACTIVIDADES DE DISEÑO DE INGENIERÍA Y CONSULTORÍA DE INGENIERÍA PARA PROYECTOS DE INGENIERÍA CIVIL, HIDRÁULICA Y DE TRÁFICO.</t>
-        </is>
-      </c>
-      <c r="V4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="W4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="X4" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Y4" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Z4" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AA4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AB4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AC4" s="4" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AD4" s="5" t="inlineStr">
-        <is>
-          <t>El ciudadano / contribuyente no registra deudas firmes, impugnadas o en facilidades de pago.</t>
-        </is>
-      </c>
-      <c r="AE4" s="5" t="inlineStr">
-        <is>
-          <t>ANEXO TRANSACCIONAL SIMPLIFICADO JUNIO 2026</t>
-        </is>
-      </c>
-      <c r="AF4" s="5" t="inlineStr">
-        <is>
-          <t>MUNICIPIO DE QUITO;</t>
-        </is>
-      </c>
-      <c r="AG4" s="135" t="n">
-        <v>2327.26</v>
-      </c>
-      <c r="AH4" s="5" t="inlineStr">
+      <c r="U4" s="59" t="inlineStr">
+        <is>
+          <t>ACTIVIDADES DE CONSULTORIA</t>
+        </is>
+      </c>
+      <c r="V4" s="60" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="W4" s="60" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="X4" s="109" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y4" s="109" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Z4" s="109" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AA4" s="60" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB4" s="60" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AC4" s="60" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AD4" s="59" t="inlineStr">
+        <is>
+          <t>El ciudadano / contribuyente no registra deudas firmes.</t>
+        </is>
+      </c>
+      <c r="AE4" s="59" t="inlineStr">
+        <is>
+          <t>AL DIA EN SUS OBLIGACIONES</t>
+        </is>
+      </c>
+      <c r="AF4" s="59" t="inlineStr">
+        <is>
+          <t>Quito / Manta</t>
+        </is>
+      </c>
+      <c r="AG4" s="110" t="inlineStr">
+        <is>
+          <t>$52.63</t>
+        </is>
+      </c>
+      <c r="AH4" s="59" t="inlineStr">
         <is>
           <t>PROVEEDOR DEL ESTADO</t>
         </is>
       </c>
-      <c r="AI4" s="5" t="inlineStr">
+      <c r="AI4" s="59" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="AJ4" s="5" t="inlineStr">
+      <c r="AJ4" s="59" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
       <c r="AK4" s="6" t="n"/>
-      <c r="AL4" s="5" t="inlineStr">
-        <is>
-          <t>RELACION DE DEPENDENCIA (IESS)</t>
-        </is>
-      </c>
-      <c r="AM4" s="5" t="inlineStr">
-        <is>
-          <t>AFILIADO VOLUNTARIO</t>
-        </is>
-      </c>
-      <c r="AN4" s="5" t="inlineStr">
-        <is>
-          <t>SI registra obligaciones patronales en mora</t>
-        </is>
-      </c>
-      <c r="AO4" s="136" t="n">
-        <v>12683.75</v>
+      <c r="AL4" s="59" t="inlineStr">
+        <is>
+          <t>Relación de Dependencia (IESS)</t>
+        </is>
+      </c>
+      <c r="AM4" s="59" t="inlineStr">
+        <is>
+          <t>Voluntario</t>
+        </is>
+      </c>
+      <c r="AN4" s="59" t="inlineStr">
+        <is>
+          <t>NO registra obligaciones patronales en mora</t>
+        </is>
+      </c>
+      <c r="AO4" s="59" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
       </c>
       <c r="AP4" s="6" t="n"/>
       <c r="AQ4" s="6" t="n"/>
-      <c r="AR4" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
+      <c r="AR4" s="59" t="inlineStr">
+        <is>
+          <t>SI Cumple con sus obligaciones</t>
         </is>
       </c>
       <c r="AS4" s="5" t="inlineStr">
@@ -4244,11 +3821,12 @@
           <t>TOTAL DE PROCESOS EN LA ACTUALIDAD</t>
         </is>
       </c>
-      <c r="EA4" s="168" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
+      <c r="CB4" s="59" t="inlineStr">
+        <is>
+          <t>01/01/2015</t>
+        </is>
+      </c>
+      <c r="EA4" s="59" t="n"/>
       <c r="EB4" s="5" t="inlineStr">
         <is>
           <t>Registro SI/NO</t>
@@ -4276,10 +3854,10 @@
       </c>
       <c r="EG4" s="5" t="inlineStr">
         <is>
-          <t>ULTIMO DE LA LISTA</t>
-        </is>
-      </c>
-      <c r="EH4" s="169" t="n"/>
+          <t xml:space="preserve">AÑO MAS ACTUAL </t>
+        </is>
+      </c>
+      <c r="EH4" s="111" t="n"/>
       <c r="EJ4" s="6" t="n"/>
       <c r="EK4" s="6" t="n"/>
       <c r="EL4" s="6" t="n"/>
@@ -4375,7 +3953,7 @@
       <c r="FG4" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="FH4" s="134" t="n">
+      <c r="FH4" s="100" t="n">
         <v>44851</v>
       </c>
       <c r="FI4" s="4" t="inlineStr">
@@ -4396,7 +3974,7 @@
       <c r="FL4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="FM4" s="134" t="inlineStr">
+      <c r="FM4" s="100" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -4438,7 +4016,7 @@
       <c r="GI4" s="6" t="n"/>
       <c r="GJ4" s="6" t="n"/>
       <c r="GK4" s="6" t="n"/>
-      <c r="GL4" s="170" t="n"/>
+      <c r="GL4" s="112" t="n"/>
       <c r="GM4" s="57" t="n"/>
       <c r="GN4" s="57" t="n"/>
     </row>
@@ -4460,7 +4038,7 @@
           <t>GUAYAS / GUAYAQUIL / TARQUI / AV. CARLOS JULIO AROSEMENA S/N</t>
         </is>
       </c>
-      <c r="G5" s="134" t="n">
+      <c r="G5" s="100" t="n">
         <v>26632</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -4487,15 +4065,15 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="P5" s="134" t="n">
+      <c r="P5" s="100" t="n">
         <v>26632</v>
       </c>
-      <c r="Q5" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="R5" s="134" t="inlineStr">
+      <c r="Q5" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="R5" s="100" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -4525,15 +4103,15 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="X5" s="134" t="n">
+      <c r="X5" s="100" t="n">
         <v>43067</v>
       </c>
-      <c r="Y5" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Z5" s="134" t="n">
+      <c r="Y5" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Z5" s="100" t="n">
         <v>43273</v>
       </c>
       <c r="AA5" s="5" t="inlineStr">
@@ -4551,72 +4129,63 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="AD5" s="5" t="inlineStr">
-        <is>
-          <t>El ciudadano / contribuyente no registra deudas firmes, impugnadas o en facilidades de pago.</t>
-        </is>
-      </c>
-      <c r="AE5" s="5" t="inlineStr">
-        <is>
-          <t>AL DIA EN SUS OBLIGACIONES</t>
-        </is>
-      </c>
-      <c r="AF5" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AG5" s="135" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH5" s="5" t="inlineStr">
-        <is>
-          <t>PROVEEDOR DEL ESTADO</t>
-        </is>
-      </c>
-      <c r="AI5" s="5" t="inlineStr">
+      <c r="AD5" s="59" t="inlineStr">
+        <is>
+          <t>El ciudadano / contribuyente registra un valor de deudas firmes de $150.00</t>
+        </is>
+      </c>
+      <c r="AE5" s="59" t="inlineStr">
+        <is>
+          <t>2011 DECLARACION DE IVA MAYO 2026 / 2012 DECLARACION DE IVA JUNIO 2026</t>
+        </is>
+      </c>
+      <c r="AF5" s="59" t="inlineStr">
+        <is>
+          <t>No existen registros en los 5 municipios</t>
+        </is>
+      </c>
+      <c r="AG5" s="110" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+      <c r="AH5" s="59" t="inlineStr">
+        <is>
+          <t>NO ES PROVEEDOR DEL ESTADO</t>
+        </is>
+      </c>
+      <c r="AI5" s="59" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="AJ5" s="5" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="AJ5" s="59" t="inlineStr">
+        <is>
+          <t>INDETERMINADO</t>
         </is>
       </c>
       <c r="AK5" s="6" t="n"/>
-      <c r="AL5" s="5" t="inlineStr">
-        <is>
-          <t>RELACION DE DEPENDENCIA (IESS)</t>
-        </is>
-      </c>
-      <c r="AM5" s="5" t="inlineStr">
-        <is>
-          <t>afiliado seguro general tiempo completo</t>
-        </is>
-      </c>
-      <c r="AN5" s="5" t="inlineStr">
-        <is>
-          <t>NO registra obligaciones patronales en mora</t>
-        </is>
-      </c>
-      <c r="AO5" s="136" t="n">
-        <v>0</v>
+      <c r="AL5" s="59" t="inlineStr"/>
+      <c r="AM5" s="59" t="inlineStr"/>
+      <c r="AN5" s="59" t="inlineStr">
+        <is>
+          <t>SI registra obligaciones patronales en mora</t>
+        </is>
+      </c>
+      <c r="AO5" s="59" t="inlineStr">
+        <is>
+          <t>$1,250.00</t>
+        </is>
       </c>
       <c r="AP5" s="6" t="n"/>
       <c r="AQ5" s="6" t="n"/>
-      <c r="AR5" s="5" t="inlineStr">
-        <is>
-          <t>SI Cumple con sus obligaciones</t>
+      <c r="AR5" s="59" t="inlineStr">
+        <is>
+          <t>NO Cumple con sus obligaciones</t>
         </is>
       </c>
       <c r="AS5" s="45" t="n"/>
       <c r="AT5" s="45" t="n"/>
-      <c r="EA5" s="5" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
       <c r="EM5" s="5" t="n">
         <v>1</v>
       </c>
@@ -4630,7 +4199,7 @@
           <t>23281202303069</t>
         </is>
       </c>
-      <c r="EP5" s="134" t="n">
+      <c r="EP5" s="100" t="n">
         <v>46038</v>
       </c>
       <c r="EQ5" s="4" t="inlineStr">
@@ -4705,7 +4274,7 @@
       <c r="FG5" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="FH5" s="134" t="n">
+      <c r="FH5" s="100" t="n">
         <v>46090</v>
       </c>
       <c r="FI5" s="4" t="inlineStr">
@@ -4726,7 +4295,7 @@
       <c r="FL5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="FM5" s="134" t="n">
+      <c r="FM5" s="100" t="n">
         <v>46051</v>
       </c>
       <c r="FN5" s="4" t="inlineStr">
@@ -4763,7 +4332,7 @@
           <t>ESMERALDAS / ESMERALDAS / 5 DE AGOSTO / A 6 Y F</t>
         </is>
       </c>
-      <c r="G6" s="134" t="n">
+      <c r="G6" s="100" t="n">
         <v>43543</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -4790,13 +4359,13 @@
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="P6" s="134" t="n">
+      <c r="P6" s="100" t="n">
         <v>43543</v>
       </c>
-      <c r="Q6" s="134" t="n">
+      <c r="Q6" s="100" t="n">
         <v>44255</v>
       </c>
-      <c r="R6" s="134" t="n">
+      <c r="R6" s="100" t="n">
         <v>45426</v>
       </c>
       <c r="S6" s="5" t="inlineStr">
@@ -4824,17 +4393,17 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="X6" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Y6" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Z6" s="134" t="inlineStr">
+      <c r="X6" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y6" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Z6" s="100" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -4869,57 +4438,19 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="AG6" s="135" t="n">
+      <c r="AG6" s="101" t="n">
         <v>0</v>
       </c>
-      <c r="AH6" s="5" t="inlineStr">
-        <is>
-          <t>NO ES PROVEEDOR DEL ESTADO</t>
-        </is>
-      </c>
-      <c r="AI6" s="5" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="AJ6" s="5" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
       <c r="AK6" s="6" t="n"/>
-      <c r="AL6" s="5" t="inlineStr">
-        <is>
-          <t>NO REGISTRA COBERTURA</t>
-        </is>
-      </c>
-      <c r="AM6" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AN6" s="5" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AO6" s="136" t="n">
-        <v>0</v>
-      </c>
       <c r="AP6" s="6" t="n"/>
       <c r="AQ6" s="6" t="n"/>
-      <c r="AR6" s="5" t="inlineStr">
+      <c r="AR6" s="59" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
       <c r="AS6" s="45" t="n"/>
       <c r="AT6" s="45" t="n"/>
-      <c r="EA6" s="5" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
       <c r="EM6" s="5" t="inlineStr">
         <is>
           <t>NA</t>
@@ -5025,7 +4556,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="FH6" s="134" t="inlineStr">
+      <c r="FH6" s="100" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -5050,7 +4581,7 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="FM6" s="134" t="inlineStr">
+      <c r="FM6" s="100" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -5087,7 +4618,7 @@
           <t>GUAYAS / GUAYAQUIL / XIMENA / LOS RIOS 1301 Y CLEMENTE BALLEN</t>
         </is>
       </c>
-      <c r="G7" s="134" t="n">
+      <c r="G7" s="100" t="n">
         <v>39694</v>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -5110,13 +4641,13 @@
           <t>SUSPENDIDO</t>
         </is>
       </c>
-      <c r="P7" s="134" t="n">
+      <c r="P7" s="100" t="n">
         <v>39694</v>
       </c>
-      <c r="Q7" s="134" t="n">
+      <c r="Q7" s="100" t="n">
         <v>45139</v>
       </c>
-      <c r="R7" s="134" t="n">
+      <c r="R7" s="100" t="n">
         <v>43469</v>
       </c>
       <c r="S7" s="5" t="inlineStr">
@@ -5144,17 +4675,17 @@
           <t>NA</t>
         </is>
       </c>
-      <c r="X7" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Y7" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="Z7" s="134" t="inlineStr">
+      <c r="X7" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Y7" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="Z7" s="100" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -5176,7 +4707,7 @@
       </c>
       <c r="AD7" s="5" t="inlineStr">
         <is>
-          <t>No registra deudas firmes</t>
+          <t>El ciudadano / contribuyente no registra deudas firmes, impugnadas o en facilidades de pago.</t>
         </is>
       </c>
       <c r="AE7" s="5" t="inlineStr">
@@ -5195,7 +4726,7 @@
           <t>17U05202600018</t>
         </is>
       </c>
-      <c r="EP7" s="134" t="inlineStr">
+      <c r="EP7" s="100" t="inlineStr">
         <is>
           <t>02/04/2026</t>
         </is>
@@ -5213,7 +4744,7 @@
           <t>09333202600398</t>
         </is>
       </c>
-      <c r="ET7" s="134" t="n">
+      <c r="ET7" s="100" t="n">
         <v>46146</v>
       </c>
       <c r="EU7" s="4" t="inlineStr">
@@ -5221,22 +4752,22 @@
           <t>282 INCUMPLIMIENTO DE DECISIONES LEGÍTIMAS DE AUTORIDAD COMPETENTE, INC.1</t>
         </is>
       </c>
-      <c r="EV7" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="EW7" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="EX7" s="134" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="EY7" s="134" t="inlineStr">
+      <c r="EV7" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="EW7" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="EX7" s="100" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="EY7" s="100" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -5251,6 +4782,25 @@
       <c r="C8" s="5" t="inlineStr">
         <is>
           <t>AMBACAR CIA. LTDA.</t>
+        </is>
+      </c>
+      <c r="AR8" s="5" t="inlineStr">
+        <is>
+          <t>NO Cumple con sus obligaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70.05" customHeight="1">
+      <c r="AR9" s="5" t="inlineStr">
+        <is>
+          <t>SI Cumple con sus obligaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70.05" customHeight="1">
+      <c r="AR10" s="5" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
@@ -5276,8 +4826,8 @@
     <mergeCell ref="CE1:DK2"/>
     <mergeCell ref="EM2:EY2"/>
     <mergeCell ref="GN1:GN3"/>
+    <mergeCell ref="N1:AC1"/>
     <mergeCell ref="FZ2:GF2"/>
-    <mergeCell ref="N1:AC1"/>
     <mergeCell ref="AN1:AR2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A3:A6 A7:B1048576">

</xml_diff>

<commit_message>
feat: URLs desde Parametrizacion, no hardcodeadas (18 sitios) + fiscalia_totem eliminado
</commit_message>
<xml_diff>
--- a/templates/Matriz Revisión Clientes.xlsx
+++ b/templates/Matriz Revisión Clientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\villacisr\Desktop\Automatizacion_PLAF\Dev\ACW-PLAFT-UAFE\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33D9CA1F-BAD8-4502-8309-2C54259DCACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3AB408-AC3A-4493-AC2D-881F4B2EC36F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="259" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="259" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametrizacion" sheetId="1" r:id="rId1"/>
@@ -389,7 +389,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="276">
   <si>
     <t>IDENTIFICACIÓN BÁSICA</t>
   </si>
@@ -1179,9 +1179,6 @@
     <t>URL_FISCALIA_NOTICIAS</t>
   </si>
   <si>
-    <t>https://www.gestiondefiscalias.gob.ec/siaf/informacion/web/noticiasdelito/index.php</t>
-  </si>
-  <si>
     <t>Fiscalía - MÓDULO DE INFORMACIÓN NOTICIAS DE DELITO</t>
   </si>
   <si>
@@ -1219,6 +1216,9 @@
   </si>
   <si>
     <t>SERCOP / INCOP - Descargar los certificados de proveedores Incumplidos</t>
+  </si>
+  <si>
+    <t>https://www.gestiondefiscalias.gob.ec/siaf/sitio/consulta_ndd_ext/redirect.php?data=L3Zhci93d3cvaHRtbC9zaWFmL2luZm9ybWFjaW9uL3dlYi9ub3RpY2lhc2RlbGl0by8uLi8uLi8uLi9zaXRpby9jb25zdWx0YV9uZGRfZXh0L2NvbnN1bHRhX2NpdWRhZGFuYS5waHA%3D</t>
   </si>
 </sst>
 </file>
@@ -1874,7 +1874,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2081,36 +2081,32 @@
     <xf numFmtId="0" fontId="12" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2126,9 +2122,6 @@
     <xf numFmtId="164" fontId="5" fillId="2" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2137,23 +2130,33 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2817,54 +2820,54 @@
         <v>261</v>
       </c>
       <c r="B18" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C18" s="3" t="s">
         <v>262</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>263</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="3" t="s">
         <v>265</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>266</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" t="s">
         <v>268</v>
-      </c>
-      <c r="C20" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>269</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="C21" t="s">
         <v>271</v>
-      </c>
-      <c r="C21" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>272</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="C22" t="s">
         <v>274</v>
-      </c>
-      <c r="C22" t="s">
-        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -2885,23 +2888,23 @@
     <hyperlink ref="B15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
     <hyperlink ref="B16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
     <hyperlink ref="B17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="B18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="B19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="B20" r:id="rId19" location="!/" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="B21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="B22" r:id="rId21" tooltip="https://www.compraspublicas.gob.ec/procesocontratacion/compras/ep/empreporteincumplidos.cpe" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B19" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="B20" r:id="rId18" location="!/" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="B21" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="B22" r:id="rId20" tooltip="https://www.compraspublicas.gob.ec/procesocontratacion/compras/ep/empreporteincumplidos.cpe" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="B18" r:id="rId21" xr:uid="{8A6122D6-6C8D-4789-AE11-C6965D0196A6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId22"/>
   <tableParts count="1">
-    <tablePart r:id="rId22"/>
+    <tablePart r:id="rId23"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:GN12"/>
+  <dimension ref="A1:GN11"/>
   <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="70.05" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" style="4" customWidth="1"/>
@@ -3097,444 +3100,444 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:196" s="10" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="76"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="104" t="s">
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="74"/>
+      <c r="J1" s="74"/>
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
+      <c r="M1" s="75"/>
+      <c r="N1" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="O1" s="76"/>
-      <c r="P1" s="76"/>
-      <c r="Q1" s="76"/>
-      <c r="R1" s="76"/>
-      <c r="S1" s="76"/>
-      <c r="T1" s="76"/>
-      <c r="U1" s="76"/>
-      <c r="V1" s="76"/>
-      <c r="W1" s="76"/>
-      <c r="X1" s="76"/>
-      <c r="Y1" s="76"/>
-      <c r="Z1" s="76"/>
-      <c r="AA1" s="76"/>
-      <c r="AB1" s="76"/>
-      <c r="AC1" s="77"/>
-      <c r="AD1" s="100" t="s">
+      <c r="O1" s="74"/>
+      <c r="P1" s="74"/>
+      <c r="Q1" s="74"/>
+      <c r="R1" s="74"/>
+      <c r="S1" s="74"/>
+      <c r="T1" s="74"/>
+      <c r="U1" s="74"/>
+      <c r="V1" s="74"/>
+      <c r="W1" s="74"/>
+      <c r="X1" s="74"/>
+      <c r="Y1" s="74"/>
+      <c r="Z1" s="74"/>
+      <c r="AA1" s="74"/>
+      <c r="AB1" s="74"/>
+      <c r="AC1" s="75"/>
+      <c r="AD1" s="106" t="s">
         <v>2</v>
       </c>
-      <c r="AE1" s="76"/>
-      <c r="AF1" s="76"/>
-      <c r="AG1" s="76"/>
-      <c r="AH1" s="76"/>
-      <c r="AI1" s="76"/>
-      <c r="AJ1" s="76"/>
-      <c r="AK1" s="77"/>
-      <c r="AL1" s="93" t="s">
+      <c r="AE1" s="74"/>
+      <c r="AF1" s="74"/>
+      <c r="AG1" s="74"/>
+      <c r="AH1" s="74"/>
+      <c r="AI1" s="74"/>
+      <c r="AJ1" s="74"/>
+      <c r="AK1" s="75"/>
+      <c r="AL1" s="91" t="s">
         <v>3</v>
       </c>
-      <c r="AM1" s="77"/>
-      <c r="AN1" s="106" t="s">
+      <c r="AM1" s="75"/>
+      <c r="AN1" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="AO1" s="76"/>
-      <c r="AP1" s="76"/>
-      <c r="AQ1" s="76"/>
-      <c r="AR1" s="77"/>
-      <c r="AS1" s="99" t="s">
+      <c r="AO1" s="74"/>
+      <c r="AP1" s="74"/>
+      <c r="AQ1" s="74"/>
+      <c r="AR1" s="75"/>
+      <c r="AS1" s="96" t="s">
         <v>5</v>
       </c>
-      <c r="AT1" s="89"/>
-      <c r="AU1" s="99" t="s">
+      <c r="AT1" s="87"/>
+      <c r="AU1" s="96" t="s">
         <v>6</v>
       </c>
-      <c r="AV1" s="76"/>
-      <c r="AW1" s="76"/>
-      <c r="AX1" s="76"/>
-      <c r="AY1" s="76"/>
-      <c r="AZ1" s="76"/>
-      <c r="BA1" s="76"/>
-      <c r="BB1" s="76"/>
-      <c r="BC1" s="76"/>
-      <c r="BD1" s="76"/>
-      <c r="BE1" s="76"/>
-      <c r="BF1" s="76"/>
-      <c r="BG1" s="76"/>
-      <c r="BH1" s="76"/>
-      <c r="BI1" s="76"/>
-      <c r="BJ1" s="76"/>
-      <c r="BK1" s="76"/>
-      <c r="BL1" s="76"/>
-      <c r="BM1" s="76"/>
-      <c r="BN1" s="76"/>
-      <c r="BO1" s="76"/>
-      <c r="BP1" s="76"/>
-      <c r="BQ1" s="76"/>
-      <c r="BR1" s="76"/>
-      <c r="BS1" s="76"/>
-      <c r="BT1" s="76"/>
-      <c r="BU1" s="76"/>
-      <c r="BV1" s="76"/>
-      <c r="BW1" s="76"/>
-      <c r="BX1" s="76"/>
-      <c r="BY1" s="76"/>
-      <c r="BZ1" s="76"/>
-      <c r="CA1" s="76"/>
-      <c r="CB1" s="76"/>
-      <c r="CC1" s="76"/>
-      <c r="CD1" s="89"/>
-      <c r="CE1" s="101" t="s">
+      <c r="AV1" s="74"/>
+      <c r="AW1" s="74"/>
+      <c r="AX1" s="74"/>
+      <c r="AY1" s="74"/>
+      <c r="AZ1" s="74"/>
+      <c r="BA1" s="74"/>
+      <c r="BB1" s="74"/>
+      <c r="BC1" s="74"/>
+      <c r="BD1" s="74"/>
+      <c r="BE1" s="74"/>
+      <c r="BF1" s="74"/>
+      <c r="BG1" s="74"/>
+      <c r="BH1" s="74"/>
+      <c r="BI1" s="74"/>
+      <c r="BJ1" s="74"/>
+      <c r="BK1" s="74"/>
+      <c r="BL1" s="74"/>
+      <c r="BM1" s="74"/>
+      <c r="BN1" s="74"/>
+      <c r="BO1" s="74"/>
+      <c r="BP1" s="74"/>
+      <c r="BQ1" s="74"/>
+      <c r="BR1" s="74"/>
+      <c r="BS1" s="74"/>
+      <c r="BT1" s="74"/>
+      <c r="BU1" s="74"/>
+      <c r="BV1" s="74"/>
+      <c r="BW1" s="74"/>
+      <c r="BX1" s="74"/>
+      <c r="BY1" s="74"/>
+      <c r="BZ1" s="74"/>
+      <c r="CA1" s="74"/>
+      <c r="CB1" s="74"/>
+      <c r="CC1" s="74"/>
+      <c r="CD1" s="87"/>
+      <c r="CE1" s="97" t="s">
         <v>7</v>
       </c>
-      <c r="CF1" s="76"/>
-      <c r="CG1" s="76"/>
-      <c r="CH1" s="76"/>
-      <c r="CI1" s="76"/>
-      <c r="CJ1" s="76"/>
-      <c r="CK1" s="76"/>
-      <c r="CL1" s="76"/>
-      <c r="CM1" s="76"/>
-      <c r="CN1" s="76"/>
-      <c r="CO1" s="76"/>
-      <c r="CP1" s="76"/>
-      <c r="CQ1" s="76"/>
-      <c r="CR1" s="76"/>
-      <c r="CS1" s="76"/>
-      <c r="CT1" s="76"/>
-      <c r="CU1" s="76"/>
-      <c r="CV1" s="76"/>
-      <c r="CW1" s="76"/>
-      <c r="CX1" s="76"/>
-      <c r="CY1" s="76"/>
-      <c r="CZ1" s="76"/>
-      <c r="DA1" s="76"/>
-      <c r="DB1" s="76"/>
-      <c r="DC1" s="76"/>
-      <c r="DD1" s="76"/>
-      <c r="DE1" s="76"/>
-      <c r="DF1" s="76"/>
-      <c r="DG1" s="76"/>
-      <c r="DH1" s="76"/>
-      <c r="DI1" s="76"/>
-      <c r="DJ1" s="76"/>
-      <c r="DK1" s="89"/>
-      <c r="DL1" s="96" t="s">
+      <c r="CF1" s="74"/>
+      <c r="CG1" s="74"/>
+      <c r="CH1" s="74"/>
+      <c r="CI1" s="74"/>
+      <c r="CJ1" s="74"/>
+      <c r="CK1" s="74"/>
+      <c r="CL1" s="74"/>
+      <c r="CM1" s="74"/>
+      <c r="CN1" s="74"/>
+      <c r="CO1" s="74"/>
+      <c r="CP1" s="74"/>
+      <c r="CQ1" s="74"/>
+      <c r="CR1" s="74"/>
+      <c r="CS1" s="74"/>
+      <c r="CT1" s="74"/>
+      <c r="CU1" s="74"/>
+      <c r="CV1" s="74"/>
+      <c r="CW1" s="74"/>
+      <c r="CX1" s="74"/>
+      <c r="CY1" s="74"/>
+      <c r="CZ1" s="74"/>
+      <c r="DA1" s="74"/>
+      <c r="DB1" s="74"/>
+      <c r="DC1" s="74"/>
+      <c r="DD1" s="74"/>
+      <c r="DE1" s="74"/>
+      <c r="DF1" s="74"/>
+      <c r="DG1" s="74"/>
+      <c r="DH1" s="74"/>
+      <c r="DI1" s="74"/>
+      <c r="DJ1" s="74"/>
+      <c r="DK1" s="87"/>
+      <c r="DL1" s="93" t="s">
         <v>8</v>
       </c>
-      <c r="DM1" s="76"/>
-      <c r="DN1" s="76"/>
-      <c r="DO1" s="76"/>
-      <c r="DP1" s="76"/>
-      <c r="DQ1" s="76"/>
-      <c r="DR1" s="76"/>
-      <c r="DS1" s="76"/>
-      <c r="DT1" s="76"/>
-      <c r="DU1" s="76"/>
-      <c r="DV1" s="76"/>
-      <c r="DW1" s="76"/>
-      <c r="DX1" s="76"/>
-      <c r="DY1" s="76"/>
-      <c r="DZ1" s="89"/>
-      <c r="EA1" s="88" t="s">
+      <c r="DM1" s="74"/>
+      <c r="DN1" s="74"/>
+      <c r="DO1" s="74"/>
+      <c r="DP1" s="74"/>
+      <c r="DQ1" s="74"/>
+      <c r="DR1" s="74"/>
+      <c r="DS1" s="74"/>
+      <c r="DT1" s="74"/>
+      <c r="DU1" s="74"/>
+      <c r="DV1" s="74"/>
+      <c r="DW1" s="74"/>
+      <c r="DX1" s="74"/>
+      <c r="DY1" s="74"/>
+      <c r="DZ1" s="87"/>
+      <c r="EA1" s="86" t="s">
         <v>9</v>
       </c>
-      <c r="EB1" s="76"/>
-      <c r="EC1" s="76"/>
-      <c r="ED1" s="76"/>
-      <c r="EE1" s="76"/>
-      <c r="EF1" s="76"/>
-      <c r="EG1" s="76"/>
-      <c r="EH1" s="76"/>
-      <c r="EI1" s="76"/>
-      <c r="EJ1" s="76"/>
-      <c r="EK1" s="76"/>
-      <c r="EL1" s="76"/>
-      <c r="EM1" s="76"/>
-      <c r="EN1" s="76"/>
-      <c r="EO1" s="76"/>
-      <c r="EP1" s="76"/>
-      <c r="EQ1" s="76"/>
-      <c r="ER1" s="76"/>
-      <c r="ES1" s="76"/>
-      <c r="ET1" s="76"/>
-      <c r="EU1" s="76"/>
-      <c r="EV1" s="76"/>
-      <c r="EW1" s="76"/>
-      <c r="EX1" s="76"/>
-      <c r="EY1" s="76"/>
-      <c r="EZ1" s="76"/>
-      <c r="FA1" s="76"/>
-      <c r="FB1" s="76"/>
-      <c r="FC1" s="76"/>
-      <c r="FD1" s="76"/>
-      <c r="FE1" s="76"/>
-      <c r="FF1" s="76"/>
-      <c r="FG1" s="76"/>
-      <c r="FH1" s="76"/>
-      <c r="FI1" s="76"/>
-      <c r="FJ1" s="76"/>
-      <c r="FK1" s="76"/>
-      <c r="FL1" s="76"/>
-      <c r="FM1" s="76"/>
-      <c r="FN1" s="76"/>
-      <c r="FO1" s="76"/>
-      <c r="FP1" s="76"/>
-      <c r="FQ1" s="76"/>
-      <c r="FR1" s="76"/>
-      <c r="FS1" s="76"/>
-      <c r="FT1" s="76"/>
-      <c r="FU1" s="76"/>
-      <c r="FV1" s="76"/>
-      <c r="FW1" s="76"/>
-      <c r="FX1" s="76"/>
-      <c r="FY1" s="76"/>
-      <c r="FZ1" s="76"/>
-      <c r="GA1" s="76"/>
-      <c r="GB1" s="76"/>
-      <c r="GC1" s="76"/>
-      <c r="GD1" s="76"/>
-      <c r="GE1" s="76"/>
-      <c r="GF1" s="89"/>
-      <c r="GG1" s="75" t="s">
+      <c r="EB1" s="74"/>
+      <c r="EC1" s="74"/>
+      <c r="ED1" s="74"/>
+      <c r="EE1" s="74"/>
+      <c r="EF1" s="74"/>
+      <c r="EG1" s="74"/>
+      <c r="EH1" s="74"/>
+      <c r="EI1" s="74"/>
+      <c r="EJ1" s="74"/>
+      <c r="EK1" s="74"/>
+      <c r="EL1" s="74"/>
+      <c r="EM1" s="74"/>
+      <c r="EN1" s="74"/>
+      <c r="EO1" s="74"/>
+      <c r="EP1" s="74"/>
+      <c r="EQ1" s="74"/>
+      <c r="ER1" s="74"/>
+      <c r="ES1" s="74"/>
+      <c r="ET1" s="74"/>
+      <c r="EU1" s="74"/>
+      <c r="EV1" s="74"/>
+      <c r="EW1" s="74"/>
+      <c r="EX1" s="74"/>
+      <c r="EY1" s="74"/>
+      <c r="EZ1" s="74"/>
+      <c r="FA1" s="74"/>
+      <c r="FB1" s="74"/>
+      <c r="FC1" s="74"/>
+      <c r="FD1" s="74"/>
+      <c r="FE1" s="74"/>
+      <c r="FF1" s="74"/>
+      <c r="FG1" s="74"/>
+      <c r="FH1" s="74"/>
+      <c r="FI1" s="74"/>
+      <c r="FJ1" s="74"/>
+      <c r="FK1" s="74"/>
+      <c r="FL1" s="74"/>
+      <c r="FM1" s="74"/>
+      <c r="FN1" s="74"/>
+      <c r="FO1" s="74"/>
+      <c r="FP1" s="74"/>
+      <c r="FQ1" s="74"/>
+      <c r="FR1" s="74"/>
+      <c r="FS1" s="74"/>
+      <c r="FT1" s="74"/>
+      <c r="FU1" s="74"/>
+      <c r="FV1" s="74"/>
+      <c r="FW1" s="74"/>
+      <c r="FX1" s="74"/>
+      <c r="FY1" s="74"/>
+      <c r="FZ1" s="74"/>
+      <c r="GA1" s="74"/>
+      <c r="GB1" s="74"/>
+      <c r="GC1" s="74"/>
+      <c r="GD1" s="74"/>
+      <c r="GE1" s="74"/>
+      <c r="GF1" s="87"/>
+      <c r="GG1" s="103" t="s">
         <v>10</v>
       </c>
-      <c r="GH1" s="76"/>
-      <c r="GI1" s="76"/>
-      <c r="GJ1" s="77"/>
-      <c r="GK1" s="82" t="s">
+      <c r="GH1" s="74"/>
+      <c r="GI1" s="74"/>
+      <c r="GJ1" s="75"/>
+      <c r="GK1" s="83" t="s">
         <v>11</v>
       </c>
-      <c r="GL1" s="94" t="s">
+      <c r="GL1" s="92" t="s">
         <v>12</v>
       </c>
-      <c r="GM1" s="85" t="s">
+      <c r="GM1" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="GN1" s="85" t="s">
+      <c r="GN1" s="70" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:196" s="10" customFormat="1" ht="25.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="78"/>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
-      <c r="H2" s="79"/>
-      <c r="I2" s="79"/>
-      <c r="J2" s="79"/>
-      <c r="K2" s="79"/>
-      <c r="L2" s="79"/>
-      <c r="M2" s="80"/>
-      <c r="N2" s="95" t="s">
+      <c r="A2" s="80"/>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
+      <c r="I2" s="81"/>
+      <c r="J2" s="81"/>
+      <c r="K2" s="81"/>
+      <c r="L2" s="81"/>
+      <c r="M2" s="82"/>
+      <c r="N2" s="105" t="s">
         <v>15</v>
       </c>
-      <c r="O2" s="71"/>
-      <c r="P2" s="71"/>
-      <c r="Q2" s="71"/>
-      <c r="R2" s="71"/>
-      <c r="S2" s="71"/>
-      <c r="T2" s="71"/>
-      <c r="U2" s="72"/>
-      <c r="V2" s="81" t="s">
+      <c r="O2" s="77"/>
+      <c r="P2" s="77"/>
+      <c r="Q2" s="77"/>
+      <c r="R2" s="77"/>
+      <c r="S2" s="77"/>
+      <c r="T2" s="77"/>
+      <c r="U2" s="78"/>
+      <c r="V2" s="104" t="s">
         <v>16</v>
       </c>
-      <c r="W2" s="71"/>
-      <c r="X2" s="71"/>
-      <c r="Y2" s="71"/>
-      <c r="Z2" s="71"/>
-      <c r="AA2" s="71"/>
-      <c r="AB2" s="71"/>
-      <c r="AC2" s="74"/>
-      <c r="AD2" s="78"/>
-      <c r="AE2" s="79"/>
-      <c r="AF2" s="79"/>
-      <c r="AG2" s="79"/>
-      <c r="AH2" s="79"/>
-      <c r="AI2" s="79"/>
-      <c r="AJ2" s="79"/>
-      <c r="AK2" s="80"/>
-      <c r="AL2" s="78"/>
-      <c r="AM2" s="80"/>
-      <c r="AN2" s="78"/>
-      <c r="AO2" s="79"/>
-      <c r="AP2" s="79"/>
-      <c r="AQ2" s="79"/>
-      <c r="AR2" s="80"/>
-      <c r="AS2" s="84"/>
-      <c r="AT2" s="98"/>
-      <c r="AU2" s="84"/>
-      <c r="AV2" s="97"/>
-      <c r="AW2" s="97"/>
-      <c r="AX2" s="97"/>
-      <c r="AY2" s="97"/>
-      <c r="AZ2" s="97"/>
-      <c r="BA2" s="97"/>
-      <c r="BB2" s="97"/>
-      <c r="BC2" s="97"/>
-      <c r="BD2" s="97"/>
-      <c r="BE2" s="97"/>
-      <c r="BF2" s="97"/>
-      <c r="BG2" s="97"/>
-      <c r="BH2" s="97"/>
-      <c r="BI2" s="97"/>
-      <c r="BJ2" s="97"/>
-      <c r="BK2" s="97"/>
-      <c r="BL2" s="97"/>
-      <c r="BM2" s="97"/>
-      <c r="BN2" s="97"/>
-      <c r="BO2" s="97"/>
-      <c r="BP2" s="97"/>
-      <c r="BQ2" s="97"/>
-      <c r="BR2" s="97"/>
-      <c r="BS2" s="97"/>
-      <c r="BT2" s="97"/>
-      <c r="BU2" s="97"/>
-      <c r="BV2" s="97"/>
-      <c r="BW2" s="97"/>
-      <c r="BX2" s="97"/>
-      <c r="BY2" s="97"/>
-      <c r="BZ2" s="97"/>
-      <c r="CA2" s="97"/>
-      <c r="CB2" s="97"/>
-      <c r="CC2" s="97"/>
-      <c r="CD2" s="98"/>
-      <c r="CE2" s="84"/>
-      <c r="CF2" s="97"/>
-      <c r="CG2" s="97"/>
-      <c r="CH2" s="97"/>
-      <c r="CI2" s="97"/>
-      <c r="CJ2" s="97"/>
-      <c r="CK2" s="97"/>
-      <c r="CL2" s="97"/>
-      <c r="CM2" s="97"/>
-      <c r="CN2" s="97"/>
-      <c r="CO2" s="97"/>
-      <c r="CP2" s="97"/>
-      <c r="CQ2" s="97"/>
-      <c r="CR2" s="97"/>
-      <c r="CS2" s="97"/>
-      <c r="CT2" s="97"/>
-      <c r="CU2" s="97"/>
-      <c r="CV2" s="97"/>
-      <c r="CW2" s="97"/>
-      <c r="CX2" s="97"/>
-      <c r="CY2" s="97"/>
-      <c r="CZ2" s="97"/>
-      <c r="DA2" s="97"/>
-      <c r="DB2" s="97"/>
-      <c r="DC2" s="97"/>
-      <c r="DD2" s="97"/>
-      <c r="DE2" s="97"/>
-      <c r="DF2" s="97"/>
-      <c r="DG2" s="97"/>
-      <c r="DH2" s="97"/>
-      <c r="DI2" s="97"/>
-      <c r="DJ2" s="97"/>
-      <c r="DK2" s="98"/>
-      <c r="DL2" s="84"/>
-      <c r="DM2" s="97"/>
-      <c r="DN2" s="97"/>
-      <c r="DO2" s="97"/>
-      <c r="DP2" s="97"/>
-      <c r="DQ2" s="97"/>
-      <c r="DR2" s="97"/>
-      <c r="DS2" s="97"/>
-      <c r="DT2" s="97"/>
-      <c r="DU2" s="97"/>
-      <c r="DV2" s="97"/>
-      <c r="DW2" s="97"/>
-      <c r="DX2" s="97"/>
-      <c r="DY2" s="97"/>
-      <c r="DZ2" s="98"/>
+      <c r="W2" s="77"/>
+      <c r="X2" s="77"/>
+      <c r="Y2" s="77"/>
+      <c r="Z2" s="77"/>
+      <c r="AA2" s="77"/>
+      <c r="AB2" s="77"/>
+      <c r="AC2" s="102"/>
+      <c r="AD2" s="80"/>
+      <c r="AE2" s="81"/>
+      <c r="AF2" s="81"/>
+      <c r="AG2" s="81"/>
+      <c r="AH2" s="81"/>
+      <c r="AI2" s="81"/>
+      <c r="AJ2" s="81"/>
+      <c r="AK2" s="82"/>
+      <c r="AL2" s="80"/>
+      <c r="AM2" s="82"/>
+      <c r="AN2" s="80"/>
+      <c r="AO2" s="81"/>
+      <c r="AP2" s="81"/>
+      <c r="AQ2" s="81"/>
+      <c r="AR2" s="82"/>
+      <c r="AS2" s="85"/>
+      <c r="AT2" s="95"/>
+      <c r="AU2" s="85"/>
+      <c r="AV2" s="94"/>
+      <c r="AW2" s="94"/>
+      <c r="AX2" s="94"/>
+      <c r="AY2" s="94"/>
+      <c r="AZ2" s="94"/>
+      <c r="BA2" s="94"/>
+      <c r="BB2" s="94"/>
+      <c r="BC2" s="94"/>
+      <c r="BD2" s="94"/>
+      <c r="BE2" s="94"/>
+      <c r="BF2" s="94"/>
+      <c r="BG2" s="94"/>
+      <c r="BH2" s="94"/>
+      <c r="BI2" s="94"/>
+      <c r="BJ2" s="94"/>
+      <c r="BK2" s="94"/>
+      <c r="BL2" s="94"/>
+      <c r="BM2" s="94"/>
+      <c r="BN2" s="94"/>
+      <c r="BO2" s="94"/>
+      <c r="BP2" s="94"/>
+      <c r="BQ2" s="94"/>
+      <c r="BR2" s="94"/>
+      <c r="BS2" s="94"/>
+      <c r="BT2" s="94"/>
+      <c r="BU2" s="94"/>
+      <c r="BV2" s="94"/>
+      <c r="BW2" s="94"/>
+      <c r="BX2" s="94"/>
+      <c r="BY2" s="94"/>
+      <c r="BZ2" s="94"/>
+      <c r="CA2" s="94"/>
+      <c r="CB2" s="94"/>
+      <c r="CC2" s="94"/>
+      <c r="CD2" s="95"/>
+      <c r="CE2" s="85"/>
+      <c r="CF2" s="94"/>
+      <c r="CG2" s="94"/>
+      <c r="CH2" s="94"/>
+      <c r="CI2" s="94"/>
+      <c r="CJ2" s="94"/>
+      <c r="CK2" s="94"/>
+      <c r="CL2" s="94"/>
+      <c r="CM2" s="94"/>
+      <c r="CN2" s="94"/>
+      <c r="CO2" s="94"/>
+      <c r="CP2" s="94"/>
+      <c r="CQ2" s="94"/>
+      <c r="CR2" s="94"/>
+      <c r="CS2" s="94"/>
+      <c r="CT2" s="94"/>
+      <c r="CU2" s="94"/>
+      <c r="CV2" s="94"/>
+      <c r="CW2" s="94"/>
+      <c r="CX2" s="94"/>
+      <c r="CY2" s="94"/>
+      <c r="CZ2" s="94"/>
+      <c r="DA2" s="94"/>
+      <c r="DB2" s="94"/>
+      <c r="DC2" s="94"/>
+      <c r="DD2" s="94"/>
+      <c r="DE2" s="94"/>
+      <c r="DF2" s="94"/>
+      <c r="DG2" s="94"/>
+      <c r="DH2" s="94"/>
+      <c r="DI2" s="94"/>
+      <c r="DJ2" s="94"/>
+      <c r="DK2" s="95"/>
+      <c r="DL2" s="85"/>
+      <c r="DM2" s="94"/>
+      <c r="DN2" s="94"/>
+      <c r="DO2" s="94"/>
+      <c r="DP2" s="94"/>
+      <c r="DQ2" s="94"/>
+      <c r="DR2" s="94"/>
+      <c r="DS2" s="94"/>
+      <c r="DT2" s="94"/>
+      <c r="DU2" s="94"/>
+      <c r="DV2" s="94"/>
+      <c r="DW2" s="94"/>
+      <c r="DX2" s="94"/>
+      <c r="DY2" s="94"/>
+      <c r="DZ2" s="95"/>
       <c r="EA2" s="63"/>
-      <c r="EB2" s="73" t="s">
+      <c r="EB2" s="101" t="s">
         <v>17</v>
       </c>
-      <c r="EC2" s="71"/>
-      <c r="ED2" s="71"/>
-      <c r="EE2" s="71"/>
-      <c r="EF2" s="71"/>
-      <c r="EG2" s="71"/>
-      <c r="EH2" s="71"/>
-      <c r="EI2" s="71"/>
-      <c r="EJ2" s="71"/>
-      <c r="EK2" s="71"/>
-      <c r="EL2" s="74"/>
-      <c r="EM2" s="102" t="s">
+      <c r="EC2" s="77"/>
+      <c r="ED2" s="77"/>
+      <c r="EE2" s="77"/>
+      <c r="EF2" s="77"/>
+      <c r="EG2" s="77"/>
+      <c r="EH2" s="77"/>
+      <c r="EI2" s="77"/>
+      <c r="EJ2" s="77"/>
+      <c r="EK2" s="77"/>
+      <c r="EL2" s="102"/>
+      <c r="EM2" s="98" t="s">
         <v>18</v>
       </c>
-      <c r="EN2" s="91"/>
-      <c r="EO2" s="91"/>
-      <c r="EP2" s="91"/>
-      <c r="EQ2" s="91"/>
-      <c r="ER2" s="91"/>
-      <c r="ES2" s="91"/>
-      <c r="ET2" s="91"/>
-      <c r="EU2" s="91"/>
-      <c r="EV2" s="91"/>
-      <c r="EW2" s="91"/>
-      <c r="EX2" s="91"/>
-      <c r="EY2" s="103"/>
-      <c r="EZ2" s="90" t="s">
+      <c r="EN2" s="89"/>
+      <c r="EO2" s="89"/>
+      <c r="EP2" s="89"/>
+      <c r="EQ2" s="89"/>
+      <c r="ER2" s="89"/>
+      <c r="ES2" s="89"/>
+      <c r="ET2" s="89"/>
+      <c r="EU2" s="89"/>
+      <c r="EV2" s="89"/>
+      <c r="EW2" s="89"/>
+      <c r="EX2" s="89"/>
+      <c r="EY2" s="99"/>
+      <c r="EZ2" s="88" t="s">
         <v>19</v>
       </c>
-      <c r="FA2" s="91"/>
-      <c r="FB2" s="91"/>
-      <c r="FC2" s="91"/>
-      <c r="FD2" s="91"/>
-      <c r="FE2" s="91"/>
-      <c r="FF2" s="91"/>
-      <c r="FG2" s="91"/>
-      <c r="FH2" s="91"/>
-      <c r="FI2" s="91"/>
-      <c r="FJ2" s="91"/>
-      <c r="FK2" s="91"/>
-      <c r="FL2" s="91"/>
-      <c r="FM2" s="91"/>
-      <c r="FN2" s="91"/>
-      <c r="FO2" s="91"/>
-      <c r="FP2" s="92"/>
-      <c r="FQ2" s="70" t="s">
+      <c r="FA2" s="89"/>
+      <c r="FB2" s="89"/>
+      <c r="FC2" s="89"/>
+      <c r="FD2" s="89"/>
+      <c r="FE2" s="89"/>
+      <c r="FF2" s="89"/>
+      <c r="FG2" s="89"/>
+      <c r="FH2" s="89"/>
+      <c r="FI2" s="89"/>
+      <c r="FJ2" s="89"/>
+      <c r="FK2" s="89"/>
+      <c r="FL2" s="89"/>
+      <c r="FM2" s="89"/>
+      <c r="FN2" s="89"/>
+      <c r="FO2" s="89"/>
+      <c r="FP2" s="90"/>
+      <c r="FQ2" s="100" t="s">
         <v>20</v>
       </c>
-      <c r="FR2" s="71"/>
-      <c r="FS2" s="71"/>
-      <c r="FT2" s="71"/>
-      <c r="FU2" s="71"/>
-      <c r="FV2" s="71"/>
-      <c r="FW2" s="71"/>
-      <c r="FX2" s="71"/>
-      <c r="FY2" s="72"/>
-      <c r="FZ2" s="105" t="s">
+      <c r="FR2" s="77"/>
+      <c r="FS2" s="77"/>
+      <c r="FT2" s="77"/>
+      <c r="FU2" s="77"/>
+      <c r="FV2" s="77"/>
+      <c r="FW2" s="77"/>
+      <c r="FX2" s="77"/>
+      <c r="FY2" s="78"/>
+      <c r="FZ2" s="76" t="s">
         <v>21</v>
       </c>
-      <c r="GA2" s="71"/>
-      <c r="GB2" s="71"/>
-      <c r="GC2" s="71"/>
-      <c r="GD2" s="71"/>
-      <c r="GE2" s="71"/>
-      <c r="GF2" s="72"/>
-      <c r="GG2" s="78"/>
-      <c r="GH2" s="79"/>
-      <c r="GI2" s="79"/>
-      <c r="GJ2" s="80"/>
-      <c r="GK2" s="83"/>
-      <c r="GL2" s="86"/>
-      <c r="GM2" s="86"/>
-      <c r="GN2" s="86"/>
+      <c r="GA2" s="77"/>
+      <c r="GB2" s="77"/>
+      <c r="GC2" s="77"/>
+      <c r="GD2" s="77"/>
+      <c r="GE2" s="77"/>
+      <c r="GF2" s="78"/>
+      <c r="GG2" s="80"/>
+      <c r="GH2" s="81"/>
+      <c r="GI2" s="81"/>
+      <c r="GJ2" s="82"/>
+      <c r="GK2" s="84"/>
+      <c r="GL2" s="71"/>
+      <c r="GM2" s="71"/>
+      <c r="GN2" s="71"/>
     </row>
     <row r="3" spans="1:196" ht="58.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
@@ -4113,10 +4116,10 @@
       <c r="GJ3" s="41" t="s">
         <v>118</v>
       </c>
-      <c r="GK3" s="84"/>
-      <c r="GL3" s="87"/>
-      <c r="GM3" s="87"/>
-      <c r="GN3" s="87"/>
+      <c r="GK3" s="85"/>
+      <c r="GL3" s="72"/>
+      <c r="GM3" s="72"/>
+      <c r="GN3" s="72"/>
     </row>
     <row r="4" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -4579,6 +4582,21 @@
       <c r="EA6" s="59" t="s">
         <v>124</v>
       </c>
+      <c r="EB6" s="59" t="s">
+        <v>138</v>
+      </c>
+      <c r="EC6" s="59" t="s">
+        <v>206</v>
+      </c>
+      <c r="EE6" s="59" t="s">
+        <v>207</v>
+      </c>
+      <c r="EF6" s="59">
+        <v>1</v>
+      </c>
+      <c r="EG6" s="59">
+        <v>2019</v>
+      </c>
       <c r="EI6" s="59" t="s">
         <v>124</v>
       </c>
@@ -4659,6 +4677,21 @@
       <c r="EA7" s="59" t="s">
         <v>138</v>
       </c>
+      <c r="EB7" s="59" t="s">
+        <v>138</v>
+      </c>
+      <c r="EC7" s="59" t="s">
+        <v>208</v>
+      </c>
+      <c r="EE7" s="59" t="s">
+        <v>209</v>
+      </c>
+      <c r="EF7" s="59">
+        <v>2</v>
+      </c>
+      <c r="EG7" s="59">
+        <v>2025</v>
+      </c>
       <c r="EI7" s="59" t="s">
         <v>138</v>
       </c>
@@ -4761,21 +4794,12 @@
     </row>
     <row r="9" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="AR9" s="5"/>
-      <c r="EB9" s="59" t="s">
-        <v>138</v>
-      </c>
-      <c r="EC9" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="EE9" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="EF9" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="EG9" s="59" t="s">
-        <v>126</v>
-      </c>
+      <c r="EB9" s="107"/>
+      <c r="EC9" s="107"/>
+      <c r="ED9" s="107"/>
+      <c r="EE9" s="107"/>
+      <c r="EF9" s="107"/>
+      <c r="EG9" s="107"/>
       <c r="EM9" s="59">
         <v>1</v>
       </c>
@@ -4866,21 +4890,12 @@
     </row>
     <row r="10" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="AR10" s="5"/>
-      <c r="EB10" s="59" t="s">
-        <v>124</v>
-      </c>
-      <c r="EC10" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="EE10" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="EF10" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="EG10" s="59" t="s">
-        <v>126</v>
-      </c>
+      <c r="EB10" s="107"/>
+      <c r="EC10" s="107"/>
+      <c r="ED10" s="107"/>
+      <c r="EE10" s="107"/>
+      <c r="EF10" s="107"/>
+      <c r="EG10" s="107"/>
       <c r="EM10" s="59" t="s">
         <v>126</v>
       </c>
@@ -4973,21 +4988,6 @@
       </c>
     </row>
     <row r="11" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="EB11" s="59" t="s">
-        <v>138</v>
-      </c>
-      <c r="EC11" s="59" t="s">
-        <v>206</v>
-      </c>
-      <c r="EE11" s="59" t="s">
-        <v>207</v>
-      </c>
-      <c r="EF11" s="59">
-        <v>1</v>
-      </c>
-      <c r="EG11" s="59">
-        <v>2019</v>
-      </c>
       <c r="EM11" s="59">
         <v>2</v>
       </c>
@@ -5026,28 +5026,17 @@
       </c>
       <c r="EY11" s="59" t="s">
         <v>126</v>
-      </c>
-    </row>
-    <row r="12" spans="1:196" ht="70.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="EB12" s="59" t="s">
-        <v>138</v>
-      </c>
-      <c r="EC12" s="59" t="s">
-        <v>208</v>
-      </c>
-      <c r="EE12" s="59" t="s">
-        <v>209</v>
-      </c>
-      <c r="EF12" s="59">
-        <v>2</v>
-      </c>
-      <c r="EG12" s="59">
-        <v>2025</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A3:GN5" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="22">
+    <mergeCell ref="EB2:EL2"/>
+    <mergeCell ref="A1:M2"/>
+    <mergeCell ref="V2:AC2"/>
+    <mergeCell ref="GG1:GJ2"/>
+    <mergeCell ref="N2:U2"/>
+    <mergeCell ref="AD1:AK2"/>
     <mergeCell ref="GN1:GN3"/>
     <mergeCell ref="N1:AC1"/>
     <mergeCell ref="FZ2:GF2"/>
@@ -5064,12 +5053,6 @@
     <mergeCell ref="CE1:DK2"/>
     <mergeCell ref="EM2:EY2"/>
     <mergeCell ref="FQ2:FY2"/>
-    <mergeCell ref="EB2:EL2"/>
-    <mergeCell ref="A1:M2"/>
-    <mergeCell ref="V2:AC2"/>
-    <mergeCell ref="GG1:GJ2"/>
-    <mergeCell ref="N2:U2"/>
-    <mergeCell ref="AD1:AK2"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:B1 A3:A6 A7:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="142"/>

</xml_diff>